<commit_message>
Curate 50 medium-focused MTSamples reports
Keep 48 medium reports and document two Allergy/Immunology length exceptions. Preserve the historical EDA and record reproducible selection checks, source IDs, and hashes.
</commit_message>
<xml_diff>
--- a/data/curated_baseline/mtsamples_curated_50.xlsx
+++ b/data/curated_baseline/mtsamples_curated_50.xlsx
@@ -523,7 +523,7 @@
     </row>
     <row r="2" ht="110" customHeight="1">
       <c r="A2" s="2" t="n">
-        <v>4995</v>
+        <v>0</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -532,26 +532,26 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Kawasaki Disease - Discharge Summary </t>
+          <t xml:space="preserve"> Allergic Rhinitis </t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> This is a 14-month-old baby boy Caucasian who came in with presumptive diagnosis of Kawasaki with fever for more than 5 days and conjunctivitis, mild arthritis with edema, rash, resolving and with elevated neutrophils and thrombocytosis, elevated CRP and ESR. </t>
+          <t xml:space="preserve"> A 23-year-old white female presents with complaint of allergies.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>ADMITTING DIAGNOSIS: , Kawasaki disease.,DISCHARGE DIAGNOSIS:,  Kawasaki disease, resolving.,HOSPITAL COURSE:,  This is a 14-month-old baby boy Caucasian who came in with presumptive diagnosis of Kawasaki with fever for more than 5 days and conjunctivitis, mild arthritis with edema, rash, resolving and with elevated neutrophils and thrombocytosis, elevated CRP and ESR.  When he was sent to the hospital, he had a fever of 102.  Subsequently, the patient was evaluated and based on the criteria, he was started on high dose of aspirin and IVIG.  Echocardiogram was also done, which was negative.  IVIG was done x1, and between 12 hours of IVIG, he spiked fever again; it was repeated twice, and then after second IVIG, he did not spike any more fever.  Today, his fever and his rash have completely resolved.  He does not have any conjunctivitis and no redness of mucous membranes.  He is more calm and quite and taking good p.o.; so with a very close followup and a cardiac followup, he will be sent home.,DISCHARGE ACTIVITIES:,  Ad-lib.,DISCHARGE DIET: , PO ad-lib.,DISCHARGE MEDICATIONS: , Aspirin high dose 340 mg q.6h. for 1 day and then aspirin low dose 40 mg q.d. for 14 days and then Prevacid also to prevent his GI from aspirin 15 mg p.o. once a day.  He will be followed by his primary doctor in 2 to 3 days.  Cardiology for echo followup in 4 to 6 weeks and instructed not to give any vaccine in less than 11 months because of IVIG, all the live virus vaccine, and if he gets any rashes, any fevers, should go to primary care doctor as soon as possible.</t>
+          <t>SUBJECTIVE:,  This 23-year-old white female presents with complaint of allergies.  She used to have allergies when she lived in Seattle but she thinks they are worse here.  In the past, she has tried Claritin, and Zyrtec.  Both worked for short time but then seemed to lose effectiveness.  She has used Allegra also.  She used that last summer and she began using it again two weeks ago.  It does not appear to be working very well.  She has used over-the-counter sprays but no prescription nasal sprays.  She does have asthma but doest not require daily medication for this and does not think it is flaring up.,MEDICATIONS: , Her only medication currently is Ortho Tri-Cyclen and the Allegra.,ALLERGIES: , She has no known medicine allergies.,OBJECTIVE:,Vitals:  Weight was 130 pounds and blood pressure 124/78.,HEENT:  Her throat was mildly erythematous without exudate.  Nasal mucosa was erythematous and swollen.  Only clear drainage was seen.  TMs were clear.,Neck:  Supple without adenopathy.,Lungs:  Clear.,ASSESSMENT:,  Allergic rhinitis.,PLAN:,1.  She will try Zyrtec instead of Allegra again.  Another option will be to use loratadine.  She does not think she has prescription coverage so that might be cheaper.,2.  Samples of Nasonex two sprays in each nostril given for three weeks.  A prescription was written as well.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>allergy / immunology, mucous membranes, conjunctivitis, ad lib, kawasaki disease, vaccine, fever, aspirin</t>
+          <t>allergy / immunology, allergic rhinitis, allergies, asthma, nasal sprays, rhinitis, nasal, erythematous, allegra, sprays, allergic,</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>270</v>
+        <v>204</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -560,28 +560,28 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Allergy / Immunology; short; discharge summary; diagnoses + symptoms + medications</t>
+          <t>Allergy / Immunology; short (documented Allergy length exception); SOAP-style; lower text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>4995</v>
+        <v>0</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>discharge summary</t>
+          <t>SOAP-style</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0.383509918845807</v>
+        <v>0.3761834986474301</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; imaging; follow-up</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; treatment plans; assessment/plan</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Allergy / Immunology; medium; other narrative/sectioned; diagnoses + symptoms + medications</t>
+          <t>Allergy / Immunology; medium; other narrative/sectioned; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J3" s="2" t="n">
@@ -647,7 +647,7 @@
     </row>
     <row r="4" ht="110" customHeight="1">
       <c r="A4" s="2" t="n">
-        <v>4996</v>
+        <v>4998</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -656,22 +656,22 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Followup on Asthma </t>
+          <t xml:space="preserve"> Allergy Evaluation Consult </t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> A female for a complete physical and follow up on asthma with allergic rhinitis.</t>
+          <t xml:space="preserve"> Acute allergic reaction, etiology uncertain, however, suspicious for Keflex.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>SUBJECTIVE: , This is a 42-year-old white female who comes in today for a complete physical and follow up on asthma.  She says her asthma has been worse over the last three months.  She has been using her inhaler daily.  Her allergies seem to be a little bit worse as well.  Her husband has been hauling corn and this seems to aggravate things.  She has not been taking Allegra daily but when she does take it, it seems to help somewhat.  She has not been taking her Flonase which has helped her in the past.  She also notes that in the past she was on Advair but she got some vaginal irritation with that.,She had been noticing increasing symptoms of irritability and PMS around her menstrual cycle.  She has been more impatient around that time.  Says otherwise her mood is normal during the rest of the month.  It usually is worse the week before her cycle and improves the day her menstrual cycle starts.  Menses have been regular but somewhat shorter than in the past.  Occasionally she will get some spotting after her cycles.  She denies any hot flashes or night sweats with this.  In reviewing the chart it is noted that she did have 3+ blood with what appeared to be a urinary tract infection previously.  Her urine has not been rechecked.  She recently had lab work and cholesterol drawn for a life insurance application and is going to send me those results when available.,REVIEW OF SYSTEMS: , As above.  No fevers, no headaches, no shortness of breath currently.  No chest pain or tightness.  No abdominal pain, no heartburn, no constipation, diarrhea or dysuria.  Occasional stress incontinence.  No muscle or joint pain.  No concerns about her skin.  No polyphagia, polydipsia or polyuria.,PAST MEDICAL HISTORY: , Significant for asthma, allergic rhinitis and cervical dysplasia.,SOCIAL HISTORY: , She is married.  She is a nonsmoker.,MEDICATIONS: , Proventil and Allegra.,ALLERGIES: , Sulfa.,OBJECTIVE:,Vital signs:  Her weight is 151 pounds.  Blood pressure is 110/60.  Pulse is 72.  Temperature is 97.1 degrees.  Respirations are 20.,General:  This is a well-developed, well-nourished 42-year-old white female, alert and oriented in no acute distress.  Affect is appropriate and is pleasant.,HEENT:  Normocephalic, atraumatic.  Tympanic membranes are clear.  Conjunctivae are clear.  Pupils are equal, round and reactive to light.  Nares without turbinate edema.  Oropharynx is nonerythematous.,Neck:  Supple without lymphadenopathy, thyromegaly, carotid bruit or JVD.,Chest:  Clear to auscultation bilaterally.,Cardiovascular:  Regular rate and rhythm without murmur.,Abdomen:  Soft, nontender, nondistended.  Normoactive bowel sounds.  No masses or organomegaly to palpation.,Extremities:  Without cyanosis or edema.,Skin:  Without abnormalities.,Breasts:  Normal symmetrical breasts without dimpling or retraction.  No nipple discharge.  No masses or lesions to palpation.  No axillary masses or lymphadenopathy.,Genitourinary:  Normal external genitalia.  The walls of the vaginal vault are visualized with normal pink rugae with no lesions noted.  Cervix is visualized without lesion.  She has a moderate amount of thick white/yellow vaginal discharge in the vaginal vault.  No cervical motion tenderness.  No adnexal tenderness or fullness.,ASSESSMENT/PLAN:,1.  Asthma.  Seems to be worse than in the past.  She is just using her Proventil inhaler but is using it daily.  We will add Flovent 44 mcg two puffs p.o. b.i.d.  May need to increase the dose.  She did get some vaginal irritation with Advair in the past but she is willing to retry that if it is necessary.  May also need to consider Singulair.  She is to call me if she is not improving.  If her shortness of breath worsens she is to call me or go into the emergency department.  We will plan on following up for reevaluation in one month.,2.  Allergic rhinitis.  We will plan on restarting Allegra and Flonase daily for the time being.,3.  Premenstrual dysphoric disorder.  She may have some perimenopausal symptoms.  We will start her on fluoxetine 20 mg one tablet p.o. q.d.,4.  Hematuria.  Likely this is secondary to urinary tract infection but we will repeat a UA to document clearing.  She does have some frequent dysuria but is not having it currently.,5.  Cervical dysplasia.  Pap smear is taken.  We will notify the patient of results.  If normal we will go back to yearly Pap smear.  She is scheduled for screening mammogram and instructed on monthly self-breast exam techniques.  Recommend she get 1200 mg of calcium and 400 U of vitamin D a day.</t>
+          <t>HISTORY: , A 34-year-old male presents today self-referred at the recommendation of Emergency Room physicians and his nephrologist to pursue further allergy evaluation and treatment.  Please refer to chart for history and physical, as well as the medical records regarding his allergic reaction treatment at ABC Medical Center for further details and studies.  In summary, the patient had an acute event of perioral swelling, etiology uncertain, occurring on 05/03/2008 requiring transfer from ABC Medical Center to XYZ Medical Center due to a history of renal failure requiring dialysis and he was admitted and treated and felt that his allergy reaction was to Keflex, which was being used to treat a skin cellulitis dialysis shunt infection.  In summary, the patient states he has some problems with tolerating grass allergies, environmental and inhalant allergies occasionally, but has never had anaphylactic or angioedema reactions.  He currently is not taking any medication for allergies.  He is taking atenolol for blood pressure control.  No further problems have been noted upon his discharge and treatment, which included corticosteroid therapy and antihistamine therapy and monitoring.,PAST MEDICAL HISTORY:,  History of urticaria, history of renal failure with hypertension possible source of renal failure, history of dialysis times 2 years and a history of hypertension.,PAST SURGICAL HISTORY:,  PermCath insertion times 3 and peritoneal dialysis.,FAMILY HISTORY: , Strong for heart disease, carcinoma, and a history of food allergies, and there is also a history of hypertension.,CURRENT MEDICATIONS: , Atenolol, sodium bicarbonate, Lovaza, and Dialyvite.,ALLERGIES: , Heparin causing thrombocytopenia.,SOCIAL HISTORY: , Denies tobacco or alcohol use.,PHYSICAL EXAMINATION:  ,VITAL SIGNS:  Age 34, blood pressure 128/78, pulse 70, temperature is 97.8, weight is 207 pounds, and height is 5 feet 7 inches.,GENERAL:  The patient is healthy appearing; alert and oriented to person, place and time; responds appropriately; in no acute distress.,HEAD:  Normocephalic.  No masses or lesions noted.,FACE:  No facial tenderness or asymmetry noted.,EYES:  Pupils are equal, round and reactive to light and accommodation bilaterally.  Extraocular movements are intact bilaterally.,EARS:  The tympanic membranes are intact bilaterally with a good light reflex.  The external auditory canals are clear with no lesions or masses noted.  Weber and Rinne tests are within normal limits.,NOSE:  The nasal cavities are patent bilaterally.  The nasal septum is midline.  There are no nasal discharges.  No masses or lesions noted.,THROAT:  The oral mucosa appears healthy.  Dental hygiene is maintained well.  No oropharyngeal masses or lesions noted.  No postnasal drip noted.,NECK:  The neck is supple with no adenopathy or masses palpated.  The trachea is midline.  The thyroid gland is of normal size with no nodules.,NEUROLOGIC:  Facial nerve is intact bilaterally.  The remaining cranial nerves are intact without focal deficit.,LUNGS:  Clear to auscultation bilaterally.  No wheeze noted.,HEART:  Regular rate and rhythm.  No murmur noted.,IMPRESSION:  ,1.  Acute allergic reaction, etiology uncertain, however, suspicious for Keflex.,2.  Renal failure requiring dialysis.,3.  Hypertension.,RECOMMENDATIONS:  ,RAST allergy testing for both food and environmental allergies was performed, and we will get the results back to the patient with further recommendations to follow.  If there is any specific food or inhalant allergen that is found to be quite high on the sensitivity scale, we would probably recommend the patient to avoid the offending agent to hold off on any further reactions.  At this point, I would recommend the patient stopping any further use of cephalosporin antibiotics, which may be the cause of his allergic reaction, and I would consider this an allergy.  Being on atenolol, the patient has a more difficult time treating acute anaphylaxis, but I do think this is medically necessary at this time and hopefully we can find specific causes for his allergic reactions.  An EpiPen was also prescribed in the event of acute angioedema or allergic reaction or sensation of impending allergic reaction and he is aware he needs to proceed directly to the emergency room for further evaluation and treatment recommendations after administration of an EpiPen.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="n">
-        <v>708</v>
+        <v>638</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -680,15 +680,15 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Allergy / Immunology; long; follow-up/progress; diagnoses + symptoms + medications</t>
+          <t>Allergy / Immunology; long (documented Allergy length exception); consultation; higher text complexity; diagnoses + medications + allergies</t>
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>4996</v>
+        <v>4998</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>follow-up/progress</t>
+          <t>consultation</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -697,17 +697,17 @@
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>0.7729936880072137</v>
+        <v>0.7756424706943192</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; vital signs; past history; treatment plans; follow-up; assessment/plan</t>
+          <t>diagnoses; medications; allergies; vital signs; past history; treatment plans; surgery</t>
         </is>
       </c>
     </row>
     <row r="5" ht="110" customHeight="1">
       <c r="A5" s="2" t="n">
-        <v>4874</v>
+        <v>4626</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -716,43 +716,43 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Chest Pain - Office Note </t>
+          <t xml:space="preserve"> Transesophageal Echocardiography Probe </t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Patient with a family history of premature coronary artery disease came in for evaluation of recurrent chest pain</t>
+          <t xml:space="preserve"> Insertion of transesophageal echocardiography probe and unsuccessful insertion of arterial venous lines.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>DISCHARGE DIAGNOSES:,1.  Chest pain.  The patient ruled out for myocardial infarction on serial troponins.  Result of nuclear stress test is pending.,2.  Elevated liver enzymes, etiology uncertain for an outpatient followup.,3.  Acid reflux disease.,TEST DONE: , Nuclear stress test, results of which are pending.,HOSPITAL COURSE: , This 32-year-old with family history of premature coronary artery disease came in for evaluation of recurrent chest pain, O2 saturation at 94% with both atypical and typical features of ischemia.  The patient ruled out for myocardial infarction with serial troponins.  Nuclear stress test has been done, results of which are pending.  The patient is stable to be discharged pending the results of nuclear stress test and cardiologist's recommendations.  He will follow up with cardiologist, Dr. X, in two weeks and with his primary physician in two to four weeks.  Discharge medications will depend on results of nuclear stress test.</t>
+          <t>INDICATIONS FOR PROCEDURE:,  Impending open heart surgery for closure of ventricular septal defect in a 4-month-old girl.,Procedures were done under general anesthesia.  The patient was already in the operating room under general anesthesia.  Antibiotic prophylaxis with cefazolin and gentamicin was already given prior to beginning the procedures.,PROCEDURE #1:,  Insertion of transesophageal echocardiography probe.,DESCRIPTION OF PROCEDURE #1: , The probe was well lubricated and with digital manipulation, was passed into the esophagus without resistance.  The probe was placed so that the larger diameter was in the anterior-posterior position during insertion.  The probe was used by the pediatric cardiologist for preoperative and postoperative diagnostic echocardiography.  At the end, it was removed without trauma and there was no blood tingeing.  It is to be noted that approximately 30 minutes after removing the cannula, I inserted a 14-French suction tube to empty the stomach and there were a few mL of blood secretions that were suctioned.  There was no overt bleeding.,PROCEDURE #2: , Attempted and unsuccessful insertion of arterial venous lines.,DESCRIPTION OF PROCEDURE #2:,  Both groins were prepped and draped.  The patient was placed at 10 degrees head-up position.  A Cook 4-French double-lumen 8-cm catheter kit was opened.  Using the 21-gauge needle that comes with the kit, several attempts were made to insert central venous and then an arterial line in the left groin.  There were several successful punctures of these vessels, but I was unable to advance Seldinger wire.  After removal of the needles, the area was compressed digitally for approximately 5 minutes.  There was a small hematoma that was not growing.  Initially, the left leg was mildly mottled with prolonged capillary refill of approximately 3 seconds.  Using 1% lidocaine, I infiltrated the vessels of the groin both medial and lateral to the vascular sheath.  Further observation, the capillary refill and circulation of the left leg became more than adequate.  The O2 saturation monitor that was on the left toe functioned well throughout the procedures, from the beginning to the end.  At the end of the procedure, the circulation of the leg was intact.,</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>cardiovascular / pulmonary, chest pain, serial troponins, premature coronary artery disease, coronary artery disease, nuclear stress test, stress test</t>
+          <t>cardiovascular / pulmonary, impending open heart surgery, ventricular septal defect, antibiotic prophylaxis, cefazolin, transesophageal echocardiography probe, arterial venous lines, groin, transesophageal echocardiography, echocardiography probe, insertion, transesophageal, arterial, venous, groins, echocardiography, probe</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>144</v>
+        <v>341</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Cardiovascular / Pulmonary; short; follow-up/progress; diagnoses + symptoms + medications</t>
+          <t>Cardiovascular / Pulmonary; medium; other narrative/sectioned; lower text complexity; diagnoses + procedures + imaging</t>
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>4874</v>
+        <v>4626</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>follow-up/progress</t>
+          <t>other narrative/sectioned</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -761,17 +761,17 @@
         </is>
       </c>
       <c r="M5" s="2" t="n">
-        <v>0.2741771866546438</v>
+        <v>0.3669972948602344</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; vital signs; past history; treatment plans; follow-up</t>
+          <t>diagnoses; procedures; imaging; surgery</t>
         </is>
       </c>
     </row>
     <row r="6" ht="110" customHeight="1">
       <c r="A6" s="2" t="n">
-        <v>4690</v>
+        <v>4720</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -780,39 +780,35 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Pulmonary Consultation - 2 </t>
+          <t xml:space="preserve"> Non-Q-wave Myocardial Infarction </t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Patient with complaints of significant coughing and wheezing.</t>
+          <t xml:space="preserve"> A patient with non-Q-wave myocardial infarction.  No definite chest pains.  The patient is breathing okay.  The patient denies orthopnea or PND.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>PAST MEDICAL HISTORY:,  Unremarkable, except for diabetes and atherosclerotic vascular disease.,ALLERGIES:,  PENICILLIN.,CURRENT MEDICATIONS:,  Include Glucovance, Seroquel, Flomax, and Nexium.,PAST SURGICAL HISTORY: , Appendectomy and exploratory laparotomy.,FAMILY HISTORY: , Noncontributory.,SOCIAL HISTORY:  ,The patient is a non-smoker.  No alcohol abuse.  The patient is married with no children.,REVIEW OF SYSTEMS:,  Significant for an old CVA.,PHYSICAL EXAMINATION:,  The patient is an elderly male alert and cooperative.  Blood pressure 96/60 mmHg.  Respirations were 20.  Pulse 94.  Afebrile.  O2 was 94% on room air.  HEENT:  Normocephalic and atraumatic.  Pupils are reactive.  Oral mucosa is grossly normal.  Neck is supple.  Lungs:  Decreased breath sounds.  Disturbed breath sounds with poor exchange.  Heart:  Regular rhythm.  Abdomen:  Soft and nontender.  No organomegaly or masses.  Extremities:  No cyanosis, clubbing, or edema.,LABORATORY DATA: , Oropharyngeal evaluation done on 11/02/2006 revealed mild oropharyngeal dysphagia with no evidence of laryngeal penetration or aspiration with food or liquid.  Slight reduction in tongue retraction resulting in mild residual remaining in the palatal sinuses, which clear with liquid swallow and double-saliva swallow.,ASSESSMENT:,1.  Cough probably multifactorial combination of gastroesophageal reflux and recurrent aspiration.,2.  Old CVA with left hemiparesis.,3.  Oropharyngeal dysphagia.,4.  Diabetes.,PLAN:,  At the present time, the patient is recommended to continue on a regular diet, continue speech pathology evaluation as well as perform double-swallow during meals with bolus sensation.  He may use Italian lemon ice during meals to help clear sinuses as well.  The patient will follow up with you.  If you need any further assistance, do not hesitate to call me.</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cardiovascular / pulmonary, pulmonary evaluation, cough, wheezing, congestion, coughing and wheezing, breath sounds, oropharyngeal dysphagia, pulmonary, breath, sounds, dysphagia, aspiration, sinuses, oropharyngeal, coughing, swallowing, </t>
-        </is>
-      </c>
+          <t>REASON FOR CONSULT: , A patient with non-Q-wave myocardial infarction.,HISTORY OF PRESENT ILLNESS: , The patient is a pleasant 52-year-old gentleman with a history of diabetes mellitus, hypertension, and renal failure, on dialysis, who presented with emesis, dizziness, and nausea for the last few weeks.  The patient reports having worsening emesis and emesis a few times.  No definite chest pains.  The patient is breathing okay.  The patient denies orthopnea or PND.,PAST MEDICAL HISTORY:,1.  Diabetes mellitus.,2.  Hypertension.,3.  Renal failure, on dialysis.,MEDICATIONS:,  Aspirin, Coreg, doxazosin, insulin, metoclopramide, simvastatin, and Starlix.,ALLERGIES:  ,NO KNOWN DRUG ALLERGIES.,SOCIAL HISTORY: , The patient denies tobacco, alcohol or drug use.,FAMILY HISTORY: , Negative for early atherosclerotic heart disease.,REVIEW OF SYSTEMS: , General:  The patient denies fever or chills.  Pulmonary:  The patient denies hemoptysis.  Cardiovascular:  Refer to HPI.  GI:  The patient denies hematemesis or melena.  The rest of systems review is negative.,PHYSICAL EXAMINATION:,VITAL SIGNS:  Pulse 71, blood pressure 120/70, and respiratory rate 18.,GENERAL:  A well-nourished, well-developed male in no acute distress.,HEENT:  Normocephalic, atraumatic.  Pupils seem to be equal, round, and reactive.  Extraocular muscles are full, but the patient has left eye ptosis.,NECK:  Supple without JVD or lymphadenopathy.,LUNGS:  Clear to auscultation bilaterally.,CARDIOVASCULAR:  PMI is displaced 0.5 cm lateral to the midclavicular line.  Regular rate and rhythm, S1, S2.  No definite S3, 2/6 holosystolic murmur at the apex radiating to the axilla.,ABDOMEN:  Positive bowel sounds, nondistended and nontender.  No hepatosplenomegaly.,EXTREMITIES:  Trace pedal edema.,EKG shows atrial fibrillation with rapid ventricular response at 164 with old anteroseptal myocardial infarction and old inferior wall myocardial infarction.  Subsequent EKG in sinus rhythm shows sinus rhythm with old inferior wall myocardial infarction and probable anteroseptal myocardial infarction with Q-waves in V1, V2, and up to V3.,LABORATORY EXAM: , WBC 28,800, hemoglobin 13.6, hematocrit 40, and platelets 266,000.  PT 11.3, INR 1.1, and PTT 24.1.  Sodium 126, potassium 4.3, chloride 86, CO2 26, glucose 371, BUN 80, and creatinine 8.4.  CK was 261, then 315, and then 529 with CK-MB of 8.06, then 8.69, and then 24.6.  Troponin was 0.051, then 0.46, and then 19.8 this morning.,IMPRESSION:,1.  Paroxysmal atrial fibrillation.  The heart rate was slowed down with IV Cardizem, the patient converted to sinus rhythm.  The patient is currently in sinus rhythm.,2.  Emesis.  The etiology is unclear.  The patient reports that the emesis is better.  The patient is just having some nausea.,3.  Non-Q-wave myocardial infarction.  EKG shows atrial fibrillation with old anteroseptal myocardial infarction and old inferior wall myocardial infarction.,4.  Diabetes mellitus.,5.  Renal failure.,6.  Hypertension.,7.  Hypercholesterolemia.,PLAN:,1.  We will start amiodarone to keep from going back into atrial fibrillation.,2.  Echocardiogram.,3.  Aspirin and IV heparin.,4.  Serial CK-MB and troponin.,5.  Cardiac catheterization, possible percutaneous coronary intervention.  The risks, benefits, and alternatives were explained to the patient through a translator.  The patient understands and wishes to proceed.,6.  IV Integrilin.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="n">
-        <v>244</v>
+        <v>458</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Cardiovascular / Pulmonary; short; consultation; diagnoses + symptoms + medications</t>
+          <t>Cardiovascular / Pulmonary; medium; consultation; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>4690</v>
+        <v>4720</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -825,11 +821,11 @@
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>0.6734107303877368</v>
+        <v>0.9004170423805229</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; past history; treatment plans; follow-up; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; assessment/plan</t>
         </is>
       </c>
     </row>
@@ -872,7 +868,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Cardiovascular / Pulmonary; medium; procedure/operative; diagnoses + medications + laboratory values</t>
+          <t>Cardiovascular / Pulmonary; medium; procedure/operative; middle text complexity; diagnoses + medications + laboratory values</t>
         </is>
       </c>
       <c r="J7" s="2" t="n">
@@ -899,7 +895,7 @@
     </row>
     <row r="8" ht="110" customHeight="1">
       <c r="A8" s="2" t="n">
-        <v>4965</v>
+        <v>4976</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
@@ -908,35 +904,35 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Atrial Fibrillation - Consult </t>
+          <t xml:space="preserve"> Abnormal Echocardiogram </t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> A 74-year-old woman for Cardiology consultation regarding atrial fibrillation and anticoagulation after a fall.  The patient denies any chest pain nor clear shortness of breath.</t>
+          <t xml:space="preserve"> Abnormal echocardiogram findings and followup.  Shortness of breath, congestive heart failure, and valvular insufficiency.   The patient complains of shortness of breath, which is worsening.  The patient underwent an echocardiogram, which shows severe mitral regurgitation and also large pleural effusion.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS:,  I was kindly asked to see Ms. ABC who is a 74-year-old woman for cardiology consultation regarding atrial fibrillation and anticoagulation after a fall.,The patient is somnolent at this time, but does arouse, but is unable to provide much history.  By review of the chart, it appears that she fell, which is what she states when she got up out of a rocking chair and could not get herself off the floor.  She states that 1-1/2 hours later she was able to get herself off the floor.,The patient denies any chest pain nor clear shortness of breath.,PAST MEDICAL HISTORY: , Includes, end-stage renal disease from hypertension.  She follows up with Dr. X in her office and has been known to have a small-to-moderate sized pericardial effusion since 11/07 that has apparently been followed and it appears that the patient was not interested in having diagnostic pericardiocentesis done.  She had an echocardiogram today (please see also that report), which shows stable and small-to-moderate sized pericardial effusion without tamponade, normal left ventricular ejection fraction at 55% with mild concentric left ventricular hypertrophy, mildly dilated right ventricular size, normal right ventricular ejection fraction, moderate mitral regurgitation and severe tricuspid regurgitation with severe pulmonary hypertension, estimated PA systolic pressure of 71 mmHg when compared to the prior echocardiogram done 08/29/07, previously the mitral regurgitation was mild and previously the PA systolic pressure was estimated at 90 mmHg.  Other findings were not significantly changed including pericardial effusion description.  She has a history of longstanding hypertension.  She has been on hemodialysis since 1997 for renal failure, history of mini-strokes documented several years ago, history of seizure disorder, she has a history of right upper extremity edema and right breast enlargement from right subclavian vein occlusion.  She has a history of hypertension, depression, hyperlipidemia, on Sensipar for tertiary hyperparathyroidism.,PAST SURGICAL HISTORY: , Includes, cholecystectomy, post fistula in the left arm, which has failed, and right arm, which is being used including number of operative procedures to the fistula.  She follows up with Dr. Y regarding neurovascular surgery.,MEDICATIONS: , On admission:,1.  Norvasc 10 mg once a day.,2.  Aspirin 81 mg once a day.,3.  Colace 200 mg two at bedtime.,4.  Labetalol 100 mg p.o. b.i.d.,5.  Nephro-Vite one tablet p.o. q.a.m.,6.  Dilantin 100 mg p.o. t.i.d.,7.  Renagel 1600 mg p.o. t.i.d.,8.  Sensipar 120 mg p.o. every day.,9.  Sertraline 100 mg p.o. nightly.,10.  Zocor 20 mg p.o. nightly.,ALLERGIES: , TO MEDICATIONS PER CHART ARE NONE.,FAMILY HISTORY:  ,Unable to obtain as the patient becomes quite sleepy when I am talking.,SOCIAL HISTORY:  ,Unable to obtain as the patient becomes quite sleepy when I am talking.,REVIEW OF SYSTEMS: , Unable to obtain as the patient becomes quite sleepy when I am talking.,PHYSICAL EXAM:  ,Temperature 99.2, blood pressure ranges from 88/41 to 108/60, pulse 70, respiratory rate, 20, O2 saturation 98%.  Height is 5 feet 1 inch, weight 147 pounds.  On general exam, she is a pleasant elderly woman who does arouse to voice, but then becomes quite sleepy and apparently that is an improvement from when she was admitted.  HEENT shows the cranium is normocephalic and atraumatic.  She has moist mucosal membranes.  Neck veins are difficult to assess, but do not appear clinically distended.  No carotid bruits.  Lungs are clear to auscultation anteriorly.  No wheezes.  Cardiac exam:  S1, S2 regular rate, 3/6 holosystolic murmur heard with radiation from the left apex towards the left axilla.  No rub, no gallop.  PMI is nondisplaced.  Abdomen:  Soft, nondistended.  CVA is benign.  Extremities with no significant edema.  Pulses appear grossly intact.  She has evidence of right upper extremity edema, which is apparently chronic.,DIAGNOSTIC DATA/LAB DATA: , EKGs are reviewed including from 07/07/09 at 08:31 a.m., which shows atrial fibrillation with left anterior fascicular block, poor R-wave progression when compared to one done on 07/06/09 at 18:25, there is really no significant change.  The atrial fibrillation appears present since at least on EKG done on 11/02/07 and this EKG is not significantly changed from the most recent one.  Echocardiogram results as above.  Chest x-ray shows mild pulmonary vascular congestion.  BNP shows 3788.  Sodium 136, potassium 4.5, chloride 94, bicarbonate 23, BUN 49, creatinine 5.90.  Troponin was 0.40 followed by 0.34.  INR 1.03 on 05/18/07.  White blood cell count 9.4, hematocrit 42, platelet count 139.,IMPRESSION: , Ms. ABC is a 74-year-old woman admitted to the hospital with a fall and she has a history of vascular dementia, so her history is somewhat unreliable it seems and she is somnolent at that time.  She does have chronic atrial fibrillation again documented at least present since 2007 and I found an EKG report by Dr. X, which shows atrial fibrillation on 08/29/07 per her report.  One of the questions we were asked was whether the patient would be a candidate for Coumadin.  Clearly given her history of small mini-strokes, I think Coumadin would be appropriate given this chronic atrial fibrillation, but the main issue is the fall risk.  If not felt to be significant fall risk then I would strongly recommend Coumadin as the patient herself states that she has only fallen twice in the past year.  I would defer that decision to Dr. Z and Dr. XY who know the patient well and it may be that physical therapy consult is appropriate to help adjudicate.,RECOMMENDATIONS:,1.  Fall assessment as per Dr. Z and Dr. XY with possible PT consult if felt appropriate and if the patient is not felt to be at significant fall risk, would put her on Coumadin.  Given her history of small strokes as documented in the chart and her chronic atrial fibrillation, she does have reasonable heart rate control on current labetalol.,2.  The patient has elevated BNP and I suspect that is due to her severe pulmonary hypertension and renal failure and in the light of normal LV function, I would not make any further evaluation of that other than aggressive diuresis.,3.  Regarding this minimal troponin elevation, I do not feel this is a diagnosis especially in the setting of pulmonary hypertension and her small-to-moderate sized stable pericardial effusion again that has been longstanding since 2007 from what I can tell and there is no evidence of tamponade.  I would defer to her usual cardiologist Dr. X whether an outpatient stress evaluation is appropriate for risk stratification.  I did find that the patient had a prior cardiac stress test in 08/07 where they felt that there was some subtle reversibility of the anterior wall, but it was felt that it may be artifact rather than true ischemia with normal LV function seen on that study as well.,4.  Continue Norvasc for history of hypertension as well as labetalol.,5.  The patient is felt to be a significant fall risk and will at least continue her aspirin 81 mg once a day for secondary CVA, thromboprophylaxis (albeit understanding that it is inferior to Coumadin).,6.  Continue Dilantin for history of seizures.</t>
+          <t>REASON FOR CONSULTATION:  ,Abnormal echocardiogram findings and followup.  Shortness of breath, congestive heart failure, and valvular insufficiency.,HISTORY OF PRESENT ILLNESS:  ,The patient is an 86-year-old female admitted for evaluation of abdominal pain and bloody stools.  The patient has colitis and also diverticulitis, undergoing treatment.  During the hospitalization, the patient complains of shortness of breath, which is worsening.  The patient underwent an echocardiogram, which shows severe mitral regurgitation and also large pleural effusion.  This consultation is for further evaluation in this regard.  As per the patient, she is an 86-year-old female, has limited activity level.  She has been having shortness of breath for many years.  She also was told that she has a heart murmur, which was not followed through on a regular basis.,CORONARY RISK FACTORS: , History of hypertension, no history of diabetes mellitus, nonsmoker, cholesterol status unclear, no prior history of coronary artery disease, and family history noncontributory.,FAMILY HISTORY:  ,Nonsignificant.,PAST SURGICAL HISTORY: , No major surgery.,MEDICATIONS: , Presently on Lasix, potassium supplementation, Levaquin, hydralazine 10 mg b.i.d., antibiotic treatments, and thyroid supplementation.,ALLERGIES:  ,AMBIEN, CARDIZEM, AND IBUPROFEN.,PERSONAL HISTORY:,  She is a nonsmoker.  Does not consume alcohol.  No history of recreational drug use.,PAST MEDICAL HISTORY:  ,Basically GI pathology with diverticulitis, colitis, hypothyroidism, arthritis, questionable hypertension, no prior history of coronary artery disease, and heart murmur.,REVIEW OF SYSTEMS,CONSTITUTIONAL:  Weakness, fatigue, and tiredness.,HEENT:  History of cataract, blurred vision, and hearing impairment.,CARDIOVASCULAR:  Shortness of breath and heart murmur.  No coronary artery disease.,RESPIRATORY:  Shortness of breath.  No pneumonia or valley fever.,GASTROINTESTINAL:  No nausea, vomiting, hematemesis, or melena.,UROLOGICAL:  No frequency or urgency.,MUSCULOSKELETAL:  Arthritis and severe muscle weakness.,SKIN:  Nonsignificant.,NEUROLOGICAL:  No TIA or CVA.  No seizure disorder.,ENDOCRINE/HEMATOLOGICAL:  As above.,PHYSICAL EXAMINATION,VITAL SIGNS:  Pulse of 84, blood pressure of 168/74, afebrile, and respiratory rate 16 per minute.,HEENT/NECK:  Head is atraumatic and normocephalic.  Neck veins flat.  No significant carotid bruits appreciated.,LUNGS:  Air entry bilaterally fair.  No obvious rales or wheezes.,HEART:  PMI displaced.  S1, S2 with systolic murmur at the precordium, grade 2/6.,ABDOMEN:  Soft and nontender.,EXTREMITIES:  Chronic skin changes.  Feeble pulses distally.  No clubbing or cyanosis.,DIAGNOSTIC DATA: , EKG:  Normal sinus rhythm.  No acute ST-T changes.,Echocardiogram report was reviewed.,LABORATORY DATA:,  H&amp;H 13 and 39.  BUN and creatinine within normal limits.  Potassium within normal limits.  BNP 9290.,IMPRESSION:,1.  The patient admitted for gastrointestinal pathology, under working treatment.,2.  History of prior heart murmur with echocardiogram findings as above.  Basically revealed normal left ventricular function with left atrial enlargement, large pleural effusion, and severe mitral regurgitation and tricuspid regurgitation.,RECOMMENDATIONS:,1.  From cardiac standpoint, conservative treatment.  Possibility of a transesophageal echocardiogram to assess valvular insufficiency adequately well discussed extensively.,2.  After extensive discussion, given her age 86, limited activity level, and no intention of undergoing any treatment in this regard from a surgical standpoint, the patient does not wish to proceed with a transesophageal echocardiogram.,3.  Based on the above findings, we will treat her medically with ACE inhibitors and diuretics and see how she fares.  She has a normal LV function.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="n">
-        <v>1143</v>
+        <v>482</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Cardiovascular / Pulmonary; long; consultation; diagnoses + symptoms + medications</t>
+          <t>Cardiovascular / Pulmonary; medium; consultation; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>4965</v>
+        <v>4976</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -949,17 +945,17 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>0.9389652840396754</v>
+        <v>0.8649684400360684</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; surgery</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; imaging; past history; treatment plans; follow-up; surgery</t>
         </is>
       </c>
     </row>
     <row r="9" ht="110" customHeight="1">
       <c r="A9" s="2" t="n">
-        <v>4447</v>
+        <v>4457</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -968,43 +964,43 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Ear Pain - Drainage </t>
+          <t xml:space="preserve"> Dietary Consultation - 1 </t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Right ear pain with drainage - otitis media and otorrhea.</t>
+          <t xml:space="preserve"> Dietary consultation for a woman with polycystic ovarian syndrome and hyperlipidemia.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>CHIEF COMPLAINT:,  Right ear pain with drainage.,HISTORY OF PRESENT ILLNESS:,  This is a 12-year-old white male here with his mother for complaints of his right ear hurting.  Mother states he has been complaining for several days.  A couple of days ago she noticed drainage from the right ear.  The patient states it has been draining for several days and it has a foul smell to it.  He has had some low-grade fever.  The patient was seen in the office about a week ago with complaints of a sore throat, headache and fever.  The patient was evaluated for Strep throat which was negative and just had been doing supportive care.  He did have a recent airplane ride a couple of weeks ago also.  There has been no cough, shortness of breath or wheezing.  No vomiting or diarrhea.,PHYSICAL EXAM:,General:  He is alert in no distress.,Vital Signs:  Temperature:  99.1 degrees.,HEENT:  Normocephalic, atraumatic.  Pupils equal, round and react to light.  The left TM is clear.  The right TM is poorly visualized secondary to purulent secretions in the right ear canal.  There is no erythema of the ear canals.  Nares is patent.  Oropharynx is clear.  The patient does wear braces.,Neck:  Supple.,Lungs:  Clear to auscultation.,Heart:  Regular.  No murmur.,ASSESSMENT:,1.  Right otitis media.,2.  Right otorrhea.,PLAN:,  Ceftin 250 mg by mouth twice a day for 10 days.  Ciprodex four drops to the right ear twice a day.  The patient is to return to the office in two weeks for followup.</t>
+          <t>SUBJECTIVE:,  This is a followup dietary consultation for polycystic ovarian syndrome and hyperlipidemia.  The patient reports that she has resumed food record keeping which she feels like it has given her greater control.  Her physical activity level has remained high.  Her struggle times are in the mid-afternoon if she has not had enough food to eat, as well as in the evening after dinner.,OBJECTIVE:, Vital Signs:  Weight is 189-1/2 pounds.  Food records were reviewed,ASSESSMENT:,  The patient has experienced a weight loss of 1-1/2 pounds in the last month.  She is commended for these efforts.  We have reviewed food records identifying that she has done a nice job keeping a calorie count for the last two or three weeks.  We discussed the value of this and how it was very difficulty to resume it, however, after she suspended the record keeping.  We also discussed its reflection that she is not getting very many fruits and vegetables on a regular basis.  We identified some ways of preventing her from feeling sluggish and having problems with low blood sugar in the middle of the afternoon by routinely planning an afternoon snack that can prevent these symptoms.  This will likely be around 2:30 or 3 p.m. for her.  We also discussed strategies for evening snacking to help put some definition and boundaries to the snacking.,PLAN:,  I recommended the patient routinely include an afternoon snack around 2:30 to 3 p.m.  It will be helpful if this snack includes some protein such as nuts or low-fat cheese.  She is also encouraged to continue with her record keeping for food choices and calorie points.  I also recommended she maintain her high level of physical activity.  Will plan to follow the patient in one month for ongoing support.  This was a 30-minute consultation.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>consult - history and phy., drainage, ear hurting, ear pain, otitis media, otorrhea, ear pain with drainage, otitis, media, ear,</t>
+          <t>consult - history and phy., dietary consultation, calorie count, calorie points, consultation, food choices, food record, hyperlipidemia, low-fat cheese, many fruits and vegetables, physical activity, polycystic ovarian syndrome, snack, dietary, polycystic, food, afternoon</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>241</v>
+        <v>295</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Consult - History and Phy.; short; other narrative/sectioned; diagnoses + symptoms + medications</t>
+          <t>Consult - History and Phy.; medium; SOAP-style; lower text complexity; diagnoses + symptoms + vital signs</t>
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>4447</v>
+        <v>4457</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>other narrative/sectioned</t>
+          <t>SOAP-style</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1013,11 +1009,11 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0.3765779981965735</v>
+        <v>0.3642921550946799</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; vital signs; past history; treatment plans; follow-up; assessment/plan</t>
+          <t>diagnoses; symptoms; vital signs; treatment plans; follow-up; assessment/plan</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1052,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Consult - History and Phy.; medium; history and physical; diagnoses + symptoms + medications</t>
+          <t>Consult - History and Phy.; medium; history and physical; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
@@ -1083,7 +1079,7 @@
     </row>
     <row r="11" ht="110" customHeight="1">
       <c r="A11" s="2" t="n">
-        <v>4427</v>
+        <v>4218</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -1092,39 +1088,39 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Erythema Nodosum - Consult </t>
+          <t xml:space="preserve"> OB/GYN - H&amp;P </t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The patient presents for a followup for history of erythema nodosum.</t>
+          <t xml:space="preserve"> Initial obstetrical examination - Normal first pregnancy.  Inadequate naternal nutrition.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>REASON FOR VISIT:,  The patient presents for a followup for history of erythema nodosum.,HISTORY OF PRESENT ILLNESS: , This is a 25-year-old woman who is attending psychology classes.  She was diagnosed with presumptive erythema nodosum in 2004 based on a biopsy consistent with erythema nodosum, but not entirely specific back in Netherlands.  At that point, she had undergone workup which was extensive for secondary diseases associated with erythema nodosum.  Part of her workup included a colonoscopy.  The findings were equivocal characterizes not clearly abnormal biopsies of the terminal ileum.,The skin biopsy, in particular, mentions some fibrosis, basal proliferation, and inflammatory cells in the subcutis.,Prior to the onset of her erythema nodosum, she had a tibia-fibula fracture several years before on the right, which was not temporarily associated with the skin lesions, which are present in both legs anyway.  Even, a jaw cosmetic surgery she underwent was long before she started developing her skin lesions.  She was seen in our clinic and by Dermatology on several occasions.  Apart from the first couple of visits when she presented stating a recurrent skin rash with a description suggestive of erythema nodosum in the lower extremities and ankle and there is discomfort pointing towards a possible inflammatory arthritis and an initial high sed rate of above 110 with an increased CRP.  In the following visits, no evident abnormality has been detected.  In the first visit, here some MTP discomfort detected.  It was thought that erythema nodosum may be present.  However, the evaluation of Dermatology did not concur and it was thought that the patient had venous stasis, which could be related to her prior fracture.  When she was initially seen here, a suspicion of IBD, sarcoid inflammatory arthropathy, and lupus was raised.  She had an equivocal rheumatoid fracture, but her CCP was negative.  She had an ANA, which was positive at 1:40 with a speckled pattern persistently, but the rest of the lupus serologies including double-stranded DNA, RNP, Smith, Ro, La were negative.  Her cardiolipin panel antibodies were negative as well.  We followed the IgM, IgG, and IgA being less than 10.  However, she did have a beta-2 glycoprotein 1 or an RVVT tested and this may be important since she has a livedo pattern.  It was thought that the onset of lupus may be the case.  It was thought that rheumatoid arthritis could not be the case since it is not associated with erythema nodosum.  For the fear of possible lymphoma, she underwent CT of the chest, abdomen, and pelvis.  It was done also in order to rule out sarcoid and the result was unremarkable.  Based on some changes in her bowel habits and evidence of B12 deficiency with a high methylmalonic and high homocystine levels along with a low normal B12 in addition to iron studies consistent with iron deficiency and an initially low MCV, the possibility of inflammatory bowel disease was employed.  The patient underwent an initially unrevealing colonoscopy and a capsule endoscopy, which was normal.  A second colonoscopy was done recently and microscopically no evidence of inflammatory bowel disease was seen.  However, eosinophil aggregations were noted in microscopy and this was told to be consistent with an allergic reaction or an emerging Crohn disease and I will need to discuss with Gastroenterology what is the significance of that.  Her possible B12 deficiency and iron deficiency were never addressed during her stay here in the United States.,In the initial appointment, she was placed on prednisone 40 mg, which was gradually titrated down this led to an exacerbation of her acne.  We decided to take her off prednisone due to adverse effects and start her on colchicine 0.6 mg daily.  While this kept things under control with the inflammatory markers being positive and no overt episodes of erythema nodosum, the patient still complains for sensitivity with less suspicious skin rash in the lower extremities and occasional ankle swelling and pain.  She was reevaluated by Dermatology for that and no evidence of erythema nodosum was felt to be present.  Out plan was to proceed with a DEXA scan, at some point check a vitamin D level, and order vitamin D and calcium over the counter for bone protection purposes.  However, the later was deferred until we have resolved the situation and find out what is the underlying cause of her disease.,Her past medical history apart from the tibia-fibular fracture and the jaw cosmetic surgery is significant for varicella and mononucleosis.,Her physical examination had shown consistently diffuse periarticular ankle edema and also venous stasis changes at least until I took over her care last August.  I have not been able to detect any erythema nodosum, however, a livedo pattern has been detected consistently.  She also has evidence of acne, which does not seem to be present at the moment.  She also was found to have a heart murmur present and we are going to proceed with an echocardiogram placed.,Her workup during the initial appointment included an ACE level, which was normal.  She also had a rather higher sed rate up to 30, but prior to that, per report, it was even higher, above 110.  Her RVVT was normal, her rheumatoid factor was negative.  Her ANA was 1:40, speckled pattern.  The double-stranded DNA was negative.  Her RNP and Smith were negative as well.  RO and LA were negative and cardiolipin antibodies were negative as well.  A urinalysis at the moment was completely normal.  A CRP was 2.3 in the initial appointment, which was high.  A CCP was negative.  Her CBC had shown microcytosis and hypochromia with a hematocrit of 37.7.  This improved later without any evidence of hypochromia, microcytosis or anemia with a hematocrit of 40.3.,The patient returns here today, as I mentioned, complaining of milder bouts of skin rash, which she calls erythema nodosum, which is accompanied by arthralgias, especially in the ankles.  I am mentioning here that photosensitivity rash was mentioned in the past.  She tells me that she had it twice back in Europe after skiing where her whole face was swollen.  Her acne has been very stable after she was taken off prednisone and was started on colchicine 0.6 daily.  Today we discussed about the effect of colchicine on a possible pregnancy.,MEDICATIONS: , Prednisone was stopped.  Vitamin D and calcium over the counter, we need to verify that.  Colchicine 0.6 mg daily which we are going to stop, ranitidine 150 mg as needed, which she does not take frequently.,FINDINGS:,  On physical examination, she is very pleasant, alert, and oriented x 3 and not in any acute distress.  There is some evidence of faint subcutaneous lesions in both shins bilaterally, but with mild tenderness, but no evidence of classic erythema nodosum.  Stasis dermatitis changes in both lower extremities present.  Mild livedo reticularis is present as well.,There is some periarticular ankle edema as well.  Laboratory data from 04/23/07, show a normal complete metabolic profile with a creatinine of 0.7, a CBC with a white count of 7880, hematocrit of 40.3, and platelets of 228.  Her microcytosis and hypochromia has resolved.  Her serum electrophoresis does not show a monoclonal abnormality.  Her vitamin D levels were 26, which suggests some mild insufficiency and she would probably benefit by vitamin D supplementation.  This points again towards some ileum pathology.  Her ANCA B and C were negative.  Her PF3 and MPO were unremarkable.  Her endomysial antibodies were negative.  Her sed rate at this time were 19.  The highest has been 30, but prior to her appointment here was even higher.  Her ANA continues to be positive with a titer of 1:40, speckled pattern.  Her double-stranded DNA is negative.  Her serum immunofixation confirmed the absence of monoclonal abnormality.  Her urine immunofixation was not performed.  Her IgG, IgA, and IgM levels are normal.  Her IgE levels are normal as well.  A urinalysis was not performed this time.  Her CRP is 0.4.  Her tissue transglutaminase antibodies are negative.  Her ASCA is normal and anti-OmpC was not tested.  Gliadin antibodies IgA is 12, which is in the borderline to be considered equivocal, but these are nonspecific.  I am reminding here that her homocystine levels have been 15.7, slightly higher, and that her methylmalonic acid was 385, which is obviously abnormal.  Her B12 levels were 216, which is rather low possibly indicating a B12 deficiency.  Her iron studies showed a ferritin of 15, a saturation of 9%, and an iron of 30.  Her TIBC was 345 pointing towards an iron deficiency anemia.  I am reminding you that her ACE levels in the past were normal and that she has a microcytosis.  Her radiologic workup including a thoracic, abdominal, and pelvic CT did not show any suspicious adenopathy, but only small aortocaval and periaortic nodes, the largest being 8 mm in short axis, likely reactive.  Her pelvic ultrasound showed normal uterus adnexa.  Her bladder was normal as well.  Subcentimeter inguinal nodes were found.  There was no large lytic or sclerotic lesion noted.  Her recent endoscopy was unremarkable, but the microscopy showed some eosinophil aggregation, which may be pointing towards allergy or an evolving Crohn disease.  Her capsule endoscopy was limited secondary to rapid transit.  There was only a tiny mucosal red spot in the proximal jejunum without active bleeding, 2 possible erosions were seen in the distal jejunum and proximal ileum.  However, no significant inflammation or bleeding was seen and this could be small bowel crisis.  Neither evidence of bleeding or inflammation were seen as well.  Specifically, the terminal ileum appeared normal.  Recent evaluation by a dermatologist did not verify the presence of erythema nodosum.,ASSESSMENT:,  This is a 25-year-old woman diagnosed with presumptive erythema nodosum in 2004.  She has been treated with prednisone as in the beginning she had also a wrist and ankle discomfort and high inflammatory markers.  Since I took over her care, I have not seen a clear-cut erythema nodosum being present.  No evidence of synovitis was there.  Her serologies apart from an ANA of 1:40 were negative.  She has a livedo pattern, which has been worrisome.  The issue here was a possibility of inflammatory bowel disease based on deficiency in vitamin B12 as indicated by high methylmalonic and homocystine levels and also iron deficiency.  She also has low vitamin D levels, which point towards terminal ileum pathology as well and she had a history of decreased MCV.  We never received the x-ray of her hands which she had and she never had a DEXA scan.  Lymphoma has been ruled out and we believe that inflammatory bowel disease, after repeated colonoscopies and the capsule endoscopy, has been ruled out as well.  Sarcoid is probably not the case since the patient did not have any lymphadenopathies and her ACE levels were normal.  We are going check a PPD to rule out tuberculosis.  We are going to order an RVVT and glycoprotein beta-1 levels in her workup to make sure that an antiphospholipid syndrome is not present given the livedo pattern.  An anti-intrinsic factor will be added as well.  Her primary care physician needs to workup the possible B12 and iron deficiency and also the vitamin D deficiency.  In the meanwhile, we feel that the patient should stop taking the colchicine and if she has a flare of her disease then she should present to her dermatologist and have the skin biopsy performed in order to have a clear-cut answer of what is the nature of this skin rash.  Regarding her heart murmur, we are going to proceed with an echocardiogram.  A PPD should be placed as well.  In her next appointment, we may fax a requisition for vitamin B replacement.,PROBLEMS/DIAGNOSES:,  1.  Recurrent erythema nodosum with ankle and wrist discomfort, ? arthritis.,2.  Iron deficiencies, according to iron studies.,3.  Borderline B12 with increased methylmalonic acid and homocystine.,4.  On chronic steroids; vitamin D and calcium is needed; she needs a DEXA scan.,5.  Typical ANCA, per records, were not verified here.  ANCA and ASCA were negative and the OmpC was not ordered.,6.  Acne.,7.  Recurrent arthralgia not present.  Rheumatoid factor, CCP negative, ANA 1:40 speckled.,8.  Livedo reticularis, beta 2-glycoprotein was not checked, we are going to check it today.  Needs vaccination for influenza and pneumonia.,9.  Vitamin D deficiency.  She needs replacement with ergocalciferol, but this may point towards ___________ pathology as this was not detected.,10.  Recurrent ankle discomfort which necessitates ankle x-rays.,PLANS:,  We can proceed with part of her workup here in clinic, PPD, echocardiogram, ankle x-rays, and anti-intrinsic factor antibodies.  We can start repleting her vitamin D with __________ weeks of ergocalciferol 50,000 weekly.  We can add an RVVT and glycoprotein to her workup in order to rule out any antiphospholipid syndrome.  She should be taking vitamin D and calcium after the completion of vitamin D replacement.  She should be seen by her primary care physician, have the iron and B12 deficiency worked up.  She should stop the colchicine and if the skin lesion recurs then she should be seen by her dermatologist.  Based on the physical examination, we do not suspect that the patient has the presence of any other disease associated with erythema nodosum.  We are going to add an amylase and lipase to evaluate her pancreatic function, RPR, HIV, __________ serologies.  Given the evidence of possible malabsorption it may be significant to proceed with an upper endoscopy to rule out Whipple disease or celiac disease which can sometimes be associated with erythema nodosum.  An anti-intrinsic factor would be added, as I mentioned.  I doubt whether the patient has Behcet disease given the absence of oral or genital ulcers.  She does not give a history of oral contraceptives or medications that could be related to erythema nodosum.  She does not have any evidence of lupus __________ mycosis.  Histoplasmosis coccidioidomycosis would be accompanied by other symptoms.  Hodgkin disease has probably been ruled out with a CAT scan.  However, we are going to add an LDH in future workup.  I need to discuss with her primary care physician regarding the need for workup of her vitamin B12 deficiency and also with her gastroenterologist regarding the need for an upper endoscopy.  The patient will return in 1 month.</t>
+          <t>CHIEF COMPLAINT,:  This 32 year-old female presents today for an initial obstetrical examination.  Home pregnancy test was positive.,The patient indicates fetal activity is not yet detected (due to early stage of pregnancy).  LMP:  02/13/2002 EDD:  11/20/2002 GW:  8.0 weeks.  Patient has been trying to conceive for 6 months.,Menses:  Onset:  12 years old.  Interval:  24-26 days.  Duration:  4-6 days.  Flow:  moderate.  Complications:  PMS - mild.,Last Pap smear taken on 11/2/2001.  Contraception:  Patient is currently using none.,ALLERGIES:,  Patient admits allergies to venom - bee/wasp resulting in difficulty breathing, severe rash, pet dander resulting in nasal stuffiness.  Medication History:  None.,PAST MEDICAL HISTORY:,  Past medical history is unremarkable.  Past Surgical History:  Patient admits past surgical history of tonsillectomy in 1980.  Social History:  Patient admits alcohol use Drinking is described as social, Patient denies illegal drug use, Patient denies STD history, Patient denies tobacco use.,FAMILY HISTORY:,  Patient admits a family history of cancer of breast associated with mother.,REVIEW OF SYSTEMS:,Neurological: (+) unremarkable.,Respiratory: (+) difficulty sleeping, (-) breathing difficulties, respiratory symptoms.,Psychiatric: (+) anxious feelings.,Cardiovascular: (-) cardiovascular problems or chest symptoms.,Genitourinary: (-) decreased libido, (-) vaginal dryness, (-) vaginal bleeding.  Diet is high in empty calories, high in fats and low in fiber.,PHYSICAL EXAM:,  BP Standing:  126/84 Resp:  22 HR:  78 Temp:  99.1 Height:  5 ft.  6 in.  Weight:  132 lbs.,Pre-Gravid Weight is 125 lbs.,Patient is a 32 year old female who appears pleasant, in no apparent distress, her given age, well developed,,well nourished and with good attention to hygiene and body habitus.,Oriented to person, place and time.,Mood and affect normal and appropriate to situation.,HEENT:Head &amp; Face:  Examination of head and face is unremarkable.,Skin:  No skin rash, subcutaneous nodules, lesions or ulcers observed.  No edema observed.,Cardiovascular:  Heart auscultation reveals no murmurs, gallop, rubs or clicks.,Respiratory:  Lungs CTA.,Breast:  Chest (Breasts):  Breast inspection and palpation shows no abnormal findings.,Abdomen:  Abdomen soft, nontender, bowel sounds present x 4 without palpable masses.,Genitourinary:  External genitalia are normal in appearance.  Examination of urethra shows no abnormalities.  Examination of vaginal vault reveals no abnormalities.  Cervix shows no pathology.  Uterine portion of bimanual exam reveals contour normal, shape regular and size normal.  Adnexa and parametria show no masses, tenderness, organomegaly or nodularity.  Examination of anus and perineum shows no abnormalities.,TEST RESULTS: , Urine pregnancy test:  positive. CBC results within normal limits.  Blood type:  O positive.  Rh:  positive.  FBS:  88 mg/dl.,IMPRESSION:,  Pregnancy, normal first.  Maternal nutrition is inadequate for protein and poor and high in empty calories and junk foods and sweets.,PLAN:,  Pap smear submitted for manual screening.  Ordered CBC.  Ordered blood type.  Ordered hemoglobin.  Ordered Rh.,Ordered fasting blood glucose.,COUNSELING:,  Counseling was given regarding adverse effects of alcohol, physical activity and sexual activity.  Educational supplies dispensed to patient.,Return to clinic in 4 week (s).,PRESCRIPTIONS:,  NatalCare Plus Dosage:  Prenatal Multivitamins tablet Sig:  QD Dispense:  60 Refills:  4 Allow Generic:  Yes,PATIENT INSTRUCTIONS:,  Patient received written information regarding pre-eclampsia and eclampsia.  Patient was instructed to restrict activity.  Patient instructed to limit caffeine use.  Patient instructed to limit salt intake.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="n">
-        <v>2332</v>
+        <v>490</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Consult - History and Phy.; long; consultation; diagnoses + symptoms + medications</t>
+          <t>Consult - History and Phy.; medium; history and physical; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>4427</v>
+        <v>4218</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>consultation</t>
+          <t>history and physical</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1133,17 +1129,17 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>0.8742110009017132</v>
+        <v>0.833633904418395</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; follow-up; surgery</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; past history; treatment plans; follow-up; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="12" ht="110" customHeight="1">
       <c r="A12" s="2" t="n">
-        <v>3963</v>
+        <v>3938</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -1152,39 +1148,35 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Discharge Summary - 14 </t>
+          <t xml:space="preserve"> Discharge Summary - COPD </t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The patient is a 60-year-old female patient who off and on for the past 10 to 12 months has had almost daily diarrhea, nausea, inability to eat. </t>
+          <t xml:space="preserve"> Chest x-ray on admission, no acute finding, no interval change.  CT angiography, negative for pulmonary arterial embolism.  Chronic obstructive pulmonary disease exacerbation improving, on steroids and bronchodilators.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS: , The patient is a 60-year-old female patient who off and on for the past 10 to 12 months has had almost daily diarrhea, nausea, inability to eat.  She had an EGD and colonoscopy with Dr. ABC a few days prior to this admission.  Colonoscopy did reveal diverticulosis and EGD showed retained bile and possible gastritis.  Biopsies were done.  The patient presented to our emergency room for worsening abdominal pain as well as swelling of the right lower leg.,PAST MEDICAL HISTORY: , Extensive and well documented in prior charts.,PHYSICAL EXAMINATION: , Abdomen was diffusely tender.  Lungs clear.  Blood pressure 129/69 on admission.  At the time of admission, she had just a trace of bilateral lower edema.,LABORATORY STUDIES: , White count 6.7, hemoglobin 13, hematocrit 39.3.  Potassium of 3.2 on 08/15/2007.,HOSPITAL COURSE: , Dr. ABC apparently could not advance the scope into the cecum and therefore warranted a barium enema.  This was done and did not really show what the cecum on the barium enema.  There was some retained stool in that area and the patient had a somewhat prolonged hospital course on the remaining barium from the colon.  She did have some enemas.  She had persistent nausea, headache, neck pain throughout this hospitalization.  Finally, she did improve enough to the point where she could be discharged home.,DISCHARGE DIAGNOSIS: , Nausea and abdominal pain of uncertain etiology.,SECONDARY DIAGNOSIS:  ,Migraine headache.,COMPLICATIONS:  ,None.,DISCHARGE CONDITION: , Guarded.,DISCHARGE PLAN:  ,Follow up with me in the office in 5 to 7 days to resume all pre-admission medications.  Diet and activity as tolerated.</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>discharge summary, diarrhea, nausea, inability to eat, egd, colonoscopy, biopsies, barium enema, cecum, barium, admission,</t>
-        </is>
-      </c>
+          <t>PROCEDURES:,1.  Chest x-ray on admission, no acute finding, no interval change.,2.  CT angiography, negative for pulmonary arterial embolism.,3.  Nuclear myocardial perfusion scan, abnormal.  Reversible defect suggestive of ischemia, ejection fraction of 55%.,DIAGNOSES ON DISCHARGE:,1.  Chronic obstructive pulmonary disease exacerbation improving, on steroids and bronchodilators.,2.  Coronary artery disease, abnormal nuclear scan, discussed with Cardiology Dr. X, who recommended to discharge the patient and follow up in the clinic.,3.  Diabetes mellitus type 2.,4.  Anemia, hemoglobin and hematocrit stable.,5.  Hypokalemia, replaced.,6.  History of coronary artery disease status post stent placement 2006-2008.,7.  Bronchitis.,HOSPITAL COURSE:  ,The patient is a 65-year-old American-native Indian male, past medical history of heavy tobacco use, history of diabetes mellitus type 2, chronic anemia, COPD, coronary artery disease status post stent placement, who presented in the emergency room with increasing shortness of breath, cough productive for sputum, and orthopnea.  The patient started on IV steroid, bronchodilator as well as antibiotics.,He also complained of chest pain that appears to be more pleuritic with history of coronary artery disease and orthopnea.  He was evaluated by Cardiology Dr. X, who proceeded with stress test.  Stress test reported positive for reversible ischemia, but Cardiology decided to follow up the patient in the clinic.  The patient's last cardiac cath was in 2008.,The patient clinically significantly improved and wants to go home.  His hemoglobin on admission was 8.8, and has remained stable.  He is afebrile, hemodynamically stable.,ALLERGIES: , LISINOPRIL AND PENICILLIN.,MEDICATIONS ON DISCHARGE:,1.  Prednisone tapering dose 40 mg p.o. daily for three days, then 30 mg p.o. daily for three days, then 20 mg p.o. daily for three days, then 10 mg p.o. daily for three days, and 5 mg p.o. daily for two days.,2.  Levaquin 750 mg p.o. daily for 5 more days.,3.  Protonix 40 mg p.o. daily.,4.  The patient can continue other current home medications at home.,FOLLOWUP APPOINTMENTS:,1.  Recommend to follow up with Cardiology Dr. X's office in a week.,2.  The patient is recommended to see Hematology Dr. Y in the office for workup of anemia.,3.  Follow up with primary care physician's office tomorrow.,SPECIAL INSTRUCTIONS:,1.  If increasing shortness of breath, chest pain, fever, any acute symptoms to return to emergency room.,2.  Discussed about discharge plan, instructions with the patient by bedside.  He understands and agreed.  Also discussed discharge plan instructions with the patient's nurse.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="n">
-        <v>260</v>
+        <v>379</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Discharge Summary; short; discharge summary; diagnoses + symptoms + medications</t>
+          <t>Discharge Summary; medium; discharge summary; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>3963</v>
+        <v>3938</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
@@ -1193,21 +1185,21 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>higher</t>
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0.6243237150586114</v>
+        <v>0.7226104598737602</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; laboratory values; vital signs; procedures; past history; treatment plans; follow-up</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; procedures; imaging; past history; treatment plans; follow-up</t>
         </is>
       </c>
     </row>
     <row r="13" ht="110" customHeight="1">
       <c r="A13" s="2" t="n">
-        <v>3962</v>
+        <v>3885</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
@@ -1216,26 +1208,26 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Death Summary - 2 </t>
+          <t xml:space="preserve"> Speech Therapy - Discharge Summary - 1 </t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Cardiac arrest, severe congestive heart failure, acute on chronic respiratory failure, osteoporosis, and depression.</t>
+          <t xml:space="preserve"> The patient was referred to Medical Center's Outpatient Rehabilitation Department for skilled speech therapy to improve her functional communication skills and swallowing function and safety.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>FINAL DIAGNOSES:,1.  Cardiac arrest.,2.  Severe congestive heart failure.,3.  Acute on chronic respiratory failure.,4.  Osteoporosis.,5.  Depression.,HISTORY OF PRESENT ILLNESS: , This 92-year-old lady with history of depression and chronic low back pain, osteoporosis, and congestive heart failure, was diagnosed having pneumonia approximately for at least 10 days prior to admission.  In the ER, she was given oral antibiotics.  She also saw me few days before admission coming for a followup.  She was doing fairly well.  She was thought to have congestive heart failure and she was advised to continue with her diuretics.  For the last few days, the patient started to have anorexia, she did not eat well, and she did not drink well.  Her family could not take care of her.  So, she was brought to the emergency room, where she was found to have rapid heart rate with a sinus tachycardia around 112 to 130s.  The ________ was found to be dry.  She was given 1 L of IV fluids and she was subsequently admitted in the hospital for further management.,COURSE IN THE HOSPITAL: , The patient stayed in the telemetry.  The patient had significant shortness of breath secondary to congestive heart failure with bilateral basilar crackles.  She was continued on IV antibiotics and general IV hydration was started initially because of low blood pressure and low perfusion status.  On subsequently improved and stopped and Lasix was started; Dr. X, cardiologist was also placed.  The patient's family wanted her to be a DNR and DNI.  They were allowing us to treat her aggressively medically for pneumonia and congestive heart failure.  However, the patient became extremely weak, mostly unresponsive.  At this time, the patient's family wanted a Hospice consult, which was requested.  By the time the Hospice could evaluate her, the patient's condition got deteriorated, she went into more bradycardiac and hypertension and subsequently expired.  Please see the hospital notes for complete details.</t>
+          <t>HISTORY: , The patient is a 67-year-old female, was referred to Medical Center's Outpatient Rehabilitation Department for skilled speech therapy to improve her functional communication skills and swallowing function and safety.  At the onset of therapy, on 03/26/08, the patient was NPO with a G-tube and the initial speech and language evaluation revealed global aphasia with an aphasia quotient of 3.6/100 based on the Western Aphasia Battery.  Since the initial evaluation, the patient has attended 60 outpatient speech therapy sessions, which have focussed on her receptive communication, expressive language, multimodality communication skills, and swallowing function and safety.,SHORT-TERM GOALS:,1.  The patient met 3 out of 4 original short-term therapy goals, which were to complete a modified barium swallow study, which she did do and which revealed no aspiration.  At this time, the patient is eating and drinking and taking all medications by mouth; however, her G-tube is still present.  The patient was instructed to talk to the primary care physician about removal of her feeding tube.,2.  The patient will increase accuracy of yes-no responses to greater than 80% accuracy.  She did accomplish this goal.  The patient is also able to identify named objects with greater than 80% accuracy.,ADDITIONAL GOALS: , Following the completion of these goals, additional goals were established.  Based on reevaluation, the patient met 2 out of these 3 initial goals and she is currently able to read and understand simple sentences with greater than 90% accuracy independently and she is able to write 10 words related to basic wants and needs with greater than 80% accuracy independently.  The patient continues to have difficulty stating verbally, yes or no, to questions as well as accurately using head gestures and to respond to yes-no questions.  The patient continues to have marked difficulty with her expressive language abilities.  She is able to write simple words to help express her basic wants and needs.  She has made great strides; however, with her receptive communication, she is able to read words as well as short phrases and able to point to named objects and answer simple-to-moderate complex yes-no questions.  A reevaluation completed on 12/01/08, revealed an aphasia quotient of 26.4.  Once again, she made significant improvement and comprehension, but continues to have unintelligible speech.  An alternative communication device was discussed with the patient and her husband, but at this time, the patient does not want to utilize a communication device.  If, in the future, the patient continues to struggle with her expressive communication, an alternative augmented communication device would be a benefit to her.  Please reconsult at that time if and when the patient is ready to use a speech generating device.  The patient is discharged from my services at this time due to a plateau in her progress.  Numerous home activities were recommended to allow her to continue to make progress at home.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">discharge summary, bradycardiac, hypertension, hospice, congestive heart failure, cardiac arrest, respiratory failure, </t>
+          <t>discharge summary, communication skills, g-tube, aphasia, language evaluation, western aphasia battery, skilled speech therapy, swallowing function, speech therapy, therapy, swallowing, aspiration, speech, communication,</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>313</v>
+        <v>471</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -1244,15 +1236,15 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Discharge Summary; medium; other narrative/sectioned; diagnoses + symptoms + vital signs</t>
+          <t>Discharge Summary; medium; discharge summary; lower text complexity; medications + treatment plans</t>
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>3962</v>
+        <v>3885</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>other narrative/sectioned</t>
+          <t>discharge summary</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1261,17 +1253,17 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0.3609670874661858</v>
+        <v>0.3477795311091073</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; vital signs; past history; treatment plans; follow-up</t>
+          <t>medications; treatment plans</t>
         </is>
       </c>
     </row>
     <row r="14" ht="110" customHeight="1">
       <c r="A14" s="2" t="n">
-        <v>3911</v>
+        <v>3925</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -1280,26 +1272,22 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Lap Chole - Discharge Summary </t>
+          <t xml:space="preserve"> Discharge Summary - Urology &amp; Nephrology  </t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Laparoscopic cholecystectomy.  Acute cholecystitis, status post laparoscopic cholecystectomy, end-stage renal disease on hemodialysis, hyperlipidemia, hypertension, congestive heart failure, skin lymphoma 5 years ago, and hypothyroidism.</t>
+          <t xml:space="preserve"> Solitary left kidney with obstruction and hypertension and chronic renal insufficiency, plus a Pseudomonas urinary tract infection.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>PROCEDURE:,  Laparoscopic cholecystectomy.,DISCHARGE DIAGNOSES:,1.  Acute cholecystitis.,2.  Status post laparoscopic cholecystectomy.,3.  End-stage renal disease on hemodialysis.,4.  Hyperlipidemia.,5.  Hypertension.,6.  Congestive heart failure.,7.  Skin lymphoma 5 years ago.,8.  Hypothyroidism.,HOSPITAL COURSE: , This is a 78-year-old female with past medical condition includes hypertension, end-stage renal disease, hyperlipidemia, hypothyroidism, and skin lymphoma who had a left AV fistula done about 3 days ago by Dr. X and the patient went later on home, but started having epigastric pain and right upper quadrant pain and mid abdominal pain, some nauseated feeling, and then she could not handle the pain, so came to the emergency room, brought by the family.  The patient's initial assessment, the patient's vital signs were stable, showed temperature 97.9, pulse was 106, and blood pressure was 156/85.  EKG was not available and ultrasound of the abdomen showed there is a renal cyst about 2 cm.  There is sludge in the gallbladder wall versus a stone in the gallbladder wall.  Thickening of the gallbladder wall with positive Murphy sign.  She has a history of cholecystitis.  Urine shows positive glucose, but negative for nitrite and creatinine was 7.1, sodium 131, potassium was 5.2, and lipase and amylase were normal.  So, the patient admitted to the Med/Surg floor initially and the patient was started on IV fluid as well as low-dose IV antibiotic and 2-D echocardiogram and EKG also was ordered.  The patient also had history of CHF in the past and recently had some workup done.  The patient does not remember initially.  Surgical consult also requested and blood culture and urine culture also ordered.  The same day, the patient was seen by Dr. Y and the patient should need cholecystectomy, but the patient also needs dialysis and also needs to be cleared by the cardiologist, so the patient later on seen by Dr. Z and cleared the patient for the surgery with moderate risk and the patient underwent laparoscopic cholecystectomy.  The patient also seen by nephrologist and underwent dialysis.  The patient's white count went down 6.1, afebrile.  On postop day #1, the patient started eating and also walking.  The patient also had chronic bronchitis.  The patient was later on feeling fine, discussed with surgery.  The patient was then able to discharge to home and follow with the surgeon in about 3-5 days.  Discharged home with Synthroid 0.5 mg 1 tablet p.o. daily, Plavix 75 mg p.o. daily, folic acid 1 mg p.o. daily, Diovan 80 mg p.o. daily, Renagel 2 tablets 800 mg p.o. twice a day, Lasix 40 mg p.o.  2 tablets twice a day, lovastatin 20 mg p.o. daily, Coreg 3.125 mg p.o. twice a day, nebulizer therapy every 3 hours as needed, also Phenergan 25 mg p.o. q.8 hours for nausea and vomiting, Pepcid 20 mg p.o. daily, Vicodin 1 tablet p.o. q.6 hours p.r.n. as needed, and Levaquin 250 mg p.o. every other day for the next 5 days.  The patient also had Premarin that she was taking, advised to discontinue because of increased risk of heart disease and stroke explained to the patient.  Discharged home.</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">discharge summary, end-stage renal disease, lymphoma, cholecystitis, congestive heart failure, skin lymphoma, gallbladder wall, laparoscopic cholecystectomy </t>
-        </is>
-      </c>
+          <t>ADMITTING DIAGNOSES:,  Solitary left kidney with obstruction, and hypertension, and chronic renal insufficiency.,DISCHARGE DIAGNOSES: , Solitary left kidney with obstruction and hypertension and chronic renal insufficiency, plus a Pseudomonas urinary tract infection.,PROCEDURES: , Cystoscopy under anesthesia, ureteroscopy, an attempted tube placement, stent removal with retrograde pyelography, percutaneous tube placement, and nephrostomy by Radiology.,PERTINENT LABORATORIES: , Creatinine of 1.4.  During the hospitalization it was decreased to 0.8 and Pseudomonas urinary tract infection, positive culture sensitive to ceftazidime and ciprofloxacin.,HISTORY OF PRESENT ILLNESS:  ,The patient is a 3-1/2-year-old boy with a solitary kidney, had a ureteropelvic junction repair performed by Dr. Y, in the past, unfortunately, it was thought still be obstructed.  A stent was placed approximately 6 weeks ago after urethroscopic placement with some difficulty.  Plan was to remove the stent.  At the time of removal, we were unable to place another tube within the collecting system, and the patient was admitted for percutaneous nephrostomy placement.  He has had no recent cold or flu.  He has problems with hypertension for which he is on enalapril at home in addition to his Macrodantin prophylaxis.,PAST MEDICAL HISTORY: , The patient has no known allergies.  Multiple urinary tract infection, solitary kidney, and previous surgeries as mentioned above.,REVIEW OF SYSTEMS:,  A 14-organ system review of systems is negative except for the history of present illness.  He also has history of being a 34-week preemie twin.,ALLERGIES: , No known allergies.,FAMILY HISTORY: , Unremarkable without any bleeding or anesthetic problems.,SOCIAL HISTORY: , The patient lives at home with his parents, 2 brothers, and a sister.,IMMUNIZATIONS:,  Up-to-date.,MEDICATIONS: , On admission was Macrodantin, hydralazine, and enalapril.,PHYSICAL EXAMINATION:,GENERAL:  The patient is an active little boy.,HEENT:  The head and neck exam was grossly normal.  He had no oral, ocular, or nasal discharge.,LUNGS:  Exam was normal without wheezing.,HEART:  Without murmur or gallops.,ABDOMEN:  Soft, without mass or tenderness with a well-healed flank incision.,GU:  Uncircumcised male with bilaterally descended testes.,EXTREMITIES:  He has full range of motion in all 4 extremities.,SKIN:  Warm, pink, and dry.,NEUROLOGIC:  Grossly intact.,BACK:  He has normal back.  Normal gait.,HOSPITAL COURSE: , The patient was admitted to the hospital after inability to place a ureteral stent via ureteroscopy and cystoscopy.  He was made NPO.  He had a fever at first time with elevated creatinine.  He was also evaluated and treated by Dr. X, for fluid management, hypertensive management, and gave him some hydralazine and Lasix to improve his urine output, in addition to manage his blood pressure.  Once the percutaneous tube was placed, we found that his urine culture grew Pseudomonas, so he was kept on Fortaz, and was switched over to ciprofloxacin without difficulty.  He, otherwise, did well with continuing decrease his creatinine at the time of discharge to home.,The patient was discharged home in stable condition with ciprofloxacin, enalapril, and recommendation for followup in Urology in 1 to 2 weeks for the surgical correction in 2 to 3 weeks of repeat pyeloplasty or possible ureterocalicostomy.  The patient had draining nephrostomy tube without difficulty.,</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="n">
-        <v>505</v>
+        <v>493</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1308,11 +1296,11 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Discharge Summary; medium; discharge summary; diagnoses + symptoms + medications</t>
+          <t>Discharge Summary; medium; discharge summary; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>3911</v>
+        <v>3925</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -1321,21 +1309,21 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>higher</t>
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>0.5958633904418396</v>
+        <v>0.7965509467989179</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; laboratory values; vital signs; procedures; imaging; past history; surgery</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; procedures; past history; treatment plans; follow-up; surgery</t>
         </is>
       </c>
     </row>
     <row r="15" ht="110" customHeight="1">
       <c r="A15" s="2" t="n">
-        <v>3966</v>
+        <v>3911</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -1344,39 +1332,39 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Discharge Summary - 10 </t>
+          <t xml:space="preserve"> Lap Chole - Discharge Summary </t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Patient with a history of a Nissen fundoplication performed six years ago for gastric reflux. </t>
+          <t xml:space="preserve"> Laparoscopic cholecystectomy.  Acute cholecystitis, status post laparoscopic cholecystectomy, end-stage renal disease on hemodialysis, hyperlipidemia, hypertension, congestive heart failure, skin lymphoma 5 years ago, and hypothyroidism.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>ADMITTING DIAGNOSES:,  Hiatal hernia, gastroesophageal reflux disease reflux.,DISCHARGE DIAGNOSES:,  Hiatal hernia, gastroesophageal reflux disease reflux.,SECONDARY DIAGNOSIS: , Postoperative ileus.,PROCEDURES DONE: , Hiatal hernia repair and Nissen fundoplication revision.,BRIEF HISTORY: , The patient is an 18-year-old male who has had a history of a Nissen fundoplication performed six years ago for gastric reflux.  Approximately one year ago, he was involved in a motor vehicle accident and CT scan at that time showed that he had a hiatal hernia.  Over the past year, this has caused him an increasing number of problems, including chest pain when he eats, and shortness of breath after large meals.  He is also having reflux symptoms again.  He presents to us for repair of the hiatal hernia and revision of the Nissen fundoplication.,HOSPITAL COURSE: , Mr. A was admitted to the adolescent floor by Brenner Children's Hospital after his procedure.  He was stable at that time.  He did complain of some nausea.  However, he did not have any vomiting at that time.  He had an NG tube in and was n.p.o.  He also had a PCA for pain management as well as Toradol.  On postoperative day #1, he complained of not being able to urinate, so a Foley catheter was placed.  Over the next several days, his hospital course proceeded as follows.  He continued to complain of some nausea; however, he did not ever have any vomiting.  Eventually, the Foley catheter was discontinued and he had excellent urine output without any complications.  He ambulated frequently.  He remained n.p.o. for three days.  He also had the NG tube in during that time.  On postoperative day #4, he began to have some flatus, and the NG tube was discontinued.  He was advanced to a liquid diet and tolerated this without any complications.  At this time, he was still using the PCA for pain control.  However, he was using it much less frequently than on days #1 and #2 postoperatively.  After tolerating the full liquid diet without any complications, he was advanced to a soft diet and his pain medications were transitioned to p.o. medications rather than the PCA.  The PCA was discontinued.  He tolerated the soft diet without any complications and continued to have flatus frequently.  On postoperative day #6, it was determined that he was stable for discharge to home as he was taking p.o. without any complications.  His pain was well controlled with p.o. pain medications.  He was passing gas frequently, had excellent urine output, and was ambulating frequently without any issues.,DISCHARGE CONDITION:,  Stable.,DISPOSITION: , Discharged to home.,DISCHARGE INSTRUCTIONS: , The patient was discharged to home with instructions for maintaining a soft diet.  It was also recommended that he does not drink any soda postoperatively.  He is instructed to keep his incision site clean and dry and it was also recommended that he avoid any heavy lifting.  He will be able to attend school when it starts in a few weeks.  However, he is not going to be able to play football in the near future.  He was given prescription for pain medication upon discharge.  He is instructed to contact Pediatric Surgery if he has any fevers, any nausea and vomiting, any chest pain, any constipation, or any other concerns.</t>
+          <t>PROCEDURE:,  Laparoscopic cholecystectomy.,DISCHARGE DIAGNOSES:,1.  Acute cholecystitis.,2.  Status post laparoscopic cholecystectomy.,3.  End-stage renal disease on hemodialysis.,4.  Hyperlipidemia.,5.  Hypertension.,6.  Congestive heart failure.,7.  Skin lymphoma 5 years ago.,8.  Hypothyroidism.,HOSPITAL COURSE: , This is a 78-year-old female with past medical condition includes hypertension, end-stage renal disease, hyperlipidemia, hypothyroidism, and skin lymphoma who had a left AV fistula done about 3 days ago by Dr. X and the patient went later on home, but started having epigastric pain and right upper quadrant pain and mid abdominal pain, some nauseated feeling, and then she could not handle the pain, so came to the emergency room, brought by the family.  The patient's initial assessment, the patient's vital signs were stable, showed temperature 97.9, pulse was 106, and blood pressure was 156/85.  EKG was not available and ultrasound of the abdomen showed there is a renal cyst about 2 cm.  There is sludge in the gallbladder wall versus a stone in the gallbladder wall.  Thickening of the gallbladder wall with positive Murphy sign.  She has a history of cholecystitis.  Urine shows positive glucose, but negative for nitrite and creatinine was 7.1, sodium 131, potassium was 5.2, and lipase and amylase were normal.  So, the patient admitted to the Med/Surg floor initially and the patient was started on IV fluid as well as low-dose IV antibiotic and 2-D echocardiogram and EKG also was ordered.  The patient also had history of CHF in the past and recently had some workup done.  The patient does not remember initially.  Surgical consult also requested and blood culture and urine culture also ordered.  The same day, the patient was seen by Dr. Y and the patient should need cholecystectomy, but the patient also needs dialysis and also needs to be cleared by the cardiologist, so the patient later on seen by Dr. Z and cleared the patient for the surgery with moderate risk and the patient underwent laparoscopic cholecystectomy.  The patient also seen by nephrologist and underwent dialysis.  The patient's white count went down 6.1, afebrile.  On postop day #1, the patient started eating and also walking.  The patient also had chronic bronchitis.  The patient was later on feeling fine, discussed with surgery.  The patient was then able to discharge to home and follow with the surgeon in about 3-5 days.  Discharged home with Synthroid 0.5 mg 1 tablet p.o. daily, Plavix 75 mg p.o. daily, folic acid 1 mg p.o. daily, Diovan 80 mg p.o. daily, Renagel 2 tablets 800 mg p.o. twice a day, Lasix 40 mg p.o.  2 tablets twice a day, lovastatin 20 mg p.o. daily, Coreg 3.125 mg p.o. twice a day, nebulizer therapy every 3 hours as needed, also Phenergan 25 mg p.o. q.8 hours for nausea and vomiting, Pepcid 20 mg p.o. daily, Vicodin 1 tablet p.o. q.6 hours p.r.n. as needed, and Levaquin 250 mg p.o. every other day for the next 5 days.  The patient also had Premarin that she was taking, advised to discontinue because of increased risk of heart disease and stroke explained to the patient.  Discharged home.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>discharge summary,</t>
+          <t xml:space="preserve">discharge summary, end-stage renal disease, lymphoma, cholecystitis, congestive heart failure, skin lymphoma, gallbladder wall, laparoscopic cholecystectomy </t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>533</v>
+        <v>505</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Discharge Summary; long; discharge summary; diagnoses + symptoms + medications</t>
+          <t>Discharge Summary; medium; discharge summary; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J15" s="2" t="n">
-        <v>3966</v>
+        <v>3911</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
@@ -1389,17 +1377,17 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0.5607529305680794</v>
+        <v>0.5958633904418396</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; procedures; imaging; past history; treatment plans; surgery</t>
+          <t>diagnoses; symptoms; medications; laboratory values; vital signs; procedures; imaging; past history; surgery</t>
         </is>
       </c>
     </row>
     <row r="16" ht="110" customHeight="1">
       <c r="A16" s="2" t="n">
-        <v>3864</v>
+        <v>3846</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
@@ -1408,35 +1396,39 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Closed Head Injury </t>
+          <t xml:space="preserve"> Fall &amp; Laceration </t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Status post a high-speed motor vehicle accident in which patient was ejected from the vehicle.</t>
+          <t xml:space="preserve"> Patient running to catch a taxi and stumbled, fell and struck his face on the sidewalk.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>CHIEF COMPLAINT:,  Status post motor vehicle accident.,HISTORY OF PRESENT ILLNESS: , The patient is a 17-year-old white male who is status post a high-speed motor vehicle accident in which he was ejected from the vehicle.  He denies loss of consciousness, although the EMT people report that he did have loss of consciousness.  The patient was stable en route.  Upon arrival, he complained of headache.,PAST MEDICAL HISTORY:,  Medical:  None.  Surgical:  None.,REVIEW OF SYSTEMS: , CARDIAC:  No history.  PULMONARY:  Some morning cough.  (Patient is a smoker.),MEDICATIONS:,  None.,ALLERGIES:,  ALLERGIC TO PENICILLIN, CAUSES SKIN RASH.,PHYSICAL EXAMINATION:,VITAL SIGNS:  Blood pressure 120/80, pulse 82, respirations 20, temperature 36.8°.,HEENT:  Contusion over right occipital area.  Tympanic membranes benign.,NECK:  Nontender.,CHEST:  Atraumatic, nontender.,LUNGS:  Clear to auscultation and percussion.,ABDOMEN:  Flat, soft, and nontender.,BACK:  Atraumatic, nontender.,PELVIS:  Stable,EXTREMITIES:  Contusion over right forearm.  No bone deformity or crepitus.,RECTAL:  Normal sphincter tone; guaiac negative.,NEUROLOGIC:  Glasgow coma scale 15.  Pupils equal, round, reactive to light.  Patient moves all 4 extremities without focal deficit.,LABORATORY DATA: , Serial hematocrits 42.4, and 40.4.  White blood count 6.3.  Ethanol:  None.  Amylase 66.  Urinalysis normal.  PT 12.6, PTT 29.  Chem-7 panel within normal limits.,X-rays of cervical spine and lumbosacral spine within normal limits.  X-rays of pelvis and chest within normal limits.,ASSESSMENT:,1.  Closed head injury.,2.  Rule out intra-abdominal injury.,PLAN:,  The patient will be admitted to the trauma surgery service for continued evaluation and treatment for closed head injury as well as possible intra-abdominal injury.</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr"/>
+          <t>CC:,  Fall and laceration.,HPI: , Mr. B is a 42-year-old man who was running to catch a taxi when he stumbled, fell and struck his face on the sidewalk.  He denies loss of consciousness but says he was dazed for a while after it happened.  He complains of pain over the chin and right forehead where he has abrasions.  He denies neck pain, back pain, extremity pain or pain in the abdomen.,PMH: , Hypertension.,MEDS:,  None.,ROS: , As above.  Otherwise negative.,PHYSICAL EXAM: , This is a gentleman in full C-spine precautions on a backboard brought by EMS.  He is in no apparent distress.  ,Vital Signs:  BP 165/95 HR 80 RR 12 Temp 98.4 SpO2 95% ,HEENT:  No palpable step offs, there is blood over the right fronto-parietal area where there is a small 1cm laceration and surrounding abrasion.  Also, 2 cm laceration over the base of the chin without communication to the oro-pharynx.  No other trauma noted.  No septal hematoma.  No other facial bony tenderness.  ,Neck:  Nontender ,Chest:  Breathing comfortably; equal breath sounds.  ,Heart:  Regular rhythm.,Abd:  Benign.,Ext:  No tenderness or deformity; pulses are equal throughout; good cap refill ,Neuro:  Awake and alert; slight slurring of speech and cognitive slowing consistent with alcohol; moves all extremities; cranial nerves normal.  ,COURSE IN THE ED:,  Patient arrived and was placed on monitors.  An IV had been placed in the field and labs were drawn.  X-rays of the C spine show no fracture and I've removed the C-collar.  The lacerations were explored and no foreign body found.  They were irrigated and closed with simple interrupted sutures.  Labs showed normal CBC, Chem-7, and U/A except there was moderate protein in the urine.  The blood alcohol returned at 0.146.  A banana bag is ordered and his care will be turned over to Dr. G for further evaluation and care.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>emergency room reports, loss of consciousness, laceration, fall, course in the ed, placed on monitors, fell and struck, abrasions,</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="n">
-        <v>232</v>
+        <v>302</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Emergency Room Reports; short; other narrative/sectioned; diagnoses + symptoms + medications</t>
+          <t>Emergency Room Reports; medium; other narrative/sectioned; lower text complexity; symptoms + laboratory values + vital signs</t>
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>3864</v>
+        <v>3846</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
@@ -1445,21 +1437,21 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>higher</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>0.6975879170423805</v>
+        <v>0.36547565374211</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; imaging; past history; treatment plans; surgery; assessment/plan</t>
+          <t>symptoms; laboratory values; vital signs; imaging</t>
         </is>
       </c>
     </row>
     <row r="17" ht="110" customHeight="1">
       <c r="A17" s="2" t="n">
-        <v>3838</v>
+        <v>3826</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
@@ -1468,22 +1460,26 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Head Injury </t>
+          <t xml:space="preserve"> Mastoiditis - Discharge Summary </t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Head injury, anxiety, and hypertensive emergency.</t>
+          <t xml:space="preserve"> Suspected mastoiditis ruled out, right acute otitis media, and severe ear pain resolving.  The patient is an 11-year-old male who was admitted from the ER after a CT scan suggested that the child had mastoiditis.  </t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>CHIEF COMPLAINT:,  Head injury.,HISTORY: , This 16-year-old female presents to Children's Hospital via paramedic ambulance with a complaint at approximately 6 p.m. while she was at band practice using her flag device.  She struck herself in the head with the flag.  There was no loss of consciousness.  She did feel dizzy.  She complained of a headache.  She was able to walk.  She continued to participate in her flag practice.  She got dizzier.  She sat down for a while and walked and during the second period of walking, she had some episodes of diplopia, felt that she might faint and was assisted to the ground and was transported via paramedic ambulance to Children's Hospital for further evaluation.,PAST MEDICAL HISTORY: , Hypertension.,ALLERGIES:,  DENIED TO ME; HOWEVER, IT IS NOTED BEFORE SEVERAL ACCORDING TO MEDITECH.,CURRENT MEDICATIONS: , Enalapril.,PAST SURGICAL HISTORY: , She had some kind of an abdominal obstruction as an infant.,SOCIAL HISTORY: , She is here with mother and father who lives at home.  There is no smoking at home.  There is second-hand smoke exposure.,FAMILY HISTORY:  ,No noted family history of infectious disease exposure.,IMMUNIZATIONS:,  She is up-to-date on her shots, otherwise negative.,REVIEW OF SYSTEMS:  ,On the 10-plus systems reviewed with the section of those noted on the template.,PHYSICAL EXAMINATION:,VITAL SIGNS:  Her temperature 100 degrees, pulse 86, respirations 20, and her initial blood pressure 166/116, and a weight of 55.8 kg.,GENERAL:  She is supine awake, alert, cooperative, and active child.,HEENT:  Head atraumatic, normocephalic.  Pupils equal, round, reactive to light.  Extraocular motions intact and conjugate.  Clear TMs, nose and oropharynx.  Moist oral mucosa without noted lesions.,NECK:  Supple, full painless nontender range motion.,CHEST:  Clear to auscultation, equal, stable to palpation.,HEART:  Regular without rubs or murmurs.,ABDOMEN:  No abdominal bruits are heard.,EXTREMITIES:  Equal femoral pulses are appreciated.  Equal radial and dorsalis pedis pulses are appreciated.  He moves all extremities without difficulty.  Nontender.  No deformity.  No swelling.,SKIN:  There was no significant bruising, lesions or rash about her abdomen.  No significant bruising, lesions or rash.,NEUROLOGIC:  Symmetric face and extremity motion.  Ambulates without difficulty.  She is awake, alert, and appropriate.,MEDICAL DECISION MAKING:,  The differential entertained includes head injury, anxiety, and hypertensive emergency.  She is evaluated in the emergency department with serial blood pressure examinations, which are noted to return to a more baseline state for her 130s/90s.  Her laboratory data shows a mildly elevated creatinine of 1.3.  Urine is within normal.  Urinalysis showing no signs of infection.  Head CT read by staff has no significant intracranial pathology.  No mass shift, bleed or fracture per Dr. X.  A 12-lead EKG reviewed preliminarily by myself noting normal sinus rhythm, normal axis rates of 90.  No significant ST-T wave changes.  No significant change from previous 09/2007 EKG.  Her headache has resolved.  She is feeling better.  I spoke with Dr. X at 0206 hours consulting Nephrology regarding this patient's presentation with the plan for home.  Follow up with her regular doctor.  Blood pressures have normalized for her.  She should return to emergency department on concern.  They are to call the family to Nephrology Clinic next week for optimization of her blood pressure control with a working diagnosis of head injury, hypertension, and syncope.</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr"/>
+          <t>DISCHARGE DIAGNOSES:  ,1.  Suspected mastoiditis ruled out.,2.  Right acute otitis media.,3.  Severe ear pain resolving.,HISTORY OF PRESENT ILLNESS: , The patient is an 11-year-old male who was admitted from the ER after a CT scan suggested that the child had mastoiditis.  The child has had very severe ear pain and blood draining from the right ear.  The child had a temperature maximum of 101.4 in the ER.  The patient was admitted and started on IV Unasyn, which he tolerated well and required Morphine and Vicodin for pain control.  In the first 12 hours after admission, the patient's pain decreased and also swelling of his cervical area decreased.  The patient was evaluated by Dr. X from the ENT while in house.  After reviewing the CT scan, it was felt that the CT scan was not consistent with mastoiditis.  The child was continued on IV fluid and narcotics for pain as well as Unasyn until the time of discharge.  At the time of discharge his pain is markedly decreased about 2/10 and swelling in the area has improved.  The patient is also able to take p.o. well.,DISCHARGE PHYSICAL EXAMINATION:,GENERAL:  The patient is alert, in no respiratory distress.,VITAL SIGNS:  His temperature is 97.6, heart rate 83, blood pressure 105/57, respiratory rate 16 on room air.,HEENT:  Right ear shows no redness.  The area behind his ear is nontender.  There is a large posterior chains node that is nontender and the swelling in this area has decreased markedly.,NECK:  Supple.,CHEST:  Clear breath sounds.,CARDIAC:  Normal S1, S2 without murmur.,ABDOMEN:  Soft.  There is no hepatosplenomegaly or tenderness.,SKIN:  Warm and well perfused.,DISCHARGE WEIGHT: , 38.7 kg.,DISCHARGE CONDITION: , Good.,DISCHARGE DIET:,  Regular as tolerated.,DISCHARGE MEDICATIONS:  ,1.  Ciprodex Otic Solution in the right ear twice daily.,2.  Augmentin 500 mg three times daily x10 days.,FOLLOW UP:  ,1.  Dr. Y in one week (ENT).,2.  The primary care physician in 2 to 3 days.,TIME SPENT: , Approximate discharge time is 28 minutes.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
       <c r="G17" s="2" t="n">
-        <v>519</v>
+        <v>318</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1492,15 +1488,15 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Emergency Room Reports; medium; other narrative/sectioned; diagnoses + symptoms + medications</t>
+          <t>Emergency Room Reports; medium; discharge summary; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J17" s="2" t="n">
-        <v>3838</v>
+        <v>3826</v>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>other narrative/sectioned</t>
+          <t>discharge summary</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1509,17 +1505,17 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>0.8070897204688909</v>
+        <v>0.631311992786294</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; imaging; past history; treatment plans; follow-up; surgery</t>
+          <t>diagnoses; symptoms; medications; vital signs; imaging; past history; follow-up</t>
         </is>
       </c>
     </row>
     <row r="18" ht="110" customHeight="1">
       <c r="A18" s="2" t="n">
-        <v>3818</v>
+        <v>3860</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
@@ -1528,39 +1524,39 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Shone complex </t>
+          <t xml:space="preserve"> Consult/ER Report - OB/GYN </t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Complete heart block with pacemaker malfunction and  a history of Shone complex.</t>
+          <t xml:space="preserve"> A female with unknown gestational age who presents to the ED after a suicide attempt.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>HISTORY AND PHYSICAL:  ,The patient is a 13-year-old, who has a history of Shone complex and has a complete heart block.  He is on the pacemaker.  He had a coarctation of the aorta and that was repaired when he was an infant.  He was followed in our Cardiology Clinic here and has been doing well.  However last night, he was sleeping, and he states he felt as if he has having a dream, and there was thunder in this dream, which woke him up.  He then felt that his defibrillator was going off and this has continued and feels like his heart rate is not normal.  Thus, his dad put him in the car and transported him here.  He has been evaluated here.  He had some scar tissue at one point when the internal pacemaker was not working properly and had to have that replaced.  It was 2 a.m. when he woke, and again, he was brought here by private vehicle.  He was well prior to going to bed.  No cough, cold, runny nose, fever.  No trauma has been noted.,PAST MEDICAL HISTORY:,  Shone complex, pacemaker dependent.,MEDICATIONS: , He is on no medications at this time.,ALLERGIES:,  He has no allergies.,IMMUNIZATIONS:,  Up to date.,SOCIAL HISTORY: , He lives with his parents.,FAMILY HISTORY: , Negative.,REVIEW OF SYSTEM: , Twelve asked, all negative, except as noted above.,PHYSICAL EXAMINATION:,GENERAL:  This is an awake, alert male, who appears to be in mild distress.,HEENT:  Pupils are equal, round, and reactive to light.  Extraocular movements are intact.  His TMs are clear.  His nares are clear.  The mucous membranes are pink and moist.  Throat is clear.,NECK:  Supple without lymphadenopathy or masses.  Trachea is midline.,LUNGS:  Clear.,HEART:  Shows bradycardia at 53.  He has good distal pulses.,ABDOMEN:  Soft, nontender.  Positive bowel sounds.  No guarding, no rebound.  No rashes are seen.,HOSPITAL COURSE:,  Initial blood pressure is 164/90.  He was moved in room 1.  He was placed on nasal cannula.  Pulse ox was 100%, which is normal.  We placed him on a monitor.  We did an EKG; it has not appear to be capturing his pacemaker at this time.  Shortly after the patient's arrival, the Medtronic technician came and worked out his pacemaker.  Medtronic representative informed me that the lead that he has in place has been recalled because it has been prone to microfractures, oversensing, and automatic defibrillation.  As noted, he was transferred to room 1, placed on a monitor, pulse ox.  An IV was placed.  A standard blood work was sent.  A chest x-ray was done showing normal heart size, lead appeared to be in placed.  There was no evidence of pulmonary edema.  His pacemaker did not appear to be capturing.  We placed him on transthoracic leads.  However, it is difficult to get good placement with these because of the area where his pacemaker was placed.  The Medtronic technician initially turned off his defibrillation mode and turned down his sensor.  However, we could not get our transthoracic pacer to capture his heart.  When the Medtronic representative turned off the pacemaker, the heart rate seemed to drop into the 40s.  The patient appeared to be in pain.  We placed it back on a rate of 60 at that time.  He has remained in sinus bradycardia, but no evidence of ectopic beats.  No widening of his QRS complex.  I spoke with Cardiology.  Cardiology service has come in, has evaluated him at bedside with me.  Again, we turned up the transthoracic pacer, but it is again not seem to be picking up, and his heart rate is still going with the Medtronic's internal pacemaker.  So with the ICU physician on call, Dr. X, he has agreed with taking this young man to the ICU.,An hour after presentation here, the ICU was ready for bed.  I accompanied the patient up to the ICU.  He remained awake and alert.  Initially, he was complaining of a lot of chest pain.  Once the defibrillator was turned off, he had no more pain.  He was transported to the Pediatrics PICU and delivered in stable condition.,LABORATORY DATA: , CBC was normal.  Chem-20 was normal as well.,IMPRESSION:  ,Complete heart block with pacemaker malfunction.,PLAN:  ,He is admitted to the ICU.,TIME SEEN: , Critical care time outside billable procedures was 45 minutes with this patient.  I should note that a 12-lead EKG was done here showing sinus bradycardia, normal intervals otherwise.</t>
+          <t>The patient states that she has abnormal menstrual periods and cannot remember the first day of her last normal menstrual period.  She states that she had spotting for three months daily until approximately two weeks ago, when she believes that she passed a fetus.  She states that upon removal of a tampon, she saw a tadpole like structure and believed it to be a fetus.  However, she states she did not know that she was pregnant at this time.  She denies any abdominal pain or vaginal bleeding.  She states that the pregnancy is unplanned; however, she would desire to continue the pregnancy.,PAST MEDICAL HISTORY:  Diabetes mellitus which resolved after weight loss associated with gastric bypass surgery.,PAST SURGICAL HISTORY:,1.  Gastric bypass.,2.  Bilateral carpal tunnel release.,3.  Laparoscopic cholecystectomy.,4.  Hernia repair after gastric bypass surgery.,5.  Thoracotomy.,6.  Knee surgery.,MEDICATIONS:,1.  Lexapro 10 mg daily.,2.  Tramadol 50 mg tablets two by mouth four times a day.,3.  Ambien 10 mg tablets one by mouth at bedtime.,ALLERGIES:  AMOXICILLIN CAUSES THROAT SWELLING.  AVELOX CAUSES IV SITE SWELLING.,SOCIAL HISTORY:  The patient denies tobacco, ethanol, or drug use.  She is currently separated from her partner who is the father of her 21-month-old daughter.  She currently lives with her parents in Greenville.  However, she was visiting the estranged boyfriend in Wilkesboro, this week.,GYN HISTORY:  The patient denies history of abnormal Pap smears or STDs.,OBSTETRICAL HISTORY:  Gravida 1 was a term spontaneous vaginal delivery, complicated only by increased blood pressures at the time of delivery.  Gravida 2 is current.,REVIEW OF SYSTEMS:  The 14-point review of systems was negative with the exception as noted in the HPI.,PHYSICAL EXAMINATION:,VITAL SIGNS:  Blood pressure 134/45, pulse 130, respirations 28.  Oxygen saturation 100%.,GENERAL:  Patient lying quietly on a stretcher.  No acute distress.,HEENT:  Normocephalic, atraumatic.  Slightly dry mucous membranes.,CARDIOVASCULAR EXAM:  Regular rate and rhythm with tachycardia.,CHEST:  Clear to auscultation bilaterally.,ABDOMEN:  Soft, nontender, nondistended with positive bowel sounds.  No rebound or guarding.,SKIN:  Normal turgor.  No jaundice.  No rashes noted.,EXTREMITIES:  No clubbing, cyanosis, or edema.,NEUROLOGIC:  Cranial nerves II through XII grossly intact.,PSYCHIATRIC:  Flat affect.  Normal verbal response.,ASSESSMENT AND PLAN:  A 34-year-old Caucasian female, gravida 2 para 1-0-0-1, at unknown gestation who presents after suicide attempt.,1.  Given the substances taken, medications are unlikely to affect the development of the fetus.  There have been no reported human anomalies associated with Ambien or tramadol use.  There is, however, a 4% risk of congenital anomalies in the general population.,2.  Recommend quantitative HCG and transvaginal ultrasound for pregnancy dating.,3.  Recommend prenatal vitamins.,4.  The patient to follow up as an outpatient for routine prenatal care.,</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="n">
-        <v>717</v>
+        <v>418</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Emergency Room Reports; long; history and physical; diagnoses + symptoms + medications</t>
+          <t>Emergency Room Reports; medium; consultation; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J18" s="2" t="n">
-        <v>3818</v>
+        <v>3860</v>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>history and physical</t>
+          <t>consultation</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1569,17 +1565,17 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>0.7195671776375112</v>
+        <v>0.8509355275022543</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; imaging; past history; treatment plans; follow-up; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="19" ht="110" customHeight="1">
       <c r="A19" s="2" t="n">
-        <v>3859</v>
+        <v>3847</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
@@ -1588,58 +1584,62 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Consult - ICU Management </t>
+          <t xml:space="preserve"> Fiberoptic Bronchoscopy with Lavage </t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Consultation for ICU management for a patient with possible portal vein and superior mesenteric vein thrombus leading to mesenteric ischemia.</t>
+          <t xml:space="preserve"> Emergent fiberoptic bronchoscopy with lavage.   Status post multiple trauma/motor vehicle accident.  Acute respiratory failure.  Acute respiratory distress/ventilator asynchrony.  Hypoxemia.  Complete atelectasis of left lung.  Clots partially obstructing the endotracheal tube and completely obstructing the entire left main stem and entire left bronchial system.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>REASON FOR CONSULTATION: , ICU management.,HISTORY OF PRESENT ILLNESS: , The patient is a 43-year-old gentleman who presented from an outside hospital with complaints of right upper quadrant pain in the abdomen, which revealed possible portal vein and superior mesenteric vein thrombus leading to mesenteric ischemia.  The patient was transferred to the ABCD Hospital where he had a weeklong course with progressive improvement in his status after aggressive care including intubation, fluid resuscitation, and watchful waiting.  The patient clinically improved; however, his white count remained elevated with the intermittent fevers prompting a CT scan.  Repeat CT scan showed a loculated area of ischemic bowel with perforation in the left upper abdomen.  The patient was taken emergently to the operating room last night by the General Surgery Service where proximal half of the jejunum was noted to be liquified with 3 perforations.  This section of small bowel was resected, and a wound VAC placed for damage control.  Plan was to return the patient to the Operating Room tomorrow for further exploration and possible re-anastomosis of the bowel.  The patient is currently intubated, sedated, and on pressors for septic shock and in the down ICU.,PAST MEDICAL HISTORY:,  Prior to coming into the hospital for this current episode, the patient had hypertension, diabetes, and GERD.,PAST SURGICAL HISTORY:,  Included a cardiac cath with no interventions taken.,HOME MEDICATIONS:,  Include Lantus insulin as well as oral hypoglycemics.,CURRENT MEDS:,  Include Levophed, Ativan, fentanyl drips, cefepime, Flagyl, fluconazole, and vancomycin.  Nexium, Synthroid, hydrocortisone, and Angiomax, which is currently on hold.,REVIEW OF SYSTEMS:,  Unable to be obtained secondary to the patient's intubated and sedated status.,ALLERGIES: , None.,FAMILY HISTORY:,  Includes diabetes on his father side of the family.  No other information is provided.,SOCIAL HISTORY:,  Includes tobacco use as well as alcohol use.,PHYSICAL EXAMINATION:,GENERAL: The patient is currently intubated and sedated on Levophed drip.,VITAL SIGNS: Temperature is 100.6, systolic is 110/60 with MAP of 80, and heart rate is 120, sinus rhythm.,NEUROLOGIC: Neurologically, he is sedated, on Ativan with fentanyl drip as well.  He does arouse with suctioning, but is unable to open his eyes to commands.,HEAD AND NECK EXAMINATION: His pupils are equal, round, reactive, and constricted.  He has no scleral icterus.  His mucous membranes are pink, but dry.  He has an EG tube, which is currently 24-cm at the lip.  He has a left-sided subclavian vein catheter, triple lumen.,NECK: His neck is without masses or lymphadenopathy or JVD.,CHEST: Chest has diminished breath sounds bilaterally.,ABDOMEN: Abdomen is soft, but distended with a wound VAC in place.  Groins demonstrate a left-sided femoral outline.,EXTREMITIES: His bilateral upper extremities are edematous as well as his bilateral lower extremities; however, his right is more than it is in the left.  His toes are cool, and pulses are not palpable.,LABORATORY EXAMINATION: , Laboratory examination reveals an ABG of 7.34, CO2 of 30, O2 of 108, base excess of -8, bicarb of 16.1, sodium of 144, potassium of 6.5, chloride of 122, CO2 18, BUN 43, creatinine 2.0, glucose 172, calcium 6.6, phosphorus 1.1, mag 1.8, albumin is 1.6, cortisone level random is 22.  After stimulation with cosyntropin, they were still 22 and then 21 at 30 and 60 minutes respectively.  LFTs are all normal.  Amylase and lipase are normal.  Triglycerides are 73, INR is 2.2, PTT is 48.3, white count 20.7, hemoglobin 9.6, and platelets of 211.  UA was done, which also shows a specific gravity of 1.047, 1+ protein, trace glucose, large amount of blood, and many bacteria.  Chest x-rays performed and show the tip of the EG tube at level of the carina with some right upper lobe congestion, but otherwise clear costophrenic angles.  Tip of the left subclavian vein catheter is appropriate, and there is no pneumothorax noted.,ASSESSMENT AND PLAN:,  This is a 43-year-old gentleman who is acutely ill, in critical condition with mesenteric ischemia secondary to visceral venous occlusion.  He is status post small bowel resection.  We plan to go back to operating room tomorrow for further debridement and possible closure.  Neurologically, the patient initially had question of encephalopathy while in the hospital secondary to slow awakening after previous intubation; however, he did clear eventually, and was able to follow commands.  I did not suspect any sort of pathologic abnormality of his neurologic status as he has further CT scan of his brain, which was normal.  Currently, we will keep him sedated and on fentanyl drip to ease pain and facilitate ventilation on the respirator.  We will form daily sedation holidays to assess his neurologic status and avoid over sedating with Ativan.,1.  Cardiovascular.  The patient currently is in septic shock requiring vasopressors maintained on MAP greater than 70.  We will continue to try to wean the vasopressin after continued volume loading, also place SvO2 catheter to assess his oxygen delivery and consumption given his state of shock.  Currently, his rhythm is of sinus tachycardia, I do not suspect AFib or any other arrhythmia at this time.  If he does not improve as expected with volume resuscitation and with resolution of his sepsis, we will obtain an echocardiogram to assess his cardiac function.  Once he is off the vasopressors, we will try low-dose beta blockade as tolerated to reduce his rate.,2.  Pulmonology.  Currently, the patient is on full vent support with a rate of 20, tidal volume of 550, pressure support of 10, PEEP of 6, and FiO2 of 60.  We will wean his FiO2 as tolerated to keep his saturation greater than 90% and wean his PEEP as tolerated to reduce preload compromise.  We will keep the head of bed elevated and start chlorhexidine as swish and swallow for VAP prevention.,3.  Gastrointestinal.  The patient has known mesenteric venous occlusion secondary to the thrombus formation at the portal vein as well as the SMV.  He is status post immediate resection of jejunum leaving a blind proximal jejunum and blind distal jejunum.  We will maintain NG tube as he has a blind stump there, and we will preclude any further administration of any meds through this NG tube.  I will keep him on GI prophylaxis as he is intubated.  We will currently hold his TPN as he is undergoing a large amount of volume changes as well as he is undergoing electrolyte changes.  He will have a long-term TPN after this acute episode.  His LFTs are all normal currently.  Once he is postop tomorrow, we will restart the Angiomax for his venous occlusion.,4.  Renal.  The patient currently is in the acute renal insufficiency with anuria and an increase in his creatinine as well as his potassium.  His critical hyperkalemia which is requiring dosing of dextrose insulin, bicarb, and calcium; we will recheck his potassium levels after this cocktail.  He currently is started to make more urine since being volume resuscitated with Hespan as well as bicarb drip.  Hopefully given his increased urine output, he will start to eliminate some potassium and will not need dialysis.  We will re-consult Nephrology at this time.,5.  Endocrine.  The patient has adrenal insufficiency based on lack of stem to cosyntropin.  We will start hydrocortisone 50 q.6h.,6.  Infectious Disease.  Currently, the patient is on broad-spectrum antibiotic prophylaxis imperially.  Given his bowel ischemia, we will continue these, and appreciate ID service's input.,7.  Hematology.  Hematologically, the patient has a hypercoagulable syndrome, also had HIT secondary to his heparin administration.  We will restart the Angiomax once he is back from the OR tomorrow.  Currently, his INR is 2.2.  Therefore, he should be covered at the moment.  Appreciate the Hematology's input in this matter.,Please note the total critical care time spent at the bedside excluding central line placement was 1 hour.</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr"/>
+          <t>PREOPERATIVE DIAGNOSES:,1.  Status post multiple trauma/motor vehicle accident.,2.  Acute respiratory failure.,3.  Acute respiratory distress/ventilator asynchrony.,4.  Hypoxemia.,5.  Complete atelectasis of left lung.,POSTOPERATIVE DIAGNOSES:,1.  Status post multiple trauma/motor vehicle accident.,2.  Acute respiratory failure.,3.  Acute respiratory distress/ventilator asynchrony.,4.  Hypoxemia.,5.  Complete atelectasis of left lung.,6.  Clots partially obstructing the endotracheal tube and completely obstructing the entire left main stem and entire left bronchial system.,PROCEDURE PERFORMED: ,Emergent fiberoptic plus bronchoscopy with lavage.,LOCATION OF PROCEDURE:  ,ICU.  Room #164.,ANESTHESIA/SEDATION:,  Propofol drip, Brevital 75 mg, morphine 5 mg, and Versed 8 mg.,HISTORY,:  The patient is a 44-year-old male who was admitted to ABCD Hospital on 09/04/03 status post MVA with multiple trauma and subsequently diagnosed with multiple spine fractures as well as bilateral pulmonary contusions, requiring ventilatory assistance.  The patient was noted with acute respiratory distress on ventilator support with both ventilator asynchrony and progressive desaturation.  Chest x-ray as noted above revealed complete atelectasis of the left lung.  The patient was subsequently sedated and received one dose of paralytic as noted above followed by emergent fiberoptic flexible bronchoscopy.,PROCEDURE DETAIL,:  A bronchoscope was inserted through the oroendotracheal tube, which was partially obstructed with blood clots.  These were lavaged with several aliquots of normal saline until cleared.  The bronchoscope required removal because the tissue/clots were obstructing the bronchoscope.  The bronchoscope was reinserted on several occasions until cleared and advanced to the main carina.  The endotracheal tube was noted to be in good position.  The bronchoscope was advanced through the distal trachea.  There was a white tissue completely obstructing the left main stem at the carina.  The bronchoscope was advanced to this region and several aliquots of normal saline lavage were instilled and suctioned.  Again this partially obstructed the bronchoscope requiring several times removing the bronchoscope to clear the lumen.  The bronchoscope subsequently was advanced into the left mainstem and subsequently left upper and lower lobes.  There was diffuse mucus impactions/tissue as well as intermittent clots.  There was no evidence of any active bleeding noted.  Bronchoscope was adjusted and the left lung lavaged until no evidence of any endobronchial obstruction is noted.  Bronchoscope was then withdrawn to the main carina and advanced into the right bronchial system.  There is no plugging or obstruction of the right bronchial system.  The bronchoscope was then withdrawn to the main carina and slowly withdrawn as the position of endotracheal tube was verified, approximately 4 cm above the main carina.  The bronchoscope was then completely withdrawn as the patient was maintained on ventilator support during and postprocedure.  Throughout the procedure, pulse oximetry was greater than 95% throughout.  There is no hemodynamic instability or variability noted during the procedure.  Postprocedure chest x-ray is pending at this time.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">emergency room reports, multiple trauma, motor vehicle accident, acute respiratory failure, acute respiratory distress, ventilator asynchrony, hypoxemia, atelectasis, bronchoscopy, lavage, fiberoptic bronchoscopy, endotracheal tube, acute respiratory, asynchrony, bronchoscope, fiberoptic, endotracheal, bronchial, ventilatory, tube, respiratory, </t>
+        </is>
+      </c>
       <c r="G19" s="2" t="n">
-        <v>1258</v>
+        <v>440</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Emergency Room Reports; long; consultation; diagnoses + symptoms + medications</t>
+          <t>Emergency Room Reports; medium; procedure/operative; middle text complexity; diagnoses + medications + vital signs</t>
         </is>
       </c>
       <c r="J19" s="2" t="n">
-        <v>3859</v>
+        <v>3847</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>consultation</t>
+          <t>procedure/operative</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>higher</t>
+          <t>middle</t>
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0.9758791704238052</v>
+        <v>0.5204012623985572</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; follow-up; surgery; assessment/plan</t>
+          <t>diagnoses; medications; vital signs; procedures; imaging</t>
         </is>
       </c>
     </row>
     <row r="20" ht="110" customHeight="1">
       <c r="A20" s="2" t="n">
-        <v>3800</v>
+        <v>3808</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
@@ -1648,62 +1648,58 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Diabetes Mellitus - SOAP Note - 2 </t>
+          <t xml:space="preserve"> Acute Cystitis &amp; Diabetes Type II </t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Patient today with ongoing issues with diabetic control.</t>
+          <t xml:space="preserve"> The patient complaining of abdominal pain, has a long-standing history of diabetes treated with Micronase daily.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>SUBJECTIVE:,  I am asked to see the patient today with ongoing issues around her diabetic control.  We have been fairly aggressively, downwardly adjusting her insulins, both the Lantus insulin, which we had been giving at night as well as her sliding scale Humalog insulin prior to meals.  Despite frequent decreases in her insulin regimen, she continues to have somewhat low blood glucoses, most notably in the morning when the glucoses have been in the 70s despite decreasing her Lantus insulin from around 84 units down to 60 units, which is a considerable change.  What I cannot explain is why her glucoses have not really climbed at all despite the decrease in insulin.  The staff reports to me that her appetite is good and that she is eating as well as ever.  I talked to Anna today.  She feels a little fatigued.  Otherwise, she is doing well.,PHYSICAL EXAMINATION:  ,Vitals as in the chart.  The patient is a pleasant and cooperative.  She is in no apparent distress.,ASSESSMENT AND PLAN: , Diabetes, still with some problematic low blood glucoses, most notably in the morning.  To address this situation, I am going to hold her Lantus insulin tonight and decrease and then change the administration time to in the morning.  She will get 55 units in the morning.  I am also decreasing once again her Humalog sliding scale insulin prior to meals.  I will review the blood glucoses again next week.,</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>endocrinology, diabetic control, insulin prior to meals, low blood glucoses, sliding scale, lantus insulin, diabetes, mellitus, lantus, glucoses,</t>
-        </is>
-      </c>
+          <t>HISTORY OF PRESENT ILLNESS: , The patient is a 45-year-old male complaining of abdominal pain.  The patient also has a long-standing history of diabetes which is treated with Micronase daily.,PAST MEDICAL HISTORY: , There is no significant past medical history noted today.,PHYSICAL EXAMINATION:,HEENT:  Patient denies ear abnormalities, nose abnormalities and throat abnormalities.,Cardio:  Patient has history of elevated cholesterol, but does not have ASHD, hypertension and PVD.,Resp:  Patient denies asthma, lung infections and lung lesions.,GI:  Patient denies colon abnormalities, gall bladder problems, liver abnormalities and peptic ulcer disease.,GU:  Patient has history of Urinary tract disorder, but does not have Bladder disorder and Kidney disorder.,Endocrine:  Patient has history of diabetes, but does not have hormonal irregularities and thyroid abnormalities.,Dermatology:  Patient denies allergic reactions, rashes and skin lesions.,MEDS:,  Micronase 2.5 mg Tab PO QAM #30.  Bactrim 400/80 Tab PO BID #30.,SOCIAL HISTORY:,  No known history of drug or alcohol abuse.  Work, diet, and exercise patterns are within normal limits.,FAMILY HISTORY:,  No significant family history.,REVIEW OF SYSTEMS:,  Non-contributory.,Vital Signs:  Height = 72 in.  Weight =184 lbs.  Upright BP = 120/80 mmHg.  Pulse = 80 bpm.  Resp =12 pm.  Patient is afebrile.,Neck:  The neck is supple.  There is no jugular venous distension.  The thyroid is nontender, or normal size and conto.,Lungs:  Lung expansion and excursions are symmetric.  The lungs are clear to auscultation and percussion.,Cardio:  There is a regular rhythm.  SI and S2 are normal.  No abnormal heart sounds are detected.  Blood pressure is equal bilaterally.,Abdomen:  Normal bowel sounds are present.  The abdomen is soft; The abdomen is nontender; without organomegaly; There is no CVA tenderness.  No hernias are noted.,Extremities:  There is no clubbing, cyanosis, or edema.,ASSESSMENT: , Diabetes type II uncontrolled.  Acute cystitis.,PLAN: , Endocrinology Consult, complete CBC.  ,RX: , Micronase 2.5 mg Tab PO QAM #30, Bactrim 400/80 Tab PO BID #30.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="n">
-        <v>237</v>
+        <v>299</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Endocrinology; short; SOAP-style; diagnoses + treatment plans + assessment/plan</t>
+          <t>Endocrinology; medium; other narrative/sectioned; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J20" s="2" t="n">
-        <v>3800</v>
+        <v>3808</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>SOAP-style</t>
+          <t>other narrative/sectioned</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>middle</t>
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>0.1243800721370604</v>
+        <v>0.5951307484220019</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; treatment plans; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; past history; treatment plans; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="21" ht="110" customHeight="1">
       <c r="A21" s="2" t="n">
-        <v>3798</v>
+        <v>3805</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
@@ -1712,26 +1708,26 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Post Hemithyroidectomy </t>
+          <t xml:space="preserve"> Completion Thyroidectomy </t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The patient with left completion hemithyroidectomy and reimplantation of the left parathyroid and left sternocleidomastoid region in the inferior 1/3rd region.  Papillary carcinoma of the follicular variant of the thyroid in the right lobe, status post right hemithyroidectomy.</t>
+          <t xml:space="preserve"> Completion thyroidectomy with limited right paratracheal node dissection.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>PREOPERATIVE DIAGNOSES: , Papillary carcinoma of the follicular variant of the thyroid in the right lobe, status post right hemithyroidectomy.,POSTOPERATIVE DIAGNOSES: , Papillary carcinoma of the follicular variant of the thyroid in the right lobe, status post right hemithyroidectomy.,PROCEDURE:  ,The patient with left completion hemithyroidectomy and reimplantation of the left parathyroid and left sternocleidomastoid region in the inferior 1/3rd region.,FINDINGS: , Normal-appearing thyroid gland with a possible lump in the inferior aspect, there was a parathyroid gland that by frozen section _________  was not thyroid, it was reimplanted to the left lower sternocleidomastoid region.,ESTIMATED BLOOD LOSS:  ,Approximately 10 mL.,FLUIDS: , Crystalloid only.,COMPLICATIONS: , None.,DRAINS: , Rubber band drain in the neck.,CONDITION:,  Stable.,PROCEDURE:  ,The patient placed supine under general anesthesia.  First, a shoulder roll was placed, 1% lidocaine and 1:100,000 epinephrine was injected into the old scar, natural skin fold, and Betadine prep.  Sterile dressing was placed.  The laryngeal monitoring was noted to be working fine.  Then, an incision was made in this area in a curvilinear fashion through the old scar, taken through the fat and the platysma level.  The strap muscles were found and there was scar tissue along the trachea and the strap muscles were elevated off of the left thyroid, the thyroid gland was then found.  Then, using bipolar cautery and a Coblation dissector, the thyroid gland inferiorly was dissected off and the parathyroid gland was left inferiorly and there was scar tissue that was released and laterally, the thyroid gland was released, then came into the Berry ligaments.  The Berry ligament was dissected off and the gland came off all the way to the superior and inferior thyroid vessels, which were crossed with the Harmonic scalpel and removed.  No bleeding was seen.  There was a small nick in the external jugular vein that was tied with a 4-0 Vicryl suture ligature.  After this was completed, on examining the specimen, there appeared to be a lobule on it and it was sent off as possibly parathyroid, therefore it was reimplanted in the left lower sternocleidomastoid region using the silk suture ligature.  After this was completed, no bleeding was seen.  The laryngeal nerve could be seen and intact and then Rubber band  drain was placed throughout the neck along the thyroid bed and 4-0 Vicryl was used to close the strap muscles in an interrupted fashion along with the platysma region and subcutaneous region and a running 5-0 nylon was used to close the skin and Mastisol and Steri-Strips were placed along the skin edges and then on awakening, both laryngeal nerves were working normally.  Procedure was then terminated at that time.</t>
+          <t>TITLE OF OPERATION:,  Completion thyroidectomy with limited right paratracheal node dissection.,INDICATION FOR SURGERY:,  A 49-year-old woman with a history of a left dominant nodule in her thyroid gland, who subsequently underwent left thyroid lobectomy and isthmusectomy, was found to have multifocal papillary thyroid carcinoma throughout her left thyroid lobe and isthmus.  Consideration given to completion thyroidectomy.  Risks, benefits, and alternatives of this procedure was discussed with the patient in great detail.  Risks included but were not limited to anesthesia, bleeding, infection, injury to nerves including vocal fold paralysis, hoarseness, low calcium, scar, cosmetic deformity, need for thyroid hormone replacement, and also need for further management.  The patient understood all of this and then wished to proceed.,PREOP DIAGNOSIS:,  Multifocal thyroid carcinoma and previous left thyroid lobectomy resection specimen.,POSTOP DIAGNOSIS: , Multifocal thyroid carcinoma and previous left thyroid lobectomy resection specimen.,PROCEDURE DETAIL:,  After identifying the patient, the patient was placed supine in the operating room table.  After establishment of general anesthesia via orotracheal intubation with a number 6 nerve integrity monitoring system endotracheal tube, the eyes were protected with Tegaderm.  Nerve integrity monitoring system endotracheal tube was confirmed to be working adequately and secured.  The previous skin incision for a thyroidectomy was then planned, then incorporated into an ellipse.  The patient was prepped and draped in a sterile fashion.  Subsequently, the ellipse around the previous incision was deformed.  The scar was then excised.  Subplatysmal flaps were raised to the thyroid notch and sternal notch respectively.  Strap muscles were isolated in the midline and dissected and mobilized from the thyroid lobe on the right side.  There was some dense fibrosis and inflammation surrounding the right thyroid lobe.  Careful dissection along the thyroid lobe allowed for identification of the superior thyroid artery and vein which were individually ligated with a Harmonic scalpel.  The right inferior and superior parathyroid glands were identified and preserved and recurrent laryngeal nerve was identified and traced superiorly, then preserved.  Of note is that there were multiple lymph nodes in the paratracheal region on the right side.  These lymph nodes were carefully dissected away from the recurrent laryngeal nerve, trachea, and the carotid artery, and sent as a separate specimen labeled right paratracheal lymph nodes.  The wound was copiously irrigated.  Valsalva maneuver was given.  Surgicel was placed in the wound bed.  Strap muscles were reapproximated in the midline with 3-0 Vicryl and incision was then closed with interrupted 3-0 Vicryl and Indermil for the skin.  The patient was extubated in the operating room table, sent to the postanesthesia care unit in good condition.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>endocrinology, thyroid, rubber band drain, berry ligaments, papillary carcinoma, follicular variant, strap muscles, thyroid gland, sternocleidomastoid, parathyroid, hemithyroidectomy,</t>
+          <t xml:space="preserve">endocrinology, multifocal thyroid carcinoma, thyroid lobectomy, thyroid, papillary, thyroid lobe, isthmus, completion thyroidectomy, thyroidectomy, paratracheal, lobectomy, </t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>434</v>
+        <v>423</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1740,15 +1736,15 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Endocrinology; medium; procedure/operative; diagnoses + procedures + surgery</t>
+          <t>Endocrinology; medium; other narrative/sectioned; middle text complexity; diagnoses + procedures + past history</t>
         </is>
       </c>
       <c r="J21" s="2" t="n">
-        <v>3798</v>
+        <v>3805</v>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>procedure/operative</t>
+          <t>other narrative/sectioned</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -1757,17 +1753,17 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>0.4576758340847611</v>
+        <v>0.4482078449053201</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; procedures; surgery</t>
+          <t>diagnoses; procedures; past history; treatment plans; surgery</t>
         </is>
       </c>
     </row>
     <row r="22" ht="110" customHeight="1">
       <c r="A22" s="2" t="n">
-        <v>3797</v>
+        <v>3811</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
@@ -1776,39 +1772,43 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Thyroid Mass Consult </t>
+          <t xml:space="preserve"> Acquired Hypothyroidism Followup </t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Thyroid mass diagnosed as papillary carcinoma.  The patient is a 16-year-old young lady with a history of thyroid mass that is now biopsy proven as papillary.  The pattern of miliary metastatic lesions in the chest is consistent with this diagnosis.</t>
+          <t xml:space="preserve"> Return visit to the endocrine clinic for acquired hypothyroidism, papillary carcinoma of the thyroid gland status post total thyroidectomy in 1992, and diabetes mellitus.</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>REASON FOR CONSULTATION: , Thyroid mass diagnosed as papillary carcinoma.,HISTORY OF PRESENT ILLNESS:  ,The patient is a 16-year-old young lady, who was referred from the Pediatric Endocrinology Department by Dr. X for evaluation and surgical recommendations regarding treatment of a mass in her thyroid, which has now been proven to be papillary carcinoma on fine needle aspiration biopsy.  The patient's parents relayed that they first noted a relatively small but noticeable mass in the middle portion of her thyroid gland about 2004.  An ultrasound examination had reportedly been done in the past and the mass is being observed.  When it began to enlarge recently, she was referred to the Pediatric Endocrinology Department and had an evaluation there.  The patient was referred for fine needle aspiration and the reports recently returned a diagnosis of papillary thyroid carcinoma.  The patient has not had any hoarseness, difficulty swallowing, or any symptoms of endocrine dysfunction.  She has no weight changes consistent with either hyper or hypothyroidism.  There is no family history of thyroid cancer in her family.  She has no notable discomfort with this lesion.  There have been no skin changes.  Historically, she does not have a history of any prior head and neck radiation or treatment of any unusual endocrinopathy.,PAST MEDICAL HISTORY:,  Essentially unremarkable.  The patient has never been hospitalized in the past for any major illnesses.  She has had no prior surgical procedures.,IMMUNIZATIONS: , Current and up to date.,ALLERGIES: , She has no known drug allergies.,CURRENT MEDICATIONS:  ,Currently taking no routine medications.  She describes her pain level currently as zero.,FAMILY HISTORY: , There is no significant family history, although the patient's father does note that his mother had a thyroid surgery at some point in life, but it was not known whether this was for cancer, but he suspects it might have been for goiter.  This was done in Tijuana.  His mom is from central portion of Mexico.  There is no family history of multiple endocrine neoplasia syndromes.,SOCIAL HISTORY:  ,The patient is a junior at Hoover High School.  She lives with her mom in Fresno.,REVIEW OF SYSTEMS: , A careful 12-system review was completely normal except for the problems related to the thyroid mass.,PHYSICAL EXAMINATION:,GENERAL:  The patient is a 55.7 kg, nondysmorphic, quiet, and perhaps slightly apprehensive young lady, who was in no acute distress.  She was alert and oriented x3 and had an appropriate affect.,HEENT:  The head and neck examination is most significant.  There is mild amount of facial acne.  The patient's head, eyes, ears, nose, and throat appeared to be grossly normal.,NECK:  There is a slightly visible midline bulge in the region of the thyroid isthmus.  A firm nodule is present there, and there is also some nodularity in the right lobe of the thyroid.  This mass is relatively hard, slightly fixed, but not tethered to surrounding tissues, skin, or muscles that I can determine.  There are some shotty adenopathy in the area.  No supraclavicular nodes were noted.,CHEST:  Excursions are symmetric with good air entry.,LUNGS:  Clear.,CARDIOVASCULAR:  Normal.  There is no tachycardia or murmur noted.,ABDOMEN:  Benign.,EXTREMITIES:  Extremities are anatomically correct with full range of motion.,GENITOURINARY:  External genitourinary exam was deferred at this time and can be performed later during anesthesia.  This is same as too for her rectal examination.,SKIN:  There is no acute rash, purpura, or petechiae.,NEUROLOGIC:  Normal and no focal deficits.  Her voice is strong and clear.  There is no evidence of dysphonia or vocal cord malfunction.,DIAGNOSTIC STUDIES: , I reviewed laboratory data from the Diagnostics Lab, which included a mild abnormality in the AST at 11, which is slightly lower than the normal range.  T4 and TSH levels were recorded as normal.  Free thyroxine was normal, and the serum pregnancy test was negative.  There was no level of thyroglobulin recorded on this.  A urinalysis and comprehensive metabolic panel was unremarkable.  A chest x-ray was obtained, which I personally reviewed.  There is a diffuse pattern of tiny nodules in both lungs typical of miliary metastatic disease that is often seen in patients with metastatic thyroid carcinoma.,IMPRESSION/PLAN: , The patient is a 16-year-old young lady with a history of thyroid mass that is now biopsy proven as papillary.  The pattern of miliary metastatic lesions in the chest is consistent with this diagnosis and is unfortunate in that it generally means a more advanced stage of disease.  I spent approximately 30 minutes with the patient and her family today discussing the surgical aspects of the treatment of this disease.  During this time, we talked about performing a total thyroidectomy to eradicate as much of the native thyroid tissue and remove the primary source of the cancer in anticipation of radioactive iodine therapy.  We talked about sentinel node dissection, and we spent significant amount of time talking about the possibility of hypoparathyroidism if all four of the parathyroid glands were damaged during this operation.  We also discussed the recurrent laryngeal and external laryngeal branches of the nerve supplying the vocal cord function and how they cane be damaged during the thyroidectomy as well.  I answered as many of the family's questions as they could mount during this stressful time with this recent information supplied to them.  I also did talk to them about the chest x-ray pattern, which was complete __________ as the film was just on the day prior to my clinic visit.  This will have some impact on the postoperative adjunctive therapy.  The radiologist commented about the risk of pulmonary fibrosis and the use of radioactive iodine in this situation, but it seems likely that is going to be necessary to attempt to treat this disease in the patient's case.  I did discuss with them the possibility of having to take large doses of calcium and vitamin D in the event of hypoparathyroidism if that does happen, and we also talked about possibly sparing parathyroid tissue and reimplanting it in a muscle belly either in the neck or forearm if that becomes a necessity.  All of the family's questions have been answered.  This is a very anxious and anxiety provoking time in the family.  I have made every effort to get the patient under schedule within the next 48 hours to have this operation done.  We are tentatively planning on proceeding this upcoming Friday afternoon with total thyroidectomy.</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr"/>
+          <t>PROBLEM LIST:,1.  Acquired hypothyroidism.,2.  Papillary carcinoma of the thyroid gland, status post total thyroidectomy in 1992.,3.  Diabetes mellitus.,4.  Insomnia with sleep apnea.,HISTORY OF PRESENT ILLNESS: , This is a return visit to the endocrine clinic for the patient with history as noted above.  She is 45 years old.  Her last visit was about 6 months ago.  Since that time, the patient states her health has remained unchanged.  Currently, primary complaint is one of fatigue that she feels throughout the day.  She states, however, she is doing well with CPAP and wakes up feeling refreshed but tends to tire out later in the day.  In terms of her thyroid issues, the patient states that she is not having signs or symptoms of thyroid excess or hypothyroidism.  She is not reporting temperature intolerance, palpitations, muscle weakness, tremors, nausea, vomiting, constipation, hyperdefecation or diarrhea.  Her weight has been stable.  She is not reporting proximal muscle weakness.,CURRENT MEDICATIONS:,1.  Levothyroxine 125 micrograms p.o. once daily.,2.  CPAP.,3.  Glucotrol.,4.  Avandamet.,5.  Synthroid.,6.  Byetta injected twice daily.,REVIEW OF SYSTEMS: , As stated in the HPI.  She is not reporting polyuria, polydipsia or polyphagia.  She is not reporting fevers, chills, sweats, visual acuity changes, nausea, vomiting, constipation or diarrhea.  She is not having any lightheadedness, weakness, chest pain, shortness of breath, difficulty breathing, orthopnea or dyspnea on exertion.,PHYSICAL EXAMINATION:,GENERAL:  She is an overweight, very pleasant woman, in no acute distress.  VITAL SIGNS:  Temperature 96.9, pulse 85, respirations not counted, blood pressure 135/65, and weight 85.7 kg.  NECK:  Reveals well healed surgical scar in the anteroinferior aspect of the neck.  There is no palpable thyroid tissue noted on this examination today.  There is no lymphadenopathy.  THORAX:  Reveals lungs that are clear, PA and lateral, without adventitious sounds.  CARDIOVASCULAR:  Demonstrated regular rate and rhythm.  S1 and S2 without murmur.  No S3, no S4 is auscultated.  EXTREMITIES:  Deep tendon reflexes 2+/4 without a delayed relaxation phase.  No fine resting tremor of the outstretched upper extremity.  SKIN, HAIR, AND NAILS:  All are unremarkable.,LABORATORY DATABASE: , Lab data on 08/29/07 showed the following:  Thyroglobulin quantitative less than 0.5 and thyroglobulin antibody less than 20, free T4 1.35, and TSH suppressed at 0.121.,ASSESSMENT AND PLAN:,This is a 45-year-old woman with history as noted above.,1.  Acquired hypothyroidism, status post total thyroidectomy for papillary carcinoma in 1992.,2.  Plan to continue following thyroglobulin levels.,3.  Plan to obtain a free T4, TSH, and thyroglobulin levels today.,4.  Have the patient call the clinic next week for followup and continued management of her hypothyroid state.,5.  Plan today is to repeat her thyroid function studies.  This case was discussed with Dr. X and the recommendation.  We are giving the patient today is for us to taper her medication to get her TSH somewhere between 0.41 or less.  Therefore, labs have been drawn.  We plan to see the patient back in approximately 6 months or sooner.  A repeat body scan will not been done, the one in 03/06 was negative.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">endocrinology, thyroid function studies, thyroid gland, diabetes mellitus, papillary carcinoma, total thyroidectomy, acquired hypothyroidism, carcinoma, thyroidectomy, thyroglobulin, hypothyroidism, </t>
+        </is>
+      </c>
       <c r="G22" s="2" t="n">
-        <v>1037</v>
+        <v>486</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Endocrinology; long; consultation; diagnoses + symptoms + medications</t>
+          <t>Endocrinology; medium; follow-up/progress; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J22" s="2" t="n">
-        <v>3797</v>
+        <v>3811</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>consultation</t>
+          <t>follow-up/progress</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -1817,17 +1817,17 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>0.8055117222723174</v>
+        <v>0.8002705139765555</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; procedures; imaging; past history; treatment plans; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; laboratory values; vital signs; past history; treatment plans; follow-up; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="23" ht="110" customHeight="1">
       <c r="A23" s="2" t="n">
-        <v>3604</v>
+        <v>3608</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
@@ -1836,39 +1836,39 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CT Abdomen &amp; Pelvis - 5 </t>
+          <t xml:space="preserve"> CT Abdomen &amp; Pelvis </t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  CT abdomen without contrast and pelvis without contrast, reconstruction.</t>
+          <t xml:space="preserve"> CT Abdomen &amp; Pelvis W&amp;WO Contrast</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>EXAM: , CT abdomen without contrast and pelvis without contrast, reconstruction.,REASON FOR EXAM: , Right lower quadrant pain, rule out appendicitis.,TECHNIQUE:  ,Noncontrast CT abdomen and pelvis.  An intravenous line could not be obtained for the use of intravenous contrast material.,FINDINGS: , The appendix is normal.  There is a moderate amount of stool throughout the colon.  There is no evidence of a small bowel obstruction or evidence of pericolonic inflammatory process.  Examination of the extreme lung bases appear clear, no pleural effusions.  The visualized portions of the liver, spleen, adrenal glands, and pancreas appear normal given the lack of contrast.  There is a small hiatal hernia.  There is no intrarenal stone or evidence of obstruction bilaterally.  There is a questionable vague region of low density in the left anterior mid pole region, this may indicate a tiny cyst, but it is not well seen given the lack of contrast.  This can be correlated with a followup ultrasound if necessary.  The gallbladder has been resected.  There is no abdominal free fluid or pathologic adenopathy.  There is abdominal atherosclerosis without evidence of an aneurysm.,Dedicated scans of the pelvis disclosed phleboliths, but no free fluid or adenopathy.  There are surgical clips present.  There is a tiny airdrop within the bladder.  If this patient has not had a recent catheterization, correlate for signs and symptoms of urinary tract infection.,IMPRESSION:,1.Normal appendix.,2.Moderate stool throughout the colon.,3.No intrarenal stones.,4.Tiny airdrop within the bladder.  If this patient has not had a recent catheterization, correlate for signs and symptoms of urinary tract infection.  The report was faxed upon dictation.</t>
+          <t>EXAM:,  CT Abdomen &amp; Pelvis W&amp;WO Contrast, ,REASON FOR EXAM: , Status post aortobiiliac graft repair. , ,TECHNIQUE: , 5 mm spiral thick spiral CT scanning was performed through the entire abdomen and pelvis utilizing intravenous dynamic bolus contrast enhancement.  No oral or rectal contrast was utilized.  Comparison is made with the prior CT abdomen and pelvis dated 10/20/05.  There has been no significant change in size of the abdominal aortic aneurysm centered roughly at the renal artery origin level which has dimensions of 3.7 cm transversely x 3.4 AP.  Just below this level is the top of the endoluminal graft repair with numerous surrounding surgical clips.  The size of the native aneurysm component at this level is stable at 5.5 cm in diameter with mural thrombus surrounding the enhancing endolumen.  There is no abnormal entrance of contrast agent into the mural thrombus to indicate an endoluminal leak.  Further distally, there is extension of the graft into both proximal common iliac arteries without evidence for endoluminal leak at this level either.  No exoluminal leakage is identified at any level.  There is no retroperitoneal hematoma present.  The findings are unchanged from the prior exam.  ,The liver, spleen, pancreas, adrenals and right kidney are unremarkable with moderate diffuse atrophy of the pancreas present.  There is advanced atrophy of the left kidney.  No hydronephrosis is present.  No acute findings are identified elsewhere in the abdomen. ,The lung bases are clear. ,Concerning the remainder of the pelvis, no acute pathology is identified.  There is prominent streak artifact from the left total hip replacement.  There is diffuse moderate sigmoid diverticulosis without evidence for diverticulitis.  The bladder grossly appears normal.  A hysterectomy has been performed.  ,IMPRESSION:,1.  No complications identified regarding endoluminal aortoiliac graft repair as described.  The findings are stable compared to the study of 10/20/04.  ,2.  Stable mild aneurysm of aortic aneurysm, centered roughly at renal artery level.  ,3.  No other acute findings noted. ,4.  Advanced left renal atrophy.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>gastroenterology, reconstruction, appendicitis, urinary tract infection, ct abdomen, abdomen, ct, pelvis, contrast, noncontrast,</t>
+          <t>gastroenterology, aortobiiliac graft repair, renal atrophy, ct abdomen &amp; pelvis, w&amp;wo contrast, aortic aneurysm, renal artery, mural thrombus, endoluminal leak, ct abdomen, ct, contrast, pelvis, abdomen,</t>
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>259</v>
+        <v>324</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Gastroenterology; short; diagnostic report; diagnoses + symptoms + procedures</t>
+          <t>Gastroenterology; medium; diagnostic report; lower text complexity; diagnoses + imaging + surgery</t>
         </is>
       </c>
       <c r="J23" s="2" t="n">
-        <v>3604</v>
+        <v>3608</v>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
@@ -1881,17 +1881,17 @@
         </is>
       </c>
       <c r="M23" s="2" t="n">
-        <v>0.3426510369702435</v>
+        <v>0.3290126239855726</v>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; procedures; imaging; follow-up; surgery</t>
+          <t>diagnoses; imaging; surgery</t>
         </is>
       </c>
     </row>
     <row r="24" ht="110" customHeight="1">
       <c r="A24" s="2" t="n">
-        <v>3472</v>
+        <v>3685</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
@@ -1900,22 +1900,26 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Rectal Bleeding - 1-year-old </t>
+          <t xml:space="preserve"> Admission History &amp; Physical - Nausea </t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Pediatric Gastroenterology - Rectal Bleeding Consult.</t>
+          <t xml:space="preserve"> Patient status post gastric bypass surgery, developed nausea and right upper quadrant pain.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS:,  This is a 1-year-old male patient who was admitted on 12/23/2007 with a history of rectal bleeding.  He was doing well until about 2 days prior to admission and when he passes hard stools, there was bright red blood in the stool.  He had one more episode that day of stool; the stool was hard with blood in it.  Then, he had one episode of rectal bleeding yesterday and again one stool today, which was soft and consistent with dark red blood in it.  No history of fever, no diarrhea, no history of easy bruising.  Excessive bleeding from minor cut.  He has been slightly fussy.,PAST MEDICAL HISTORY:  ,Nothing significant.,PREGNANCY DELIVERY AND NURSERY COURSE: , He was born full term without complications.,PAST SURGICAL HISTORY: , None.,SIGNIFICANT ILLNESS AND REVIEW OF SYSTEMS: , Negative for heart disease, lung disease, history of cancer, blood pressure problems, or bleeding problems.,DIET:,  Regular table food, 24 ounces of regular milk.  He is n.p.o. now.,TRAVEL HISTORY: , Negative.,IMMUNIZATION: , Up-to-date.,ALLERGIES: , None.,MEDICATIONS: , None, but he is on IV Zantac now.,SOCIAL HISTORY: , He lives with parents and siblings.,FAMILY HISTORY:,  Nothing significant.,LABORATORY EVALUATION: , On 12/24/2007, WBC 8.4, hemoglobin 7.6, hematocrit 23.2 and platelets 314,000.  Sodium 135, potassium 4.7, chloride 110, CO2 20, BUN 6 and creatinine 0.3.  Albumin 3.3.  AST 56 and ALT 26.  CRP less than 0.3.  Stool rate is still negative.,DIAGNOSTIC DATA: , CT scan of the abdomen was read as normal.,PHYSICAL EXAMINATION:  ,VITAL SIGNS:  Temperature 99.5 degrees Fahrenheit, pulse 142 per minute and respirations 28 per minute.  Weight 9.6 kilogram.,GENERAL:  He is alert and active child in no apparent distress.,HEENT:  Atraumatic and normocephalic.  Pupils are equal, round and reactive to light.  Extraocular movements, conjunctivae and sclerae fair.  Nasal mucosa pink and moist.  Pharynx is clear.,NECK:  Supple without thyromegaly or masses.,LUNGS:  Good air entry bilaterally.  No rales or wheezing.,ABDOMEN:  Soft and nondistended.  Bowel sounds positive.  No mass palpable.,GENITALIA:  Normal male.,RECTAL:  Deferred, but there was no perianal lesion.,MUSCULOSKELETAL:  Full range of movement.  No edema.  No cyanosis.,CNS:  Alert, active and playful.,IMPRESSION: , A 1-year-old male patient with history of rectal bleeding.  Possibilities include Meckel's diverticulum, polyp, infection and vascular malformation.,PLAN:,  To proceed with Meckel scan today.  If Meckel scan is negative, we will consider upper endoscopy and colonoscopy.  We will start colon clean out if Meckel scan is negative.  We will send his stool for C. diff toxin, culture, blood for RAST test for cow milk, soy, wheat and egg.  Monitor hemoglobin.</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr"/>
+          <t>CHIEF COMPLAINT: , Nausea.,PRESENT ILLNESS: , The patient is a 28-year-old, who is status post gastric bypass surgery nearly one year ago.  He has lost about 200 pounds and was otherwise doing well until yesterday evening around 7:00-8:00 when he developed nausea and right upper quadrant pain, which apparently wrapped around toward his right side and back.  He feels like he was on it but has not done so.  He has overall malaise and a low-grade temperature of 100.3.  He denies any prior similar or lesser symptoms.  His last normal bowel movement was yesterday.  He denies any outright chills or blood per rectum.,PAST MEDICAL HISTORY: , Significant for hypertension and morbid obesity, now resolved.,PAST SURGICAL HISTORY: , Gastric bypass surgery in December 2007.,MEDICATIONS:  ,Multivitamins and calcium.,ALLERGIES: , None known.,FAMILY HISTORY:  ,Positive for diabetes mellitus in his father, who is now deceased.,SOCIAL HISTORY: , He denies tobacco or alcohol.  He has what sounds like a data entry computer job.,REVIEW OF SYSTEMS:  ,Otherwise negative.,PHYSICAL EXAMINATION:,  His temperature is 100.3, blood pressure 129/59, respirations 16, heart rate 84.  He is drowsy, but easily arousable and appropriate with conversation.  He is oriented to person, place, and situation.  He is normocephalic, atraumatic.  His sclerae are anicteric.  His mucous membranes are somewhat tacky.  His neck is supple and symmetric.  His respirations are unlabored and clear.  He has a regular rate and rhythm.  His abdomen is soft.  He has diffuse right upper quadrant tenderness, worse focally, but no rebound or guarding.  He otherwise has no organomegaly, masses, or abdominal hernias evident.  His extremities are symmetrical with no edema.  His posterior tibial pulses are palpable and symmetric.  He is grossly nonfocal neurologically.,STUDIES:,  His white blood cell count is 8.4 with 79 segs.  His hematocrit is 41.  His electrolytes are normal.  His bilirubin is 2.8.  His AST 349, ALT 186, alk-phos 138 and lipase is normal at 239.,ASSESSMENT: , Choledocholithiasis, ? cholecystitis.,PLAN: , He will be admitted and placed on IV antibiotics.  We will get an ultrasound this morning.  He will need his gallbladder out, probably with intraoperative cholangiogram.  Hopefully, the stone will pass this way.  Due to his anatomy, an ERCP would prove quite difficult if not impossible unless laparoscopic assisted.  Dr. X will see him later this morning and discuss the plan further.  The patient understands.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gastroenterology, gastric bypass surgery, nausea, choledocholithiasis, cholecystitis, ercp, gastric bypass, bypass surgery, </t>
+        </is>
+      </c>
       <c r="G24" s="2" t="n">
-        <v>410</v>
+        <v>379</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -1924,15 +1928,15 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Gastroenterology; medium; other narrative/sectioned; diagnoses + symptoms + medications</t>
+          <t>Gastroenterology; medium; history and physical; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>3472</v>
+        <v>3685</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>other narrative/sectioned</t>
+          <t>history and physical</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -1941,17 +1945,17 @@
         </is>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0.800777727682597</v>
+        <v>0.7628494138863842</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; imaging; past history; treatment plans; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="25" ht="110" customHeight="1">
       <c r="A25" s="2" t="n">
-        <v>3525</v>
+        <v>3606</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
@@ -1960,58 +1964,62 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> GI Consultation - 3 </t>
+          <t xml:space="preserve"> CT Abdomen &amp; Pelvis - 3 </t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> GI Consultation for Chrohn's disease.</t>
+          <t xml:space="preserve"> CT of the abdomen and pelvis without contrast.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>PROBLEM:  ,Prescription evaluation for Crohn's disease., ,HISTORY: , This is a 46-year-old male who is here for a refill of Imuran.  He is taking it at a dose of 100 mg per day.  He is status post resection of the terminal ileum and has experienced intermittent obstructive symptoms for the past several years.  In fact, he had an episode three weeks ago in which he was seen at the emergency room after experiencing sudden onset of abdominal pain and vomiting. An x-ray was performed, which showed no signs of obstruction per his report.  He thinks that the inciting factor of this incident was too many grapes eaten the day before.  He has had similar symptoms suggestive of obstruction when eating oranges or other high-residue fruits in the past.  The patient's normal bowel pattern is loose stools and this is unchanged recently.  He has not had any rectal bleeding. He asks today about a rope-like vein on his anterior right arm that has been a little tender and enlarged after he was in the emergency room and they had difficulty with IV insertion.  He has not had any fever, red streaking up the arm, or enlargement of lymph nodes.  The tenderness has now completely resolved.  , ,He had a colonoscopy performed in August of 2003, by Dr. S.  An anastomotic stricture was found at the terminal ileum/cecum junction.  Dr. S recommended that if the patient experienced crampy abdominal pain or other symptoms of obstruction, that he may consider balloon dilation.  No active Crohn's disease was found during the colonoscopy.  , ,Earlier this year, he experienced a non-specific hepatitis with elevation of his liver function tests.  At that time he was taking a lot of Tylenol for migraine-type headaches.  Under Dr. S's recommendation, he stopped the Imuran for one month and reduced his dose of Tylenol.  Since that time his liver enzymes have normalized and he has restarted the Imuran with no problems.  , ,He also reports heartburn that is occurring on a slightly more frequent basis than it has in the past.  It used to occur once a week only, but has now increased in frequency to twice a week.  He takes over-the-counter H2 blockers as needed, as well as Tums.  He associates the onset of his symptoms with eating spicy Mexican food., ,PAST MEDICAL HISTORY: , Reviewed and unchanged.,ALLERGIES: , No known allergies to medications.,OPERATIONS: , Unchanged.,ILLNESSES: , Crohn's disease, vitamin B12 deficiency.,MEDICATIONS:,  Imuran, Nascobal, Vicodin p.r.n., ,REVIEW OF SYSTEMS: , Dated 08/04/04 is reviewed and noted.  Please see pertinent GI issues as discussed above.  Otherwise unremarkable., ,PHYSICAL EXAMINATION:  , GENERAL:  Pleasant male in no acute distress.  Well nourished and well developed. SKIN: indurated, cord-like superficial vein on the right anterior forearm, approx. 3 cm in length.  Non-tender to palpation. No erythema or red streaking.  No edema. LYMPH:  No epitrochlear or axillary lymph node enlargement or tenderness on the right side. , ,DATA REVIEWED: Labs from June 8th and July 19th reviewed.  Liver function tests normal with AST 14 and ALT 44.  WBCs were slightly low at 4.8.  Hemoglobin dropped slightly from 14.1 on 6/8 to 12.9 on 7/19. Hematocrit dropped slightly as well from 43.2 on 6/804 to 40.0 on 7/19/04.  These results were reviewed by Dr. S and lab results letter sent., ,IMPRESSION:  ,1. Crohn's disease, status post terminal ileum resection, on Imuran.  Intermittent symptoms of bowel obstruction.  Last episode three weeks ago.,2.  History of non-specific hepatitis while taking high doses of Tylenol.  Now resolved. ,2.  Increased frequency of reflux symptoms.,3.  Superficial thrombophlebitis, resolving. ,4.  Slightly low H&amp;H., ,PLAN:  ,1.  We discussed Dr. S's recommendation that the patient undergo balloon dilation for recurrent bowel obstruction type symptoms.  The patient emphatically states that he does not want to consider dilation at this time.  The patient is strongly encouraged to call us when he does experience any obstructive symptoms, including abdominal pain, nausea, vomiting, or change in bowel habits.  He states understanding of this. Advised to maintain low residue diet to avoid obstructions. ,2.  Continue with liver panel and ABC every month per Dr. S's instructions.,3.  Continue Imuran 100 mg per day.,4.  Continue to minimize Tylenol use.  The patient is wondering if he can take another type of medication for migraines that is not Tylenol or antiinflammatories or aspirin.  Dr. S is consulted and agrees that Imitrex is an acceptable alternative for migraine headaches since he does not have advanced liver disease. The patient will make an appointment with his primary care provider to discuss this further. ,5.  Reviewed the importance of prophylactic treatment of reflux-type symptoms.  Encouraged the patient to take over-the-counter H2 blockers on a daily basis to prevent symptoms from occurring.  The patient will try this and if he remains symptomatic, then he will call our office and a prescription for Zantac 150 mg per day will be provided.  Reviewed the potential need for upper endoscopy should his symptoms continue or become more frequent.  He does not want to undergo any type of procedure such as that at this time.,6.</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr"/>
+          <t>EXAM: , CT of the abdomen and pelvis without contrast.,HISTORY: , Lower abdominal pain.,FINDINGS:,  Limited views of the lung bases demonstrate linear density most likely representing dependent atelectasis.  There is a 1.6 cm nodular density at the left posterior sulcus.,Noncontrast technique limits evaluation of the solid abdominal organs.  Cardiomegaly and atherosclerotic calcifications are seen.,Hepatomegaly is observed.  There is calcification within the right lobe of the liver likely related to granulomatous changes.  Subtle irregularity of the liver contour is noted, suggestive of cirrhosis.  There is splenomegaly seen.  There are two low-attenuation lesions seen in the posterior aspect of the spleen, which are incompletely characterized that may represent splenic cyst.  The pancreas appears atrophic.  There is a left renal nodule seen, which measures 1.9 cm with a Hounsfield unit density of approximately 29, which is indeterminate.,There is mild bilateral perinephric stranding.  There is an 8-mm fat density lesion in the anterior inner polar region of the left kidney, compatible in appearance with angiomyolipoma.  There is a 1-cm low-attenuation lesion in the upper pole of the right kidney, likely representing a cyst, but incompletely characterized on this examination.  Bilateral ureters appear normal in caliber along their visualized course.  The bladder is partially distended with urine, but otherwise unremarkable.,Postsurgical changes of hysterectomy are noted.  There are pelvic phlebolith seen.  There is a calcified soft tissue density lesion in the right pelvis, which may represent an ovary with calcification, as it appears continuous with the right gonadal vein.,Scattered colonic diverticula are observed.  The appendix is within normal limits.  The small bowel is unremarkable.  There is an anterior abdominal wall hernia noted containing herniated mesenteric fat.  The hernia neck measures approximately 2.7 cm.  There is stranding of the fat within the hernia sac.,There are extensive degenerative changes of the right hip noted with changes suggestive of avascular necrosis.  Degenerative changes of the spine are observed.,IMPRESSION:,1.  Anterior abdominal wall hernia with mesenteric fat-containing stranding, suggestive of incarcerated fat.,2.  Nodule in the left lower lobe, recommend follow up in 3 months.,3.  Indeterminate left adrenal nodule, could be further assessed with dedicated adrenal protocol CT or MRI.,4.  Hepatomegaly with changes suggestive of cirrhosis.  There is also splenomegaly observed.,5.  Low-attenuation lesions in the spleen may represent cyst, that are incompletely characterized on this examination.,6.  Fat density lesion in the left kidney, likely represents angiomyolipoma.,7.  Fat density soft tissue lesion in the region of the right adnexa, this contains calcifications and may represent an ovary or possibly dermoid cyst.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>gastroenterology, abdominal pain, cardiomegaly, atherosclerotic calcifications, hepatomegaly, perinephric stranding, low attenuation lesions, abdominal, calcifications, lesions, abdomen,</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="n">
-        <v>833</v>
+        <v>408</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Gastroenterology; long; consultation; diagnoses + symptoms + medications</t>
+          <t>Gastroenterology; medium; diagnostic report; middle text complexity; diagnoses + symptoms + imaging</t>
         </is>
       </c>
       <c r="J25" s="2" t="n">
-        <v>3525</v>
+        <v>3606</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>consultation</t>
+          <t>diagnostic report</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>higher</t>
+          <t>middle</t>
         </is>
       </c>
       <c r="M25" s="2" t="n">
-        <v>0.9021077547339945</v>
+        <v>0.472497745716862</v>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; procedures; imaging; past history; treatment plans; follow-up; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; imaging; treatment plans; follow-up</t>
         </is>
       </c>
     </row>
     <row r="26" ht="110" customHeight="1">
       <c r="A26" s="2" t="n">
-        <v>3362</v>
+        <v>3341</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
@@ -2020,39 +2028,39 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Gen Med Consult - 23 </t>
+          <t xml:space="preserve"> Gen Med Consult - 41 </t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Patient in with mom for possible ear infection.</t>
+          <t xml:space="preserve"> Backache, stomachache, and dysuria for the last two days - Urinary dysuria, left flank pain, pharyngitis.</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>SUBJECTIVE:,  Mom brings the patient in today for possible ear infection.  He is complaining of left ear pain today.  He was treated on 04/14/2004, with amoxicillin for left otitis and Mom said he did seem to get better but just started complaining of the left ear pain today.  He has not had any fever but the congestion has continued to be very thick and purulent.  It has never really resolved.  He has a loose, productive-sounding cough but not consistently and not keeping him up at night.  No wheezing or shortness of breath.,PAST MEDICAL HISTORY:,  He has had some wheezing in the past but nothing recently.,FAMILY HISTORY: , All siblings are on antibiotics for ear infections and URIs.,OBJECTIVE:,General:  The patient is a 5-year-old male.  Alert and cooperative.  No acute distress.,Neck:  Supple without adenopathy.,HEENT:  Ear canals clear.  TMs, bilaterally, have distorted light reflexes but no erythema.  Gray in color.  Oropharynx pink and moist with a lot of postnasal discharge.  Nares are swollen and red.  Thick, purulent drainage.  Eyes are a little puffy.,Chest:  Respirations regular, nonlabored.,Lungs:  Clear to auscultation throughout.,Heart:  Regular rhythm without murmur.,Skin:  Warm, dry, pink.  Moist mucus membranes.  No rash.,ASSESSMENT:,  Ongoing purulent rhinitis.  Probable sinusitis and serous otitis.,PLAN:,  Change to Omnicef two teaspoons daily for 10 days.  Frequent saline in the nose.  Also, there was some redness around the nares with a little bit of yellow crusting.  It appeared to be the start of impetigo, so hold off on the Rhinocort for a few days and then restart.  Use a little Neosporin for now.</t>
+          <t>SUBJECTIVE:,  The patient complains of backache, stomachache, and dysuria for the last two days.  Fever just started today and cough.  She has history of kidney stones less than a year ago and had a urinary tract infection at that time.  Her back started hurting last night.,PAST MEDICAL HISTORY:,  She denies sexual activities since two years ago.  Her last menstrual period was 06/01/2004.  Her periods have been irregular.  She started menarche at 10 years of age and she is still irregular and it runs in Mom’s side of the family.  Mom and maternal aunt have had total hysterectomies.  She also is diagnosed with abnormal valve has to be on SBE prophylaxis, sees Dr. XYZ Allen.  She avoids decongestants.  She is limited on her activity secondary to her heart condition.,MEDICATION:,  Cylert.,ALLERGIES: , No known drug allergies.,OBJECTIVE:,Vital Signs:  Blood pressure is 124/72.  Temperature 99.2.  Respirations 20 unlabored.  Weight:  137 pounds.,HEENT:  Normocephalic.  Conjunctivae noninjected.  No mattering noted.  Her TMs are bilaterally clear, nonerythematous.  Throat clear, good mucous membrane moisture, but she did have erythema and edema at her posterior soft palate.,Neck:  Supple.  Increased lymphadenopathy noted in the submandibular nodes, but no axillary nodes and no hepatosplenomegaly.,Respiratory:  Clear.  No wheezes, no crackles, no tachypnea, and no retractions.,Cardiovascular:  Regular rate and rhythm.  S1 and S2 normal, no murmur.,Abdomen:  Soft.  No organomegaly.  She did have exquisite tenderness to palpation of the left upper quadrant and flank area, but the spleen was not palpable.  She has no suprapubic tenderness.,Extremities:  She has good range of motion of upper and lower extremities.  Good ambulation.,Her UA was positive for 2+ leukocyte esterase, positive nitrites, 1+ protein, 2+ ketones, 4+ blood, greater than 50 white blood cells, 10-20 rbc’s, and 1+ bacteria.  Culture and sensitivity is pending.  Her Strep test is negative.  Culture is pending.,ASSESSMENT:,1.  Urinary dysuria.,2.  Left flank pain.,3.  Pharyngitis.,PLAN:,  A 1 g of Rocephin IM was given.  Call Dr. B's office tomorrow morning incase a second IM dose is needed.  If not then she will fill a prescription for Omnicef 300 mg capsule 1 p.o. b.i.d. for 10 days total and then we will await the culture and sensitivity results to see if this is appropriate drug.  Push fluids.  Await strep culture report.  Follow up with Dr. XYZ if no better or symptoms worsen.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>general medicine, ear infection, productive-sounding cough, purulent rhinitis, serous otitis, sinusitis, wheezing, ear, amoxicillin,</t>
+          <t xml:space="preserve">general medicine, backache, stomachache, dysuria, cylert, urinary dysuria, pharyngitis, culture and sensitivity, tenderness, urinary, infection, </t>
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>253</v>
+        <v>374</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>General Medicine; short; SOAP-style; diagnoses + symptoms + past history</t>
+          <t>General Medicine; medium; SOAP-style; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J26" s="2" t="n">
-        <v>3362</v>
+        <v>3341</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -2061,21 +2069,21 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>higher</t>
         </is>
       </c>
       <c r="M26" s="2" t="n">
-        <v>0.3677299368800721</v>
+        <v>0.6918958521190262</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; past history; treatment plans; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; past history; treatment plans; follow-up; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="27" ht="110" customHeight="1">
       <c r="A27" s="2" t="n">
-        <v>3375</v>
+        <v>3319</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
@@ -2084,26 +2092,22 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Gen Med Consult - 15 </t>
+          <t xml:space="preserve"> Gen Med H&amp;P - 2 </t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Complaint of mood swings and tearfulness.</t>
+          <t xml:space="preserve"> Weakness, malaise dyspnea on exertion, 15-pound weight loss - Bilateral pneumonia, hepatitis, renal insufficiency, </t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS:,  A 50-year-old female comes to the clinic with complaint of mood swings and tearfulness.  This has been problematic over the last several months and is just worsening to the point where it is impairing her work.  Her boss asks her if she was actually on drugs in which she said no.  She stated may be she needed to be, meaning taking some medications.  The patient had been prescribed Wellbutrin in the past and responded well to it; however, at that time it was prescribed for obsessive-compulsive type disorder relating to overeating and therefore her insurance would not cover the medication.  She has not been on any other antidepressants in the past.  She is not having any suicidal ideation but is having difficulty concentrating, rapid mood swings with tearfulness, and insomnia.  She denies any hot flashes or night sweats.  She underwent TAH with BSO in December of 2003.,FAMILY HISTORY: , Benign breast lump in her mother; however, her paternal grandmother had breast cancer.  The patient denies any palpitations, urinary incontinence, hair loss, or other concerns.  She was recently treated for sinusitis.,ALLERGIES:,  She is allergic to Sulfa.,CURRENT MEDICATIONS:,  Recently finished Minocin and Duraphen II DM.,PHYSICAL EXAMINATION:,General:  A well-developed and well-nourished female, conscious, alert, oriented times three in no acute distress.  Mood is dysthymic.  Affect is tearful.,Skin:  Without rash.,Eyes:  PERRLA.  Conjunctivae are clear.,Neck:  Supple with adenopathy or thyromegaly.,Lungs:  Clear.,Heart:  Regular rate and rhythm without murmur.,ASSESSMENT:,1.  Postsurgical menopause.,2.  Mood swings.,PLAN:,  I spent about 30 minutes with the patient discussing treatment options.  I do believe that her moods would greatly benefit from hormone replacement therapy; however, she is reluctant to do this because of family history of breast cancer.  We will try starting her back on Wellbutrin XL 150 mg daily.  She may increase to 300 mg daily after three to seven days.  Samples provided initially.  If she is not obtaining adequate relief from medication alone, we will then suggest that we explore the use of hormone replacement therapy.  I also recommended increasing her exercise.  We will also obtain some screening lab work including CBC, UA, TSH, chemistry panel, and lipid profile.  Follow up here in two weeks or sooner if any other problems.  She is needing her annual breast exam as well.</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>general medicine, tearfulness, mood swings, menopause, postsurgical menopause, mood swings and tearfulness, hormone replacement therapy, breast cancer, wellbutrin,</t>
-        </is>
-      </c>
+          <t>HISTORY OF PRESENT ILLNESS: , This is a 43-year-old black man with no apparent past medical history who presented to the emergency room with the chief complaint of weakness, malaise and dyspnea on exertion for approximately one month.  The patient also reports a 15-pound weight loss.  He denies fever, chills and sweats.  He denies cough and diarrhea.  He has mild anorexia.,PAST MEDICAL HISTORY:,  Essentially unremarkable except for chest wall cysts which apparently have been biopsied by a dermatologist in the past, and he was given a benign diagnosis.  He had a recent PPD which was negative in August 1994.,MEDICATIONS: , None.,ALLERGIES: , No known drug allergies.,SOCIAL HISTORY: , He occasionally drinks and is a nonsmoker.  The patient participated in homosexual activity in Haiti during 1982 which he described as "very active." Denies intravenous drug use.  The patient is currently employed.,FAMILY HISTORY:,  Unremarkable.,PHYSICAL EXAMINATION:,GENERAL:  This is a thin, black cachectic man speaking in full sentences with oxygen.,VITAL SIGNS:  Blood pressure 96/56, heart rate 120.  No change with orthostatics.  Temperature 101.6 degrees Fahrenheit.  Respirations 30.,HEENT:  Funduscopic examination normal.  He has oral thrush.,LYMPH:  He has marked adenopathy including right bilateral epitrochlear and posterior cervical nodes.,NECK:  No goiter, no jugular venous distention.,CHEST:  Bilateral basilar crackles, and egophony at the right and left middle lung fields.,HEART:  Regular rate and rhythm, no murmur, rub or gallop.,ABDOMEN:  Soft and nontender.,GENITOURINARY:  Normal.,RECTAL:  Unremarkable.,SKIN:  The patient has multiple, subcutaneous mobile nodules on the chest wall that are nontender.  He has very pale palms., ,LABORATORY AND X-RAY DATA: , Sodium 133, potassium 5.3, BUN 29, creatinine 1.8.  Hemoglobin 14, white count 7100, platelet count 515.  Total protein 10, albumin 3.1, AST 131, ALT 31.  Urinalysis shows 1+ protein, trace blood.  Total bilirubin 2.4, direct bilirubin 0.1.  Arterial blood gases:  pH 7.46, pC02 32, p02 46 on room air.  Electrocardiogram shows normal sinus rhythm.  Chest x-ray shows bilateral alveolar and interstitial infiltrates.,IMPRESSION:,1.  Bilateral pneumonia; suspect atypical pneumonia, rule out Pneumocystis carinii pneumonia and tuberculosis.,2.  Thrush.,3.  Elevated unconjugated bilirubins.,4.  Hepatitis.,5.  Elevated globulin fraction.,6.  Renal insufficiency.,7.  Subcutaneous nodules.,8.  Risky sexual behavior in 1982 in Haiti.,PLAN:,1.  Induced sputum, rule out Pneumocystis carinii pneumonia and tuberculosis.,2.  Begin intravenous Bactrim and erythromycin.,3.  Begin prednisone.,4.  Oxygen.,5.  Nystatin swish and swallow.,6.  Dermatologic biopsy of lesions.,7.  Check HIV and RPR.,8.  Administer Pneumovax, tetanus shot and Heptavax if indicated.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="n">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -2112,34 +2116,34 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>General Medicine; medium; consultation; diagnoses + symptoms + medications</t>
+          <t>General Medicine; medium; history and physical; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J27" s="2" t="n">
-        <v>3375</v>
+        <v>3319</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>consultation</t>
+          <t>history and physical</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>higher</t>
         </is>
       </c>
       <c r="M27" s="2" t="n">
-        <v>0.5342087466185753</v>
+        <v>0.8847497745716864</v>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; past history; treatment plans; follow-up; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="28" ht="110" customHeight="1">
       <c r="A28" s="2" t="n">
-        <v>3319</v>
+        <v>3381</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
@@ -2148,22 +2152,22 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Gen Med H&amp;P - 2 </t>
+          <t xml:space="preserve"> Gen Med Consult - 13 </t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Weakness, malaise dyspnea on exertion, 15-pound weight loss - Bilateral pneumonia, hepatitis, renal insufficiency, </t>
+          <t xml:space="preserve"> Consult for hypertension and a med check.  History of osteoarthritis, osteoporosis, hypothyroidism, allergic rhinitis and kidney stones.</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS: , This is a 43-year-old black man with no apparent past medical history who presented to the emergency room with the chief complaint of weakness, malaise and dyspnea on exertion for approximately one month.  The patient also reports a 15-pound weight loss.  He denies fever, chills and sweats.  He denies cough and diarrhea.  He has mild anorexia.,PAST MEDICAL HISTORY:,  Essentially unremarkable except for chest wall cysts which apparently have been biopsied by a dermatologist in the past, and he was given a benign diagnosis.  He had a recent PPD which was negative in August 1994.,MEDICATIONS: , None.,ALLERGIES: , No known drug allergies.,SOCIAL HISTORY: , He occasionally drinks and is a nonsmoker.  The patient participated in homosexual activity in Haiti during 1982 which he described as "very active." Denies intravenous drug use.  The patient is currently employed.,FAMILY HISTORY:,  Unremarkable.,PHYSICAL EXAMINATION:,GENERAL:  This is a thin, black cachectic man speaking in full sentences with oxygen.,VITAL SIGNS:  Blood pressure 96/56, heart rate 120.  No change with orthostatics.  Temperature 101.6 degrees Fahrenheit.  Respirations 30.,HEENT:  Funduscopic examination normal.  He has oral thrush.,LYMPH:  He has marked adenopathy including right bilateral epitrochlear and posterior cervical nodes.,NECK:  No goiter, no jugular venous distention.,CHEST:  Bilateral basilar crackles, and egophony at the right and left middle lung fields.,HEART:  Regular rate and rhythm, no murmur, rub or gallop.,ABDOMEN:  Soft and nontender.,GENITOURINARY:  Normal.,RECTAL:  Unremarkable.,SKIN:  The patient has multiple, subcutaneous mobile nodules on the chest wall that are nontender.  He has very pale palms., ,LABORATORY AND X-RAY DATA: , Sodium 133, potassium 5.3, BUN 29, creatinine 1.8.  Hemoglobin 14, white count 7100, platelet count 515.  Total protein 10, albumin 3.1, AST 131, ALT 31.  Urinalysis shows 1+ protein, trace blood.  Total bilirubin 2.4, direct bilirubin 0.1.  Arterial blood gases:  pH 7.46, pC02 32, p02 46 on room air.  Electrocardiogram shows normal sinus rhythm.  Chest x-ray shows bilateral alveolar and interstitial infiltrates.,IMPRESSION:,1.  Bilateral pneumonia; suspect atypical pneumonia, rule out Pneumocystis carinii pneumonia and tuberculosis.,2.  Thrush.,3.  Elevated unconjugated bilirubins.,4.  Hepatitis.,5.  Elevated globulin fraction.,6.  Renal insufficiency.,7.  Subcutaneous nodules.,8.  Risky sexual behavior in 1982 in Haiti.,PLAN:,1.  Induced sputum, rule out Pneumocystis carinii pneumonia and tuberculosis.,2.  Begin intravenous Bactrim and erythromycin.,3.  Begin prednisone.,4.  Oxygen.,5.  Nystatin swish and swallow.,6.  Dermatologic biopsy of lesions.,7.  Check HIV and RPR.,8.  Administer Pneumovax, tetanus shot and Heptavax if indicated.</t>
+          <t>SUBJECTIVE:,  The patient is a 76-year-old white female who presents to the clinic today originally for hypertension and a med check.  She has a history of hypertension, osteoarthritis, osteoporosis, hypothyroidism, allergic rhinitis and kidney stones.  Since her last visit she has been followed by Dr. Kumar.  Those issues are stable.  She has had no fever or chills, cough, congestion, nausea, vomiting, chest pain, chest pressure.,PAST MEDICAL HISTORY:,  She has an intolerance to Prevacid.,CURRENT MEDICATIONS:,  Evista 60 daily, Levothroid 0.05 mg daily, Claritin 10 daily, Celebrex 200 daily, HCTZ 25 daily and amitriptyline p.r.n.,PAST SURGICAL HISTORY:,  Bilateral mastectomies, tonsillectomy, EGD, flex sig in 2001 and a heart cath.,FAMILY HISTORY: , Father passed away at 81; mother of multiple myeloma at 83.,SOCIAL HISTORY:,  She is married.  A 76-year-old who used to smoke a pack a day and quit in 1985.  She is retired.,REVIEW OF SYSTEMS:,  Essentially negative in HEENT, chest, cardiovascular, GI, GU, musculoskeletal, or neurologic.,OBJECTIVE:,  Temperature is 97.5 degrees.  Blood pressure is 168/70.  Pulse is 88.  Weight is 129 pounds.,GENERAL:  She is an elderly 76-year-old in no acute distress.,HEENT:  Atraumatic.  Extraocular muscles were intact.  Pupils equal, round and reactive to light and accommodation.  Tympanic membranes are clear, dry and intact.  Sinuses and throat are clear.  Neck is soft, supple.  No meningeal signs are present.  No thyromegaly is present.,CHEST:  Clear to auscultation.,CARDIOVASCULAR:  Regular rate and rhythm without murmur.,ABDOMEN:  Soft, nontender.  Bowel sounds are positive.  No organomegaly or peritoneal signs are present.,EXTREMITIES:  Moving all extremities.  Peripheral pulses are normal.  No edema is present.,NEUROLOGIC:  Alert and oriented.  Cranial nerves II-XII grossly intact.  Strength 5+/5 globally.  Reflexes 2+/IV globally.  Romberg is negative.  There is no numbness, tingling, weakness or other neurologic deficit present.,BREASTS:  Surgically absent but there are no lumps, lesions, masses, discharge or adenopathy present.,BACK:  Straight.,SKIN:  Clear.,GENITALIA:  Deferred as she has been followed by Dr. XYZ many times this year.  She does have a history of some elevated cholesterol.,ASSESSMENT:,1.  Hypertension, suboptimal control.,2.  Hypothyroidism.,3.  Arthritis.,4.  Allergic rhinitis.,5.  History of kidney stones.,6.  Osteoporosis.,PLAN:,1.  CBC, complete metabolic profile, UA for hypertension.,2.  Chest x-ray for history of breast cancer.,3.  DEXA scan, full body for osteoporosis.,4.  Flex is up to date.,5.  Pneumovax has been given in the last five years.,6.  Lipid profile for elevated cholesterol.,7.  Refill meds.,8.  Follow up every three to six months for blood pressure check or sooner p.r.n. problems.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="n">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -2172,15 +2176,15 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>General Medicine; medium; history and physical; diagnoses + symptoms + medications</t>
+          <t>General Medicine; medium; SOAP-style; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J28" s="2" t="n">
-        <v>3319</v>
+        <v>3381</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>history and physical</t>
+          <t>SOAP-style</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -2189,17 +2193,17 @@
         </is>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0.8847497745716864</v>
+        <v>0.8136271415689811</v>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; imaging; past history; treatment plans; follow-up; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="29" ht="110" customHeight="1">
       <c r="A29" s="2" t="n">
-        <v>3287</v>
+        <v>3290</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
@@ -2208,35 +2212,35 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> H&amp;P - Gen Med - 2 </t>
+          <t xml:space="preserve"> H&amp;P - Gen Med - 1  </t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> History of diabetes, osteoarthritis, atrial fibrillation, hypertension, asthma, obstructive sleep apnea on CPAP, diabetic foot ulcer, anemia, and left lower extremity cellulitis.</t>
+          <t xml:space="preserve"> An 85-year-old female with diarrhea, vomiting, and abdominal pain.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS:, The patient is a 71-year-old Caucasian female with a history of diabetes, osteoarthritis, atrial fibrillation, hypertension, asthma, obstructive sleep apnea on CPAP, diabetic foot ulcer, anemia and left lower extremity cellulitis. She was brought in by the EMS service to Erlanger emergency department with pulseless electrical activity. Her husband states that he was at home with his wife, when she presented to him complaining of fever and chills. She became acutely unresponsive. She was noted to have worsening of her breathing. She took several of her MDIs and then was placed on her CPAP. He went to notify EMS and when he returned, she was found to not be breathing. He stated that she was noted to have no breathing in excess of 10 minutes. He states that the EMS system arrived at the home and she was found not breathing. The patient was intubated at the scene and upon arrival to Erlanger Medical Center, she was found to have pupils fixed and dilated. She was seen by me in the emergency department and was on Neo-Synephrine, dopamine with a blood pressure of 97/22 with a rapid heart rate and again, in an unresponsive state.,REVIEW OF SYSTEMS:, Review of systems was not obtainable.,PAST MEDICAL HISTORY:, Diabetes, osteoarthritis, hypertension, asthma, atrial fibrillation, diabetic foot ulcer and anemia.,PAST SURGICAL HISTORY:, Noncontributory to above.,FAMILY HISTORY:, Mother with history of coronary artery disease.,SOCIAL HISTORY:, The patient is married. She uses no ethanol, no tobacco and no illicits. She has a very support family unit.,MEDICATIONS:, Augmentin; Detrol LA; lisinopril.,IMMUNIZATIONS:, Immunizations were up to date for influenza, negative for Pneumovax.,ALLERGIES:, PENICILLIN.,LABORATORY AT PRESENTATION:, White blood cell count 11, hemoglobin 10.5, hematocrit 32.2, platelets 175,000. Sodium 148, potassium 5.2, BUN 30, creatinine 2.2 and glucose 216. PT was 22.4.,RADIOLOGIC DATA:, Chest x-ray revealed a diffuse pulmonary edema.,PHYSICAL EXAMINATION:,VITAL SIGNS: Blood pressure 97/52, pulse of 79, respirations 16, O2 sat 100%.,HEENT: The patient's pupils were again, fixed and dilated and intubated on the monitor.,CHEST: Poor air movement bilateral with bilateral rales.,CARDIOVASCULAR: Regular rate and rhythm.,ABDOMEN: The abdomen was obese, nondistended and nontender.,EXTREMITIES: Left diabetic foot had oozing pus drainage from the foot.,GU: Foley catheter was in place.,IMPRESSION AND PLAN:,1. Acute cardiac arrest with pulseless electrical activity with hypotensive shock and respiratory failure: Will continue ventilator support. Will rule out pulmonary embolus, rule out myocardial infarction. Continue pressors. The patient is currently on dopamine, Neo-Synephrine and Levophed.,2. Acute respiratory distress syndrome: Will continue ventilatory support.,3. Questionable sepsis: Will obtain blood cultures, intravenous vancomycin and Rocephin given.,4. Hypotensive shock: Will continue pressors. Will check random cortisol. Hydrocortisone was added.,Further inpatient management for this patient will be provided by Dr. R. The patient's status was discussed with her daughter and her husband. The husband states that his wife has been very ill in the past with multiple admissions, but he had never seen her as severely ill as with this event. He states that she completely was not breathing at all and he is aware of the severity of her illness and the gravity of her current prognosis. Will obtain the assistance with cardiology with this admission and will continue pressors and supportive therapy. The family will make an assessment and final decision concerning her long-term management after a 24 hour period.</t>
+          <t>CHIEF COMPLAINT:, Diarrhea, vomiting, and abdominal pain.,HISTORY OF PRESENT ILLNESS:, The patient is an 85-year-old female who presents with a chief complaint as described above. The patient is a very poor historian and is extremely hard of hearing, and therefore, very little history is available. She was found by EMS sitting on the toilet having diarrhea, and apparently had also just vomited. Upon my questioning of the patient, she can confirm that she has been sick to her stomach and has vomited. She cannot tell me how many times. She is also unable to describe the vomitus. She also tells me that her belly has been hurting. I am unable to get any further history from the patient because, again, she is an extremely poor historian and very hard of hearing.,PAST MEDICAL HISTORY:, Per the ER documentation is hypertension, diverticulosis, blindness, and sciatica.,MEDICATIONS:, Lorazepam 0.5 mg, dosing interval is not noted; Tylenol PM; Klor-Con 10 mEq; Lexapro; calcium with vitamin D.,ALLERGIES:, SHE IS ALLERGIC TO PENICILLIN.,FAMILY HISTORY:, Unknown.,SOCIAL HISTORY:, Also unknown.,REVIEW OF SYSTEMS:, Unobtainable secondary to the patient's condition.,PHYSICAL EXAMINATION:,VITAL SIGNS: Pulse 80. Respiratory rate 18. Blood pressure 130/80. Temperature 97.6.,GENERAL: Elderly black female who is initially sleeping upon my evaluation, but is easily arousable.,NECK: No JVD. No thyromegaly.,EARS, NOSE, AND THROAT: Her oropharynx is dry. Her hearing is very diminished.,CARDIOVASCULAR: Regular rhythm. No lower extremity edema.,GI: Mild epigastric tenderness to palpation without guarding or rebound. Bowel sounds are normoactive.,RESPIRATORY: Clear to auscultation bilaterally with a normal effort.,SKIN: Warm, dry, no erythema.,NEUROLOGICAL: The patient attempts to answer questions when asked, but is very hard of hearing. She is seen to move all extremities spontaneously.,DIAGNOSTIC DATA:, White count 9.6, hemoglobin 15.9, hematocrit 48.2, platelet count 345, PTT 24, PT 13.3, INR 0.99, sodium 135, potassium 3.3, chloride 95, bicarb 20, BUN 54, creatinine 2.2, glucose 165, calcium 10.3, magnesium 2.5, total protein 8.2, albumin 3.8, AST 33, ALT 26, alkaline phosphatase 92. Cardiac isoenzymes negative x1. EKG shows sinus rhythm with a rate of 96 and a prolonged QT interval.,ASSESSMENT AND PLAN:,1. Pancreatitis. Will treat symptomatically with morphine and Zofran, and also IV fluids. Will keep NPO.,2. Diarrhea. Will check stool studies.,3. Volume depletion. IV fluids.,4. Hyperglycemia. It is unknown whether the patient is diabetic. I will treat her with sliding scale insulin.,5. Hypertension. If the patient takes blood pressure medications, it is not listed on the only medication listing that is available. I will prescribe clonidine as needed.,6. Renal failure. Her baseline is unknown. This is at least partly prerenal. Will replace volume with IV fluids and monitor her renal function.,7. Hypokalemia. Will replace per protocol.,8. Hypercalcemia. This is actually rather severe when adjusted for the patient's low albumin. Her true calcium level comes out to somewhere around 12. For now, I will just treat her with IV fluids and Lasix, and monitor her calcium level.,9. Protein gap. This, in combination with the calcium, may be suggestive of multiple myeloma. It is my understanding that the family is seeking hospice placement for the patient right now. I would have to discuss with the family before undertaking any workup for multiple myeloma or other malignancy.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="n">
-        <v>545</v>
+        <v>524</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>General Medicine; long; history and physical; diagnoses + symptoms + medications</t>
+          <t>General Medicine; medium; history and physical; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J29" s="2" t="n">
-        <v>3287</v>
+        <v>3290</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
@@ -2249,17 +2253,17 @@
         </is>
       </c>
       <c r="M29" s="2" t="n">
-        <v>0.8654756537421101</v>
+        <v>0.8744364292155093</v>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; past history; treatment plans; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="30" ht="110" customHeight="1">
       <c r="A30" s="2" t="n">
-        <v>3150</v>
+        <v>3186</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
@@ -2268,39 +2272,39 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Lymph Node Excisional Biopsy </t>
+          <t xml:space="preserve"> Biopsy - Cervical Lymph Node </t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Left axillary lymph node excisional biopsy.  Left axillary adenopathy.</t>
+          <t xml:space="preserve"> Excisional biopsy of right cervical lymph node.</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>PREOPERATIVE DIAGNOSIS: , Left axillary adenopathy.,POSTOPERATIVE DIAGNOSIS: , Left axillary adenopathy.,PROCEDURE: , Left axillary lymph node excisional biopsy.,ANESTHESIA:,  LMA.,INDICATIONS: , Patient is a very pleasant woman who in 2006 had breast conservation therapy with radiation only.  Note, she refused her CMF adjuvant therapy and this was for a triple-negative infiltrating ductal carcinoma of the breast.  Patient has been following with Dr. Diener and Dr. Wilmot.  I believe that genetic counseling had been recommended to her and obviously the CMF was recommended, but she declined both.  She presented to the office with left axillary adenopathy in view of the high-risk nature of her lesion.  I recommended that she have this lymph node removed.  The procedure, purpose, risk, expected benefits, potential complications, alternative forms of therapy were discussed with her and she was agreeable to surgery.,TECHNIQUE: , Patient was identified, then taken into the operating room where after induction of appropriate anesthesia, her left chest, neck, axilla, and arm were prepped with Betadine solution, draped in a sterile fashion.  An incision was made at the hairline, carried down by sharp dissection through the clavipectoral fascia.  I was able to easily palpate the lymph node and grasp it with a figure-of-eight 2-0 silk suture and by sharp dissection, was carried to hemoclip all attached structures.  The lymph node was excised in its entirety.  The wound was irrigated.  The lymph node sent to pathology.  The wound was then closed.  Hemostasis was assured and the patient was taken to recovery room in stable condition.</t>
+          <t>PREOPERATIVE DIAGNOSIS: , Cervical lymphadenopathy.,POSTOPERATIVE DIAGNOSIS:,  Cervical lymphadenopathy.,PROCEDURE: , Excisional biopsy of right cervical lymph node.,ANESTHESIA: , General endotracheal anesthesia.,SPECIMEN: , Right cervical lymph node.,EBL: , 10 cc.,COMPLICATIONS: , None.,FINDINGS:,  Enlarged level 2 lymph node was identified and removed and sent for pathologic examination.,FLUIDS: , Please see anesthesia report.,URINE OUTPUT: , None recorded during the case.,INDICATIONS FOR PROCEDURE: , This is a 43-year-old female with a several-year history of persistent cervical lymphadenopathy.  She reports that it is painful to palpation on the right and has had multiple CT scans as well as an FNA which were all nondiagnostic.  After risks and benefits of surgery were discussed with the patient, an informed consent was obtained.  She was scheduled for an excisional biopsy of the right cervical lymph node.,PROCEDURE IN DETAIL: , The patient was taken to the operating room and placed in the supine position.  She was anesthetized with general endotracheal anesthesia.  The neck was then prepped and draped in the sterile fashion.  Again, noted on palpation there was an enlarged level 2 cervical lymph node.,A 3-cm horizontal incision was made over this lymph node.  Dissection was carried down until the sternocleidomastoid muscle was identified.  The enlarged lymph node that measured approximately 2 cm in diameter was identified and was removed and sent to Pathology for touch prep evaluation.  The area was then explored for any other enlarged lymph nodes.  None were identified, and hemostasis was achieved with electrocautery.  A quarter-inch Penrose drain was placed in the wound.,The wound was then irrigated and closed with 3-0 interrupted Vicryl sutures for a deep closure followed by a running 4-0 Prolene subcuticular suture.  Mastisol and Steri-Strip were placed over the incision, and sterile bandage was applied.  The patient tolerated this procedure well and was extubated without complications and transported to the recovery room in stable condition.  She will return to the office tomorrow in followup to have the Penrose drain removed.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>hematology - oncology, axillary lymph node excisional biopsy, sharp dissection, excisional biopsy, lymph node, axillary, excisional, biopsy</t>
+          <t xml:space="preserve">hematology - oncology, lymphadenopathy, excisional biopsy, fna, mastisol, penrose drain, cervical, cervical lymph node, endotracheal anesthesia, lymph node, sternocleidomastoid, cervical lymph, lymph, anesthesia, </t>
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>249</v>
+        <v>318</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Hematology - Oncology; short; procedure/operative; diagnoses + procedures + treatment plans</t>
+          <t>Hematology - Oncology; medium; procedure/operative; middle text complexity; diagnoses + procedures + imaging</t>
         </is>
       </c>
       <c r="J30" s="2" t="n">
-        <v>3150</v>
+        <v>3186</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
@@ -2309,15 +2313,15 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>middle</t>
         </is>
       </c>
       <c r="M30" s="2" t="n">
-        <v>0.3123872858431019</v>
+        <v>0.5526375112714157</v>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; procedures; treatment plans; surgery</t>
+          <t>diagnoses; procedures; imaging; past history; follow-up; surgery</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2364,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Hematology - Oncology; medium; follow-up/progress; diagnoses + symptoms + laboratory values</t>
+          <t>Hematology - Oncology; medium; follow-up/progress; higher text complexity; diagnoses + symptoms + laboratory values</t>
         </is>
       </c>
       <c r="J31" s="2" t="n">
@@ -2387,7 +2391,7 @@
     </row>
     <row r="32" ht="110" customHeight="1">
       <c r="A32" s="2" t="n">
-        <v>3119</v>
+        <v>3159</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
@@ -2396,62 +2400,58 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Symes Amputation - Hallux </t>
+          <t xml:space="preserve"> Hematology Consult </t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Excision of mass, left second toe and distal Symes amputation, left hallux with excisional biopsy.  Mass, left second toe.  Tumor.  Left hallux bone invasion of the distal phalanx.</t>
+          <t xml:space="preserve"> Leukocytosis, acute deep venous thrombosis, right lower extremity with bilateral pulmonary embolism, on intravenous heparin complicated with acute renal failure for evaluation.</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>PREOPERATIVE DIAGNOSES:,1.  Mass, left second toe.,2.  Tumor.,3.  Left hallux bone invasion of the distal phalanx.,POSTOPERATIVE DIAGNOSES:,1.  Mass, left second toe.,2.  Tumor.,3.  Left hallux with bone invasion of the distal phalanx.,PROCEDURE PERFORMED:,1.  Excision of mass, left second toe.,2.  Distal Syme's amputation, left hallux with excisional biopsy.,HISTORY: , This 47-year-old Caucasian male presents to ABCD General Hospital with a history of tissue mass on his left foot.  The patient states that the mass has been present for approximately two weeks and has been rapidly growing in size.  The patient also has history of shave biopsy in the past.  The patient does state that he desires surgical excision at this time.,PROCEDURE IN DETAIL:,  An IV was instituted by the Department of Anesthesia in the preoperative holding area.  The patient was transported from the operating room and placed on the operating room table in the supine position with the safety belt across his lap.  Copious amount of Webril was placed around the left ankle followed by a blood pressure cuff.  After adequate sedation by the Department of Anesthesia, a total of 6 cc mixed with 1% lidocaine plain with 0.5% Marcaine plain was injected in a digital block fashion at the base of the left hallux as well as the left second toe.,The foot was then prepped and draped in the usual sterile orthopedic fashion.  The foot was elevated from the operating table and exsanguinated with an Esmarch bandage.  Care was taken with the exsanguination to perform exsanguination below the level of the digits so as not to rupture the masses.  The foot was lowered to the operating table.  The stockinet was reflected and the foot was cleansed with wet and dry sponge.  A distal Syme's incision was planned over the distal aspect of the left hallux.  The incision was performed with a #10 blade and deepened with #15 down to the level of bone.  The dorsal skin flap was removed and dissected in toto off of the distal phalanx.  There was noted to be in growth of the soft tissue mass into the dorsal cortex with erosion in the dorsal cortex and exposure of cortical bone at the distal phalanx.  The tissue was sent to Pathology where Dr. Green stated that a frozen sample would be of less use for examining for cancer.  Dr. Green did state that he felt that there was an adequate incomplete excision of the soft tissue for specimen.  At this time, a sagittal saw was then used to resect all ends of bone of the distal phalanx.  The area was inspected for any remaining suspicious tissues.  Any suspicious tissue was removed.  The area was then flushed with copious amounts of sterile saline.  The skin was then reapproximated with #4-0 nylon with a combination of simple and vertical mattress sutures.,Attention was then directed to the left second toe.  There was noted to be a dorsolateral mass over the dorsal distal aspect of the left second toe.  A linear incision was made just medial to the tissue mass.  The mass was then dissected from the overlying skin and off of the underlying capsule.  This tissue mass was hard, round, and pearly-gray in appearance.  It does not invade into any other surrounding tissues.  The area was then flushed with copious amounts of sterile saline and the skin was closed with #4-0 nylon.  Dressings consisted of Owen silk soaked in Betadine, 4x4s, Kling, Kerlix, and an Ace wrap.  The pneumatic ankle tourniquet was released and immediate hyperemic flush was noted to all five digits of the left foot.  The patient tolerated the above procedure and anesthesia well without complications.  The patient was transported to PACU with vital signs stable and vascular status intact.  The patient was given postoperative pain prescription for Vicodin and instructed to follow up with Dr. Bonnani in his office as directed.  The patient will be contacted immediately pending the results of pathology.  Cultures obtained in the case were aerobic and anaerobic gram stain, Silver stain, and a CBC.</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>hematology - oncology, distal phalanx, mass, tumor., hallux bone, phalanx, symes amputation, excisional biopsy, distal, amputation, invasion, toe, symes, incision, flushed, excision, tissue, hallux</t>
-        </is>
-      </c>
+          <t>REASON FOR CONSULTATION:,  Acute deep venous thrombosis, right lower extremity with bilateral pulmonary embolism, on intravenous heparin complicated with acute renal failure for evaluation.,HISTORY OF PRESENTING ILLNESS:  ,Briefly, this is a 36-year-old robust Caucasian gentleman with no significant past medical or surgical history, who works as a sales representative, doing a lot of traveling by plane and car and attending several sales shows, developed acute shortness of breath with an episode of syncope this weekend and was brought in by paramedics to Hospital.  A V/Q scan revealed multiple pulmonary perfusion defects consistent with high probability pulmonary embolism.  A Doppler venous study of the lower extremity also revealed nonocclusive right popliteal vein thrombosis.  A CT of the abdomen and pelvis revealed normal-appearing liver, spleen, and pancreas; however, the right kidney appeared smaller compared to left and suggesting possibility of renal infarct.  Renal function on admission was within normal range; however, serial renal function showed rapid increase in creatinine to 5 today.  He has been on intravenous heparin and hemodialysis is being planned for tomorrow.  Reviewing his history, there is no family members with hypercoagulable state or prior history of any thrombotic complication.  He denies any recent injury to his lower extremity and in fact denied any calf pain or swelling.,PAST MEDICAL AND SURGICAL HISTORY:  ,Unremarkable.,SOCIAL HISTORY: , He is married and has 1 son.  He has a brother who is healthy.  There is no history of tobacco use or alcohol use.,FAMILY HISTORY:,  No family history of hypercoagulable condition.,MEDICATIONS:  ,Advil p.r.n.,ALLERGIES: , NONE.,REVIEW OF SYSTEMS: , Essentially unremarkable except for sudden onset dyspnea on easy exertion complicated with episode of syncope.  He denied any hemoptysis.  He denied any calf swelling or pain.  Lately, he has been traveling and has been sitting behind a desk for a long period of time.,PHYSICAL EXAMINATION:,GENERAL:  He is a robust young gentleman, awake, alert, and hemodynamically stable.,HEENT:  Sclerae anicteric.  Conjunctivae normal.  Oropharynx normal.,NECK:  No adenopathy or thyromegaly.  No jugular venous distention.,HEART:  Regular.,LUNGS:  Bilateral air entry.,ABDOMEN:  Obese and benign.,EXTREMITIES:  No calf swelling or calf tenderness appreciated.,SKIN:  No petechiae or ecchymosis.,NEUROLOGIC:  Nonfocal.,LABORATORY FINDINGS:,  Blood count obtained showed a white count of 16.8, hemoglobin 14.8 g percent, hematocrit 44.6%, MCV 94, and platelet count 209,000.  Liver profile normal.  Thyroid study revealed a TSH of 1.3.  Prothrombin time/INR 1.5, partial thromboplastin time 78.6 seconds.  Renal function, BUN 44 and creatinine 5.7.  Echocardiogram revealed left ventricular hypertrophy with ejection fraction of 65%, no intramural thrombus noted.,IMPRESSION:,1.  Bilateral pulmonary embolism, most consistent with emboli from right lower extremity, on intravenous heparin, rule out hereditary hypercoagulable state.,2.  Leukocytosis, most likely leukemoid reaction secondary to acute pulmonary embolism/renal infarction, doubt presence of myeloproliferative disorder.,3.  Acute renal failure secondary to embolic right renal infarction.,4.  Obesity.,PLAN: , From hematologic standpoint, we will await hypercoagulable studies, which have all been sent on admission to see if a hereditary component is at play.  For now, we will continue intravenous heparin and subsequent oral anticoagulation with Coumadin.  In view of worsening renal function, may need temporary hemodialysis until renal function improves.  I discussed at length with the patient's wife at the bedside.</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="n">
-        <v>660</v>
+        <v>512</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Hematology - Oncology; long; procedure/operative; diagnoses + symptoms + medications</t>
+          <t>Hematology - Oncology; medium; consultation; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J32" s="2" t="n">
-        <v>3119</v>
+        <v>3159</v>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>procedure/operative</t>
+          <t>consultation</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>higher</t>
         </is>
       </c>
       <c r="M32" s="2" t="n">
-        <v>0.5547790802524797</v>
+        <v>0.845299819657349</v>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; procedures; past history; follow-up; surgery</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; imaging; past history; treatment plans; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="33" ht="110" customHeight="1">
       <c r="A33" s="2" t="n">
-        <v>2920</v>
+        <v>2964</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
@@ -2460,39 +2460,39 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CT Head - 2 </t>
+          <t xml:space="preserve"> Carotid Ultrasound </t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The patient is a 79-year-old man with adult hydrocephalus who was found to have large bilateral effusions on a CT scan.  The patient's subdural effusions are still noticeable, but they are improving.</t>
+          <t xml:space="preserve"> Bilateral carotid ultrasound.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>REASON FOR CT SCAN: , The patient is a 79-year-old man with adult hydrocephalus who was found to have large bilateral effusions on a CT scan performed on January 16, 2008.  I changed the shunt setting from 1.5 to 2.0 on February 12, 2008 and his family obtained this repeat CT scan to determine whether his subdural effusions were improving.,CT scan from 03/11/2008 demonstrates frontal horn span at the level of foramen of Munro of 2.6 cm.  The 3rd ventricular contour which is flat with a 3rd ventricular span of 10 mm.  There is a single shunt, which enters on the right occipital side and ends in the left lateral ventricle.  He has symmetric bilateral subdurals that are less than 1 cm in breadth each, which is a reduction from the report from January 16, 2008, which states that he had a subdural hygroma, maximum size 1.3 cm on the right and 1.1 cm on the left.,ASSESSMENT: , The patient's subdural effusions are still noticeable, but they are improving at the setting of 2.0.,PLAN: , I would like to see the patient with a new head CT in about three months, at which time we can decide whether 2.0 is the appropriate setting for him to remain at or whether we can consider changing the shunt setting.</t>
+          <t>EXAM:,  Bilateral carotid ultrasound.,REASON FOR EXAM: , Headache.,TECHNIQUE:  ,Color grayscale and Doppler analysis is employed.,FINDINGS:,  On the grayscale images, the right common carotid artery demonstrates patency with mild intimal thickening only.  At the level of the carotid bifurcation, there is heterogeneous hard plaque present, but without grayscale evidence of greater than 50% stenosis.  Right common carotid waveform is normal with a peak systolic velocity of 0.474 m/second and an end-diastolic velocity of 0.131 m/second.  The right ECA is patent as well with the velocity measurement 0.910 m/second.,The right internal carotid artery at the bifurcation demonstrates plaque formation, but no evidence of greater than 50% stenosis.  Proximal peak systolic velocity in the internal carotid artery is 0.463 m/second with proximal end-diastolic velocity of 0.170.  The mid internal carotid peak systolic velocity is 0.564 m/second, and mid ICA end-diastolic velocity is 0.199 m/second.  Right ICA distal PSV 0.580 m/second, right ICA distal EDV 0.204 m/second.  Vertebral flow is antegrade on the right at 0.469 m/second.,On the left, the common carotid artery demonstrates intimal thickening, but is otherwise patent.  At the level of the bifurcation, however, there is more pronounced plaque formation with approximately 50% stenosis by the grayscale analysis.  See the velocity measurements below:,Left carotid ECA measurement 0.938 m/second.  Left common carotid PSV 0.686 m/second, and left common carotid end-diastolic velocity 0.137 m/second.,Left internal carotid artery again demonstrates prominent focus of hard plaque with up to at least 50% stenosis.  This should be further assessed with CTA for more precise measurement.  The left proximal ICA/PSV 0.955 m/second, left proximal ICA/EDV 0.287 m/second.  There is spectral broadening in the proximal aspect of the carotid waveform.  The left carotid ICA mid PSV 0.895, left carotid ICA mid EDV 0.278 with also spectral broadening present.,The left distal ICA/PSV 0.561, left distal ICA/EDV 0.206, again the spectral broadening present.  Vertebral flow is antegrade at 0.468 m/second.,IMPRESSION: , The study demonstrates bilateral hard plaque at the bifurcation, left greater than right.  There is at least 50% stenosis of the left internal carotid artery at its bifurcation and a followup CTA is recommended for further assessment.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>neurology, ct scan, subdural, adult hydrocephalus, bilateral effusions, shunt setting, subdural effusions, hydrocephalus, ventricular, scan, ct,</t>
+          <t>neurology, doppler analysis, headache, edv, ica, eca, psv, distal ica/edv, hard plaque, bilateral carotid ultrasound, peak systolic velocity, internal carotid artery, plaque formation, carotid ultrasound, carotid artery, carotid, stenosis, proximal, artery, velocity</t>
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>217</v>
+        <v>348</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Neurology; short; diagnostic report; diagnoses + imaging + treatment plans</t>
+          <t>Neurology; medium; diagnostic report; middle text complexity; diagnoses + imaging + treatment plans</t>
         </is>
       </c>
       <c r="J33" s="2" t="n">
-        <v>2920</v>
+        <v>2964</v>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
@@ -2501,21 +2501,21 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>middle</t>
         </is>
       </c>
       <c r="M33" s="2" t="n">
-        <v>0.2989179440937781</v>
+        <v>0.3897655545536519</v>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; imaging; treatment plans; assessment/plan</t>
+          <t>diagnoses; imaging; treatment plans; follow-up</t>
         </is>
       </c>
     </row>
     <row r="34" ht="110" customHeight="1">
       <c r="A34" s="2" t="n">
-        <v>2868</v>
+        <v>2936</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
@@ -2524,62 +2524,62 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Headache - Office Visit </t>
+          <t xml:space="preserve"> Craniotomy - Frontotemporal - 1 </t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The patient with continued problems with her headaches. </t>
+          <t xml:space="preserve"> Acute left subdural hematoma.  Left frontal temporal craniotomy for evacuation of acute subdural hematoma.  CT imaging reveals an acute left subdural hematoma, which is hemispheric.</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>She also had EMG/nerve conduction studies since she was last seen in our office that showed severe left ulnar neuropathy, moderate right ulnar neuropathy, bilateral mild-to-moderate carpal tunnel and diabetic neuropathy.  She was referred to Dr. XYZ and will be seeing him on August 8, 2006.,She was also never referred to the endocrine clinic to deal with her poor diabetes control.  Her last hemoglobin A1c was 10.,PAST MEDICAL HISTORY:,  Diabetes, hypertension, elevated lipids, status post CVA, and diabetic retinopathy.,MEDICATIONS: , Glyburide, Avandia, metformin, lisinopril, Lipitor, aspirin, metoprolol and Zonegran.,PHYSICAL EXAMINATION:,  Blood pressure was 140/70, heart rate was 76, respiratory rate was 18, and weight was 226 pounds.  On general exam she has an area of tenderness on palpation in the left parietal region of her scalp.  Neurological exam is detailed on our H&amp;P form.  Her neurological exam is within normal limits.,IMPRESSION AND PLAN:,  For her headaches we are going to titrate Zonegran up to 200 mg q.h.s. to try to maximize the Zonegran therapy.  If this is not effective, when she comes back on August 7, 2006 we will then consider other anticonvulsants such as Neurontin or Lyrica.  We also discussed with Ms. Hawkins the possibility of nerve block injection; however, at this point she is not interested.,She will be seeing Dr. XYZ for her neuropathies.,We made an appointment in endocrine clinic today for a counseling in terms of better diabetes control and she is responsible for trying to get her referral from her primary care physician to go for this consult.</t>
+          <t>PREOPERATIVE DIAGNOSIS:,  Acute left subdural hematoma.,POSTOPERATIVE DIAGNOSIS:,  Acute left subdural hematoma.,PROCEDURE:,  Left frontal temporal craniotomy for evacuation of acute subdural hematoma.,DESCRIPTION OF PROCEDURE: , This is a 76-year-old man who has a history of acute leukemia.  He is currently in the phase of his therapy where he has developed a profound thrombocytopenia and white cell deficiency.  He presents after a fall in the hospital in which he apparently struck his head and now has a progressive neurologic deterioration consistent with an intracerebral injury.  His CT imaging reveals an acute left subdural hematoma, which is hemispheric.,The patient was brought to the operating room, placed under satisfactory general endotracheal anesthesia.  He had previously been intubated and taken to the Intensive Care Unit and now is brought for emergency craniotomy.  The images were brought up on the electronic imaging and confirmed that this was a left-sided condition.  He was fixed in a three-point headrest.  His scalp was shaved and prepared with Betadine, iodine and alcohol.  We made a small curved incision over the temporal, parietal, frontal region.  The scalp was reflected.  A single bur hole was made at the frontoparietal junction and then a 4x6cm bur hole was created.  After completing the bur hole flap, the dura was opened and a gelatinous mass of subdural was peeled away from the brain.  The brain actually looked relatively relaxed; and after removal of the hematoma, the brain sort of slowly came back up.  We investigated the subdural space forward and backward as we could and yet careful not to disrupt any venous bleeding as we close to the midline.  After we felt that we had an adequate decompression, the dura was reapproximated and we filled the subdural space with saline.  We placed a small drain in the extra dural space and then replaced the bone flap and secured this with the bone plates.  The scalp was reapproximated, and the patient was awakened and taken to the CT scanner for a postoperative scan to ensure that there was no new hemorrhage or any other intracerebral pathology that warranted treatment.  Given that this actual skin looked good with apparent removal of about 80% of the subdural we elected to take patient to the Intensive Care Unit for further management.,I was present for the entire procedure and supervised this.  I confirmed prior to closing the skin that we had correct sponge and needle counts and the only foreign body was the drain.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>neurology, nerve conduction studies, emg, zonegran therapy, ulnar neuropathy, endocrine clinic, diabetes control, neurological exam, headache, zonegran</t>
+          <t xml:space="preserve">neurology, subdural, hematoma, temporal craniotomy, craniotomy, subdural space, bur hole, subdural hematoma, </t>
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>252</v>
+        <v>404</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Neurology; short; follow-up/progress; diagnoses + medications + laboratory values</t>
+          <t>Neurology; medium; procedure/operative; lower text complexity; diagnoses + procedures + imaging</t>
         </is>
       </c>
       <c r="J34" s="2" t="n">
-        <v>2868</v>
+        <v>2936</v>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>follow-up/progress</t>
+          <t>procedure/operative</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="M34" s="2" t="n">
-        <v>0.4283701532912534</v>
+        <v>0.3485685302073941</v>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; medications; laboratory values; vital signs; past history; treatment plans; follow-up; assessment/plan</t>
+          <t>diagnoses; procedures; imaging; past history; treatment plans; surgery</t>
         </is>
       </c>
     </row>
     <row r="35" ht="110" customHeight="1">
       <c r="A35" s="2" t="n">
-        <v>2964</v>
+        <v>2756</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
@@ -2588,26 +2588,26 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Carotid Ultrasound </t>
+          <t xml:space="preserve"> Wilson's Disease - Letter </t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Bilateral carotid ultrasound.</t>
+          <t xml:space="preserve"> A pleasant gentleman with a history of Wilson's disease who has been treated with penicillamine.</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>EXAM:,  Bilateral carotid ultrasound.,REASON FOR EXAM: , Headache.,TECHNIQUE:  ,Color grayscale and Doppler analysis is employed.,FINDINGS:,  On the grayscale images, the right common carotid artery demonstrates patency with mild intimal thickening only.  At the level of the carotid bifurcation, there is heterogeneous hard plaque present, but without grayscale evidence of greater than 50% stenosis.  Right common carotid waveform is normal with a peak systolic velocity of 0.474 m/second and an end-diastolic velocity of 0.131 m/second.  The right ECA is patent as well with the velocity measurement 0.910 m/second.,The right internal carotid artery at the bifurcation demonstrates plaque formation, but no evidence of greater than 50% stenosis.  Proximal peak systolic velocity in the internal carotid artery is 0.463 m/second with proximal end-diastolic velocity of 0.170.  The mid internal carotid peak systolic velocity is 0.564 m/second, and mid ICA end-diastolic velocity is 0.199 m/second.  Right ICA distal PSV 0.580 m/second, right ICA distal EDV 0.204 m/second.  Vertebral flow is antegrade on the right at 0.469 m/second.,On the left, the common carotid artery demonstrates intimal thickening, but is otherwise patent.  At the level of the bifurcation, however, there is more pronounced plaque formation with approximately 50% stenosis by the grayscale analysis.  See the velocity measurements below:,Left carotid ECA measurement 0.938 m/second.  Left common carotid PSV 0.686 m/second, and left common carotid end-diastolic velocity 0.137 m/second.,Left internal carotid artery again demonstrates prominent focus of hard plaque with up to at least 50% stenosis.  This should be further assessed with CTA for more precise measurement.  The left proximal ICA/PSV 0.955 m/second, left proximal ICA/EDV 0.287 m/second.  There is spectral broadening in the proximal aspect of the carotid waveform.  The left carotid ICA mid PSV 0.895, left carotid ICA mid EDV 0.278 with also spectral broadening present.,The left distal ICA/PSV 0.561, left distal ICA/EDV 0.206, again the spectral broadening present.  Vertebral flow is antegrade at 0.468 m/second.,IMPRESSION: , The study demonstrates bilateral hard plaque at the bifurcation, left greater than right.  There is at least 50% stenosis of the left internal carotid artery at its bifurcation and a followup CTA is recommended for further assessment.</t>
+          <t>Doctor's Address,Dear Doctor:,This letter is an introduction to my patient, A, who you will be seeing in the near future.  He is a pleasant gentleman with a history of Wilson's disease.  It has been treated with penicillamine.  He was diagnosed with this at age 14.  He was on his way to South Carolina for a trip when he developed shortness of breath, palpitations, and chest discomfort.  He went to the closest hospital that they were near in Randolph, North Carolina and he was found to be in atrial fibrillation with rapid rate.  He was admitted there and observed.  He converted to normal sinus rhythm spontaneously and so he required no further interventions.  He was started on Lopressor, which he has tolerated well.  An echocardiogram was performed, which revealed mild-to-moderate left atrial enlargement.  Normal ejection fraction.  No other significant valvular abnormality.  He reported to physicians there that he had cirrhosis related to his Wilson's disease.  Therefore hepatologist was consulted.  There was a recommendation to avoid Coumadin secondary to his questionable significant liver disease, therefore he was placed on aspirin 325 mg once a day.,In discussion with Mr. A and review of his chart that I have available, it is unclear as to the status of his liver disease, however, he has never had a liver biopsy, so his diagnosis of cirrhosis that they were concerned about in North Carolina is in doubt.  His LFTs have remained normal and his copper level has been undetectable on his current dose of penicillamine.,I would appreciate your input into the long term management of his anticoagulation and also any recommendations you would have about rhythm control.  He is in normal sinus rhythm as of my evaluation of him on 06/12/2008.  He is tolerating his metoprolol and aspirin without any difficulty.  I guess the big question remains is what level of risk that is entailed by placing him on Coumadin therapy due to his potentially paroxysmal atrial fibrillation and evidence of left atrial enlargement that would place him in increased risk of recurrent episodes.,I appreciate your input regarding this friendly gentleman.  His current medicines include penicillamine 250 mg p.o. four times a day, metoprolol 12.5 mg twice a day, and aspirin 325 mg a day.,If you have any questions regarding his care, please feel free to call me to discuss his case.  Otherwise, I will look forward to hearing back from you regarding his evaluation.  Thank you as always for your care of our patient.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>neurology, doppler analysis, headache, edv, ica, eca, psv, distal ica/edv, hard plaque, bilateral carotid ultrasound, peak systolic velocity, internal carotid artery, plaque formation, carotid ultrasound, carotid artery, carotid, stenosis, proximal, artery, velocity</t>
+          <t>neurology, atrial enlargement, wilson's disease, penicillamine,</t>
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>348</v>
+        <v>409</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
@@ -2616,34 +2616,34 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Neurology; medium; diagnostic report; diagnoses + imaging + treatment plans</t>
+          <t>Neurology; medium; other narrative/sectioned; lower text complexity; diagnoses + medications + procedures</t>
         </is>
       </c>
       <c r="J35" s="2" t="n">
-        <v>2964</v>
+        <v>2756</v>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>diagnostic report</t>
+          <t>other narrative/sectioned</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="M35" s="2" t="n">
-        <v>0.3897655545536519</v>
+        <v>0.3789449954914337</v>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; imaging; treatment plans; follow-up</t>
+          <t>diagnoses; medications; procedures; imaging; past history; treatment plans</t>
         </is>
       </c>
     </row>
     <row r="36" ht="110" customHeight="1">
       <c r="A36" s="2" t="n">
-        <v>2796</v>
+        <v>2946</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
@@ -2652,35 +2652,35 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Neurologic Consultation - 5 </t>
+          <t xml:space="preserve"> Consult - Migraine </t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Approximately one and a half years ago, patient fell down while walking in the living room from the bedroom.  At that time, he reports both legs gave away on him and he fell.  He reported that he had some lightheadedness just before he fell and was slightly confused, but was aware of what was happening around him.</t>
+          <t xml:space="preserve"> The patient is a 36-year-old female with past medical history of migraine headaches, who was brought to the ER after she was having uncontrolled headaches.  In the ER, the patient had a CT scan done, which was reported negative, and lumbar puncture with normal pressure and the cell count, and was admitted for followup.</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS: ,The patient is a 79-year-old right-handed man who reports that approximately one and a half years ago, he fell down while walking in the living room from the bedroom.  At that time, he reports both legs gave away on him and he fell.  He reported that he had some lightheadedness just before he fell and was slightly confused, but was aware of what was happening around him.  He was able to get up shortly after falling and according to the patient and his son, subsequently returned back to normal.,He was then well until the 3rd of July 2008 when his legs again gave way on him.  This was not preceded by lightheadedness.  He was rushed to the hospital and was found to have pneumonia, and the fall was blamed on the pneumonia.  He started using a walker from that time, prior to that he was able to walk approximately two miles per day.  He again had a fall in August of 2008 after his legs gave way.  Again, there was no lightheadedness associated with this.  He was again found to have pneumonia and again was admitted to hospital after which he went to rehabilitation and was able to use his walker again after this.  He did not, however, return to the pre-July baseline.  In October of 2008, after another fall, he was found to have pneumonia again and shingles.  He is currently in a Chronic Rehabilitation Unit.  He cannot use a walker and uses a wheelchair for everything.  He states that his hands have been numb, involving all the fingers of both hands for the past three weeks.  He is also losing muscle bulk in his hands and has noticed some general weakness of his hands.  He does, however, note that strength in his hands has not been normal since July 2008, but it is clearly getting worse.  He has been aware of some fasciculations in his legs starting in August 2008, these are present both in the lower legs and the thighs.  He does not report any cramps, problems with swallowing or problems with breathing.  He reports that he has had constipation alternating with diarrhea, although there has been no loss of control of either his bowel or bladder.  He has had some problems with blood pressure drops, and does feel presyncopal when he stands.  He also reports that he has no feeling in his feet, and that his feet feel like sponges.  This has been present for about nine months.  He has also lost joint position sense in his feet for approximately nine months.,PAST MEDICAL HISTORY:,1.  Pneumonia.  He has had recurrent episodes of pneumonia, which started at approximately age 20.  These have been treated repeatedly over the years, and on average he has tended to have an episode of pneumonia once every five years, although this has been far more frequent in the past year.  He is usually treated with antibiotics and then discharged.  There is no known history of bronchiectasis, inherited lung disease or another chronic pulmonary cause for the repeated pneumonia.,2.  He has had a catheter placed for urinary retention, his urologist has told him that he thinks that this may be due to prostate enlargement.  The patient does not have any history of diabetes and does not report any other medical problems.  He has lost approximately 18 pounds in the past month.,3.  He had an appendectomy in the 1940s.,4.  He had an ankle resection in 1975.,SOCIAL HISTORY:  ,The patient stopped smoking 27 years ago, he smoked approximately two packs a day with combined cigarettes and cigars.  He has not smoked for the past 27 years.  He hardly ever uses alcohol.  He is currently retired.,FAMILY HISTORY: , There is no family history of neuropathy, pes cavus, foot deformities, or neuromuscular diseases.  His aunt has a history of type II diabetes.,CURRENT MEDICATIONS: , Fludrocortisone 0.1 mg p.o. q.d., midodrine 5 mg p.o. q.i.d., Cymbalta 30 mg p.o. per day, Prilosec 20 mg p.o. per day, Lortab 10 mg p.o. per day, Amoxil 500 mg p.o. per day, vitamin B12 1000 mcg weekly, vitamin D 1000 units per day, Metamucil p.r.n., enteric-coated aspirin once a day, Colace 200 mg p.o. q.d., Senokot three tablets p.o. p.r.n., Reglan 10 mg p.o. q.6h., Xanax 0.25 mg p.o. q.8h. p.r.n., Ambien 5 mg p.o. q.h.s. p.r.n. and Dilaudid 2 mg tablets p.o. q.3h. p.r.n., Protonix 40 mg per day, and Megace 400 mg per day.,ALLERGIES:,  He has no medication or food allergies.,REVIEW OF SYSTEMS:,  Please see the health questionnaire and clinical notes from today.,GENERAL PHYSICAL EXAMINATION:,VITAL SIGNS:  BP was 137/60, P was 89, and his weight could not be measured because he was in a wheelchair.  His pain score was 0.,APPEARANCE:  No acute distress.  He is pleasant and well-groomed.,HEENT:  Atraumatic, normocephalic.  No carotid bruits appreciated.,LUNGS:  There were few coarse crackles in both lung bases.,CARDIOVASCULAR:  Revealed a normal first and second heart sound, with no third or fourth heart sound and no murmurs.  The pulse was regular and of normal volume.,ABDOMEN:  Soft with no masses and normal bowel sounds.  There were no carotid bruits.,EXTREMITIES:  No contractures appreciated.,NEUROLOGICAL EXAM:,MSE:  His orientation, language, calculations, 100-7 tests were all normal.  There was atrophy and fasciculations in both the arms and legs.,CRANIAL NERVES:  Cranial nerve examination was normal with the exception that there was some mild atrophy of his tongue and possible fasciculations.  His palatal movement was normal and gag reflex was normal.,MOTOR:  Strength was decreased in all muscle groups as follows:  Deltoid 4/4, biceps 4+/4+, triceps 5/5, wrist extensors 4+/4+, finger extensors 4-/4-, finger flexors 4-/4-, interossei 4-/4-, hip flexors 4+/4+, hip extensors 4+/4+, knee extensors 4/4, and knee flexors 4/4.  Foot dorsiflexion, plantar flexion, eversion, toe extension and toe flexion was all 0 to 1.  There was atrophy in both hands and general atrophy of the lower limb muscles.  The feet were both cold and showed dystrophic features.  Fasciculations were present mainly in the hands.  There was evidence of dysmetria and past pointing in the left hand.,REFLEXES:  Reflexes were 0 in all sites in the arms and legs.  The jaw reflex was 2+.  Vibration was severely decreased at the elbow and wrist and was absent in the fingers.  Vibration was absent in the toes and ankle bilaterally and was severely decreased at the knee.  Joint position sense was absent in the toes and severely decreased in the fingers.  Pin perception was absent in the feet and was decreased to the upper thighs.  Pin was decreased or absent in the fingers and decreased above the elbows.  The same distribution of sensory loss was found with monofilament testing.,COORDINATION:  Coordination was barely normal in the right hand.  Rapid alternating movements were decreased in the left hand greater than the right hand.  The patient was unable to stand and therefore gait, Romberg's test and balance could not be assessed.,DIAGNOSTIC STUDIES: , Previous diagnostic studies and patient reports.  There were extensive patient reports, all of which were reviewed.  A previous x-ray study of the lateral chest performed in October 2008 showed poor inspiration with basilar atelectasis and an infiltrate.  An x-ray of the cervical, thoracic and lumbar spine showed some evidence of lumbar spinal stenosis.  A CTA of the neck with and without contrast performed in November 2008 showed minor stenosis in the left carotid, a mild hard and soft plaque in the right carotid with approximately 55% stenosis.  The posterior circulation showed a slightly dominant right vertebral artery with no stenosis.  There was no significant stenosis, but there was minor extracranial stenosis noted.  An MRI of the brain with and without contrast performed in November 2008 showed no evidence of an acute infarct, major vascular occlusion, and no abnormal enhancement with gadolinium administration.  There was also no significant sinusitis or mastoiditis.  This was an essentially normal brain MRI.  A CBC performed in January 2009 showed an elevated white cell count of 11.3, a low red cell count of 3.43, elevated MCH of 32.4 and the rest of the study was normal.  An electrolyte study performed in January 2009 showed a sodium which was low at 127, a calcium which was low at 8.3, and a low protein of 5.2 and albumin of 3.1.  The glucose was 86.  TSH performed in January 2009 was 1.57, which is within the normal range.  Vitamin B12 was greater than a 1000, which is normal and the folate was 18.2, which was normal.  A myocardial stress study performed in December 2008 showed normal myocardial perfusion with Persantine Cardiolite SPECT.  The ECG was non-diagnostic.  There was normal regional wall motion of the left ventricle.  The left ventricular ejection fraction was 68%, which is within the normal range for males.  A CT of the lumbar spine without contrast performed in December 2008 showed a broad-based disc bulge at L1-L2, L2-L3, L3-L4 and L4-L5.  At L5-S1, in addition to the broad-based disc bulge, there was also an osteophyte complex and evidence of flavum hypertrophy without canal stenosis.  There was severe bilateral neural foraminal stenosis at L5-S1 and moderate neural foraminal stenosis at L1-L4.  An echocardiogram was performed in November 2008 and showed mild left atrial enlargement, normal left ventricular systolic function, mild concentric left ventricular hypertrophy, scleral degenerative changes in the aortic and mitral apparatus, mild mitral regurgitation, mild tricuspid regurgitation and mild to moderate aortic regurgitation.,DIAGNOSTIC IMPRESSION:  ,The patient presents with a severe neuropathy with marked large fiber sensory as well as motor findings.  He is diffusely weak as well as atrophic in all muscle groups both in his upper and lower extremities, although he is disproportionately weak in his lower extremities.  His proprioceptive and vibratory loss is severe in both the distal upper and lower extremities, signifying that he either has a severe sensory neuropathy or has involvement of the dorsal root ganglia.  According to the history, which was carefully checked, the initial onset of these symptoms goes back one and a half years, although there has only been significant progression in his condition since July 2008.  As indicated below, further diagnostic studies including a detailed nerve conduction and EMG test today showed evidence of a severe sensory, motor, and axonal neuropathy and in addition there was evidence of a diffuse polyradiculopathy.  There was no involvement of the tongue on EMG.  The laboratory testing as indicated below failed to show a specific cause for the neuropathy.  We are still, however, waiting for the paraneoplastic antibodies, which were send out lab to the Mayo Clinic.  This type of very severe sensorimotor neuropathy with significant proprioceptive loss may be seen in several conditions including peripheral nerve vasculitis due to a variety of disorders such as SLE, Sjogren's, rheumatoid arthritis, and mixed connective tissue disease.  In addition, it may also be seen with certain toxins, particularly chemotherapeutic agents.  The patient did not receive any of these.  It may also be seen as part of a paraneoplastic syndrome.  Although the patient does not have any specific clinical symptoms of a cancer, it is noted that he has had an 18-pound weight loss in the past month and does have a remote history of smoking.  We have requested that he obtain a CT of his chest, abdomen and pelvis while he is in Acute Rehabilitation.  The verbal reports of these possibly did not show any evidence of a cancer.  We did also request that he obtain a gallium scan to see if there was any evidence of an unsuspected neoplasm.  The patient did undergo a nerve and muscle biopsy, this was a radial nerve and biceps muscle biopsy from the left arm.  This showed evidence of severe axonal loss.  There was no evidence of a vasculitis.  The vessels did show some mild intimal changes that would be consistent with atherosclerosis.  There were a few perivascular changes; however, there was no clear evidence of a necrotizing vasculitis even on multiple sections.  The muscle biopsy showed severe muscle fiber atrophy, with evidence of fiber grouping.  Again, there was no evidence of inflammation or vasculitis.  Evaluation so far has also shown no evidence of an amyloid neuropathy, no evidence of a monoclonal gammopathy, of sarcoidosis, and again there is no past history of a significant toxin or infective cause for the neuropathy.  Specifically, there is no history of HIV exposure.  We would await the results of the gallium scan and of the paraneoplastic antibodies to see if these are helpful in making a diagnosis.  At this point, because of the severity and the axonal nature of the neuropathy, there is no specific therapy that will reverse the course of the illness, unless we find a specific etiology that can be stopped or reversed.  I have discussed these issues at length with the patient and with his son.  We also addressed whether or not there might be a previously undiagnosed inherited neuropathy.  I think this is unlikely given the short history and the rapid progression of the disorder.,There is also no family history that we can detect a neuropathy, and the patient does not have the typical phenotype for a chronic inherited neuropathy such as Charcot-Marie-Tooth disease type 2.  However, since I have only seen the patient on one occasion and do not know what his previous examination showed two years ago, I cannot be certain that there may not have been the presence of a neuropathy preceding this.,PLAN:,1.  Nerve conduction and EMG will be performed today.  The results were indicated above.,2.  The following laboratory studies were requested including electrolytes, CBC, thyroid function tests, B12, ANA, C-reactive protein, complement, cryoglobulins, double-stranded DNA antibodies, folate level, hemoglobin A1c, immunofixation electrophoresis, P-ANCA, C-ANCA, protein electrophoresis, rheumatoid factor, paraneoplastic antibody studies requested from the Mayo Clinic, B12.  These studies showed minor changes, which included a low sodium level of 129 as previously noted, a low creatinine of 0.74, low calcium of 8.6, low total protein of 5.7.  The B12 was greater than 2000.  The immunoelectrophoresis, ANA, double-stranded DNA, ANCA, hemoglobin A1c, folate, cryoglobulins, complement, C-reactive protein were all normal or negative.  The B12 level was greater than 2000.  Liver function tests were normal.  The glucose was 90.  ESR was 10.  Hemoglobin A1c was 5.5.,3.  A left radial sensory and left biceps biopsy were requested and have been performed and interpreted as indicated above.,4.  CT of chest, abdomen and pelvis.,5.  Whole body gallium scan for evidence of an underlying neoplasm.,6.  The patient will go to the Rehabilitation Facility for Acute Rehabilitation and Training.,7.  We have not made any changes to his medication.  He does have some mild orthostatic changes; however, he is adequately controlled with midodrine at a dose of 2.5 mg three times a day as needed up to 5 mg four times a day.  Usually, he uses a lower dose of 2.5 three times a day to 5 mg three times a day.,8.  Followup will be as determined by the family.</t>
+          <t>HISTORY OF PRESENT ILLNESS: , The patient is a 36-year-old female with past medical history of migraine headaches, who was brought to the ER after she was having uncontrolled headaches.  In the ER, the patient had a CT scan done, which was reported negative, and lumbar puncture with normal pressure and the cell count, and was admitted for followup.  Neurology consult was called to evaluate the patient in view of the current symptomatology.  The headaches were refractory to the treatment.  The patient has been on Topamax and Maxalt in the past, but did not work and according to the patient she got more confused.,PAST MEDICAL HISTORY: , History of migraine.,PAST SURGICAL HISTORY:  ,Significant for partial oophorectomy, appendectomy, and abdominoplasty.,SOCIAL HISTORY:  ,No history of any smoking, alcohol, or drug abuse.  The patient is a registered nurse by profession.,MEDICATIONS: , Currently taking no medication.,ALLERGIES: , No known allergies.,FAMILY HISTORY:,  Nothing significant.,REVIEW OF SYSTEMS: , The patient was considered to ask systemic review including neurology, psychiatry, sleep, ENT, ophthalmology, pulmonary, cardiology, gastroenterology, genitourinary, hematology, rheumatology, dermatology, allergy, immunology, endocrinology, toxicology, oncology, and was found to be positive for the symptoms mentioned in the history of the presenting illness.,PHYSICAL EXAMINATION,VITAL SIGNS:  Blood pressure of 115/66, heart rate of 69, respiratory rate of 13, temperature normal, and pulse oximetry 98% on room air at the time of initial evaluation.,HEENT:  Head, normocephalic, atraumatic.  Neck supple.  Throat clear.  No discharge from the ears or nose.  No discoloration of conjunctivae and sclerae.  No bruits auscultated over temple, orbits, or the neck.,LUNGS:  Clear to auscultation.,CARDIOVASCULAR:  Normal heart sounds.,ABDOMEN:  Benign.,EXTREMITIES:  No edema, clubbing or cyanosis.,SKIN:  No rash.  No neurocutaneous disorder.,MENTAL STATUS:  The patient is awake, alert and oriented to place and person.  Speech is fluent.  No language deficits.  Mood normal.  Affect is clear.  Memory and insight is normal.  No abnormality with thought processing and thought content.  Cranial nerve examination intact II through XII.  Motor examination:  Normal bulk, tone and power.  Deep tendon reflexes symmetrical.  Downgoing toes.  No sign of any myelopathy.  Cortical sensation intact.  Peripheral sensation grossly intact.  Vibratory sense not tested.  Gait not tested.  Coordination is normal with no dysmetria.,IMPRESSION: , Intractable headaches, by description to be migraines.  Complicated migraines by clinical criteria.  Rule out sinusitis.  Rule out vasculitis including temporal and arthritis, lupus, polyarthritis, moyamoya disease, Takayasu and Kawasaki disease.,PLAN AND RECOMMENDATIONS: , The patient to be given a trial of the prednisone with a plan to taper off in 6 days, as she already had received 50 mg today.  Depakote as a part of migraine prophylaxis and Fioricet on p.r.n. basis.,The patient to get vasculitis workup, as it has not been ordered by the primary care physician initially.  The patient already had MRI of the brain and the cervical spine.  MRI of the brain reported negative and cervical spine as shown signs of disk protrusion at C5 and C6 level, which will not explain of the temporal headache.  Plan and followup discussed with the patient in detail.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="2" t="n">
-        <v>2460</v>
+        <v>490</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Neurology; long; consultation; diagnoses + symptoms + medications</t>
+          <t>Neurology; medium; consultation; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J36" s="2" t="n">
-        <v>2796</v>
+        <v>2946</v>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
@@ -2693,17 +2693,17 @@
         </is>
       </c>
       <c r="M36" s="2" t="n">
-        <v>0.9954350766456268</v>
+        <v>0.7585099188458071</v>
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; follow-up; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; imaging; past history; treatment plans; follow-up; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="37" ht="110" customHeight="1">
       <c r="A37" s="2" t="n">
-        <v>2270</v>
+        <v>2359</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
@@ -2712,56 +2712,52 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Closed Reduction - 1 </t>
+          <t xml:space="preserve"> Ankle Sprain - H&amp;P </t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Right distal both-bone forearm fracture.  Closed reduction under conscious sedation and application of a splint was warranted.</t>
+          <t xml:space="preserve"> History and Physical for right ankle sprain</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>PREOPERATIVE DIAGNOSIS: , Right distal both-bone forearm fracture.,POSTOPERATIVE DIAGNOSIS: , Right distal both-bone forearm fracture.,INDICATIONS:,  Mr. ABC is a 10-year-old boy who suffered a fall resulting in a right distal both-bone forearm fracture.  Upon evaluation by Orthopedic Surgery team in the emergency department, it was determined that a closed reduction under conscious sedation and application of a splint was warranted.  This was discussed with the parents who expressed verbal and written consent.,PROCEDURE:,  Conscious sedation was achieved via propofol via the emergency department staff.  Afterwards, traction with re-creation of the injury pattern was utilized to achieve reduction of the patient's fracture.  This was confirmed with image intensifier.  Subsequently, the patient was placed into a splint.  The patient was aroused from conscious sedation and at this time it was noted that he had full sensation throughout radial, median, and ulnar nerve distributions and positive extensor pollicis longus, flexor pollicis longus, dorsal and palmar interossei.,DISPOSITION:  ,Post-reduction x-rays revealed good alignment in the AP x-rays.  The lateral x-rays also revealed adequate reduction.  At this time, we will allow the patient to be discharged home and have him follow up with Dr. XYZ in one week.</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">orthopedic, closed reduction, distal both bone forearm, emergency department, pollicis longus, bone forearm, forearm fracture, conscious sedation, emergency, department, pollicis, longus, splint, distal, bone, forearm, conscious, sedation, fracture, reduction, </t>
-        </is>
-      </c>
+          <t>CHIEF COMPLAINT:,  Right ankle sprain.,HISTORY OF PRESENT ILLNESS: , This is a 56-year-old female who fell on November 26, 2007 at 11:30 a.m. while at work.  She did not recall the specifics of her injury but she thinks that her right foot inverted and subsequently noticed pain in the right ankle.  She describes no other injury at this time.,PAST MEDICAL HISTORY: , Hypertension and anxiety.,PAST SURGICAL HISTORY: , None.,MEDICATIONS: , She takes Lexapro and a blood pressure pill, but does not know anything more about the names and the doses.,ALLERGIES:,  No known drug allergies.,SOCIAL HISTORY: , The patient lives here locally.  She does not report any significant alcohol or illicit drug use.  She works full time.,FAMILY HISTORY:,  Noncontributory.,REVIEW OF SYSTEMS:,Pulm:  No cough, No wheezing, No shortness of breath,CV:  No chest pain or palpitations,GI:  No abdominal pain.  No nausea, vomiting, or diarrhea.,PHYSICAL EXAM:,GENERAL APPEARANCE:  No acute distress,VITAL SIGNS:  Temperature 97.8, blood pressure 122/74, heart rate 76, respirations 24, weight 250 lbs, O2 sat 95% on R.A.,NECK:  Supple.  No lymphadenopathy.  No thyromegaly.,CHEST:  Clear to auscultation bilaterally.,HEART:  Regular rate and rhythm.  No murmurs.,ABDOMEN:  Non-distended, nontender, normal active bowel sounds.,EXTREMITIES:  No Clubbing, No Cyanosis, No edema.,MUSCULOSKELETAL:  The spine is straight and there is no significant muscle spasm or tenderness there.  Both knees appear to be non-traumatic with no deformity or significant tenderness.  The right ankle has some swelling just below the right lateral malleolus and the dorsum of the foot is tender.  There is decreased range of motion and some mild ecchymosis noted around the ankle.,DIAGNOSTIC DATA: , X-ray of the right ankle reveals no acute fracture by my observation.  Radiologic interpretation is pending., ,IMPRESSION:,  Right ankle sprain.,PLAN:,1.  Motrin 800 mg t.i.d.,2.  Tylenol 1 gm q.i.d. as needed.,3.  Walking cast is prescribed.,4.  I told the patient to call back if any problems.  The next morning she called back complaining of worsening pain and I called in some Vicodin ES 1-2 p.o. q.  8 hours p.r.n. pain #60 with no refills.</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr"/>
       <c r="G37" s="2" t="n">
-        <v>191</v>
+        <v>326</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Orthopedic; short; procedure/operative; diagnoses + procedures + imaging</t>
+          <t>Orthopedic; medium; history and physical; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J37" s="2" t="n">
-        <v>2270</v>
+        <v>2359</v>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>procedure/operative</t>
+          <t>history and physical</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>higher</t>
         </is>
       </c>
       <c r="M37" s="2" t="n">
-        <v>0.2753043282236249</v>
+        <v>0.7403629395852119</v>
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; procedures; imaging; follow-up; surgery</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; imaging; past history; treatment plans; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2800,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Orthopedic; medium; other narrative/sectioned; diagnoses + symptoms + medications</t>
+          <t>Orthopedic; medium; other narrative/sectioned; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J38" s="2" t="n">
@@ -2831,7 +2827,7 @@
     </row>
     <row r="39" ht="110" customHeight="1">
       <c r="A39" s="2" t="n">
-        <v>2078</v>
+        <v>2059</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
@@ -2840,39 +2836,39 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Physical Therapy - Low Back Pain  </t>
+          <t xml:space="preserve"> Rotator cuff syndrome - H&amp;P </t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The patient is a 26-year-old female, referred to Physical Therapy for low back pain.  The patient has a history of traumatic injury to low back.</t>
+          <t xml:space="preserve"> Shoulder pain, right shoulder diffusely - Rotator cuff syndrome, right.</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS: , The patient is a 26-year-old female, referred to Physical Therapy for low back pain.  The patient has a history of traumatic injury to low back.  The patient stated initial injury occurred eight years ago, when she fell at a ABC Store.  The patient stated she received physical therapy, one to two visits and received modality treatment only, specifically electrical stimulation and heat pack per patient recollection.  The patient stated that she has had continuous low-back pain at varying degrees for the past eight years since that fall.  The patient gave birth in August 2008 and since the childbirth, has experienced low back pain.  The patient also states that she fell four to five days ago, while mopping her floor.  The patient stated that she landed on her tailbone and symptoms have increased since that fall.  The patient stated that her initial physician examination with Dr. X was on 01/10/09, and has a followup appointment on 02/10/09.,PAST MEDICAL HISTORY: , The patient denies high blood pressure, diabetes, heart disease, lung disease, thyroid, kidney, or bladder dysfunctions.  The patient stated that she quit smoking prior to her past childbirth and is currently not pregnant.  The patient has had a C-section and also an appendectomy.  The patient was involved in a motor vehicle accident four to five years ago and at that time, the patient did not require any physical therapy nor did she report any complaints of increased back pain following that accident.,MEDICATIONS: , Patient currently states she is taking:,1.  Vicodin 500 mg two times a day.,2.  Risperdal.,3.  Zoloft.,4.  Stool softeners.,5.  Prenatal pills.,DIAGNOSTIC IMAGERY:  ,The patient states she has not had an MRI performed on her lumbar spine.  The patient also states that Dr. X took x-rays two weeks ago, and no fractures were found at that time.  Per physician note, dated 12/10/08, Dr. X dictated that the x-ray showed an anterior grade 1 spondylolisthesis of L5 over S1, and requested Physical Therapy to evaluate and treat.,SUBJECTIVE:  ,The patient states that pain is constant in nature with a baseline of 6-7/10 with pain increasing to 10/10 during the night or in cold weather.  The patient states that pain is dramatically less, when the weather is warmer.  The patient also states that pain worsens as the day progresses, in that she also hard time getting out of bed in the morning.  The patient states that she does not sleep at night well and sleeps less than one hour at a time.,Aggravating factors include, sitting for periods greater than 20 minutes or lying supine on her back.  Easing factors include side lying position in she attempts to sleep.,OBJECTIVE: , AGE:  26 years old.  HEIGHT:  5 feet 2 inches.  WEIGHT:  The patient is an obese 26-year-old female.,ACTIVE RANGE OF MOTION: , Lumbar spine, flexion, lateral flexion and rotation all within functional limits without complaints of pain or soreness while performing them during evaluation.,PALPATION:  ,The patient complained of bilateral SI joint point tenderness.  The patient also complained of left greater trochanter hip point tenderness.  The patient also complained of bilateral paraspinal tenderness on cervical spine to lumbar spine.,STRENGTH:  ,RIGHT LOWER EXTREMITY:,Knee extension 5/5, hip flexion 5/5, knee flexion 4/5, internal and external hip rotation was 4/5.  With manual muscle testing of knee flexion, hip, internal and external rotation, the patient reports an increase in right SI joint pain to 8/10.,LEFT LOWER EXTREMITY:,Hip flexion 5/5, knee extension 5/5, knee flexion 4/5, hip internal and external rotation 4/5, with slight increase in pain level with manual muscle testing and resistance.  It must be noted that PT did not apply as much resistance during manual muscle testing, secondary to the 8/10 pain elicited during the right lower extremity.,NEUROLOGICAL:  ,The patient subjectively complains of numbness with tingling in her bilateral extremities when she sits longer than 25 minutes.  However, they subside when she stands.  The patient did complain of this numbness and tingling during the evaluation and the patient was seated for a period of 20 minutes.  Upon standing, the patient stated that the numbness and tingling subsides almost immediately.  The patient stated that Dr. X told her that he believes that during her past childbirth when the epidural was being administered that there was a possibility that a sensory nerve may have been also affected during the epidural less causing the numbness and tingling in her bilateral lower extremities.  The patient does not demonstrate any sensation deficits with gentle pressure to the lumbar spine and during manual muscle testing.,GAIT:  ,The patient ambulated out of the examination room, while carrying her baby in a car seat.,ASSESSMENT:  ,The patient is a 26-year-old overweight female, referred to Physical Therapy for low back pain.  The patient presents with lower extremity weakness, which may be contributing to her lumbosacral pain, in that she has poor lumbar stabilization with dynamic ADLs, transfers, and gait activity when fatigued.  At this time, the patient may benefit from skilled physical therapy to address her decreased strength and core stability in order to improve her ADL, transfer, and mobility skills.,PROGNOSIS: , The patient's prognosis for physical therapy is good for dictated goals.,SHORT-TERM GOALS TO BE ACHIEVED IN TWO WEEKS:,1.  The patient will be able to sit for greater than 25 minutes without complaints of paraesthesia or pain in her bilateral lower extremities or bilateral SI joints.,2.  The patient will increase bilateral hip internal and external rotation to 4/5 with SI joint pain less than or equal to 5/10.,3.  The patient will report 25% improvement in her functional and ADL activities.,4.  Pain will be less than 4/10 while performing __________ while at PT session.,LONG-TERM GOALS TO BE ACCOMPLISHED IN ONE MONTH:,1.  The patient will be independent with home exercise program.,2.  Bilateral hamstring, bilateral hip internal and external rotation strength to be 4+/5 with SI joint pain less than or equal to 2/10, while performing manual muscle test.,3.  The patient will report 60% improvement or greater in functional transfers in general ADL activity.,4.  The patient will be able to sit greater than or equal to 45 minutes without complaint of lumbosacral pain.,5.  The patient will be able to sleep greater than 2 hours without pain.,TREATMENT PLAN:,1.  Therapeutic exercises to increase lower extremity strength and assist with lumbar sacral stability.</t>
+          <t>CHIEF COMPLAINT:  ,This 18 year old male presents today with shoulder pain right.  Location:  He indicates the problem location is the right shoulder diffusely.  Quality:  Quality of the pain is described by the patient as aching, throbbing and tolerable.  Patient relates pain on a scale from 0 to 10 as 5/10.  Severity:  The severity has worsened over the past 3 months.  Timing (onset/frequency):  Onset was gradual and after pitching a baseball game.  Modifying Factors:  Patient's condition is aggravated by throwing.  He participates with difficulty in basketball.  Past conservative treatments include NSAID and muscle relaxant medications.,ALLERGIES: , No known medical allergies.,MEDICATION HISTORY:,  None.,PAST MEDICAL HISTORY:  ,Childhood Illnesses: (+) strep throat (+) mumps (+) chickenpox,PAST SURGICAL HISTORY:,  No previous surgeries.,FAMILY HISTORY:,  Patient admits a family history of arthritis associated with mother.,SOCIAL HISTORY: , Patient denies smoking, alcohol abuse, illicit drug use and STDs.,REVIEW OF SYSTEMS:,Musculoskeletal: (+) joint or musculoskeletal symptoms (+) stiffness in AM.,Psychiatric: (-) psychiatric or emotional difficulties.,Eyes: (-) visual disturbance or change.,Neurological: (-) neurological symptoms or problems Endocrine: (-) endocrine-related symptoms.,Allergic / Immunologic: (-) allergic or immunologic symptoms.,Ears, Nose, Mouth, Throat: (-) symptoms involving ear, nose, mouth, or throat.,Gastrointestinal: (-) GI symptoms.,Genitourinary: (-) GU symptoms.,Constitutional Symptoms: (-) constitutional symptoms such as fever, headache, nausea, dizziness.,Cardiovascular: (-) cardiovascular problems or chest symptoms.,Respiratory: (-)breathing difficulties, respiratory symptoms.,Physical Exam:  BP Standing:  116/68 Resp:  16 HR:  68 Temp:  98.1 Height:  5 ft.  11 in.  Weight:  165 lbs.  Patient is a 18 year old male who appears pleasant, in no apparent distress, his given age, well developed, well nourished and with good attention to hygiene and body habitus.  Oriented to person, place and time.  Right shoulder shows evidence of swelling and tenderness.  Radial pulses are 2 /4, bilateral.  Brachial pulses are 2 /4, bilateral.,Appearance:  Normal.,Tenderness:  Anterior - moderate, Biceps - none, Posterior - moderate and Subacromial - moderate right.,Range of Motion:  Right shoulder ROM shows decreased flexion, decreased extension, decreased adduction, decreased abduction, decreased internal rotation, decreased external rotation.  L shoulder normal.,Strength:  External rotation - fair.  Internal rotation - poor right.,AC Joint:  Pain with ABD and cross-chest - mild right.,Rotator Cuff:  Impingement - moderate.  Painful arc - moderate right.,Instability:  None.,TEST &amp; X-RAY RESULTS:,  X-rays of the shoulder were performed.  X-ray of right shoulder reveals cuff arthropathy present.,IMPRESSION: , Rotator cuff syndrome, right.,PLAN: , Diagnosis of a rotator cuff tendinitis and shoulder impingement were discussed.  I noted that this is a very common condition resulting in significant difficulties with use of the arm.  Several treatment options and their potential benefits were described.  Nonsteroidal anti-inflammatories can be helpful but typically are slow acting.  Cortisone shots can be very effective and are quite safe.  Often more than one injection may be required.  Physical therapy can also be helpful, particularly if there is any loss of shoulder mobility or strength.  If these treatments fail to resolve symptoms, an MRI or shoulder arthrogram may be required to rule out a rotator cuff tear.  Injected shoulder joint and with Celestone Soluspan 1.0 cc .  Ordered x-rays of shoulder right.,PRESCRIPTIONS:,  Vioxx Dosage:  25 mg tablet Sig:  TID Dispense:  60 Refills:  0 Allow Generic:  Yes,PATIENT INSTRUCTIONS:,  Patient was instructed to restrict activity.  Patient was given instructions on RICE therapy.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr"/>
       <c r="G39" s="2" t="n">
-        <v>1033</v>
+        <v>526</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Orthopedic; long; SOAP-style; diagnoses + symptoms + medications</t>
+          <t>Orthopedic; medium; history and physical; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J39" s="2" t="n">
-        <v>2078</v>
+        <v>2059</v>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>SOAP-style</t>
+          <t>history and physical</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -2881,17 +2877,17 @@
         </is>
       </c>
       <c r="M39" s="2" t="n">
-        <v>0.8933724075743913</v>
+        <v>0.8419183949504058</v>
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; imaging; past history; treatment plans; follow-up; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; imaging; past history; treatment plans; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="40" ht="110" customHeight="1">
       <c r="A40" s="2" t="n">
-        <v>1618</v>
+        <v>1571</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
@@ -2900,39 +2896,39 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Mayoview </t>
+          <t xml:space="preserve"> MRI Knee - 4 </t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Resting Myoview and adenosine Myoview SPECT</t>
+          <t xml:space="preserve"> MRI left knee without contrast.</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>PROCEDURE DONE:  ,Resting Myoview and adenosine Myoview SPECT.,INDICATIONS:,  Chest pain.,PROCEDURE:,  13.3 mCi of Tc-99m tetrofosmin was injected and resting Myoview SPECT was obtained.  Pharmacologic stress testing was done using adenosine infusion.  Patient received 38 mg of adenosine infused at 140 mcg/kg/minute over a period of four minutes.  Two minutes during adenosine infusion, 31.6 mCi of Tc-99m tetrofosmin was injected.  Resting heart rate was 90 beats per minute.  Resting blood pressure was 130/70.  Peak heart rate obtained during adenosine infusion was 102 beats per minute.  Blood pressure obtained during adenosine infusion was 112/70.  During adenosine infusion, patient experienced dizziness and shortness of breath.  No significant ST segment, T wave changes, or arrhythmias were seen.,Resting Myoview and adenosine Myoview SPECT showed uniform uptake of isotope throughout myocardium without any perfusion defect.  Gated dynamic imaging showed normal wall motion and normal systolic thickening throughout left ventricular myocardium.  Left ventricular ejection fraction obtained during adenosine Myoview SPECT was 77%.  Lung heart ratio was 0.40.  TID ratio was 0.88.,IMPRESSION:,  Normal adenosine Myoview myocardial perfusion SPECT.  Normal left ventricular regional and global function with left ventricular ejection fraction of 77%.</t>
+          <t>EXAM:,MRI OF THE LEFT KNEE WITHOUT CONTRAST,CLINICAL:,Left knee pain. Twisting injury.,FINDINGS:,The images reveal a sizable joint effusion. The joint effusion appears to be complex with mixed signal intensity material within. The patella is slightly laterally tilted towards the left. The mid portion of the patella cartilage shows some increased signal and focal injury to the patellar cartilage is suspected. Mildly increased bone signal overlying the inferolateral portion of the patella is identified. No significant degenerative changes about the patella can be seen. The quadriceps tendon as well as the infrapatellar ligament both look intact. There is some prepatellar soft tissue edema.,The bone signal shows a couple of small areas of cystic change in the proximal aspect of the tibia. NO significant areas of bone edema are appreciated.,There is soft tissue edema along the lateral aspect of the knee. There is a partial tear of the lateral collateral ligament complex. The medial collateral ligament complex looks intact. A small amount of edema is identified immediately adjacent to the medial collateral ligament complex.,The posterior cruciate ligament looks intact. The anterior cruciate ligament is thickened with significant increased signal. I suspect at least a high grade partial tear.,The posterior horn of the medial meniscus shows some myxoid degenerative changes. The posterior horn and anterior horn of the lateral meniscus likewise shows myxoid degenerative type changes. I don’t see a definite tear extending to the articular surface.,IMPRESSION:,Sizeable joint effusion which is complex and may contain blood products.,Myxoid degenerative type changes medial and lateral meniscus with no definite evidence of a tear.,Soft tissue swelling and partial tear of the lateral collateral ligament complex.,At least high grade partial tear of the anterior cruciate ligament with significant thickening and increased signal of this structure.,The posterior cruciate ligament is intact.,Injury to the patellar cartilage as above.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>radiology, myoview, gated dynamic imaging, myoview spect, resting myoview, spect, tc-99m, adenosine myoview, adenosine infusion, ejection fraction, myocardium, systolic thickening, tetrofosmin, adenosine myoview spect, adenosine,</t>
+          <t>radiology, lateral collateral ligament, medial collateral ligament, posterior cruciate ligament, anterior cruciate ligament, collateral ligament complex, myxoid degenerative, partial tear, collateral ligament, ligament complex, cruciate ligament, mri, effusion, cartilage, collateral, cruciate, knee, tear, ligament</t>
         </is>
       </c>
       <c r="G40" s="2" t="n">
-        <v>184</v>
+        <v>298</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Radiology; short; diagnostic report; diagnoses + symptoms + medications</t>
+          <t>Radiology; medium; diagnostic report; lower text complexity; diagnoses + symptoms + imaging</t>
         </is>
       </c>
       <c r="J40" s="2" t="n">
-        <v>1618</v>
+        <v>1571</v>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
@@ -2945,17 +2941,17 @@
         </is>
       </c>
       <c r="M40" s="2" t="n">
-        <v>0.3524008115419297</v>
+        <v>0.147204688908927</v>
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; vital signs; procedures; imaging</t>
+          <t>diagnoses; symptoms; imaging</t>
         </is>
       </c>
     </row>
     <row r="41" ht="110" customHeight="1">
       <c r="A41" s="2" t="n">
-        <v>1663</v>
+        <v>1516</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
@@ -2964,26 +2960,26 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CT-Guided Biopsy - Kidney </t>
+          <t xml:space="preserve"> Transesophageal Echocardiogram - 3 </t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CT-guided needle placement, CT-guided biopsy of right renal mass, and embolization of biopsy tract with gelfoam.</t>
+          <t xml:space="preserve"> Transesophageal echocardiographic examination report.   Aortic valve replacement.  Assessment of stenotic valve.  Evaluation for thrombus on the valve.</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>REASON FOR EXAM:  This 60-year-old female who was found to have a solid indeterminate mass involving the inferior pole of the right kidney was referred for percutaneous biopsy under CT guidance at the request of Dr. X.,PROCEDURE:  The procedure risks and possible complications including, but not limited to severe hemorrhage which could result in emergent surgery, were explained to the patient.  The patient understood.  All questions were answered, and informed consent was obtained.  With the patient in the prone position, noncontrasted CT localization images were obtained through the kidney.  Conscious sedation was utilized with the patient being monitored.  The patient was administered divided dose of Versed and fentanyl intravenously.,Following sterile preparation and local anesthesia to the posterior aspect of the right flank, an 18-gauge co-axial Temno-type needle was directed into the inferior pole right renal mass from the posterior oblique approach.  Two biopsy specimens were obtained and placed in 10% formalin solution.  CT documented needle placement.  Following the biopsy, there was active bleeding through the stylet, as well as a small hematoma about the inferior aspect of the right kidney posteriorly.  I placed several torpedo pledgets of Gelfoam through the co-axial sheath into the site of bleeding.  The bleeding stopped.  The co-axial sheath was then removed.  Bandage was applied.  Hemostasis was obtained.  The patient was placed in the supine position.  Postbiopsy CT images were then obtained.  The patient's hematoma appeared stable.  The patient was without complaints of pain or discomfort.  The patient was then sent to her room with plans of observing for approximately 4 hours and then to be discharged, as stable.  The patient was instructed to remain at bedrest for the remaining portions of the day at home and patient is to followup with Dr. Fieldstone for the results and follow-up care.,FINDINGS:  Initial noncontrasted CT localization images reveals the presence of an approximately 2.1 cm cortical mass involving the posterior aspect of the inferior pole of the right kidney.  Images obtained during the biopsy reveals the cutting portion of the biopsy needle to extend through the mass.  Images obtained following the biopsy reveals the development of a small hematoma posterior to the right kidney in its inferior pole adjacent to the mass.  There are small droplets of air within the hematoma.  No hydronephrosis is identified.,CONCLUSION:,1.  Percutaneous biopsy of inferior pole right renal mass under computed tomography guidance with specimen sent to laboratory in 10% formalin solution.,2.  Development of a small hematoma adjacent to the inferior pole of the right kidney with active bleeding through the biopsy needle stopped by tract embolization with Gelfoam pledgets.</t>
+          <t>REASON FOR EXAM: , Aortic valve replacement.  Assessment of stenotic valve.  Evaluation for thrombus on the valve.,PREOPERATIVE DIAGNOSIS:  ,Atrial valve replacement.,POSTOPERATIVE DIAGNOSES:,  Moderate stenosis of aortic valve replacement.  Mild mitral regurgitation.  Normal left ventricular function.,PROCEDURES IN DETAIL: , The procedure was explained to the patient with risks and benefits.  The patient agreed and signed the consent form.  The patient received a total of 3 mg of Versed and 50 mcg of fentanyl for conscious sedation and pain control.  The oropharynx anesthetized with benzocaine spray and lidocaine solution.,Esophageal intubation was done with no difficulty with the second attempt.  In a semi-Fowler position, the probe was passed to transthoracic views at about 40 to 42 cm.  Multiple pictures obtained.  Assessment of the peak velocity was done later.,The probe was pulled to the mid esophageal level.  Different pictures including short-axis views of the aortic valve was done.  Extubation done with no problems and no blood on the probe.  The patient tolerated the procedure well with no immediate postprocedure complications.,INTERPRETATION: , The left atrium was mildly dilated.  No masses or thrombi were seen.  The left atrial appendage was free of thrombus.  Pulse wave interrogation showed peak velocities of 60 cm per second.,The left ventricle was normal in size and contractility with mild LVH.  EF is normal and preserved.,The right atrium and right ventricle were both normal in size.,Mitral valve showed no vegetations or prolapse.  There was mild-to-moderate regurgitation on color flow interrogation.  Aortic valve was well-seated mechanical valve, bileaflet with acoustic shadowing beyond the valve noticed.  No perivalvular leak was noticed.  There was increased velocity across the valve with peak velocity of 3.2 m/sec with calculated aortic valve area by continuity equation at 1.2 cm2 indicative of moderate aortic valve stenosis based on criteria for native heart valves.,No AIC.,Pulmonic valve was somewhat difficult to see because of acoustic shadowing from the aortic valve.  Overall showed no abnormalities.  The tricuspid valve was structurally normal.,Interatrial septum appeared to be intact, confirmed by color flow interrogation as well as agitated saline contrast study.,The aorta and aortic arch were unremarkable.  No dissection.,IMPRESSION:,1.  Mildly dilated left atrium.,2.  Mild-to-moderate regurgitation.,3.  Well-seated mechanical aortic valve with peak velocity of 3.2 m/sec and calculated valve area of 1.2 cm2 consistent with moderate aortic stenosis.  Reevaluation in two to three years with transthoracic echocardiogram will be recommended.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>radiology, embolization, ct localization, gelfoam pledgets, ct guided needle placement, ct guided biopsy, needle placement, renal mass, ct guided, inferior pole, ct, biopsy, hematoma, kidney, mass,</t>
+          <t xml:space="preserve">radiology, aortic valve replacement, stenotic valve, thrombus, stenosis, ventricular, esophageal, peak velocity, valve replacement, aortic valve, aortic, transesophageal, valve, oropharynx, atrium, interrogation, atrial, moderate, </t>
         </is>
       </c>
       <c r="G41" s="2" t="n">
-        <v>426</v>
+        <v>384</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
@@ -2992,15 +2988,15 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Radiology; medium; diagnostic report; symptoms + laboratory values + procedures</t>
+          <t>Radiology; medium; procedure/operative; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J41" s="2" t="n">
-        <v>1663</v>
+        <v>1516</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>diagnostic report</t>
+          <t>procedure/operative</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
@@ -3009,17 +3005,17 @@
         </is>
       </c>
       <c r="M41" s="2" t="n">
-        <v>0.3975428313796213</v>
+        <v>0.5675157799819658</v>
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>symptoms; laboratory values; procedures; imaging; follow-up; surgery</t>
+          <t>diagnoses; symptoms; medications; vital signs; procedures; imaging; treatment plans</t>
         </is>
       </c>
     </row>
     <row r="42" ht="110" customHeight="1">
       <c r="A42" s="2" t="n">
-        <v>1639</v>
+        <v>1663</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
@@ -3028,39 +3024,39 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Fetal Anatomical Survey </t>
+          <t xml:space="preserve"> CT-Guided Biopsy - Kidney </t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The patient is a 39-year-old gravida 3, para 2, who is now at 20 weeks and 2 days gestation.  This pregnancy is a twin gestation.  The patient presents for her fetal anatomical survey.  </t>
+          <t xml:space="preserve"> CT-guided needle placement, CT-guided biopsy of right renal mass, and embolization of biopsy tract with gelfoam.</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>PAST MEDICAL HISTORY:  ,The patient denies any significant past medical history.,PAST SURGICAL HISTORY: , The patient denies any significant surgical history.,MEDICATIONS: , The patient takes no medications.,ALLERGIES: , No known drug allergies.,SOCIAL HISTORY: , She denies use of cigarettes, alcohol or drugs.,FAMILY HISTORY: , No family history of birth defects, mental retardation or any psychiatric history.,DETAILS: , I performed a transabdominal ultrasound today using a 4 MHz transducer.  There is a twin gestation in the vertex transverse lie with an anterior placenta and a normal amount of amniotic fluid surrounding both of the twins.  The fetal biometry of twin A is as follows.  The biparietal diameter is 4.9 cm consistent with 20 weeks and 5 days, head circumference 17.6 cm consistent with 20 weeks and 1 day, the abdominal circumference is 15.0 cm consistent with 20 weeks and 2 days, and femur length is 3.1 cm consistent with 19 weeks and 5 days, and the humeral length is 3.0 cm consistent with 20 weeks and 0 day.  The average gestational age by ultrasound is 20 weeks and 1 day and the estimated fetal weight is 353 g.  The following structures are seen as normal on the fetal anatomical survey, the shape of the fetal head, the choroid plexuses, the cerebellum, nuchal fold thickness, the fetal spine and fetal face, the four-chamber view of the fetal heart, the outflow tracts of the fetal heart, the stomach, the kidneys, and cord insertion site, the bladder, the extremities, the genitalia, the cord, which appeared to have three vessels and the placenta.,Limited in views of baby A with a nasolabial region.,The following is the fetal biometry for twin B. The biparietal diameter is 4.7 cm consistent with 20 weeks and 2 days, head circumference 17.5 cm consistent with 20 weeks and 0 day, the abdominal circumference is 15.5 cm consistent with 20 weeks and 5 days, the femur length is 3.3 cm consistent with 20 weeks and 3 days, and the humeral length is 3.1 cm consistent with 20 weeks and 2 days, the average gestational age by ultrasound is 22 weeks and 2 days, and the estimated fetal weight is 384 g.  The following structures were seen as normal on the fetal anatomical survey.  The shape of the fetal head, the choroid plexuses, the cerebellum, nuchal fold thickness, the fetal spine and fetal face, the four-chamber view of the fetal heart, the outflow tracts of the fetal heart, the stomach, the kidneys, and cord insertion site, the bladder, the extremities, the genitalia, the cord, which appeared to have three vessels, and the placenta.  Limited on today's ultrasound the views of nasolabial region.,In summary, this is a twin gestation, which may well be monochorionic at 20 weeks and 1 day.  There is like gender and a single placenta.  One cannot determine with certainty whether or not this is a monochorionic or dichorionic gestation from the ultrasound today.,I sat with the patient and her husband and discussed alternative findings and the complications.  We focused our discussion today on the association of twin pregnancy with preterm delivery.  We discussed the fact that the average single intrauterine pregnancy delivers at 40 weeks' gestation while the average twin delivery occurs at 35 weeks' gestation.  We discussed the fact that 15% of twins deliver prior to 32 weeks' gestation.  These are the twins which we have the most concern regarding the long-term prospects of prematurity.  We discussed several etiologies of preterm delivery including preterm labor, incompetent cervix, premature rupture of the fetal membranes as well as early delivery from preeclampsia and growth restriction.  We discussed the use of serial transvaginal ultrasound to assess for early cervical change and the use of serial transabdominal ultrasound to assess for normal interval growth.  We discussed the need for frequent office visits to screen for preeclampsia.  We also discussed treatment options such as cervical cerclage, bedrest, tocolytic medications, and antenatal steroids.  I would recommend that the patient return in two weeks for further cervical assessment and assessment of fetal growth and well-being.,In closing, I do want to thank you very much for involving me in the care of your delightful patient.  I did review all of the above findings and recommendations with the patient today at the time of her visit.  Please do not hesitate to contact me if I could be of any further help to you.,Total visit time 40 minutes.</t>
+          <t>REASON FOR EXAM:  This 60-year-old female who was found to have a solid indeterminate mass involving the inferior pole of the right kidney was referred for percutaneous biopsy under CT guidance at the request of Dr. X.,PROCEDURE:  The procedure risks and possible complications including, but not limited to severe hemorrhage which could result in emergent surgery, were explained to the patient.  The patient understood.  All questions were answered, and informed consent was obtained.  With the patient in the prone position, noncontrasted CT localization images were obtained through the kidney.  Conscious sedation was utilized with the patient being monitored.  The patient was administered divided dose of Versed and fentanyl intravenously.,Following sterile preparation and local anesthesia to the posterior aspect of the right flank, an 18-gauge co-axial Temno-type needle was directed into the inferior pole right renal mass from the posterior oblique approach.  Two biopsy specimens were obtained and placed in 10% formalin solution.  CT documented needle placement.  Following the biopsy, there was active bleeding through the stylet, as well as a small hematoma about the inferior aspect of the right kidney posteriorly.  I placed several torpedo pledgets of Gelfoam through the co-axial sheath into the site of bleeding.  The bleeding stopped.  The co-axial sheath was then removed.  Bandage was applied.  Hemostasis was obtained.  The patient was placed in the supine position.  Postbiopsy CT images were then obtained.  The patient's hematoma appeared stable.  The patient was without complaints of pain or discomfort.  The patient was then sent to her room with plans of observing for approximately 4 hours and then to be discharged, as stable.  The patient was instructed to remain at bedrest for the remaining portions of the day at home and patient is to followup with Dr. Fieldstone for the results and follow-up care.,FINDINGS:  Initial noncontrasted CT localization images reveals the presence of an approximately 2.1 cm cortical mass involving the posterior aspect of the inferior pole of the right kidney.  Images obtained during the biopsy reveals the cutting portion of the biopsy needle to extend through the mass.  Images obtained following the biopsy reveals the development of a small hematoma posterior to the right kidney in its inferior pole adjacent to the mass.  There are small droplets of air within the hematoma.  No hydronephrosis is identified.,CONCLUSION:,1.  Percutaneous biopsy of inferior pole right renal mass under computed tomography guidance with specimen sent to laboratory in 10% formalin solution.,2.  Development of a small hematoma adjacent to the inferior pole of the right kidney with active bleeding through the biopsy needle stopped by tract embolization with Gelfoam pledgets.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>radiology, vaginal delivery, transducer, transabdominal ultrasound, placenta, amniotic fluid, fetal anatomical survey, preterm delivery, twin gestation, gestation, infant, fetal, anatomical, delivery, ultrasound,</t>
+          <t>radiology, embolization, ct localization, gelfoam pledgets, ct guided needle placement, ct guided biopsy, needle placement, renal mass, ct guided, inferior pole, ct, biopsy, hematoma, kidney, mass,</t>
         </is>
       </c>
       <c r="G42" s="2" t="n">
-        <v>729</v>
+        <v>426</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Radiology; long; diagnostic report; diagnoses + medications + allergies</t>
+          <t>Radiology; medium; diagnostic report; middle text complexity; symptoms + laboratory values + procedures</t>
         </is>
       </c>
       <c r="J42" s="2" t="n">
-        <v>1639</v>
+        <v>1663</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -3069,21 +3065,21 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>higher</t>
+          <t>middle</t>
         </is>
       </c>
       <c r="M42" s="2" t="n">
-        <v>0.738334084761046</v>
+        <v>0.3975428313796213</v>
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; medications; allergies; imaging; past history; treatment plans; follow-up; surgery</t>
+          <t>symptoms; laboratory values; procedures; imaging; follow-up; surgery</t>
         </is>
       </c>
     </row>
     <row r="43" ht="110" customHeight="1">
       <c r="A43" s="2" t="n">
-        <v>1307</v>
+        <v>1394</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
@@ -3092,43 +3088,43 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> SOAP - Temporal Mass </t>
+          <t xml:space="preserve"> Fundoplication &amp; Gastrostomy Followup </t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> MRI demonstrated right contrast-enhancing temporal mass.</t>
+          <t xml:space="preserve"> Followup of laparoscopic fundoplication and gastrostomy.  Laparoscopic fundoplication and gastrostomy was done because of the need for enteral feeding access.</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>SUBJECTIVE: , The patient is a 55-year-old African-American male that was last seen in clinic on 07/29/2008 with diagnosis of new onset seizures and an MRI scan, which demonstrated right contrast-enhancing temporal mass.  Given the characteristics of this mass and his new onset seizures, it is significantly concerning for a high-grade glioma.  ,OBJECTIVE: , The patient is alert and oriented times three, GCS of 15.  Cranial nerves II to XII are grossly intact.  Motor exam demonstrates 5/5 strength in all four extremities.  Sensation is intact to light touch, pain, temperature, and proprioception.  Cerebellar exam is intact.  Gait is normal and tandem on heels and toes.  Speech is appropriate.  Judgment is intact.  Pupils are equal and reactive to light.,ASSESSMENT AND PLAN: , The patient is a 55-year-old African-American male with a new diagnosis of rim-enhancing right temporal mass.  Given the characteristics of the MRI scan, it is highly likely that he demonstrates high-grade glioma and concerning for glioblastoma multiforme.  We have discussed in length the possible benefits of biopsy, surgical resection, medical management, as well as chemotherapy, radiation treatments, and doing nothing.  Given the high probability that the mass represents a high-grade glioma, the patient, after weighing the risks and the benefits of surgery, has agreed to undergo a surgical biopsy and resection of the mass as well as concomitant chemotherapy and radiation as the diagnosis demonstrates a high-grade glioma.  The patient has signed consent for his right temporal craniotomy for biopsy and likely resection of right temporal brain tumor.  He agrees that he will be n.p.o. after mid night on Wednesday night.  He is sent for preoperative assessment with the Anesthesiology tomorrow morning.  He has undergone vocational rehab assessment.</t>
+          <t>REASON FOR VISIT: , Followup of laparoscopic fundoplication and gastrostomy.,HISTORY OF PRESENT ILLNESS: , The patient is a delightful baby girl, who is now nearly 8 months of age and had a tracheostomy for subglottic stenosis.  Laparoscopic fundoplication and gastrostomy was done because of the need for enteral feeding access and to protect her airway at a time when it is either going to heal enough to improve and allow decannulation or eventually prove that she will need laryngotracheoplasty.  Dr. X is following The patient for this and currently plans are to perform a repeat endoscopic exam every couple of months to assist the status of her airway caliber.,The patient had a laparoscopic fundoplication and gastrostomy on 10/05/2007.  She has done well since that time.  She has had some episodes of retching intermittently and these seemed to be unpredictable.  She also had some diarrhea and poor feeding tolerance about a week ago but that has also resolved.  The patient currently takes about 1 ounce to 1.5 ounce of her feedings by mouth and the rest is given by G-tube.  She seems otherwise happy and is not having an excessive amount of stools.  Her parents have not noted any significant problems with the gastrostomy site.,The patient's exam today is excellent.  Her belly is soft and nontender.  All of her laparoscopic trocar sites are healing with a normal amount of induration, but there is no evidence of hernia or infection.  We removed The patient's gastrostomy button today and showed her parents how to reinsert one without difficulty.  The site of the gastrostomy is excellent.  There is not even a hint of granulation tissue or erythema, and I am very happy with the overall appearance.,IMPRESSION: , The patient is doing exceptionally well status post laparoscope fundoplication and gastrostomy.  Hopefully, the exquisite control of acid reflux by fundoplication will help her airway heal, and if she does well, allow decannulation in the future.  If she does require laryngotracheoplasty, the protection from acid reflux will be important to healing of that procedure as well.,PLAN:  ,The patient will follow up as needed for problems related to gastrostomy.  We will see her when she comes in the hospital for endoscopic exams and possibly laryngotracheoplasty in the future.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>soap / chart / progress notes, new onset seizures, temporal mass, cerebellar exam, glioma, temporal, massNOTE</t>
+          <t xml:space="preserve">soap / chart / progress notes, decannulation, enteral feeding, feeding access, laparoscopic fundoplication, gastrostomy, airway, laryngotracheoplasty, laparoscopic, fundoplication, </t>
         </is>
       </c>
       <c r="G43" s="2" t="n">
-        <v>279</v>
+        <v>370</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>SOAP / Chart / Progress Notes; short; SOAP-style; diagnoses + symptoms + procedures</t>
+          <t>SOAP / Chart / Progress Notes; medium; follow-up/progress; lower text complexity; diagnoses + procedures + past history</t>
         </is>
       </c>
       <c r="J43" s="2" t="n">
-        <v>1307</v>
+        <v>1394</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>SOAP-style</t>
+          <t>follow-up/progress</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -3137,17 +3133,17 @@
         </is>
       </c>
       <c r="M43" s="2" t="n">
-        <v>0.3710550045085662</v>
+        <v>0.345299819657349</v>
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; procedures; imaging; treatment plans; surgery; assessment/plan</t>
+          <t>diagnoses; procedures; past history; treatment plans; follow-up; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="44" ht="110" customHeight="1">
       <c r="A44" s="2" t="n">
-        <v>1396</v>
+        <v>1384</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
@@ -3156,26 +3152,26 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Gen Med Progress Note - 11 </t>
+          <t xml:space="preserve"> Gen Med Progress Note - 7 </t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 5-month recheck on type II diabetes mellitus, as well as hypertension.</t>
+          <t xml:space="preserve"> Patient with a three-day history of emesis and a four-day history of diarrhea</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>SUBJECTIVE:,  The patient is a 66-year-old female who presents to the clinic today for a five-month recheck on her type II diabetes mellitus, as well as hypertension.  While here she had a couple of other issues as well.  She stated that she has been having some right shoulder pain.  She denies any injury but certain range of motion does cause it to hurt.  No weakness, numbness or tingling.  As far as her diabetes she states that she only checks her blood sugars in the morning and those have all been ranging less than 100.  She has not been checking any two hours after meals.  Her blood pressures when she does check them have been running normal as well but she does not have any record of these present with her.  No other issues or concerns.  Upon review of her chart it did show that she had a benign breast biopsy done back on 06/11/04 and was told to have a repeat mammogram in six months but she has never had that done so she is needing to have this done as well.,ALLERGIES: , None.,MEDICATIONS:,  She is on Hyzaar 50/12.5 one-half p.o. daily, coated aspirin daily, lovastatin 40 mg one-half tab p.o. daily, multivitamin daily, metformin 500 mg one tab p.o. b.i.d.; however, she has been skipping her second dose during the day.,SOCIAL HISTORY:,  She is a nonsmoker.,REVIEW OF SYSTEMS:,  As noted above.,OBJECTIVE:,Vital Signs:  Temperature:  98.2.  Pulse:  64.  Respirations:  16.  Blood pressure:  110/56.  Weight:  169.,General:  Alert and oriented x 3.  No acute distress noted.,Neck:  No lymphadenopathy, thyromegaly, JVD or bruits.,Lungs:  Clear to auscultation.,Heart:  Regular rate and rhythm without murmur or gallops present.,Breasts:  Exam performed with a female nurse present.  The breasts do have some scars present underneath them bilaterally from prior breast reduction surgery.  There is no axillary adenopathy or tenderness.  Breasts appear to be symmetric.  There was no nipple discharge or retraction.  No breast tissue retraction noted in either the sitting or the supine position.  Upon palpation there were no palpable lumps or bumps and no palpable discharge.,Musculoskeletal:  She did have full range of motion of her shoulders.  She did have tenderness upon palpation over the right bicipital tendon.  There is no swelling, crepitus or discoloration noted.,MEDICAL DECISION MAKING:  Most recent hemoglobin A1c was 5.6% back in October 2004.  Most recent lipid checks were obtained back in July 2004.  We have not had this checked since that time.,ASSESSMENT:,1.  Type II diabetes mellitus.,2.  Hypertension.,3.  Right shoulder pain.,4.  Hyperlipidemia.,PLAN:,1.  She is going to go to lab to obtain a hemoglobin A1c, BMP, lipids, CPK, liver enzymes and quantitative microalbumin.,2.  We are going to set her up for a diagnostic bilateral mammogram due to a history of abnormal mammogram in the past which subsequently showed a benign breast cyst.,3.  I told her for her shoulder to take ibuprofen 600 mg three times daily with her meals for a minimum of the next one week.,4.  She is going to follow up in the clinic in three months for a complete comprehensive examination.  If any questions, concerns or problems arise between now and then she should let us know.</t>
+          <t>SUBJECTIVE:,  The patient is a 7-year-old male who comes in today with a three-day history of emesis and a four-day history of diarrhea.  Apparently, his brother had similar symptoms.  They had eaten some chicken and then ate some more of it the next day, and I could not quite understand what the problem was because there is a little bit of language barrier, although dad was trying very hard to explain to me what had happened.  But any way, after he and his brother got done eating with chicken, they both felt bad and have continued to feel bad.  The patient has had diarrhea five to six times a day for the last four days and then he had emesis pretty frequently three days ago and then has just had a couple of it each day in the last two days.  He has not had any emesis today.  He has urinated this morning.  His parents are both concerned because he had a fever of 103 last night.  Also, he ate half of a hamburger yesterday and he tried drinking some milk and that is when he had an emesis.  He has been drinking Pedialyte, Gatorade, white grape juice, and 7Up, otherwise he has not been eating anything.,MEDICATIONS:  ,None.,ALLERGIES:  ,He has no known drug allergies.,REVIEW OF SYSTEMS:,  Negative as far as sore throat, earache, or cough.,PHYSICAL EXAMINATION:,General:  He is awake and alert, no acute distress.,Vital Signs:  Blood pressure:  106/75.  Temperature:  99.  Pulse:  112.  Weight is 54 pounds.,HEENT:  His TMs are normal bilaterally.  Posterior pharynx is unremarkable.,Neck:  Without adenopathy or thyromegaly.,Lungs:  Clear to auscultation.,Heart:  Regular rate and rhythm without murmur.,Abdomen:  Benign.,Skin:  Turgor is intact.  His capillary refill is less than 3 seconds.,LABORATORY: , White blood cell count is 5.3 with 69 segs, 15 lymphs, and 13 monos.  His platelet count on his CBC is 215.,ASSESSMENT:,  Viral gastroenteritis.,PLAN:,  The parents did point out to me a rash that he had on his buttock.  There were some small almost pinpoint erythematous patches of papules that have a scab on them.  I did not see any evidence of petechiae.  Therefore, I just reassured them that this is a viral gastroenteritis.  I recommended that they stop giving him juice and just go with the Gatorade and water.  He is to stay away from milk products until his diarrhea and stomach upset have calmed down.  We talked about BRAT diet and slowly advancing his diet as he tolerates.  They have used some Kaopectate, which did not really help with the diarrhea.  Otherwise follow up as needed.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve">soap / chart / progress notes, diarrhea, emesis, history of, gastroenteritis, viral, brat diet, progress note, </t>
         </is>
       </c>
       <c r="G44" s="2" t="n">
-        <v>514</v>
+        <v>419</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -3184,34 +3180,34 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>SOAP / Chart / Progress Notes; medium; SOAP-style; diagnoses + symptoms + medications</t>
+          <t>SOAP / Chart / Progress Notes; medium; follow-up/progress; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J44" s="2" t="n">
-        <v>1396</v>
+        <v>1384</v>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>SOAP-style</t>
+          <t>follow-up/progress</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>higher</t>
+          <t>middle</t>
         </is>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0.7346145175834085</v>
+        <v>0.6001465284039675</v>
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; past history; treatment plans; follow-up; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; past history; treatment plans; follow-up; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="45" ht="110" customHeight="1">
       <c r="A45" s="2" t="n">
-        <v>1392</v>
+        <v>1396</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
@@ -3220,39 +3216,39 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Foot Pain - SOAP </t>
+          <t xml:space="preserve"> Gen Med Progress Note - 11 </t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Patient having foot pain.</t>
+          <t xml:space="preserve"> 5-month recheck on type II diabetes mellitus, as well as hypertension.</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>SUBJECTIVE:,  This 32-year-old female comes in again still having not got a primary care physician.  She said she was at Dr. XYZ office today for her appointment, and they cancelled her appointment because she has not gotten her Project Access insurance into affect.  She says that Project Access is trying to find her a doctor.  She is not currently on Project Access, and so she is here to get something for the pain in her foot.  I did notice that she went in to see Dr. XYZ for a primary care physician on 05/14/2004.  She said she does not have a primary care physician.  She was in here just last week and saw Dr. XYZ for back pain and was put on pain medicines and muscle relaxers.  She has been in here multiple times for different kinds of pain.  This pain she is having is in her foot.  She had surgery on it, and she has plates and screws.  She said she was suppose to see Dr. XYZ about getting some of the hardware out of it.  The appointment was cancelled, and that is why she came here.  It started hurting a lot yesterday, but she had this previous appointment with Dr. XYZ so she thought she would take care of it there, but they would not see her.  She did not injure her foot in any way recently.  It is chronically painful.  Every time she does very much exercise it hurts more.  We have x-rayed it in the past.  She has some hardware there.  It does not appear to be grossly abnormal or causing any loosening or problems on x-ray.,PHYSICAL EXAM: , Examination of her foot shows some well-healed surgical scars.  On the top of her foot she has two, and then on the lateral aspect below her ankle she has a long scar.  They are all old, and the surgery was done over a year ago.  She is walking with a very slight limp.  There is no redness.  No heat.  No swelling of the foot or the ankle.  It is mildly tender around the medial side of the foot just inferior to the medial malleolus.  It is not warm or red.,ASSESSMENT:,  Foot pain.,PLAN:,  She has been in here before.  She seems very pleasant.  Thought maybe she certainly might be having some significant pain, so I gave her some Lortab 7.5 to take with a refill.  After she left, I got to thinking about it and looked into her record.  She has been in here multiple times for pain medicine.  She has a primary care physician, and now she is telling us she does not have a primary care physician even though she had seen Dr. XYZ not too long ago.  We called Dr. XYZ office.  Dr. XYZ nurse said that the patient did not have an appointment today.  She has an appointment on June 15, 2004, for a postop check.  They did not tell her they would not see her today because of insurance, so the patient was lying to me.  We will keep that in mind the next time she returns, because she will likely be back.  She did say that Project Access will be approving her insurance next week, so she will be able to see Dr. XYZ soon.</t>
+          <t>SUBJECTIVE:,  The patient is a 66-year-old female who presents to the clinic today for a five-month recheck on her type II diabetes mellitus, as well as hypertension.  While here she had a couple of other issues as well.  She stated that she has been having some right shoulder pain.  She denies any injury but certain range of motion does cause it to hurt.  No weakness, numbness or tingling.  As far as her diabetes she states that she only checks her blood sugars in the morning and those have all been ranging less than 100.  She has not been checking any two hours after meals.  Her blood pressures when she does check them have been running normal as well but she does not have any record of these present with her.  No other issues or concerns.  Upon review of her chart it did show that she had a benign breast biopsy done back on 06/11/04 and was told to have a repeat mammogram in six months but she has never had that done so she is needing to have this done as well.,ALLERGIES: , None.,MEDICATIONS:,  She is on Hyzaar 50/12.5 one-half p.o. daily, coated aspirin daily, lovastatin 40 mg one-half tab p.o. daily, multivitamin daily, metformin 500 mg one tab p.o. b.i.d.; however, she has been skipping her second dose during the day.,SOCIAL HISTORY:,  She is a nonsmoker.,REVIEW OF SYSTEMS:,  As noted above.,OBJECTIVE:,Vital Signs:  Temperature:  98.2.  Pulse:  64.  Respirations:  16.  Blood pressure:  110/56.  Weight:  169.,General:  Alert and oriented x 3.  No acute distress noted.,Neck:  No lymphadenopathy, thyromegaly, JVD or bruits.,Lungs:  Clear to auscultation.,Heart:  Regular rate and rhythm without murmur or gallops present.,Breasts:  Exam performed with a female nurse present.  The breasts do have some scars present underneath them bilaterally from prior breast reduction surgery.  There is no axillary adenopathy or tenderness.  Breasts appear to be symmetric.  There was no nipple discharge or retraction.  No breast tissue retraction noted in either the sitting or the supine position.  Upon palpation there were no palpable lumps or bumps and no palpable discharge.,Musculoskeletal:  She did have full range of motion of her shoulders.  She did have tenderness upon palpation over the right bicipital tendon.  There is no swelling, crepitus or discoloration noted.,MEDICAL DECISION MAKING:  Most recent hemoglobin A1c was 5.6% back in October 2004.  Most recent lipid checks were obtained back in July 2004.  We have not had this checked since that time.,ASSESSMENT:,1.  Type II diabetes mellitus.,2.  Hypertension.,3.  Right shoulder pain.,4.  Hyperlipidemia.,PLAN:,1.  She is going to go to lab to obtain a hemoglobin A1c, BMP, lipids, CPK, liver enzymes and quantitative microalbumin.,2.  We are going to set her up for a diagnostic bilateral mammogram due to a history of abnormal mammogram in the past which subsequently showed a benign breast cyst.,3.  I told her for her shoulder to take ibuprofen 600 mg three times daily with her meals for a minimum of the next one week.,4.  She is going to follow up in the clinic in three months for a complete comprehensive examination.  If any questions, concerns or problems arise between now and then she should let us know.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>soap / chart / progress notes, soap, foot pain, primary care physician, project access, insurance, foot, project, access, care, appointment</t>
+          <t> </t>
         </is>
       </c>
       <c r="G45" s="2" t="n">
-        <v>543</v>
+        <v>514</v>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>SOAP / Chart / Progress Notes; long; SOAP-style; diagnoses + symptoms + medications</t>
+          <t>SOAP / Chart / Progress Notes; medium; SOAP-style; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J45" s="2" t="n">
-        <v>1392</v>
+        <v>1396</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
@@ -3261,21 +3257,21 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>higher</t>
         </is>
       </c>
       <c r="M45" s="2" t="n">
-        <v>0.3392132551848512</v>
+        <v>0.7346145175834085</v>
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; imaging; treatment plans; follow-up; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; past history; treatment plans; follow-up; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="46" ht="110" customHeight="1">
       <c r="A46" s="2" t="n">
-        <v>783</v>
+        <v>343</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
@@ -3284,39 +3280,39 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Foreign Body Removal - Thigh </t>
+          <t xml:space="preserve"> Shockwave Lithotripsy </t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Removal of foreign body of right thigh.  Foreign body of the right thigh, sewing needle.</t>
+          <t xml:space="preserve"> Right shockwave lithotripsy, cystoscopy, and stent removal x2.</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>PREPROCEDURE DIAGNOSIS:,  Foreign body of the right thigh.,POSTOPERATIVE DIAGNOSIS: , Foreign body of the right thigh, sewing needle.,PROCEDURE:  ,Removal of foreign body of right thigh.,HISTORY:  ,This is a 71-year-old lady who has been referred because there is a mass in the right thigh.  The patient comes with an ultrasound and apparently was diagnosed with a blood clot.  On physical examination, blood pressure was 152/76 and temperature was 95.0.  The patient is 5 feet 1 inch and weighs 170.  On examination of her right thigh, there is a transverse area of ecchymosis in the upper third of the thigh.  There is a palpation of a very sharp object just under the skin.  The patient desires for this to be removed.,DESCRIPTION OF PROCEDURE: , After obtaining informed consent in our office, the area was prepped and draped in usual fashion.  Xylocaine 1% was infiltrated in the end of the object that was the sharpest and a small incision was made there and then I pushed the foreign body through partially and then grabbed it with a hemostat and took it out and it was a 1-1/2-inch sewing needle.,Compression was applied for a few minutes and then a Band-Aid was applied.,The patient was given a tetanus toxoid 0.5 cc IM shot injection and then she was dismissed with instructions of return if inflammatory signs develop.</t>
+          <t>PREOPERATIVE DIAGNOSIS:,  Right renal stone.,POSTOPERATIVE DIAGNOSIS:  ,Right renal stone.,PROCEDURE: , Right shockwave lithotripsy, cystoscopy, and stent removal x2.,ANESTHESIA: , LMA.,ESTIMATED BLOOD LOSS:,  Minimal.  The patient was given antibiotics preoperatively.,HISTORY: , This is a 47-year-old male who presented with right renal stone and right UPJ stone.  The right UPJ stone was removed using ureteroscopy and laser lithotripsy and the stone in the kidney.  The plan was for shockwave lithotripsy.  The patient had duplicated system on the right side.  Risk of anesthesia, bleeding, infection, pain, MI, DVT, PE was discussed.  Options such as watchful waiting, passing the stone on its own, and shockwave lithotripsy were discussed.  The patient wanted to proceed with the shockwave to break the stone into small pieces as possible to allow the stones to pass easily.  Consent was obtained.,DETAILS OF THE OPERATION:  ,The patient was brought to the OR.  Anesthesia was applied.  The patient was placed in the supine position.  Using Dornier lithotriptor total of 2500 shocks were applied.  Energy levels were slowly started at O2 increased up to 7; gradually the stone seem to have broken into smaller pieces as the number of shocks went up.  The shocks were started at 60 per minute and slowly increased up to 90 per minute.  The patient's heart rate and blood pressure were stable throughout the entire procedure.,After the end of the shockwave lithotripsy the patient was placed in dorsal lithotomy position.  The patient was prepped and draped in usual sterile fashion and cystoscopy was done.  Using graspers, the stent was grasped x2 and pulled out, both stents were removed.  The patient tolerated the procedure well.  The patient was brought to recovery in stable condition.  The plan was for the patient to follow up with us and plan for KUB in about two to three months.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>surgery, removal of foreign body, sewing needle, foreign body</t>
+          <t>surgery, renal stone, stent removal, upj stone, shockwave lithotripsy, cystoscopy, stent, renal, shocks, upj, shockwave, lithotripsy, stone</t>
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>222</v>
+        <v>296</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Surgery; short; procedure/operative; diagnoses + vital signs + procedures</t>
+          <t>Surgery; medium; procedure/operative; lower text complexity; diagnoses + symptoms + procedures</t>
         </is>
       </c>
       <c r="J46" s="2" t="n">
-        <v>783</v>
+        <v>343</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
@@ -3329,17 +3325,17 @@
         </is>
       </c>
       <c r="M46" s="2" t="n">
-        <v>0.3787759242560866</v>
+        <v>0.3752254283137962</v>
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; vital signs; procedures; imaging; follow-up; surgery</t>
+          <t>diagnoses; symptoms; procedures; treatment plans; follow-up; surgery</t>
         </is>
       </c>
     </row>
     <row r="47" ht="110" customHeight="1">
       <c r="A47" s="2" t="n">
-        <v>422</v>
+        <v>1190</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
@@ -3348,26 +3344,26 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Plantar Fasciotomy </t>
+          <t xml:space="preserve"> AV Fistula - 4 </t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Plantar fascitis, left foot.  Partial plantar fasciotomy.</t>
+          <t xml:space="preserve"> Creation of autologous right brachiobasilic arteriovenous fistula - first stage.</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>PREOPERATIVE DIAGNOSIS:,  Plantar fascitis, left foot.,POSTOPERATIVE DIAGNOSIS: , Plantar fascitis, left foot.,PROCEDURE PERFORMED: , Partial plantar fasciotomy, left foot.,ANESTHESIA:,  10 cc of 0.5% Marcaine plain with TIVA.,HISTORY:  ,This 35-year-old Caucasian female presents to ABCD General Hospital with above chief complaint.  The patient states she has extreme pain with plantar fascitis in her left foot and has attempted conservative treatment including orthotics without long-term relief of symptoms and desires surgical treatment.  The patient has been NPO since mid night.  Consent is signed and in the chart.  No known drug allergies.,Details Of Procedure:  An IV was instituted by the Department of Anesthesia in the preoperative holding area.  The patient was transported to the operating room and placed on the operating table in supine position with a safety belt across the stomach.  Copious amounts of Webril were placed on the left ankle followed by blood pressure cuff.  After adequate sedation by the Department of Anesthesia, a total of 10 cc of 0.5% Marcaine plain was injected into the surgical site both medially and laterally across the plantar fascia.  The foot was then prepped and draped in the usual sterile orthopedic fashion.  An Esmarch bandage was applied for exsanguination and the pneumatic ankle tourniquet was inflated to 250 mmHg.  The foot was then reflected on the operating, stockinet reflected, and the foot cleansed with a wet and dry sponge.  Attention was then directed to the plantar medial aspect of the left heel.  An approximately 0.75 cm incision was then created in the plantar fat pad over the area of maximal tenderness.,The incision was then deepened with a combination of sharp and blunt dissection until the plantar fascia was palpated.  A #15 blade was then used to transect the medial and central bands of the plantar fascia.  Care was taken to preserve the lateral fibroids.  The foot was dorsiflexed against resistance as the fibers were released and there was noted to be increased laxity after release of the fibers on the plantar aspect of the foot indicating that plantar fascia has in fact been transacted.  The air was then flushed with copious amounts of sterile saline.  The skin incision was then closed with #3-0 nylon in simple interrupted fashion.  Dressings consisted of #0-1 silk, 4 x 4s, Kling, Kerlix, and Coban.  The pneumatic ankle tourniquet was released and immediate hyperemic flush was noted throughout all digits of the left foot.  The patient tolerated the above procedure and anesthesia well without complications.  The patient was transported to the PACU with vital signs stable and vascular status intact to the left foot.  Intraoperatively, an additional 80 cc of 1% lidocaine was injected for additional anesthesia in the case.  The patient is to be nonweightbearing on the left lower extremity with crutches.  The patient is given postoperative pain prescriptions for Vicodin ES, one q3-4h. p.o. p.r.n. for pain as well as Celebrex 200 mg one p.o. b.i.d.  The patient is to follow-up with Dr. X as directed.</t>
+          <t>PREOPERATIVE DIAGNOSES,1.  End-stage renal disease.,2.  Left subclavian vein occlusion.,3.  Status post chronic tracheostomy.,4.  Status post coronary artery bypass grafting.,5.  Right subclavian vein stenosis.,POSTOPERATIVE DIAGNOSES,1.  End-stage renal disease.,2.  Left subclavian vein occlusion.,3.  Status post chronic tracheostomy.,4.  Status post coronary artery bypass grafting.,5.  Right subclavian vein stenosis.,OPERATIVE PROCEDURE,Creation of autologous right brachiobasilic arteriovenous fistula - first stage.,INDICATIONS FOR THE PROCEDURE,This patient has a known left subclavian vein occlusion.  The right subclavian vein has an estimated 50% stenosis.  The patient has a catheter traversed in the right innominate vein.  The right basilic vein was judged to be suitable for usage on vein mapping.,OPERATIVE FINDINGS,The basilic vein was of an adequate size, but somewhat sclerotic.  A first stage autologous right brachiobasilic arteriovenous fistula was created.  A grade 2 was felt at completion.,OPERATIVE PROCEDURE IN DETAIL,After informed consent was obtained, the patient was taken to the operating room.  The patient was placed in the supine position.  The patient received regional nerve block.  The patient also received intravenous sedation.  The right arm was prepped and draped in the usual sterile fashion.  We used ultrasound to locate the basilic vein at the cubital fossa.,A small transverse incision was made slightly above the basilic vein.  The basilic vein was identified and immobilized.  The basilic vein was of a good size, but somewhat sclerotic.  The underlying fascia was incised and the brachial artery was identified and immobilized.  The brachial artery was normal.  We then divided the basilic vein distally.  The distal end was ligated using silk suture.  The brachial artery was clamped proximally and distally.  A small longitudinal arteriotomy was made in the brachial artery.  We did not give heparin.  The end of the basilic vein was then sewn end-to-side to the brachial artery using a running 7-0 Prolene suture.  ,Just prior to completion of the anastomosis, it was flushed and anastomosis was completed.  Flow was then established.  A grade 2 was felt in the outflow basilic fistula.  Hemostasis was secured.  The wound was then closed in layers using interrupted PDS sutures for the fascia and a running 4-0 Monocryl subcuticular suture for the skin.  A sterile dry dressing was applied.,The patient tolerated the procedure well.  There were no operative complications.  The sponge, instrument, and needle counts were correct at the end of the case.  I was present and participated in all aspects of the procedure.  The patient was transferred to the recovery room in satisfactory condition.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>surgery, foot, plantar fasciotomy, plantar fascitis, plantar fascia, plantar, fasciotomy, ankle, medially, fascitis, fascia</t>
+          <t xml:space="preserve">surgery, end-stage renal disease, left subclavian vein occlusion, arteriovenous fistula, artery bypass grafting, autologous, basilic vein, brachial artery, brachiobasilic, clamped, fistula, sclerotic, subclavian vein, subclavian vein stenosis, tracheostomy, brachiobasilic arteriovenous fistula, subclavian vein occlusion, vein occlusion, subclavian, basilic, artery, </t>
         </is>
       </c>
       <c r="G47" s="2" t="n">
-        <v>489</v>
+        <v>398</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
@@ -3376,34 +3372,34 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>Surgery; medium; procedure/operative; diagnoses + symptoms + medications</t>
+          <t>Surgery; medium; other narrative/sectioned; lower text complexity; diagnoses + procedures + imaging</t>
         </is>
       </c>
       <c r="J47" s="2" t="n">
-        <v>422</v>
+        <v>1190</v>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>procedure/operative</t>
+          <t>other narrative/sectioned</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0.5703899909828674</v>
+        <v>0.3529643823264202</v>
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; procedures; treatment plans; follow-up; surgery</t>
+          <t>diagnoses; procedures; imaging; surgery</t>
         </is>
       </c>
     </row>
     <row r="48" ht="110" customHeight="1">
       <c r="A48" s="2" t="n">
-        <v>768</v>
+        <v>422</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
@@ -3412,39 +3408,39 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Gangrene Surgery </t>
+          <t xml:space="preserve"> Plantar Fasciotomy </t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Gangrene osteomyelitis, right second toe.  The patient is a 58-year-old female with poorly controlled diabetes with severe lower extremity lymphedema.  The patient has history of previous right foot infection requiring first ray resection.</t>
+          <t xml:space="preserve"> Plantar fascitis, left foot.  Partial plantar fasciotomy.</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>PREOPERATIVE DIAGNOSIS: , Gangrene osteomyelitis, right second toe.,POSTOPERATIVE DIAGNOSIS: , Gangrene osteomyelitis, right second toe.,OPERATIVE REPORT:  ,The patient is a 58-year-old female with poorly controlled diabetes with severe lower extremity lymphedema.  The patient has history of previous right foot infection requiring first ray resection.  The patient has ulcerations of right second toe dorsally at the proximal interphalangeal joint, which has failed to respond to conservative treatment.  The patient now has exposed bone and osteomyelitis in the second toe.  The patient has been on IV antibiotics as an outpatient and has failed to respond to these and presents today for surgical intervention.,After an IV was started by the Department of Anesthesia, the patient was taken back to the operating room and placed on the operative table in the supine position.  A restraint belt was placed around the patient's waist using copious amounts of Webril and an ankle pneumatic tourniquet was placed around the patient's right ankle and the patient was made comfortable by the Department of Anesthesia.  After adequate amounts of sedation had been given to the patient, we administered a block of 10 cc of 0.5% Marcaine plain in proximal digital block around the second digit.  The foot and ankle were then prepped in the normal sterile orthopedic manner.  The foot was elevated and an Esmarch bandage applied to exsanguinate the foot.  The tourniquet was then inflated to 250 mmHg and the foot was brought back onto the table.  Using Band-Aid scissors, the stockinet was cut and reflected and using a wet and dry sponge, the foot was wiped, cleaned, and the second toe identified.,Using a skin scrape, a racket type incision was planned around the second toe to allow also remodelling of previous operative site.  Using a fresh #10 blade, skin incision was made circumferentially in the racket-shaped manner around the second digit.  Then, using a fresh #15 blade, the incision was deepened and was taken down to the level of the second metatarsophalangeal joint.  Care was taken to identify bleeders and cautery was used as necessary for hemostasis.  After cleaning up all the soft tissue attachments, the second digit was disarticulated down to the level of the metatarsophalangeal joint.  The head of the second metatarsal was inspected and was noted to have good glistening white cartilage with no areas of erosion evident by visual examination.  Attention was then directed to closure of the wound.  All remaining tissue was noted to be healthy and granular in appearance with no necrotic tissue evident.  Areas of subcutaneous tissue were then removed through a sharp dissection in order to allow better approximation of the skin edges.  Due to long-standing lower extremity lymphedema and postoperative changes on previous surgery, I thought that we were unable to close the incision in entirety.  Therefore, after copious amounts of irrigation using sterile saline, it was determined to use modified dental rolls using #4-0 gauze to remove tension from the skin.  Deep vertical mattress sutures were used in order to reapproximate more closely, the skin edges and bring the plantar flap of skin up to the dorsal skin.  This was obtained using #2-0 nylon suture.  Following this, the remaining exposed tissue from the wound was covered using moist to dry saline soaked 4 x 4 gauze.  The wound was then dressed using 4 x 4 gauze fluffed with abdominal pads, then using Kling and Kerlix and an ACE bandage to provide compression.  The tourniquet was deflated at 42 minutes' time and hemostasis was noted to be achieved.  The ACE bandage was extended up to just below the knee and no bleeding striking to the bandages was appreciated.  The patient tolerated the procedure well and was escorted to the Postanesthesia Care Unit with vital signs stable and vascular status intact, as was evidenced by capillary bleeding, which was present during the procedure.  Sedation was given postoperative introductions, which include to remain nonweightbearing to her right foot.  The patient was instructed to keep the foot elevated and to apply ice behind her knee as necessary, no more than 20 minutes each hour.  The patient was instructed to continue her regular medications.  The patient was to continue IV antibiotic course and was given prescription for Vicoprofen to be taken q.4h. p.r.n. for moderate to severe pain #30.  The patient will followup with Podiatry on Monday morning at 8:30 in the Podiatry Clinic for dressing change and evaluation of her foot at that time.,The patient was instructed as to signs and symptoms of infection, was instructed to return to the Emergency Department immediately if these should present.  The second digit was sent to Pathology for gross and micro.</t>
+          <t>PREOPERATIVE DIAGNOSIS:,  Plantar fascitis, left foot.,POSTOPERATIVE DIAGNOSIS: , Plantar fascitis, left foot.,PROCEDURE PERFORMED: , Partial plantar fasciotomy, left foot.,ANESTHESIA:,  10 cc of 0.5% Marcaine plain with TIVA.,HISTORY:  ,This 35-year-old Caucasian female presents to ABCD General Hospital with above chief complaint.  The patient states she has extreme pain with plantar fascitis in her left foot and has attempted conservative treatment including orthotics without long-term relief of symptoms and desires surgical treatment.  The patient has been NPO since mid night.  Consent is signed and in the chart.  No known drug allergies.,Details Of Procedure:  An IV was instituted by the Department of Anesthesia in the preoperative holding area.  The patient was transported to the operating room and placed on the operating table in supine position with a safety belt across the stomach.  Copious amounts of Webril were placed on the left ankle followed by blood pressure cuff.  After adequate sedation by the Department of Anesthesia, a total of 10 cc of 0.5% Marcaine plain was injected into the surgical site both medially and laterally across the plantar fascia.  The foot was then prepped and draped in the usual sterile orthopedic fashion.  An Esmarch bandage was applied for exsanguination and the pneumatic ankle tourniquet was inflated to 250 mmHg.  The foot was then reflected on the operating, stockinet reflected, and the foot cleansed with a wet and dry sponge.  Attention was then directed to the plantar medial aspect of the left heel.  An approximately 0.75 cm incision was then created in the plantar fat pad over the area of maximal tenderness.,The incision was then deepened with a combination of sharp and blunt dissection until the plantar fascia was palpated.  A #15 blade was then used to transect the medial and central bands of the plantar fascia.  Care was taken to preserve the lateral fibroids.  The foot was dorsiflexed against resistance as the fibers were released and there was noted to be increased laxity after release of the fibers on the plantar aspect of the foot indicating that plantar fascia has in fact been transacted.  The air was then flushed with copious amounts of sterile saline.  The skin incision was then closed with #3-0 nylon in simple interrupted fashion.  Dressings consisted of #0-1 silk, 4 x 4s, Kling, Kerlix, and Coban.  The pneumatic ankle tourniquet was released and immediate hyperemic flush was noted throughout all digits of the left foot.  The patient tolerated the above procedure and anesthesia well without complications.  The patient was transported to the PACU with vital signs stable and vascular status intact to the left foot.  Intraoperatively, an additional 80 cc of 1% lidocaine was injected for additional anesthesia in the case.  The patient is to be nonweightbearing on the left lower extremity with crutches.  The patient is given postoperative pain prescriptions for Vicodin ES, one q3-4h. p.o. p.r.n. for pain as well as Celebrex 200 mg one p.o. b.i.d.  The patient is to follow-up with Dr. X as directed.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>surgery, dorsally, toe, ulcerations, foot infection, ray resection, metatarsophalangeal joint, ace bandage, gangrene osteomyelitis, foot, infection, gangrene, digital,</t>
+          <t>surgery, foot, plantar fasciotomy, plantar fascitis, plantar fascia, plantar, fasciotomy, ankle, medially, fascitis, fascia</t>
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>767</v>
+        <v>489</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Surgery; long; procedure/operative; diagnoses + symptoms + medications</t>
+          <t>Surgery; medium; procedure/operative; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J48" s="2" t="n">
-        <v>768</v>
+        <v>422</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
@@ -3457,17 +3453,17 @@
         </is>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0.6022317403065824</v>
+        <v>0.5703899909828674</v>
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; procedures; past history; treatment plans; follow-up; surgery</t>
+          <t>diagnoses; symptoms; medications; allergies; procedures; treatment plans; follow-up; surgery</t>
         </is>
       </c>
     </row>
     <row r="49" ht="110" customHeight="1">
       <c r="A49" s="2" t="n">
-        <v>113</v>
+        <v>85</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
@@ -3476,43 +3472,43 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Hydrocelectomy. </t>
+          <t xml:space="preserve"> Neurogenic Bladder - Consult </t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Left hydrocelectomy.   This is a 67-year-old male with pain, left scrotum.  He has had an elevated PSA and also has erectile dysfunction.  He comes in now for a left hydrocelectomy.  Physical exam confirmed obvious hydrocele, left scrotum.</t>
+          <t xml:space="preserve"> Neurogenic bladder, in a patient catheterizing himself 3 times a day, changing his catheter 3 times a week</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>PREOPERATIVE DIAGNOSIS: , Left hydrocele.,OPERATION: , Left hydrocelectomy.,POSTOPERATIVE DIAGNOSIS: , Left hydrocele.,ANESTHESIA: , General,INDICATIONS AND STUDIES: , This is a 67-year-old male with pain, left scrotum.  He has had an elevated PSA and also has erectile dysfunction.  He comes in now for a left hydrocelectomy.  Physical exam confirmed obvious hydrocele, left scrotum, approximately 8 cm.  Laboratory data included a hematocrit of 43.5, hemoglobin of 15.0, and white count 4700.  Creatinine 1.3, sodium 141, and potassium 4.0.  Calcium 8.6.  Chest x-ray was unremarkable.  EKG was normal.,PROCEDURE: , The patient was satisfactorily given general anesthesia, prepped and draped in supine position, and left scrotal incision was made, carried down to the tunica vaginalis forming the hydrocele.  This was dissected free from the scrotal wall back to the base of the testicle and then excised back to the spermatic cord.  In the fashion, the hydrocele was excised and fluid drained.,Cord was infiltrated with 5 mL of 0.25% Marcaine.  The edges of the tunica vaginalis adjacent to the spermatic cord were oversewn with interrupted 3-0 Vicryl sutures for hemostasis.  The left testicle was replaced into the left scrotal compartment and affixed to the overlying Dartos fascia with a 3-0 Vicryl suture through the edge of the tunica vaginalis and the overlying Dartos fascia.,The left scrotal incision was closed, first closing the Dartos fascia with interrupted 3-0 Vicryl sutures.  Skin was closed with an interrupted running 4-0 chromic suture.  A sterile dressing was applied.  The patient was sent to the recovery room in good condition, upon awakening from general anesthesia.  Plan is to discharge the patient and see him back in the office in a week or 2 in followup.  Further plans will depend upon how he does.</t>
+          <t>HISTORY OF PRESENT ILLNESS: , The patient presents today as a consultation from Dr. ABC's office regarding the above.  He has history of neurogenic bladder, and on intermittent self-catheterization 3 times a day.  However, June 24, 2008, he was seen in the ER, and with fever, weakness, possible urosepsis.  He had a blood culture, which was positive for Staphylococcus epidermidis, as well as urine culture noted for same bacteria.  He was treated on IV antibiotics, Dr. XYZ also saw the patient.  Discharged home.  Not taking any antibiotics.  Today in the office, the patient denies any dysuria, gross hematuria, fever, chills.  He is catheterizing 3 times a day, changing his catheter weekly.  Does have history of renal transplant, which has been followed by Dr. X and is on chronic steroids.  Renal ultrasound, June 23, 2008, was noted for mild hydronephrosis of renal transplant with fluid in the pericapsular space.  Creatinine, July 7, 2008 was 2.0, BUN 36, and patient tells me this is being followed by Dr. X.  No interval complaints today, no issues with catheterization or any gross hematuria.,IMPRESSION:  ,1.  Neurogenic bladder, in a patient catheterizing himself 3 times a day, changing his catheter 3 times a week, we again reviewed the technique of catheterization, and he has no issues with this.,2.  Recurrent urinary tract infection, in a patient who has been hospitalized twice within the last few months, he is on steroids for renal transplant, which has most likely been overall reducing his immune system.  He is asymptomatic today.  No complaints today.,PLAN:,  Following a detailed discussion with the patient, we elected to proceed with intermittent self-catheterization, changing catheter weekly, and technique has been discussed as above.  Based on the recent culture, we will place him on Keflex nighttime prophylaxis, for the next three months or so.  He will call if any concerns.  Follow up as previously scheduled in September for re-assessment.  All questions answered.  The patient is seen and evaluated by myself.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>urology, hydrocele, erectile dysfunction, spermatic cord, tunica vaginalis, vicryl sutures, dartos fascia, hydrocelectomy, psa, testicle, scrotum, scrotal,</t>
+          <t>urology, neurogenic bladder, catheterizing, catheter, urinary tract infection, self-catheterization, intermittent self catheterization, renal transplant, catheterization,</t>
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>283</v>
+        <v>323</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Urology; short; procedure/operative; diagnoses + symptoms + laboratory values</t>
+          <t>Urology; medium; consultation; middle text complexity; diagnoses + symptoms + laboratory values</t>
         </is>
       </c>
       <c r="J49" s="2" t="n">
-        <v>113</v>
+        <v>85</v>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>procedure/operative</t>
+          <t>consultation</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
@@ -3521,17 +3517,17 @@
         </is>
       </c>
       <c r="M49" s="2" t="n">
-        <v>0.5389990982867449</v>
+        <v>0.4687218214607755</v>
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; laboratory values; procedures; imaging; treatment plans; follow-up; surgery</t>
+          <t>diagnoses; symptoms; laboratory values; procedures; imaging; past history; treatment plans; follow-up; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="50" ht="110" customHeight="1">
       <c r="A50" s="2" t="n">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
@@ -3540,26 +3536,26 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Erectile Dysfunction - Followup </t>
+          <t xml:space="preserve"> Flank Pain - Consult - 1 </t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Some improvement of erectile dysfunction, on low dose of Cialis, with no side effects.  </t>
+          <t xml:space="preserve"> Left flank pain, ureteral stone.</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS: , The patient presents today for followup, history of erectile dysfunction, last visit started on Cialis 10 mg.  He indicates that he has noticed some mild improvement of his symptoms, with no side effect.  On this dose, he is having firm erection, able to penetrate, lasting for about 10 or so minutes.  No chest pain, no nitroglycerin usage, no fever, no chills.  No dysuria, gross hematuria, fever, chills.  Daytime frequency every three hours, nocturia times 0, good stream.  He does have a history of elevated PSA and biopsy June of this year was noted for high grade PIN, mid left biopsy, with two specimens being too small to evaluate.  PSA 11.6.  Dr. X's notes are reviewed.,IMPRESSION:  ,1.  Some improvement of erectile dysfunction, on low dose of Cialis, with no side effects.  The patient has multiple risk factors, but denies using any nitroglycerin or any cardiac issues at this time.  We reviewed options of increasing the medication, versus trying other medications, options of penile prosthesis, Caverject injection use as well as working pump is reviewed.,2.  Elevated PSA in a patient with a recent biopsy showing high-grade PIN, as well as two specimens not being large enough to evaluate.  The patient tells me he has met with his primary care physician and after discussion, he is in consideration of repeating a prostate ultrasound and biopsy.  However, he would like to meet with Dr. X to discuss these prior to biopsy.,PLAN: , Following detailed discussion, the patient wishes to proceed with Cialis 20 mg, samples are provided as well as Levitra 10 mg, may increase this to 20 mg and understand administration of each and contraindication as well as potential side effects are reviewed.  The patient not to use them at the same time.  Will call if any other concern.  In the meantime, he is scheduled to meet with Dr. X, with a prior PSA in consideration of a possible repeating prostate ultrasound and biopsy.  He declined scheduling this at this time.  All questions answered.</t>
+          <t>REASON FOR CONSULTATION: , Left flank pain, ureteral stone.,BRIEF HISTORY: , The patient is a 76-year-old female who was referred to us from Dr. X for left flank pain.  The patient was found to have a left ureteral stone measuring about 1.3 cm in size per the patient's history.  The patient has had pain in the abdomen and across the back for the last four to five days.  The patient has some nausea and vomiting.  The patient wants something done for the stone.  The patient denies any hematuria, dysuria, burning or pain.  The patient denies any fevers.,PAST MEDICAL HISTORY: , Negative.,PAST SURGICAL HISTORY:  ,Years ago she had surgery that she does not recall.,MEDICATIONS: , None.,ALLERGIES: , None.,REVIEW OF SYSTEMS: , Denies any seizure disorder, chest pain, denies any shortness of breath, denies any dysuria, burning or pain, denies any nausea or vomiting at this time.  The patient does have a history of nausea and vomiting, but is doing better.,PHYSICAL EXAMINATION:,VITAL SIGNS:  The patient is afebrile.  Vitals are stable.,HEART:  Regular rate and rhythm.,ABDOMEN:  Soft, left-sided flank pain and left lower abdominal pain.,The rest of the exam is benign.,LABORATORY DATA: , White count of 7.8, hemoglobin 13.8, and platelets 234,000.  The patient's creatinine is 0.92.,ASSESSMENT:,1.  Left flank pain.,2.  Left ureteral stone.,3.  Nausea and vomiting.,PLAN: , Plan for laser lithotripsy tomorrow.  Options such as watchful waiting, laser lithotripsy, and shockwave lithotripsy were discussed.  The patient has a pretty enlarged stone.  Failure of the procedure if the stone is significantly impacted into the ureteral wall was discussed.  The patient understood that the success of the surgery may be or may not be 100%, that she may require shockwave lithotripsy if we are unable to get the entire stone out in one sitting.  The patient understood all the risk, benefits of the procedure and wanted to proceed.  Need for stent was also discussed with the patient.  The patient will be scheduled for surgery tomorrow.  Plan for continuation of the antibiotics, obtain urinalysis and culture, and plan for KUB to evaluate for the exact location of the stone prior to surgery tomorrow.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>urology, improvement of erectile dysfunction, erectile dysfunction, erectile, dysfunction, cialis, psa, biopsy,</t>
+          <t xml:space="preserve">urology, flank pain, ureteral stone, shockwave lithotripsy, shockwave, nausea, vomiting, lithotripsy, ureteral, stone, </t>
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -3568,15 +3564,15 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Urology; medium; follow-up/progress; diagnoses + symptoms + medications</t>
+          <t>Urology; medium; consultation; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J50" s="2" t="n">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>follow-up/progress</t>
+          <t>consultation</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
@@ -3585,17 +3581,17 @@
         </is>
       </c>
       <c r="M50" s="2" t="n">
-        <v>0.3959084761045987</v>
+        <v>0.5969341749323716</v>
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; procedures; imaging; past history; treatment plans; follow-up; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; procedures; past history; treatment plans; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="51" ht="110" customHeight="1">
       <c r="A51" s="2" t="n">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
@@ -3604,52 +3600,56 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Elevated PSA - H&amp;P </t>
+          <t xml:space="preserve"> I&amp;D - Penoscrotal Abscess </t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Abnormal serum PSA of 16 ng/ml, dribbling urine, inability to empty bladder, nocturia, urinary hesitancy and slow urine stream.</t>
+          <t xml:space="preserve"> Incision and drainage of the penoscrotal abscess, packing, penile biopsy, cystoscopy, and urethral dilation.</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>CHIEF COMPLAINT:, This 61-year-old male presents today with recent finding of abnormal serum PSA of 16 ng/ml. Associated signs and symptoms: Associated signs and symptoms include dribbling urine, inability to empty bladder, nocturia, urinary hesitancy and urine stream is slow.  Timing (onset/frequency): Onset was 6 months ago. Patient denies fever and chills and denies flank pain.,ALLERGIES: ,Patient admits allergies to adhesive tape resulting in severe rash. Patient denies an allergy to anesthesia.,MEDICATION HISTORY:, Patient is not currently taking any medications.,PAST MEDICAL HISTORY:, Childhood Illnesses: (+) asthma, Cardiovascular Hx: (-) angina, Renal / Urinary Hx: (-) kidney problems.,PAST SURGICAL HISTORY:, Patient admits past surgical history of appendectomy in 1992.,SOCIAL HISTORY:, Patient admits alcohol use, Drinking is described as heavy, Patient denies illegal drug use, Patient denies STD history, Patient denies tobacco use.,FAMILY HISTORY:, Patient admits a family history of gout attacks associated with father.,REVIEW OF SYSTEMS:, Unremarkable with exception of chief complaint.,PHYSICAL EXAM: ,BP Sitting: 120/80 Resp: 20 HR: 72 Temp: 98.6,The patient is a pleasant, 61-year-old male in no apparent distress who looks his given age, is well-developed and nourished with good attention to hygiene and body habitus.,Neck: Neck is normal and symmetrical, without swelling or tenderness. Thyroid is smooth and symmetric with no enlargement, tenderness or masses noted.,Respiratory: Respirations are even without use of accessory muscles and no intercostal retractions noted. Breathing is not labored, diaphragmatic, or abdominal. Lungs clear to auscultation with no rales, rhonchi, wheezes, or rubs noted.,Cardiovascular: Normal S1 and S2 without murmurs, gallop, rubs or clicks.  Peripheral pulses full to palpation, no varicosities, extremities warm with no edema or tenderness.,Gastrointestinal: Abdominal organs, bladder, kidney: No abnormalities, without masses, tenderness, or rigidity. Hernia: absent; no inguinal, femoral, or ventral hernias noted. Liver and/or Spleen: no abnormalities, tenderness, or masses noted. Stool specimen not indicated.,Genitourinary: Anus and perineum: no abnormalities. No fissures, edema, dimples, or tenderness noted.,Scrotum: no abnormalities. No lesions, rash, or sebaceous cyst noted.,Epididymides: no abnormalities, masses, or spermatocele, without enlargement, induration, or tenderness.,Testes: symmetrical; no abnormalities, tenderness, hydrocele, or masses noted.,Urethral Meatus: no abnormalities; no hypospadias, lesions, polyps, or discharge noted.,Penis: no abnormalities; circumcised; no phimosis, Peyronie's, condylomata, or lumps noted.,Prostate: size 60 gr, RT&gt;LT and firm.,Seminal Vesicles: no abnormalities; symmetrical; no tenderness, induration, or nodules noted.,Sphincter tone: no abnormalities; good tone; without hemorrhoids or masses.,Skin/Extremities: Skin is warm and dry with normal turgor and there is no icterus. No skin rash, subcutaneous nodules, lesions or ulcers observed.,Neurological/Psychiatric: Oriented to person, place and time. Mood and affect normal, appropriate to situation, without depression, anxiety, or agitation.,TEST RESULTS:, No tests to report at this time.,IMPRESSION: ,Elevated prostate specific antigen (PSA).,PLAN:, Cystoscopy in the office.,DIAGNOSTIC &amp; LAB ORDERS:, Ordered serum creatinine. Urinalysis and C &amp; S ordered using clean-catch specimen. Ordered free prostate specific antigen (PSA). Ordered ultrasound of prostate.,I have discussed the findings of this follow-up evaluation with the patient. The discussion included a complete verbal explanation of any changes in the examination results, diagnosis and current treatment plan. Discussed the possibility of a TURP surgical procedure; risks, complications, benefits, and alternative measures discussed. There are no activity restrictions . Instructed Ben to avoid caffeinated or alcoholic beverages and excessively spiced foods. Questions answered. If any questions should arise after returning home I have encouraged the patient to feel free to call the office at 327-8850.,PRESCRIPTIONS: , Proscar Dosage: 5 mg tablet Sig: once daily Dispense: 30 Refills: 0 Allow Generic: No,PATIENT INSTRUCTIONS:,  Patient completed benign prostatic hypertrophy questionnaire.</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr"/>
+          <t>PREOPERATIVE DIAGNOSIS: , Penoscrotal abscess.,POSTOPERATIVE DIAGNOSIS:,  Penoscrotal abscess.,OPERATION: , Incision and drainage of the penoscrotal abscess, packing, penile biopsy, cystoscopy, and urethral dilation.,BRIEF HISTORY: , The patient is a 75-year-old male presented with penoscrotal abscess.  Options such as watchful waiting, drainage, and antibiotics were discussed.  Risks of anesthesia, bleeding, infection, pain, MI, DVT, PE, completely the infection turning into necrotizing fascitis, Fournier's gangrene were discussed.  The patient already had significant phimotic changes and disfigurement of the penis.  For further debridement the patient was told that his penis is not going to be viable, he may need a total or partial penectomy now or in the future.  Risks of decreased penile sensation, pain, Foley, other unexpected issues were discussed.  The patient understood all the complications and wanted to proceed with the procedure.,DETAIL OF THE OPERATION:  ,The patient was brought to the OR.  The patient was placed in dorsal lithotomy position.  The patient was prepped and draped in the usual fashion.  Pictures were taken prior to starting the procedure for documentation.  The patient had an open sore on the right side of the penis measuring about 1 cm in size with pouring pus out using blunt dissection.  The penile area was opened up distally to allow the pus to come out.  The dissection around the proximal scrotum was done to make sure there are no other pus pockets.  The corporal body was intact, but the distal part of the corpora was completely eroded and had a fungating mass, which was biopsied and sent for permanent pathology analysis.,Urethra was identified at the distal tip, which was dilated and using 23-French cystoscope cystoscopy was done, which showed some urethral narrowing in the distal part of the urethra.  The rest of the bladder appeared normal.  The prostatic urethra was slightly enlarged.  There are no stones or tumors inside the bladder.  There were moderate trabeculations inside the bladder.  Otherwise, the bladder and the urethra appeared normal.  There was a significantly fungating mass involving the distal part of the urethra almost possibility to have including the fungating wart or fungating squamous cell carcinoma.  Again biopsies were sent for pathology analysis.  Prior to urine irrigation anaerobic aerobic cultures were sent, irrigation with over 2 L of fluid was performed.  After irrigation, packing was done with Kerlix.  The patient was brought to recovery in a stable condition.  Please note that 18-French Foley was kept in place.  Electrocautery was used at the end of the procedure to obtain hemostasis as much as possible, but there was fungating mass with slight bleeding packing was done and tight scrotal Kling was applied.  The patient was brought to Recovery in a stable condition after applying 0.5% Marcaine about 20 mL were injected around for local anesthesia.</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">urology, i&amp;d, penoscrotal, penile biopsy, cystoscopy, urethral dilation, incision and drainage, fungating mass, penoscrotal abscess, abscess, urethral, </t>
+        </is>
+      </c>
       <c r="G51" s="2" t="n">
-        <v>574</v>
+        <v>453</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Urology; long; history and physical; diagnoses + symptoms + medications</t>
+          <t>Urology; medium; procedure/operative; lower text complexity; diagnoses + symptoms + procedures</t>
         </is>
       </c>
       <c r="J51" s="2" t="n">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>history and physical</t>
+          <t>procedure/operative</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>higher</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="M51" s="2" t="n">
-        <v>0.8476104598737602</v>
+        <v>0.3762962128043282</v>
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; vital signs; procedures; imaging; past history; treatment plans; follow-up; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; procedures; surgery</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Curate 50 medium-focused MTSamples reports (#14)
Keep 48 medium reports and document two Allergy/Immunology length exceptions. Preserve the historical EDA and record reproducible selection checks, source IDs, and hashes.
</commit_message>
<xml_diff>
--- a/data/curated_baseline/mtsamples_curated_50.xlsx
+++ b/data/curated_baseline/mtsamples_curated_50.xlsx
@@ -523,7 +523,7 @@
     </row>
     <row r="2" ht="110" customHeight="1">
       <c r="A2" s="2" t="n">
-        <v>4995</v>
+        <v>0</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -532,26 +532,26 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Kawasaki Disease - Discharge Summary </t>
+          <t xml:space="preserve"> Allergic Rhinitis </t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> This is a 14-month-old baby boy Caucasian who came in with presumptive diagnosis of Kawasaki with fever for more than 5 days and conjunctivitis, mild arthritis with edema, rash, resolving and with elevated neutrophils and thrombocytosis, elevated CRP and ESR. </t>
+          <t xml:space="preserve"> A 23-year-old white female presents with complaint of allergies.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>ADMITTING DIAGNOSIS: , Kawasaki disease.,DISCHARGE DIAGNOSIS:,  Kawasaki disease, resolving.,HOSPITAL COURSE:,  This is a 14-month-old baby boy Caucasian who came in with presumptive diagnosis of Kawasaki with fever for more than 5 days and conjunctivitis, mild arthritis with edema, rash, resolving and with elevated neutrophils and thrombocytosis, elevated CRP and ESR.  When he was sent to the hospital, he had a fever of 102.  Subsequently, the patient was evaluated and based on the criteria, he was started on high dose of aspirin and IVIG.  Echocardiogram was also done, which was negative.  IVIG was done x1, and between 12 hours of IVIG, he spiked fever again; it was repeated twice, and then after second IVIG, he did not spike any more fever.  Today, his fever and his rash have completely resolved.  He does not have any conjunctivitis and no redness of mucous membranes.  He is more calm and quite and taking good p.o.; so with a very close followup and a cardiac followup, he will be sent home.,DISCHARGE ACTIVITIES:,  Ad-lib.,DISCHARGE DIET: , PO ad-lib.,DISCHARGE MEDICATIONS: , Aspirin high dose 340 mg q.6h. for 1 day and then aspirin low dose 40 mg q.d. for 14 days and then Prevacid also to prevent his GI from aspirin 15 mg p.o. once a day.  He will be followed by his primary doctor in 2 to 3 days.  Cardiology for echo followup in 4 to 6 weeks and instructed not to give any vaccine in less than 11 months because of IVIG, all the live virus vaccine, and if he gets any rashes, any fevers, should go to primary care doctor as soon as possible.</t>
+          <t>SUBJECTIVE:,  This 23-year-old white female presents with complaint of allergies.  She used to have allergies when she lived in Seattle but she thinks they are worse here.  In the past, she has tried Claritin, and Zyrtec.  Both worked for short time but then seemed to lose effectiveness.  She has used Allegra also.  She used that last summer and she began using it again two weeks ago.  It does not appear to be working very well.  She has used over-the-counter sprays but no prescription nasal sprays.  She does have asthma but doest not require daily medication for this and does not think it is flaring up.,MEDICATIONS: , Her only medication currently is Ortho Tri-Cyclen and the Allegra.,ALLERGIES: , She has no known medicine allergies.,OBJECTIVE:,Vitals:  Weight was 130 pounds and blood pressure 124/78.,HEENT:  Her throat was mildly erythematous without exudate.  Nasal mucosa was erythematous and swollen.  Only clear drainage was seen.  TMs were clear.,Neck:  Supple without adenopathy.,Lungs:  Clear.,ASSESSMENT:,  Allergic rhinitis.,PLAN:,1.  She will try Zyrtec instead of Allegra again.  Another option will be to use loratadine.  She does not think she has prescription coverage so that might be cheaper.,2.  Samples of Nasonex two sprays in each nostril given for three weeks.  A prescription was written as well.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>allergy / immunology, mucous membranes, conjunctivitis, ad lib, kawasaki disease, vaccine, fever, aspirin</t>
+          <t>allergy / immunology, allergic rhinitis, allergies, asthma, nasal sprays, rhinitis, nasal, erythematous, allegra, sprays, allergic,</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>270</v>
+        <v>204</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -560,28 +560,28 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Allergy / Immunology; short; discharge summary; diagnoses + symptoms + medications</t>
+          <t>Allergy / Immunology; short (documented Allergy length exception); SOAP-style; lower text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>4995</v>
+        <v>0</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>discharge summary</t>
+          <t>SOAP-style</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0.383509918845807</v>
+        <v>0.3761834986474301</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; imaging; follow-up</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; treatment plans; assessment/plan</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Allergy / Immunology; medium; other narrative/sectioned; diagnoses + symptoms + medications</t>
+          <t>Allergy / Immunology; medium; other narrative/sectioned; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J3" s="2" t="n">
@@ -647,7 +647,7 @@
     </row>
     <row r="4" ht="110" customHeight="1">
       <c r="A4" s="2" t="n">
-        <v>4996</v>
+        <v>4998</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -656,22 +656,22 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Followup on Asthma </t>
+          <t xml:space="preserve"> Allergy Evaluation Consult </t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> A female for a complete physical and follow up on asthma with allergic rhinitis.</t>
+          <t xml:space="preserve"> Acute allergic reaction, etiology uncertain, however, suspicious for Keflex.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>SUBJECTIVE: , This is a 42-year-old white female who comes in today for a complete physical and follow up on asthma.  She says her asthma has been worse over the last three months.  She has been using her inhaler daily.  Her allergies seem to be a little bit worse as well.  Her husband has been hauling corn and this seems to aggravate things.  She has not been taking Allegra daily but when she does take it, it seems to help somewhat.  She has not been taking her Flonase which has helped her in the past.  She also notes that in the past she was on Advair but she got some vaginal irritation with that.,She had been noticing increasing symptoms of irritability and PMS around her menstrual cycle.  She has been more impatient around that time.  Says otherwise her mood is normal during the rest of the month.  It usually is worse the week before her cycle and improves the day her menstrual cycle starts.  Menses have been regular but somewhat shorter than in the past.  Occasionally she will get some spotting after her cycles.  She denies any hot flashes or night sweats with this.  In reviewing the chart it is noted that she did have 3+ blood with what appeared to be a urinary tract infection previously.  Her urine has not been rechecked.  She recently had lab work and cholesterol drawn for a life insurance application and is going to send me those results when available.,REVIEW OF SYSTEMS: , As above.  No fevers, no headaches, no shortness of breath currently.  No chest pain or tightness.  No abdominal pain, no heartburn, no constipation, diarrhea or dysuria.  Occasional stress incontinence.  No muscle or joint pain.  No concerns about her skin.  No polyphagia, polydipsia or polyuria.,PAST MEDICAL HISTORY: , Significant for asthma, allergic rhinitis and cervical dysplasia.,SOCIAL HISTORY: , She is married.  She is a nonsmoker.,MEDICATIONS: , Proventil and Allegra.,ALLERGIES: , Sulfa.,OBJECTIVE:,Vital signs:  Her weight is 151 pounds.  Blood pressure is 110/60.  Pulse is 72.  Temperature is 97.1 degrees.  Respirations are 20.,General:  This is a well-developed, well-nourished 42-year-old white female, alert and oriented in no acute distress.  Affect is appropriate and is pleasant.,HEENT:  Normocephalic, atraumatic.  Tympanic membranes are clear.  Conjunctivae are clear.  Pupils are equal, round and reactive to light.  Nares without turbinate edema.  Oropharynx is nonerythematous.,Neck:  Supple without lymphadenopathy, thyromegaly, carotid bruit or JVD.,Chest:  Clear to auscultation bilaterally.,Cardiovascular:  Regular rate and rhythm without murmur.,Abdomen:  Soft, nontender, nondistended.  Normoactive bowel sounds.  No masses or organomegaly to palpation.,Extremities:  Without cyanosis or edema.,Skin:  Without abnormalities.,Breasts:  Normal symmetrical breasts without dimpling or retraction.  No nipple discharge.  No masses or lesions to palpation.  No axillary masses or lymphadenopathy.,Genitourinary:  Normal external genitalia.  The walls of the vaginal vault are visualized with normal pink rugae with no lesions noted.  Cervix is visualized without lesion.  She has a moderate amount of thick white/yellow vaginal discharge in the vaginal vault.  No cervical motion tenderness.  No adnexal tenderness or fullness.,ASSESSMENT/PLAN:,1.  Asthma.  Seems to be worse than in the past.  She is just using her Proventil inhaler but is using it daily.  We will add Flovent 44 mcg two puffs p.o. b.i.d.  May need to increase the dose.  She did get some vaginal irritation with Advair in the past but she is willing to retry that if it is necessary.  May also need to consider Singulair.  She is to call me if she is not improving.  If her shortness of breath worsens she is to call me or go into the emergency department.  We will plan on following up for reevaluation in one month.,2.  Allergic rhinitis.  We will plan on restarting Allegra and Flonase daily for the time being.,3.  Premenstrual dysphoric disorder.  She may have some perimenopausal symptoms.  We will start her on fluoxetine 20 mg one tablet p.o. q.d.,4.  Hematuria.  Likely this is secondary to urinary tract infection but we will repeat a UA to document clearing.  She does have some frequent dysuria but is not having it currently.,5.  Cervical dysplasia.  Pap smear is taken.  We will notify the patient of results.  If normal we will go back to yearly Pap smear.  She is scheduled for screening mammogram and instructed on monthly self-breast exam techniques.  Recommend she get 1200 mg of calcium and 400 U of vitamin D a day.</t>
+          <t>HISTORY: , A 34-year-old male presents today self-referred at the recommendation of Emergency Room physicians and his nephrologist to pursue further allergy evaluation and treatment.  Please refer to chart for history and physical, as well as the medical records regarding his allergic reaction treatment at ABC Medical Center for further details and studies.  In summary, the patient had an acute event of perioral swelling, etiology uncertain, occurring on 05/03/2008 requiring transfer from ABC Medical Center to XYZ Medical Center due to a history of renal failure requiring dialysis and he was admitted and treated and felt that his allergy reaction was to Keflex, which was being used to treat a skin cellulitis dialysis shunt infection.  In summary, the patient states he has some problems with tolerating grass allergies, environmental and inhalant allergies occasionally, but has never had anaphylactic or angioedema reactions.  He currently is not taking any medication for allergies.  He is taking atenolol for blood pressure control.  No further problems have been noted upon his discharge and treatment, which included corticosteroid therapy and antihistamine therapy and monitoring.,PAST MEDICAL HISTORY:,  History of urticaria, history of renal failure with hypertension possible source of renal failure, history of dialysis times 2 years and a history of hypertension.,PAST SURGICAL HISTORY:,  PermCath insertion times 3 and peritoneal dialysis.,FAMILY HISTORY: , Strong for heart disease, carcinoma, and a history of food allergies, and there is also a history of hypertension.,CURRENT MEDICATIONS: , Atenolol, sodium bicarbonate, Lovaza, and Dialyvite.,ALLERGIES: , Heparin causing thrombocytopenia.,SOCIAL HISTORY: , Denies tobacco or alcohol use.,PHYSICAL EXAMINATION:  ,VITAL SIGNS:  Age 34, blood pressure 128/78, pulse 70, temperature is 97.8, weight is 207 pounds, and height is 5 feet 7 inches.,GENERAL:  The patient is healthy appearing; alert and oriented to person, place and time; responds appropriately; in no acute distress.,HEAD:  Normocephalic.  No masses or lesions noted.,FACE:  No facial tenderness or asymmetry noted.,EYES:  Pupils are equal, round and reactive to light and accommodation bilaterally.  Extraocular movements are intact bilaterally.,EARS:  The tympanic membranes are intact bilaterally with a good light reflex.  The external auditory canals are clear with no lesions or masses noted.  Weber and Rinne tests are within normal limits.,NOSE:  The nasal cavities are patent bilaterally.  The nasal septum is midline.  There are no nasal discharges.  No masses or lesions noted.,THROAT:  The oral mucosa appears healthy.  Dental hygiene is maintained well.  No oropharyngeal masses or lesions noted.  No postnasal drip noted.,NECK:  The neck is supple with no adenopathy or masses palpated.  The trachea is midline.  The thyroid gland is of normal size with no nodules.,NEUROLOGIC:  Facial nerve is intact bilaterally.  The remaining cranial nerves are intact without focal deficit.,LUNGS:  Clear to auscultation bilaterally.  No wheeze noted.,HEART:  Regular rate and rhythm.  No murmur noted.,IMPRESSION:  ,1.  Acute allergic reaction, etiology uncertain, however, suspicious for Keflex.,2.  Renal failure requiring dialysis.,3.  Hypertension.,RECOMMENDATIONS:  ,RAST allergy testing for both food and environmental allergies was performed, and we will get the results back to the patient with further recommendations to follow.  If there is any specific food or inhalant allergen that is found to be quite high on the sensitivity scale, we would probably recommend the patient to avoid the offending agent to hold off on any further reactions.  At this point, I would recommend the patient stopping any further use of cephalosporin antibiotics, which may be the cause of his allergic reaction, and I would consider this an allergy.  Being on atenolol, the patient has a more difficult time treating acute anaphylaxis, but I do think this is medically necessary at this time and hopefully we can find specific causes for his allergic reactions.  An EpiPen was also prescribed in the event of acute angioedema or allergic reaction or sensation of impending allergic reaction and he is aware he needs to proceed directly to the emergency room for further evaluation and treatment recommendations after administration of an EpiPen.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="n">
-        <v>708</v>
+        <v>638</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -680,15 +680,15 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Allergy / Immunology; long; follow-up/progress; diagnoses + symptoms + medications</t>
+          <t>Allergy / Immunology; long (documented Allergy length exception); consultation; higher text complexity; diagnoses + medications + allergies</t>
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>4996</v>
+        <v>4998</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>follow-up/progress</t>
+          <t>consultation</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -697,17 +697,17 @@
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>0.7729936880072137</v>
+        <v>0.7756424706943192</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; vital signs; past history; treatment plans; follow-up; assessment/plan</t>
+          <t>diagnoses; medications; allergies; vital signs; past history; treatment plans; surgery</t>
         </is>
       </c>
     </row>
     <row r="5" ht="110" customHeight="1">
       <c r="A5" s="2" t="n">
-        <v>4874</v>
+        <v>4626</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -716,43 +716,43 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Chest Pain - Office Note </t>
+          <t xml:space="preserve"> Transesophageal Echocardiography Probe </t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Patient with a family history of premature coronary artery disease came in for evaluation of recurrent chest pain</t>
+          <t xml:space="preserve"> Insertion of transesophageal echocardiography probe and unsuccessful insertion of arterial venous lines.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>DISCHARGE DIAGNOSES:,1.  Chest pain.  The patient ruled out for myocardial infarction on serial troponins.  Result of nuclear stress test is pending.,2.  Elevated liver enzymes, etiology uncertain for an outpatient followup.,3.  Acid reflux disease.,TEST DONE: , Nuclear stress test, results of which are pending.,HOSPITAL COURSE: , This 32-year-old with family history of premature coronary artery disease came in for evaluation of recurrent chest pain, O2 saturation at 94% with both atypical and typical features of ischemia.  The patient ruled out for myocardial infarction with serial troponins.  Nuclear stress test has been done, results of which are pending.  The patient is stable to be discharged pending the results of nuclear stress test and cardiologist's recommendations.  He will follow up with cardiologist, Dr. X, in two weeks and with his primary physician in two to four weeks.  Discharge medications will depend on results of nuclear stress test.</t>
+          <t>INDICATIONS FOR PROCEDURE:,  Impending open heart surgery for closure of ventricular septal defect in a 4-month-old girl.,Procedures were done under general anesthesia.  The patient was already in the operating room under general anesthesia.  Antibiotic prophylaxis with cefazolin and gentamicin was already given prior to beginning the procedures.,PROCEDURE #1:,  Insertion of transesophageal echocardiography probe.,DESCRIPTION OF PROCEDURE #1: , The probe was well lubricated and with digital manipulation, was passed into the esophagus without resistance.  The probe was placed so that the larger diameter was in the anterior-posterior position during insertion.  The probe was used by the pediatric cardiologist for preoperative and postoperative diagnostic echocardiography.  At the end, it was removed without trauma and there was no blood tingeing.  It is to be noted that approximately 30 minutes after removing the cannula, I inserted a 14-French suction tube to empty the stomach and there were a few mL of blood secretions that were suctioned.  There was no overt bleeding.,PROCEDURE #2: , Attempted and unsuccessful insertion of arterial venous lines.,DESCRIPTION OF PROCEDURE #2:,  Both groins were prepped and draped.  The patient was placed at 10 degrees head-up position.  A Cook 4-French double-lumen 8-cm catheter kit was opened.  Using the 21-gauge needle that comes with the kit, several attempts were made to insert central venous and then an arterial line in the left groin.  There were several successful punctures of these vessels, but I was unable to advance Seldinger wire.  After removal of the needles, the area was compressed digitally for approximately 5 minutes.  There was a small hematoma that was not growing.  Initially, the left leg was mildly mottled with prolonged capillary refill of approximately 3 seconds.  Using 1% lidocaine, I infiltrated the vessels of the groin both medial and lateral to the vascular sheath.  Further observation, the capillary refill and circulation of the left leg became more than adequate.  The O2 saturation monitor that was on the left toe functioned well throughout the procedures, from the beginning to the end.  At the end of the procedure, the circulation of the leg was intact.,</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>cardiovascular / pulmonary, chest pain, serial troponins, premature coronary artery disease, coronary artery disease, nuclear stress test, stress test</t>
+          <t>cardiovascular / pulmonary, impending open heart surgery, ventricular septal defect, antibiotic prophylaxis, cefazolin, transesophageal echocardiography probe, arterial venous lines, groin, transesophageal echocardiography, echocardiography probe, insertion, transesophageal, arterial, venous, groins, echocardiography, probe</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>144</v>
+        <v>341</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Cardiovascular / Pulmonary; short; follow-up/progress; diagnoses + symptoms + medications</t>
+          <t>Cardiovascular / Pulmonary; medium; other narrative/sectioned; lower text complexity; diagnoses + procedures + imaging</t>
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>4874</v>
+        <v>4626</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>follow-up/progress</t>
+          <t>other narrative/sectioned</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -761,17 +761,17 @@
         </is>
       </c>
       <c r="M5" s="2" t="n">
-        <v>0.2741771866546438</v>
+        <v>0.3669972948602344</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; vital signs; past history; treatment plans; follow-up</t>
+          <t>diagnoses; procedures; imaging; surgery</t>
         </is>
       </c>
     </row>
     <row r="6" ht="110" customHeight="1">
       <c r="A6" s="2" t="n">
-        <v>4690</v>
+        <v>4720</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -780,39 +780,35 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Pulmonary Consultation - 2 </t>
+          <t xml:space="preserve"> Non-Q-wave Myocardial Infarction </t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Patient with complaints of significant coughing and wheezing.</t>
+          <t xml:space="preserve"> A patient with non-Q-wave myocardial infarction.  No definite chest pains.  The patient is breathing okay.  The patient denies orthopnea or PND.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>PAST MEDICAL HISTORY:,  Unremarkable, except for diabetes and atherosclerotic vascular disease.,ALLERGIES:,  PENICILLIN.,CURRENT MEDICATIONS:,  Include Glucovance, Seroquel, Flomax, and Nexium.,PAST SURGICAL HISTORY: , Appendectomy and exploratory laparotomy.,FAMILY HISTORY: , Noncontributory.,SOCIAL HISTORY:  ,The patient is a non-smoker.  No alcohol abuse.  The patient is married with no children.,REVIEW OF SYSTEMS:,  Significant for an old CVA.,PHYSICAL EXAMINATION:,  The patient is an elderly male alert and cooperative.  Blood pressure 96/60 mmHg.  Respirations were 20.  Pulse 94.  Afebrile.  O2 was 94% on room air.  HEENT:  Normocephalic and atraumatic.  Pupils are reactive.  Oral mucosa is grossly normal.  Neck is supple.  Lungs:  Decreased breath sounds.  Disturbed breath sounds with poor exchange.  Heart:  Regular rhythm.  Abdomen:  Soft and nontender.  No organomegaly or masses.  Extremities:  No cyanosis, clubbing, or edema.,LABORATORY DATA: , Oropharyngeal evaluation done on 11/02/2006 revealed mild oropharyngeal dysphagia with no evidence of laryngeal penetration or aspiration with food or liquid.  Slight reduction in tongue retraction resulting in mild residual remaining in the palatal sinuses, which clear with liquid swallow and double-saliva swallow.,ASSESSMENT:,1.  Cough probably multifactorial combination of gastroesophageal reflux and recurrent aspiration.,2.  Old CVA with left hemiparesis.,3.  Oropharyngeal dysphagia.,4.  Diabetes.,PLAN:,  At the present time, the patient is recommended to continue on a regular diet, continue speech pathology evaluation as well as perform double-swallow during meals with bolus sensation.  He may use Italian lemon ice during meals to help clear sinuses as well.  The patient will follow up with you.  If you need any further assistance, do not hesitate to call me.</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cardiovascular / pulmonary, pulmonary evaluation, cough, wheezing, congestion, coughing and wheezing, breath sounds, oropharyngeal dysphagia, pulmonary, breath, sounds, dysphagia, aspiration, sinuses, oropharyngeal, coughing, swallowing, </t>
-        </is>
-      </c>
+          <t>REASON FOR CONSULT: , A patient with non-Q-wave myocardial infarction.,HISTORY OF PRESENT ILLNESS: , The patient is a pleasant 52-year-old gentleman with a history of diabetes mellitus, hypertension, and renal failure, on dialysis, who presented with emesis, dizziness, and nausea for the last few weeks.  The patient reports having worsening emesis and emesis a few times.  No definite chest pains.  The patient is breathing okay.  The patient denies orthopnea or PND.,PAST MEDICAL HISTORY:,1.  Diabetes mellitus.,2.  Hypertension.,3.  Renal failure, on dialysis.,MEDICATIONS:,  Aspirin, Coreg, doxazosin, insulin, metoclopramide, simvastatin, and Starlix.,ALLERGIES:  ,NO KNOWN DRUG ALLERGIES.,SOCIAL HISTORY: , The patient denies tobacco, alcohol or drug use.,FAMILY HISTORY: , Negative for early atherosclerotic heart disease.,REVIEW OF SYSTEMS: , General:  The patient denies fever or chills.  Pulmonary:  The patient denies hemoptysis.  Cardiovascular:  Refer to HPI.  GI:  The patient denies hematemesis or melena.  The rest of systems review is negative.,PHYSICAL EXAMINATION:,VITAL SIGNS:  Pulse 71, blood pressure 120/70, and respiratory rate 18.,GENERAL:  A well-nourished, well-developed male in no acute distress.,HEENT:  Normocephalic, atraumatic.  Pupils seem to be equal, round, and reactive.  Extraocular muscles are full, but the patient has left eye ptosis.,NECK:  Supple without JVD or lymphadenopathy.,LUNGS:  Clear to auscultation bilaterally.,CARDIOVASCULAR:  PMI is displaced 0.5 cm lateral to the midclavicular line.  Regular rate and rhythm, S1, S2.  No definite S3, 2/6 holosystolic murmur at the apex radiating to the axilla.,ABDOMEN:  Positive bowel sounds, nondistended and nontender.  No hepatosplenomegaly.,EXTREMITIES:  Trace pedal edema.,EKG shows atrial fibrillation with rapid ventricular response at 164 with old anteroseptal myocardial infarction and old inferior wall myocardial infarction.  Subsequent EKG in sinus rhythm shows sinus rhythm with old inferior wall myocardial infarction and probable anteroseptal myocardial infarction with Q-waves in V1, V2, and up to V3.,LABORATORY EXAM: , WBC 28,800, hemoglobin 13.6, hematocrit 40, and platelets 266,000.  PT 11.3, INR 1.1, and PTT 24.1.  Sodium 126, potassium 4.3, chloride 86, CO2 26, glucose 371, BUN 80, and creatinine 8.4.  CK was 261, then 315, and then 529 with CK-MB of 8.06, then 8.69, and then 24.6.  Troponin was 0.051, then 0.46, and then 19.8 this morning.,IMPRESSION:,1.  Paroxysmal atrial fibrillation.  The heart rate was slowed down with IV Cardizem, the patient converted to sinus rhythm.  The patient is currently in sinus rhythm.,2.  Emesis.  The etiology is unclear.  The patient reports that the emesis is better.  The patient is just having some nausea.,3.  Non-Q-wave myocardial infarction.  EKG shows atrial fibrillation with old anteroseptal myocardial infarction and old inferior wall myocardial infarction.,4.  Diabetes mellitus.,5.  Renal failure.,6.  Hypertension.,7.  Hypercholesterolemia.,PLAN:,1.  We will start amiodarone to keep from going back into atrial fibrillation.,2.  Echocardiogram.,3.  Aspirin and IV heparin.,4.  Serial CK-MB and troponin.,5.  Cardiac catheterization, possible percutaneous coronary intervention.  The risks, benefits, and alternatives were explained to the patient through a translator.  The patient understands and wishes to proceed.,6.  IV Integrilin.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="n">
-        <v>244</v>
+        <v>458</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Cardiovascular / Pulmonary; short; consultation; diagnoses + symptoms + medications</t>
+          <t>Cardiovascular / Pulmonary; medium; consultation; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>4690</v>
+        <v>4720</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -825,11 +821,11 @@
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>0.6734107303877368</v>
+        <v>0.9004170423805229</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; past history; treatment plans; follow-up; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; assessment/plan</t>
         </is>
       </c>
     </row>
@@ -872,7 +868,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Cardiovascular / Pulmonary; medium; procedure/operative; diagnoses + medications + laboratory values</t>
+          <t>Cardiovascular / Pulmonary; medium; procedure/operative; middle text complexity; diagnoses + medications + laboratory values</t>
         </is>
       </c>
       <c r="J7" s="2" t="n">
@@ -899,7 +895,7 @@
     </row>
     <row r="8" ht="110" customHeight="1">
       <c r="A8" s="2" t="n">
-        <v>4965</v>
+        <v>4976</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
@@ -908,35 +904,35 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Atrial Fibrillation - Consult </t>
+          <t xml:space="preserve"> Abnormal Echocardiogram </t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> A 74-year-old woman for Cardiology consultation regarding atrial fibrillation and anticoagulation after a fall.  The patient denies any chest pain nor clear shortness of breath.</t>
+          <t xml:space="preserve"> Abnormal echocardiogram findings and followup.  Shortness of breath, congestive heart failure, and valvular insufficiency.   The patient complains of shortness of breath, which is worsening.  The patient underwent an echocardiogram, which shows severe mitral regurgitation and also large pleural effusion.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS:,  I was kindly asked to see Ms. ABC who is a 74-year-old woman for cardiology consultation regarding atrial fibrillation and anticoagulation after a fall.,The patient is somnolent at this time, but does arouse, but is unable to provide much history.  By review of the chart, it appears that she fell, which is what she states when she got up out of a rocking chair and could not get herself off the floor.  She states that 1-1/2 hours later she was able to get herself off the floor.,The patient denies any chest pain nor clear shortness of breath.,PAST MEDICAL HISTORY: , Includes, end-stage renal disease from hypertension.  She follows up with Dr. X in her office and has been known to have a small-to-moderate sized pericardial effusion since 11/07 that has apparently been followed and it appears that the patient was not interested in having diagnostic pericardiocentesis done.  She had an echocardiogram today (please see also that report), which shows stable and small-to-moderate sized pericardial effusion without tamponade, normal left ventricular ejection fraction at 55% with mild concentric left ventricular hypertrophy, mildly dilated right ventricular size, normal right ventricular ejection fraction, moderate mitral regurgitation and severe tricuspid regurgitation with severe pulmonary hypertension, estimated PA systolic pressure of 71 mmHg when compared to the prior echocardiogram done 08/29/07, previously the mitral regurgitation was mild and previously the PA systolic pressure was estimated at 90 mmHg.  Other findings were not significantly changed including pericardial effusion description.  She has a history of longstanding hypertension.  She has been on hemodialysis since 1997 for renal failure, history of mini-strokes documented several years ago, history of seizure disorder, she has a history of right upper extremity edema and right breast enlargement from right subclavian vein occlusion.  She has a history of hypertension, depression, hyperlipidemia, on Sensipar for tertiary hyperparathyroidism.,PAST SURGICAL HISTORY: , Includes, cholecystectomy, post fistula in the left arm, which has failed, and right arm, which is being used including number of operative procedures to the fistula.  She follows up with Dr. Y regarding neurovascular surgery.,MEDICATIONS: , On admission:,1.  Norvasc 10 mg once a day.,2.  Aspirin 81 mg once a day.,3.  Colace 200 mg two at bedtime.,4.  Labetalol 100 mg p.o. b.i.d.,5.  Nephro-Vite one tablet p.o. q.a.m.,6.  Dilantin 100 mg p.o. t.i.d.,7.  Renagel 1600 mg p.o. t.i.d.,8.  Sensipar 120 mg p.o. every day.,9.  Sertraline 100 mg p.o. nightly.,10.  Zocor 20 mg p.o. nightly.,ALLERGIES: , TO MEDICATIONS PER CHART ARE NONE.,FAMILY HISTORY:  ,Unable to obtain as the patient becomes quite sleepy when I am talking.,SOCIAL HISTORY:  ,Unable to obtain as the patient becomes quite sleepy when I am talking.,REVIEW OF SYSTEMS: , Unable to obtain as the patient becomes quite sleepy when I am talking.,PHYSICAL EXAM:  ,Temperature 99.2, blood pressure ranges from 88/41 to 108/60, pulse 70, respiratory rate, 20, O2 saturation 98%.  Height is 5 feet 1 inch, weight 147 pounds.  On general exam, she is a pleasant elderly woman who does arouse to voice, but then becomes quite sleepy and apparently that is an improvement from when she was admitted.  HEENT shows the cranium is normocephalic and atraumatic.  She has moist mucosal membranes.  Neck veins are difficult to assess, but do not appear clinically distended.  No carotid bruits.  Lungs are clear to auscultation anteriorly.  No wheezes.  Cardiac exam:  S1, S2 regular rate, 3/6 holosystolic murmur heard with radiation from the left apex towards the left axilla.  No rub, no gallop.  PMI is nondisplaced.  Abdomen:  Soft, nondistended.  CVA is benign.  Extremities with no significant edema.  Pulses appear grossly intact.  She has evidence of right upper extremity edema, which is apparently chronic.,DIAGNOSTIC DATA/LAB DATA: , EKGs are reviewed including from 07/07/09 at 08:31 a.m., which shows atrial fibrillation with left anterior fascicular block, poor R-wave progression when compared to one done on 07/06/09 at 18:25, there is really no significant change.  The atrial fibrillation appears present since at least on EKG done on 11/02/07 and this EKG is not significantly changed from the most recent one.  Echocardiogram results as above.  Chest x-ray shows mild pulmonary vascular congestion.  BNP shows 3788.  Sodium 136, potassium 4.5, chloride 94, bicarbonate 23, BUN 49, creatinine 5.90.  Troponin was 0.40 followed by 0.34.  INR 1.03 on 05/18/07.  White blood cell count 9.4, hematocrit 42, platelet count 139.,IMPRESSION: , Ms. ABC is a 74-year-old woman admitted to the hospital with a fall and she has a history of vascular dementia, so her history is somewhat unreliable it seems and she is somnolent at that time.  She does have chronic atrial fibrillation again documented at least present since 2007 and I found an EKG report by Dr. X, which shows atrial fibrillation on 08/29/07 per her report.  One of the questions we were asked was whether the patient would be a candidate for Coumadin.  Clearly given her history of small mini-strokes, I think Coumadin would be appropriate given this chronic atrial fibrillation, but the main issue is the fall risk.  If not felt to be significant fall risk then I would strongly recommend Coumadin as the patient herself states that she has only fallen twice in the past year.  I would defer that decision to Dr. Z and Dr. XY who know the patient well and it may be that physical therapy consult is appropriate to help adjudicate.,RECOMMENDATIONS:,1.  Fall assessment as per Dr. Z and Dr. XY with possible PT consult if felt appropriate and if the patient is not felt to be at significant fall risk, would put her on Coumadin.  Given her history of small strokes as documented in the chart and her chronic atrial fibrillation, she does have reasonable heart rate control on current labetalol.,2.  The patient has elevated BNP and I suspect that is due to her severe pulmonary hypertension and renal failure and in the light of normal LV function, I would not make any further evaluation of that other than aggressive diuresis.,3.  Regarding this minimal troponin elevation, I do not feel this is a diagnosis especially in the setting of pulmonary hypertension and her small-to-moderate sized stable pericardial effusion again that has been longstanding since 2007 from what I can tell and there is no evidence of tamponade.  I would defer to her usual cardiologist Dr. X whether an outpatient stress evaluation is appropriate for risk stratification.  I did find that the patient had a prior cardiac stress test in 08/07 where they felt that there was some subtle reversibility of the anterior wall, but it was felt that it may be artifact rather than true ischemia with normal LV function seen on that study as well.,4.  Continue Norvasc for history of hypertension as well as labetalol.,5.  The patient is felt to be a significant fall risk and will at least continue her aspirin 81 mg once a day for secondary CVA, thromboprophylaxis (albeit understanding that it is inferior to Coumadin).,6.  Continue Dilantin for history of seizures.</t>
+          <t>REASON FOR CONSULTATION:  ,Abnormal echocardiogram findings and followup.  Shortness of breath, congestive heart failure, and valvular insufficiency.,HISTORY OF PRESENT ILLNESS:  ,The patient is an 86-year-old female admitted for evaluation of abdominal pain and bloody stools.  The patient has colitis and also diverticulitis, undergoing treatment.  During the hospitalization, the patient complains of shortness of breath, which is worsening.  The patient underwent an echocardiogram, which shows severe mitral regurgitation and also large pleural effusion.  This consultation is for further evaluation in this regard.  As per the patient, she is an 86-year-old female, has limited activity level.  She has been having shortness of breath for many years.  She also was told that she has a heart murmur, which was not followed through on a regular basis.,CORONARY RISK FACTORS: , History of hypertension, no history of diabetes mellitus, nonsmoker, cholesterol status unclear, no prior history of coronary artery disease, and family history noncontributory.,FAMILY HISTORY:  ,Nonsignificant.,PAST SURGICAL HISTORY: , No major surgery.,MEDICATIONS: , Presently on Lasix, potassium supplementation, Levaquin, hydralazine 10 mg b.i.d., antibiotic treatments, and thyroid supplementation.,ALLERGIES:  ,AMBIEN, CARDIZEM, AND IBUPROFEN.,PERSONAL HISTORY:,  She is a nonsmoker.  Does not consume alcohol.  No history of recreational drug use.,PAST MEDICAL HISTORY:  ,Basically GI pathology with diverticulitis, colitis, hypothyroidism, arthritis, questionable hypertension, no prior history of coronary artery disease, and heart murmur.,REVIEW OF SYSTEMS,CONSTITUTIONAL:  Weakness, fatigue, and tiredness.,HEENT:  History of cataract, blurred vision, and hearing impairment.,CARDIOVASCULAR:  Shortness of breath and heart murmur.  No coronary artery disease.,RESPIRATORY:  Shortness of breath.  No pneumonia or valley fever.,GASTROINTESTINAL:  No nausea, vomiting, hematemesis, or melena.,UROLOGICAL:  No frequency or urgency.,MUSCULOSKELETAL:  Arthritis and severe muscle weakness.,SKIN:  Nonsignificant.,NEUROLOGICAL:  No TIA or CVA.  No seizure disorder.,ENDOCRINE/HEMATOLOGICAL:  As above.,PHYSICAL EXAMINATION,VITAL SIGNS:  Pulse of 84, blood pressure of 168/74, afebrile, and respiratory rate 16 per minute.,HEENT/NECK:  Head is atraumatic and normocephalic.  Neck veins flat.  No significant carotid bruits appreciated.,LUNGS:  Air entry bilaterally fair.  No obvious rales or wheezes.,HEART:  PMI displaced.  S1, S2 with systolic murmur at the precordium, grade 2/6.,ABDOMEN:  Soft and nontender.,EXTREMITIES:  Chronic skin changes.  Feeble pulses distally.  No clubbing or cyanosis.,DIAGNOSTIC DATA: , EKG:  Normal sinus rhythm.  No acute ST-T changes.,Echocardiogram report was reviewed.,LABORATORY DATA:,  H&amp;H 13 and 39.  BUN and creatinine within normal limits.  Potassium within normal limits.  BNP 9290.,IMPRESSION:,1.  The patient admitted for gastrointestinal pathology, under working treatment.,2.  History of prior heart murmur with echocardiogram findings as above.  Basically revealed normal left ventricular function with left atrial enlargement, large pleural effusion, and severe mitral regurgitation and tricuspid regurgitation.,RECOMMENDATIONS:,1.  From cardiac standpoint, conservative treatment.  Possibility of a transesophageal echocardiogram to assess valvular insufficiency adequately well discussed extensively.,2.  After extensive discussion, given her age 86, limited activity level, and no intention of undergoing any treatment in this regard from a surgical standpoint, the patient does not wish to proceed with a transesophageal echocardiogram.,3.  Based on the above findings, we will treat her medically with ACE inhibitors and diuretics and see how she fares.  She has a normal LV function.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="n">
-        <v>1143</v>
+        <v>482</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Cardiovascular / Pulmonary; long; consultation; diagnoses + symptoms + medications</t>
+          <t>Cardiovascular / Pulmonary; medium; consultation; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>4965</v>
+        <v>4976</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -949,17 +945,17 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>0.9389652840396754</v>
+        <v>0.8649684400360684</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; surgery</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; imaging; past history; treatment plans; follow-up; surgery</t>
         </is>
       </c>
     </row>
     <row r="9" ht="110" customHeight="1">
       <c r="A9" s="2" t="n">
-        <v>4447</v>
+        <v>4457</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -968,43 +964,43 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Ear Pain - Drainage </t>
+          <t xml:space="preserve"> Dietary Consultation - 1 </t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Right ear pain with drainage - otitis media and otorrhea.</t>
+          <t xml:space="preserve"> Dietary consultation for a woman with polycystic ovarian syndrome and hyperlipidemia.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>CHIEF COMPLAINT:,  Right ear pain with drainage.,HISTORY OF PRESENT ILLNESS:,  This is a 12-year-old white male here with his mother for complaints of his right ear hurting.  Mother states he has been complaining for several days.  A couple of days ago she noticed drainage from the right ear.  The patient states it has been draining for several days and it has a foul smell to it.  He has had some low-grade fever.  The patient was seen in the office about a week ago with complaints of a sore throat, headache and fever.  The patient was evaluated for Strep throat which was negative and just had been doing supportive care.  He did have a recent airplane ride a couple of weeks ago also.  There has been no cough, shortness of breath or wheezing.  No vomiting or diarrhea.,PHYSICAL EXAM:,General:  He is alert in no distress.,Vital Signs:  Temperature:  99.1 degrees.,HEENT:  Normocephalic, atraumatic.  Pupils equal, round and react to light.  The left TM is clear.  The right TM is poorly visualized secondary to purulent secretions in the right ear canal.  There is no erythema of the ear canals.  Nares is patent.  Oropharynx is clear.  The patient does wear braces.,Neck:  Supple.,Lungs:  Clear to auscultation.,Heart:  Regular.  No murmur.,ASSESSMENT:,1.  Right otitis media.,2.  Right otorrhea.,PLAN:,  Ceftin 250 mg by mouth twice a day for 10 days.  Ciprodex four drops to the right ear twice a day.  The patient is to return to the office in two weeks for followup.</t>
+          <t>SUBJECTIVE:,  This is a followup dietary consultation for polycystic ovarian syndrome and hyperlipidemia.  The patient reports that she has resumed food record keeping which she feels like it has given her greater control.  Her physical activity level has remained high.  Her struggle times are in the mid-afternoon if she has not had enough food to eat, as well as in the evening after dinner.,OBJECTIVE:, Vital Signs:  Weight is 189-1/2 pounds.  Food records were reviewed,ASSESSMENT:,  The patient has experienced a weight loss of 1-1/2 pounds in the last month.  She is commended for these efforts.  We have reviewed food records identifying that she has done a nice job keeping a calorie count for the last two or three weeks.  We discussed the value of this and how it was very difficulty to resume it, however, after she suspended the record keeping.  We also discussed its reflection that she is not getting very many fruits and vegetables on a regular basis.  We identified some ways of preventing her from feeling sluggish and having problems with low blood sugar in the middle of the afternoon by routinely planning an afternoon snack that can prevent these symptoms.  This will likely be around 2:30 or 3 p.m. for her.  We also discussed strategies for evening snacking to help put some definition and boundaries to the snacking.,PLAN:,  I recommended the patient routinely include an afternoon snack around 2:30 to 3 p.m.  It will be helpful if this snack includes some protein such as nuts or low-fat cheese.  She is also encouraged to continue with her record keeping for food choices and calorie points.  I also recommended she maintain her high level of physical activity.  Will plan to follow the patient in one month for ongoing support.  This was a 30-minute consultation.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>consult - history and phy., drainage, ear hurting, ear pain, otitis media, otorrhea, ear pain with drainage, otitis, media, ear,</t>
+          <t>consult - history and phy., dietary consultation, calorie count, calorie points, consultation, food choices, food record, hyperlipidemia, low-fat cheese, many fruits and vegetables, physical activity, polycystic ovarian syndrome, snack, dietary, polycystic, food, afternoon</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>241</v>
+        <v>295</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Consult - History and Phy.; short; other narrative/sectioned; diagnoses + symptoms + medications</t>
+          <t>Consult - History and Phy.; medium; SOAP-style; lower text complexity; diagnoses + symptoms + vital signs</t>
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>4447</v>
+        <v>4457</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>other narrative/sectioned</t>
+          <t>SOAP-style</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1013,11 +1009,11 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0.3765779981965735</v>
+        <v>0.3642921550946799</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; vital signs; past history; treatment plans; follow-up; assessment/plan</t>
+          <t>diagnoses; symptoms; vital signs; treatment plans; follow-up; assessment/plan</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1052,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Consult - History and Phy.; medium; history and physical; diagnoses + symptoms + medications</t>
+          <t>Consult - History and Phy.; medium; history and physical; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
@@ -1083,7 +1079,7 @@
     </row>
     <row r="11" ht="110" customHeight="1">
       <c r="A11" s="2" t="n">
-        <v>4427</v>
+        <v>4218</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -1092,39 +1088,39 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Erythema Nodosum - Consult </t>
+          <t xml:space="preserve"> OB/GYN - H&amp;P </t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The patient presents for a followup for history of erythema nodosum.</t>
+          <t xml:space="preserve"> Initial obstetrical examination - Normal first pregnancy.  Inadequate naternal nutrition.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>REASON FOR VISIT:,  The patient presents for a followup for history of erythema nodosum.,HISTORY OF PRESENT ILLNESS: , This is a 25-year-old woman who is attending psychology classes.  She was diagnosed with presumptive erythema nodosum in 2004 based on a biopsy consistent with erythema nodosum, but not entirely specific back in Netherlands.  At that point, she had undergone workup which was extensive for secondary diseases associated with erythema nodosum.  Part of her workup included a colonoscopy.  The findings were equivocal characterizes not clearly abnormal biopsies of the terminal ileum.,The skin biopsy, in particular, mentions some fibrosis, basal proliferation, and inflammatory cells in the subcutis.,Prior to the onset of her erythema nodosum, she had a tibia-fibula fracture several years before on the right, which was not temporarily associated with the skin lesions, which are present in both legs anyway.  Even, a jaw cosmetic surgery she underwent was long before she started developing her skin lesions.  She was seen in our clinic and by Dermatology on several occasions.  Apart from the first couple of visits when she presented stating a recurrent skin rash with a description suggestive of erythema nodosum in the lower extremities and ankle and there is discomfort pointing towards a possible inflammatory arthritis and an initial high sed rate of above 110 with an increased CRP.  In the following visits, no evident abnormality has been detected.  In the first visit, here some MTP discomfort detected.  It was thought that erythema nodosum may be present.  However, the evaluation of Dermatology did not concur and it was thought that the patient had venous stasis, which could be related to her prior fracture.  When she was initially seen here, a suspicion of IBD, sarcoid inflammatory arthropathy, and lupus was raised.  She had an equivocal rheumatoid fracture, but her CCP was negative.  She had an ANA, which was positive at 1:40 with a speckled pattern persistently, but the rest of the lupus serologies including double-stranded DNA, RNP, Smith, Ro, La were negative.  Her cardiolipin panel antibodies were negative as well.  We followed the IgM, IgG, and IgA being less than 10.  However, she did have a beta-2 glycoprotein 1 or an RVVT tested and this may be important since she has a livedo pattern.  It was thought that the onset of lupus may be the case.  It was thought that rheumatoid arthritis could not be the case since it is not associated with erythema nodosum.  For the fear of possible lymphoma, she underwent CT of the chest, abdomen, and pelvis.  It was done also in order to rule out sarcoid and the result was unremarkable.  Based on some changes in her bowel habits and evidence of B12 deficiency with a high methylmalonic and high homocystine levels along with a low normal B12 in addition to iron studies consistent with iron deficiency and an initially low MCV, the possibility of inflammatory bowel disease was employed.  The patient underwent an initially unrevealing colonoscopy and a capsule endoscopy, which was normal.  A second colonoscopy was done recently and microscopically no evidence of inflammatory bowel disease was seen.  However, eosinophil aggregations were noted in microscopy and this was told to be consistent with an allergic reaction or an emerging Crohn disease and I will need to discuss with Gastroenterology what is the significance of that.  Her possible B12 deficiency and iron deficiency were never addressed during her stay here in the United States.,In the initial appointment, she was placed on prednisone 40 mg, which was gradually titrated down this led to an exacerbation of her acne.  We decided to take her off prednisone due to adverse effects and start her on colchicine 0.6 mg daily.  While this kept things under control with the inflammatory markers being positive and no overt episodes of erythema nodosum, the patient still complains for sensitivity with less suspicious skin rash in the lower extremities and occasional ankle swelling and pain.  She was reevaluated by Dermatology for that and no evidence of erythema nodosum was felt to be present.  Out plan was to proceed with a DEXA scan, at some point check a vitamin D level, and order vitamin D and calcium over the counter for bone protection purposes.  However, the later was deferred until we have resolved the situation and find out what is the underlying cause of her disease.,Her past medical history apart from the tibia-fibular fracture and the jaw cosmetic surgery is significant for varicella and mononucleosis.,Her physical examination had shown consistently diffuse periarticular ankle edema and also venous stasis changes at least until I took over her care last August.  I have not been able to detect any erythema nodosum, however, a livedo pattern has been detected consistently.  She also has evidence of acne, which does not seem to be present at the moment.  She also was found to have a heart murmur present and we are going to proceed with an echocardiogram placed.,Her workup during the initial appointment included an ACE level, which was normal.  She also had a rather higher sed rate up to 30, but prior to that, per report, it was even higher, above 110.  Her RVVT was normal, her rheumatoid factor was negative.  Her ANA was 1:40, speckled pattern.  The double-stranded DNA was negative.  Her RNP and Smith were negative as well.  RO and LA were negative and cardiolipin antibodies were negative as well.  A urinalysis at the moment was completely normal.  A CRP was 2.3 in the initial appointment, which was high.  A CCP was negative.  Her CBC had shown microcytosis and hypochromia with a hematocrit of 37.7.  This improved later without any evidence of hypochromia, microcytosis or anemia with a hematocrit of 40.3.,The patient returns here today, as I mentioned, complaining of milder bouts of skin rash, which she calls erythema nodosum, which is accompanied by arthralgias, especially in the ankles.  I am mentioning here that photosensitivity rash was mentioned in the past.  She tells me that she had it twice back in Europe after skiing where her whole face was swollen.  Her acne has been very stable after she was taken off prednisone and was started on colchicine 0.6 daily.  Today we discussed about the effect of colchicine on a possible pregnancy.,MEDICATIONS: , Prednisone was stopped.  Vitamin D and calcium over the counter, we need to verify that.  Colchicine 0.6 mg daily which we are going to stop, ranitidine 150 mg as needed, which she does not take frequently.,FINDINGS:,  On physical examination, she is very pleasant, alert, and oriented x 3 and not in any acute distress.  There is some evidence of faint subcutaneous lesions in both shins bilaterally, but with mild tenderness, but no evidence of classic erythema nodosum.  Stasis dermatitis changes in both lower extremities present.  Mild livedo reticularis is present as well.,There is some periarticular ankle edema as well.  Laboratory data from 04/23/07, show a normal complete metabolic profile with a creatinine of 0.7, a CBC with a white count of 7880, hematocrit of 40.3, and platelets of 228.  Her microcytosis and hypochromia has resolved.  Her serum electrophoresis does not show a monoclonal abnormality.  Her vitamin D levels were 26, which suggests some mild insufficiency and she would probably benefit by vitamin D supplementation.  This points again towards some ileum pathology.  Her ANCA B and C were negative.  Her PF3 and MPO were unremarkable.  Her endomysial antibodies were negative.  Her sed rate at this time were 19.  The highest has been 30, but prior to her appointment here was even higher.  Her ANA continues to be positive with a titer of 1:40, speckled pattern.  Her double-stranded DNA is negative.  Her serum immunofixation confirmed the absence of monoclonal abnormality.  Her urine immunofixation was not performed.  Her IgG, IgA, and IgM levels are normal.  Her IgE levels are normal as well.  A urinalysis was not performed this time.  Her CRP is 0.4.  Her tissue transglutaminase antibodies are negative.  Her ASCA is normal and anti-OmpC was not tested.  Gliadin antibodies IgA is 12, which is in the borderline to be considered equivocal, but these are nonspecific.  I am reminding here that her homocystine levels have been 15.7, slightly higher, and that her methylmalonic acid was 385, which is obviously abnormal.  Her B12 levels were 216, which is rather low possibly indicating a B12 deficiency.  Her iron studies showed a ferritin of 15, a saturation of 9%, and an iron of 30.  Her TIBC was 345 pointing towards an iron deficiency anemia.  I am reminding you that her ACE levels in the past were normal and that she has a microcytosis.  Her radiologic workup including a thoracic, abdominal, and pelvic CT did not show any suspicious adenopathy, but only small aortocaval and periaortic nodes, the largest being 8 mm in short axis, likely reactive.  Her pelvic ultrasound showed normal uterus adnexa.  Her bladder was normal as well.  Subcentimeter inguinal nodes were found.  There was no large lytic or sclerotic lesion noted.  Her recent endoscopy was unremarkable, but the microscopy showed some eosinophil aggregation, which may be pointing towards allergy or an evolving Crohn disease.  Her capsule endoscopy was limited secondary to rapid transit.  There was only a tiny mucosal red spot in the proximal jejunum without active bleeding, 2 possible erosions were seen in the distal jejunum and proximal ileum.  However, no significant inflammation or bleeding was seen and this could be small bowel crisis.  Neither evidence of bleeding or inflammation were seen as well.  Specifically, the terminal ileum appeared normal.  Recent evaluation by a dermatologist did not verify the presence of erythema nodosum.,ASSESSMENT:,  This is a 25-year-old woman diagnosed with presumptive erythema nodosum in 2004.  She has been treated with prednisone as in the beginning she had also a wrist and ankle discomfort and high inflammatory markers.  Since I took over her care, I have not seen a clear-cut erythema nodosum being present.  No evidence of synovitis was there.  Her serologies apart from an ANA of 1:40 were negative.  She has a livedo pattern, which has been worrisome.  The issue here was a possibility of inflammatory bowel disease based on deficiency in vitamin B12 as indicated by high methylmalonic and homocystine levels and also iron deficiency.  She also has low vitamin D levels, which point towards terminal ileum pathology as well and she had a history of decreased MCV.  We never received the x-ray of her hands which she had and she never had a DEXA scan.  Lymphoma has been ruled out and we believe that inflammatory bowel disease, after repeated colonoscopies and the capsule endoscopy, has been ruled out as well.  Sarcoid is probably not the case since the patient did not have any lymphadenopathies and her ACE levels were normal.  We are going check a PPD to rule out tuberculosis.  We are going to order an RVVT and glycoprotein beta-1 levels in her workup to make sure that an antiphospholipid syndrome is not present given the livedo pattern.  An anti-intrinsic factor will be added as well.  Her primary care physician needs to workup the possible B12 and iron deficiency and also the vitamin D deficiency.  In the meanwhile, we feel that the patient should stop taking the colchicine and if she has a flare of her disease then she should present to her dermatologist and have the skin biopsy performed in order to have a clear-cut answer of what is the nature of this skin rash.  Regarding her heart murmur, we are going to proceed with an echocardiogram.  A PPD should be placed as well.  In her next appointment, we may fax a requisition for vitamin B replacement.,PROBLEMS/DIAGNOSES:,  1.  Recurrent erythema nodosum with ankle and wrist discomfort, ? arthritis.,2.  Iron deficiencies, according to iron studies.,3.  Borderline B12 with increased methylmalonic acid and homocystine.,4.  On chronic steroids; vitamin D and calcium is needed; she needs a DEXA scan.,5.  Typical ANCA, per records, were not verified here.  ANCA and ASCA were negative and the OmpC was not ordered.,6.  Acne.,7.  Recurrent arthralgia not present.  Rheumatoid factor, CCP negative, ANA 1:40 speckled.,8.  Livedo reticularis, beta 2-glycoprotein was not checked, we are going to check it today.  Needs vaccination for influenza and pneumonia.,9.  Vitamin D deficiency.  She needs replacement with ergocalciferol, but this may point towards ___________ pathology as this was not detected.,10.  Recurrent ankle discomfort which necessitates ankle x-rays.,PLANS:,  We can proceed with part of her workup here in clinic, PPD, echocardiogram, ankle x-rays, and anti-intrinsic factor antibodies.  We can start repleting her vitamin D with __________ weeks of ergocalciferol 50,000 weekly.  We can add an RVVT and glycoprotein to her workup in order to rule out any antiphospholipid syndrome.  She should be taking vitamin D and calcium after the completion of vitamin D replacement.  She should be seen by her primary care physician, have the iron and B12 deficiency worked up.  She should stop the colchicine and if the skin lesion recurs then she should be seen by her dermatologist.  Based on the physical examination, we do not suspect that the patient has the presence of any other disease associated with erythema nodosum.  We are going to add an amylase and lipase to evaluate her pancreatic function, RPR, HIV, __________ serologies.  Given the evidence of possible malabsorption it may be significant to proceed with an upper endoscopy to rule out Whipple disease or celiac disease which can sometimes be associated with erythema nodosum.  An anti-intrinsic factor would be added, as I mentioned.  I doubt whether the patient has Behcet disease given the absence of oral or genital ulcers.  She does not give a history of oral contraceptives or medications that could be related to erythema nodosum.  She does not have any evidence of lupus __________ mycosis.  Histoplasmosis coccidioidomycosis would be accompanied by other symptoms.  Hodgkin disease has probably been ruled out with a CAT scan.  However, we are going to add an LDH in future workup.  I need to discuss with her primary care physician regarding the need for workup of her vitamin B12 deficiency and also with her gastroenterologist regarding the need for an upper endoscopy.  The patient will return in 1 month.</t>
+          <t>CHIEF COMPLAINT,:  This 32 year-old female presents today for an initial obstetrical examination.  Home pregnancy test was positive.,The patient indicates fetal activity is not yet detected (due to early stage of pregnancy).  LMP:  02/13/2002 EDD:  11/20/2002 GW:  8.0 weeks.  Patient has been trying to conceive for 6 months.,Menses:  Onset:  12 years old.  Interval:  24-26 days.  Duration:  4-6 days.  Flow:  moderate.  Complications:  PMS - mild.,Last Pap smear taken on 11/2/2001.  Contraception:  Patient is currently using none.,ALLERGIES:,  Patient admits allergies to venom - bee/wasp resulting in difficulty breathing, severe rash, pet dander resulting in nasal stuffiness.  Medication History:  None.,PAST MEDICAL HISTORY:,  Past medical history is unremarkable.  Past Surgical History:  Patient admits past surgical history of tonsillectomy in 1980.  Social History:  Patient admits alcohol use Drinking is described as social, Patient denies illegal drug use, Patient denies STD history, Patient denies tobacco use.,FAMILY HISTORY:,  Patient admits a family history of cancer of breast associated with mother.,REVIEW OF SYSTEMS:,Neurological: (+) unremarkable.,Respiratory: (+) difficulty sleeping, (-) breathing difficulties, respiratory symptoms.,Psychiatric: (+) anxious feelings.,Cardiovascular: (-) cardiovascular problems or chest symptoms.,Genitourinary: (-) decreased libido, (-) vaginal dryness, (-) vaginal bleeding.  Diet is high in empty calories, high in fats and low in fiber.,PHYSICAL EXAM:,  BP Standing:  126/84 Resp:  22 HR:  78 Temp:  99.1 Height:  5 ft.  6 in.  Weight:  132 lbs.,Pre-Gravid Weight is 125 lbs.,Patient is a 32 year old female who appears pleasant, in no apparent distress, her given age, well developed,,well nourished and with good attention to hygiene and body habitus.,Oriented to person, place and time.,Mood and affect normal and appropriate to situation.,HEENT:Head &amp; Face:  Examination of head and face is unremarkable.,Skin:  No skin rash, subcutaneous nodules, lesions or ulcers observed.  No edema observed.,Cardiovascular:  Heart auscultation reveals no murmurs, gallop, rubs or clicks.,Respiratory:  Lungs CTA.,Breast:  Chest (Breasts):  Breast inspection and palpation shows no abnormal findings.,Abdomen:  Abdomen soft, nontender, bowel sounds present x 4 without palpable masses.,Genitourinary:  External genitalia are normal in appearance.  Examination of urethra shows no abnormalities.  Examination of vaginal vault reveals no abnormalities.  Cervix shows no pathology.  Uterine portion of bimanual exam reveals contour normal, shape regular and size normal.  Adnexa and parametria show no masses, tenderness, organomegaly or nodularity.  Examination of anus and perineum shows no abnormalities.,TEST RESULTS: , Urine pregnancy test:  positive. CBC results within normal limits.  Blood type:  O positive.  Rh:  positive.  FBS:  88 mg/dl.,IMPRESSION:,  Pregnancy, normal first.  Maternal nutrition is inadequate for protein and poor and high in empty calories and junk foods and sweets.,PLAN:,  Pap smear submitted for manual screening.  Ordered CBC.  Ordered blood type.  Ordered hemoglobin.  Ordered Rh.,Ordered fasting blood glucose.,COUNSELING:,  Counseling was given regarding adverse effects of alcohol, physical activity and sexual activity.  Educational supplies dispensed to patient.,Return to clinic in 4 week (s).,PRESCRIPTIONS:,  NatalCare Plus Dosage:  Prenatal Multivitamins tablet Sig:  QD Dispense:  60 Refills:  4 Allow Generic:  Yes,PATIENT INSTRUCTIONS:,  Patient received written information regarding pre-eclampsia and eclampsia.  Patient was instructed to restrict activity.  Patient instructed to limit caffeine use.  Patient instructed to limit salt intake.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="n">
-        <v>2332</v>
+        <v>490</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Consult - History and Phy.; long; consultation; diagnoses + symptoms + medications</t>
+          <t>Consult - History and Phy.; medium; history and physical; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>4427</v>
+        <v>4218</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>consultation</t>
+          <t>history and physical</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1133,17 +1129,17 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>0.8742110009017132</v>
+        <v>0.833633904418395</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; follow-up; surgery</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; past history; treatment plans; follow-up; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="12" ht="110" customHeight="1">
       <c r="A12" s="2" t="n">
-        <v>3963</v>
+        <v>3938</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -1152,39 +1148,35 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Discharge Summary - 14 </t>
+          <t xml:space="preserve"> Discharge Summary - COPD </t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The patient is a 60-year-old female patient who off and on for the past 10 to 12 months has had almost daily diarrhea, nausea, inability to eat. </t>
+          <t xml:space="preserve"> Chest x-ray on admission, no acute finding, no interval change.  CT angiography, negative for pulmonary arterial embolism.  Chronic obstructive pulmonary disease exacerbation improving, on steroids and bronchodilators.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS: , The patient is a 60-year-old female patient who off and on for the past 10 to 12 months has had almost daily diarrhea, nausea, inability to eat.  She had an EGD and colonoscopy with Dr. ABC a few days prior to this admission.  Colonoscopy did reveal diverticulosis and EGD showed retained bile and possible gastritis.  Biopsies were done.  The patient presented to our emergency room for worsening abdominal pain as well as swelling of the right lower leg.,PAST MEDICAL HISTORY: , Extensive and well documented in prior charts.,PHYSICAL EXAMINATION: , Abdomen was diffusely tender.  Lungs clear.  Blood pressure 129/69 on admission.  At the time of admission, she had just a trace of bilateral lower edema.,LABORATORY STUDIES: , White count 6.7, hemoglobin 13, hematocrit 39.3.  Potassium of 3.2 on 08/15/2007.,HOSPITAL COURSE: , Dr. ABC apparently could not advance the scope into the cecum and therefore warranted a barium enema.  This was done and did not really show what the cecum on the barium enema.  There was some retained stool in that area and the patient had a somewhat prolonged hospital course on the remaining barium from the colon.  She did have some enemas.  She had persistent nausea, headache, neck pain throughout this hospitalization.  Finally, she did improve enough to the point where she could be discharged home.,DISCHARGE DIAGNOSIS: , Nausea and abdominal pain of uncertain etiology.,SECONDARY DIAGNOSIS:  ,Migraine headache.,COMPLICATIONS:  ,None.,DISCHARGE CONDITION: , Guarded.,DISCHARGE PLAN:  ,Follow up with me in the office in 5 to 7 days to resume all pre-admission medications.  Diet and activity as tolerated.</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>discharge summary, diarrhea, nausea, inability to eat, egd, colonoscopy, biopsies, barium enema, cecum, barium, admission,</t>
-        </is>
-      </c>
+          <t>PROCEDURES:,1.  Chest x-ray on admission, no acute finding, no interval change.,2.  CT angiography, negative for pulmonary arterial embolism.,3.  Nuclear myocardial perfusion scan, abnormal.  Reversible defect suggestive of ischemia, ejection fraction of 55%.,DIAGNOSES ON DISCHARGE:,1.  Chronic obstructive pulmonary disease exacerbation improving, on steroids and bronchodilators.,2.  Coronary artery disease, abnormal nuclear scan, discussed with Cardiology Dr. X, who recommended to discharge the patient and follow up in the clinic.,3.  Diabetes mellitus type 2.,4.  Anemia, hemoglobin and hematocrit stable.,5.  Hypokalemia, replaced.,6.  History of coronary artery disease status post stent placement 2006-2008.,7.  Bronchitis.,HOSPITAL COURSE:  ,The patient is a 65-year-old American-native Indian male, past medical history of heavy tobacco use, history of diabetes mellitus type 2, chronic anemia, COPD, coronary artery disease status post stent placement, who presented in the emergency room with increasing shortness of breath, cough productive for sputum, and orthopnea.  The patient started on IV steroid, bronchodilator as well as antibiotics.,He also complained of chest pain that appears to be more pleuritic with history of coronary artery disease and orthopnea.  He was evaluated by Cardiology Dr. X, who proceeded with stress test.  Stress test reported positive for reversible ischemia, but Cardiology decided to follow up the patient in the clinic.  The patient's last cardiac cath was in 2008.,The patient clinically significantly improved and wants to go home.  His hemoglobin on admission was 8.8, and has remained stable.  He is afebrile, hemodynamically stable.,ALLERGIES: , LISINOPRIL AND PENICILLIN.,MEDICATIONS ON DISCHARGE:,1.  Prednisone tapering dose 40 mg p.o. daily for three days, then 30 mg p.o. daily for three days, then 20 mg p.o. daily for three days, then 10 mg p.o. daily for three days, and 5 mg p.o. daily for two days.,2.  Levaquin 750 mg p.o. daily for 5 more days.,3.  Protonix 40 mg p.o. daily.,4.  The patient can continue other current home medications at home.,FOLLOWUP APPOINTMENTS:,1.  Recommend to follow up with Cardiology Dr. X's office in a week.,2.  The patient is recommended to see Hematology Dr. Y in the office for workup of anemia.,3.  Follow up with primary care physician's office tomorrow.,SPECIAL INSTRUCTIONS:,1.  If increasing shortness of breath, chest pain, fever, any acute symptoms to return to emergency room.,2.  Discussed about discharge plan, instructions with the patient by bedside.  He understands and agreed.  Also discussed discharge plan instructions with the patient's nurse.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="n">
-        <v>260</v>
+        <v>379</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Discharge Summary; short; discharge summary; diagnoses + symptoms + medications</t>
+          <t>Discharge Summary; medium; discharge summary; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>3963</v>
+        <v>3938</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
@@ -1193,21 +1185,21 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>higher</t>
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0.6243237150586114</v>
+        <v>0.7226104598737602</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; laboratory values; vital signs; procedures; past history; treatment plans; follow-up</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; procedures; imaging; past history; treatment plans; follow-up</t>
         </is>
       </c>
     </row>
     <row r="13" ht="110" customHeight="1">
       <c r="A13" s="2" t="n">
-        <v>3962</v>
+        <v>3885</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
@@ -1216,26 +1208,26 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Death Summary - 2 </t>
+          <t xml:space="preserve"> Speech Therapy - Discharge Summary - 1 </t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Cardiac arrest, severe congestive heart failure, acute on chronic respiratory failure, osteoporosis, and depression.</t>
+          <t xml:space="preserve"> The patient was referred to Medical Center's Outpatient Rehabilitation Department for skilled speech therapy to improve her functional communication skills and swallowing function and safety.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>FINAL DIAGNOSES:,1.  Cardiac arrest.,2.  Severe congestive heart failure.,3.  Acute on chronic respiratory failure.,4.  Osteoporosis.,5.  Depression.,HISTORY OF PRESENT ILLNESS: , This 92-year-old lady with history of depression and chronic low back pain, osteoporosis, and congestive heart failure, was diagnosed having pneumonia approximately for at least 10 days prior to admission.  In the ER, she was given oral antibiotics.  She also saw me few days before admission coming for a followup.  She was doing fairly well.  She was thought to have congestive heart failure and she was advised to continue with her diuretics.  For the last few days, the patient started to have anorexia, she did not eat well, and she did not drink well.  Her family could not take care of her.  So, she was brought to the emergency room, where she was found to have rapid heart rate with a sinus tachycardia around 112 to 130s.  The ________ was found to be dry.  She was given 1 L of IV fluids and she was subsequently admitted in the hospital for further management.,COURSE IN THE HOSPITAL: , The patient stayed in the telemetry.  The patient had significant shortness of breath secondary to congestive heart failure with bilateral basilar crackles.  She was continued on IV antibiotics and general IV hydration was started initially because of low blood pressure and low perfusion status.  On subsequently improved and stopped and Lasix was started; Dr. X, cardiologist was also placed.  The patient's family wanted her to be a DNR and DNI.  They were allowing us to treat her aggressively medically for pneumonia and congestive heart failure.  However, the patient became extremely weak, mostly unresponsive.  At this time, the patient's family wanted a Hospice consult, which was requested.  By the time the Hospice could evaluate her, the patient's condition got deteriorated, she went into more bradycardiac and hypertension and subsequently expired.  Please see the hospital notes for complete details.</t>
+          <t>HISTORY: , The patient is a 67-year-old female, was referred to Medical Center's Outpatient Rehabilitation Department for skilled speech therapy to improve her functional communication skills and swallowing function and safety.  At the onset of therapy, on 03/26/08, the patient was NPO with a G-tube and the initial speech and language evaluation revealed global aphasia with an aphasia quotient of 3.6/100 based on the Western Aphasia Battery.  Since the initial evaluation, the patient has attended 60 outpatient speech therapy sessions, which have focussed on her receptive communication, expressive language, multimodality communication skills, and swallowing function and safety.,SHORT-TERM GOALS:,1.  The patient met 3 out of 4 original short-term therapy goals, which were to complete a modified barium swallow study, which she did do and which revealed no aspiration.  At this time, the patient is eating and drinking and taking all medications by mouth; however, her G-tube is still present.  The patient was instructed to talk to the primary care physician about removal of her feeding tube.,2.  The patient will increase accuracy of yes-no responses to greater than 80% accuracy.  She did accomplish this goal.  The patient is also able to identify named objects with greater than 80% accuracy.,ADDITIONAL GOALS: , Following the completion of these goals, additional goals were established.  Based on reevaluation, the patient met 2 out of these 3 initial goals and she is currently able to read and understand simple sentences with greater than 90% accuracy independently and she is able to write 10 words related to basic wants and needs with greater than 80% accuracy independently.  The patient continues to have difficulty stating verbally, yes or no, to questions as well as accurately using head gestures and to respond to yes-no questions.  The patient continues to have marked difficulty with her expressive language abilities.  She is able to write simple words to help express her basic wants and needs.  She has made great strides; however, with her receptive communication, she is able to read words as well as short phrases and able to point to named objects and answer simple-to-moderate complex yes-no questions.  A reevaluation completed on 12/01/08, revealed an aphasia quotient of 26.4.  Once again, she made significant improvement and comprehension, but continues to have unintelligible speech.  An alternative communication device was discussed with the patient and her husband, but at this time, the patient does not want to utilize a communication device.  If, in the future, the patient continues to struggle with her expressive communication, an alternative augmented communication device would be a benefit to her.  Please reconsult at that time if and when the patient is ready to use a speech generating device.  The patient is discharged from my services at this time due to a plateau in her progress.  Numerous home activities were recommended to allow her to continue to make progress at home.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">discharge summary, bradycardiac, hypertension, hospice, congestive heart failure, cardiac arrest, respiratory failure, </t>
+          <t>discharge summary, communication skills, g-tube, aphasia, language evaluation, western aphasia battery, skilled speech therapy, swallowing function, speech therapy, therapy, swallowing, aspiration, speech, communication,</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>313</v>
+        <v>471</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -1244,15 +1236,15 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Discharge Summary; medium; other narrative/sectioned; diagnoses + symptoms + vital signs</t>
+          <t>Discharge Summary; medium; discharge summary; lower text complexity; medications + treatment plans</t>
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>3962</v>
+        <v>3885</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>other narrative/sectioned</t>
+          <t>discharge summary</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1261,17 +1253,17 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0.3609670874661858</v>
+        <v>0.3477795311091073</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; vital signs; past history; treatment plans; follow-up</t>
+          <t>medications; treatment plans</t>
         </is>
       </c>
     </row>
     <row r="14" ht="110" customHeight="1">
       <c r="A14" s="2" t="n">
-        <v>3911</v>
+        <v>3925</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -1280,26 +1272,22 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Lap Chole - Discharge Summary </t>
+          <t xml:space="preserve"> Discharge Summary - Urology &amp; Nephrology  </t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Laparoscopic cholecystectomy.  Acute cholecystitis, status post laparoscopic cholecystectomy, end-stage renal disease on hemodialysis, hyperlipidemia, hypertension, congestive heart failure, skin lymphoma 5 years ago, and hypothyroidism.</t>
+          <t xml:space="preserve"> Solitary left kidney with obstruction and hypertension and chronic renal insufficiency, plus a Pseudomonas urinary tract infection.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>PROCEDURE:,  Laparoscopic cholecystectomy.,DISCHARGE DIAGNOSES:,1.  Acute cholecystitis.,2.  Status post laparoscopic cholecystectomy.,3.  End-stage renal disease on hemodialysis.,4.  Hyperlipidemia.,5.  Hypertension.,6.  Congestive heart failure.,7.  Skin lymphoma 5 years ago.,8.  Hypothyroidism.,HOSPITAL COURSE: , This is a 78-year-old female with past medical condition includes hypertension, end-stage renal disease, hyperlipidemia, hypothyroidism, and skin lymphoma who had a left AV fistula done about 3 days ago by Dr. X and the patient went later on home, but started having epigastric pain and right upper quadrant pain and mid abdominal pain, some nauseated feeling, and then she could not handle the pain, so came to the emergency room, brought by the family.  The patient's initial assessment, the patient's vital signs were stable, showed temperature 97.9, pulse was 106, and blood pressure was 156/85.  EKG was not available and ultrasound of the abdomen showed there is a renal cyst about 2 cm.  There is sludge in the gallbladder wall versus a stone in the gallbladder wall.  Thickening of the gallbladder wall with positive Murphy sign.  She has a history of cholecystitis.  Urine shows positive glucose, but negative for nitrite and creatinine was 7.1, sodium 131, potassium was 5.2, and lipase and amylase were normal.  So, the patient admitted to the Med/Surg floor initially and the patient was started on IV fluid as well as low-dose IV antibiotic and 2-D echocardiogram and EKG also was ordered.  The patient also had history of CHF in the past and recently had some workup done.  The patient does not remember initially.  Surgical consult also requested and blood culture and urine culture also ordered.  The same day, the patient was seen by Dr. Y and the patient should need cholecystectomy, but the patient also needs dialysis and also needs to be cleared by the cardiologist, so the patient later on seen by Dr. Z and cleared the patient for the surgery with moderate risk and the patient underwent laparoscopic cholecystectomy.  The patient also seen by nephrologist and underwent dialysis.  The patient's white count went down 6.1, afebrile.  On postop day #1, the patient started eating and also walking.  The patient also had chronic bronchitis.  The patient was later on feeling fine, discussed with surgery.  The patient was then able to discharge to home and follow with the surgeon in about 3-5 days.  Discharged home with Synthroid 0.5 mg 1 tablet p.o. daily, Plavix 75 mg p.o. daily, folic acid 1 mg p.o. daily, Diovan 80 mg p.o. daily, Renagel 2 tablets 800 mg p.o. twice a day, Lasix 40 mg p.o.  2 tablets twice a day, lovastatin 20 mg p.o. daily, Coreg 3.125 mg p.o. twice a day, nebulizer therapy every 3 hours as needed, also Phenergan 25 mg p.o. q.8 hours for nausea and vomiting, Pepcid 20 mg p.o. daily, Vicodin 1 tablet p.o. q.6 hours p.r.n. as needed, and Levaquin 250 mg p.o. every other day for the next 5 days.  The patient also had Premarin that she was taking, advised to discontinue because of increased risk of heart disease and stroke explained to the patient.  Discharged home.</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">discharge summary, end-stage renal disease, lymphoma, cholecystitis, congestive heart failure, skin lymphoma, gallbladder wall, laparoscopic cholecystectomy </t>
-        </is>
-      </c>
+          <t>ADMITTING DIAGNOSES:,  Solitary left kidney with obstruction, and hypertension, and chronic renal insufficiency.,DISCHARGE DIAGNOSES: , Solitary left kidney with obstruction and hypertension and chronic renal insufficiency, plus a Pseudomonas urinary tract infection.,PROCEDURES: , Cystoscopy under anesthesia, ureteroscopy, an attempted tube placement, stent removal with retrograde pyelography, percutaneous tube placement, and nephrostomy by Radiology.,PERTINENT LABORATORIES: , Creatinine of 1.4.  During the hospitalization it was decreased to 0.8 and Pseudomonas urinary tract infection, positive culture sensitive to ceftazidime and ciprofloxacin.,HISTORY OF PRESENT ILLNESS:  ,The patient is a 3-1/2-year-old boy with a solitary kidney, had a ureteropelvic junction repair performed by Dr. Y, in the past, unfortunately, it was thought still be obstructed.  A stent was placed approximately 6 weeks ago after urethroscopic placement with some difficulty.  Plan was to remove the stent.  At the time of removal, we were unable to place another tube within the collecting system, and the patient was admitted for percutaneous nephrostomy placement.  He has had no recent cold or flu.  He has problems with hypertension for which he is on enalapril at home in addition to his Macrodantin prophylaxis.,PAST MEDICAL HISTORY: , The patient has no known allergies.  Multiple urinary tract infection, solitary kidney, and previous surgeries as mentioned above.,REVIEW OF SYSTEMS:,  A 14-organ system review of systems is negative except for the history of present illness.  He also has history of being a 34-week preemie twin.,ALLERGIES: , No known allergies.,FAMILY HISTORY: , Unremarkable without any bleeding or anesthetic problems.,SOCIAL HISTORY: , The patient lives at home with his parents, 2 brothers, and a sister.,IMMUNIZATIONS:,  Up-to-date.,MEDICATIONS: , On admission was Macrodantin, hydralazine, and enalapril.,PHYSICAL EXAMINATION:,GENERAL:  The patient is an active little boy.,HEENT:  The head and neck exam was grossly normal.  He had no oral, ocular, or nasal discharge.,LUNGS:  Exam was normal without wheezing.,HEART:  Without murmur or gallops.,ABDOMEN:  Soft, without mass or tenderness with a well-healed flank incision.,GU:  Uncircumcised male with bilaterally descended testes.,EXTREMITIES:  He has full range of motion in all 4 extremities.,SKIN:  Warm, pink, and dry.,NEUROLOGIC:  Grossly intact.,BACK:  He has normal back.  Normal gait.,HOSPITAL COURSE: , The patient was admitted to the hospital after inability to place a ureteral stent via ureteroscopy and cystoscopy.  He was made NPO.  He had a fever at first time with elevated creatinine.  He was also evaluated and treated by Dr. X, for fluid management, hypertensive management, and gave him some hydralazine and Lasix to improve his urine output, in addition to manage his blood pressure.  Once the percutaneous tube was placed, we found that his urine culture grew Pseudomonas, so he was kept on Fortaz, and was switched over to ciprofloxacin without difficulty.  He, otherwise, did well with continuing decrease his creatinine at the time of discharge to home.,The patient was discharged home in stable condition with ciprofloxacin, enalapril, and recommendation for followup in Urology in 1 to 2 weeks for the surgical correction in 2 to 3 weeks of repeat pyeloplasty or possible ureterocalicostomy.  The patient had draining nephrostomy tube without difficulty.,</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="n">
-        <v>505</v>
+        <v>493</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1308,11 +1296,11 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Discharge Summary; medium; discharge summary; diagnoses + symptoms + medications</t>
+          <t>Discharge Summary; medium; discharge summary; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>3911</v>
+        <v>3925</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -1321,21 +1309,21 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>higher</t>
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>0.5958633904418396</v>
+        <v>0.7965509467989179</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; laboratory values; vital signs; procedures; imaging; past history; surgery</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; procedures; past history; treatment plans; follow-up; surgery</t>
         </is>
       </c>
     </row>
     <row r="15" ht="110" customHeight="1">
       <c r="A15" s="2" t="n">
-        <v>3966</v>
+        <v>3911</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -1344,39 +1332,39 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Discharge Summary - 10 </t>
+          <t xml:space="preserve"> Lap Chole - Discharge Summary </t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Patient with a history of a Nissen fundoplication performed six years ago for gastric reflux. </t>
+          <t xml:space="preserve"> Laparoscopic cholecystectomy.  Acute cholecystitis, status post laparoscopic cholecystectomy, end-stage renal disease on hemodialysis, hyperlipidemia, hypertension, congestive heart failure, skin lymphoma 5 years ago, and hypothyroidism.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>ADMITTING DIAGNOSES:,  Hiatal hernia, gastroesophageal reflux disease reflux.,DISCHARGE DIAGNOSES:,  Hiatal hernia, gastroesophageal reflux disease reflux.,SECONDARY DIAGNOSIS: , Postoperative ileus.,PROCEDURES DONE: , Hiatal hernia repair and Nissen fundoplication revision.,BRIEF HISTORY: , The patient is an 18-year-old male who has had a history of a Nissen fundoplication performed six years ago for gastric reflux.  Approximately one year ago, he was involved in a motor vehicle accident and CT scan at that time showed that he had a hiatal hernia.  Over the past year, this has caused him an increasing number of problems, including chest pain when he eats, and shortness of breath after large meals.  He is also having reflux symptoms again.  He presents to us for repair of the hiatal hernia and revision of the Nissen fundoplication.,HOSPITAL COURSE: , Mr. A was admitted to the adolescent floor by Brenner Children's Hospital after his procedure.  He was stable at that time.  He did complain of some nausea.  However, he did not have any vomiting at that time.  He had an NG tube in and was n.p.o.  He also had a PCA for pain management as well as Toradol.  On postoperative day #1, he complained of not being able to urinate, so a Foley catheter was placed.  Over the next several days, his hospital course proceeded as follows.  He continued to complain of some nausea; however, he did not ever have any vomiting.  Eventually, the Foley catheter was discontinued and he had excellent urine output without any complications.  He ambulated frequently.  He remained n.p.o. for three days.  He also had the NG tube in during that time.  On postoperative day #4, he began to have some flatus, and the NG tube was discontinued.  He was advanced to a liquid diet and tolerated this without any complications.  At this time, he was still using the PCA for pain control.  However, he was using it much less frequently than on days #1 and #2 postoperatively.  After tolerating the full liquid diet without any complications, he was advanced to a soft diet and his pain medications were transitioned to p.o. medications rather than the PCA.  The PCA was discontinued.  He tolerated the soft diet without any complications and continued to have flatus frequently.  On postoperative day #6, it was determined that he was stable for discharge to home as he was taking p.o. without any complications.  His pain was well controlled with p.o. pain medications.  He was passing gas frequently, had excellent urine output, and was ambulating frequently without any issues.,DISCHARGE CONDITION:,  Stable.,DISPOSITION: , Discharged to home.,DISCHARGE INSTRUCTIONS: , The patient was discharged to home with instructions for maintaining a soft diet.  It was also recommended that he does not drink any soda postoperatively.  He is instructed to keep his incision site clean and dry and it was also recommended that he avoid any heavy lifting.  He will be able to attend school when it starts in a few weeks.  However, he is not going to be able to play football in the near future.  He was given prescription for pain medication upon discharge.  He is instructed to contact Pediatric Surgery if he has any fevers, any nausea and vomiting, any chest pain, any constipation, or any other concerns.</t>
+          <t>PROCEDURE:,  Laparoscopic cholecystectomy.,DISCHARGE DIAGNOSES:,1.  Acute cholecystitis.,2.  Status post laparoscopic cholecystectomy.,3.  End-stage renal disease on hemodialysis.,4.  Hyperlipidemia.,5.  Hypertension.,6.  Congestive heart failure.,7.  Skin lymphoma 5 years ago.,8.  Hypothyroidism.,HOSPITAL COURSE: , This is a 78-year-old female with past medical condition includes hypertension, end-stage renal disease, hyperlipidemia, hypothyroidism, and skin lymphoma who had a left AV fistula done about 3 days ago by Dr. X and the patient went later on home, but started having epigastric pain and right upper quadrant pain and mid abdominal pain, some nauseated feeling, and then she could not handle the pain, so came to the emergency room, brought by the family.  The patient's initial assessment, the patient's vital signs were stable, showed temperature 97.9, pulse was 106, and blood pressure was 156/85.  EKG was not available and ultrasound of the abdomen showed there is a renal cyst about 2 cm.  There is sludge in the gallbladder wall versus a stone in the gallbladder wall.  Thickening of the gallbladder wall with positive Murphy sign.  She has a history of cholecystitis.  Urine shows positive glucose, but negative for nitrite and creatinine was 7.1, sodium 131, potassium was 5.2, and lipase and amylase were normal.  So, the patient admitted to the Med/Surg floor initially and the patient was started on IV fluid as well as low-dose IV antibiotic and 2-D echocardiogram and EKG also was ordered.  The patient also had history of CHF in the past and recently had some workup done.  The patient does not remember initially.  Surgical consult also requested and blood culture and urine culture also ordered.  The same day, the patient was seen by Dr. Y and the patient should need cholecystectomy, but the patient also needs dialysis and also needs to be cleared by the cardiologist, so the patient later on seen by Dr. Z and cleared the patient for the surgery with moderate risk and the patient underwent laparoscopic cholecystectomy.  The patient also seen by nephrologist and underwent dialysis.  The patient's white count went down 6.1, afebrile.  On postop day #1, the patient started eating and also walking.  The patient also had chronic bronchitis.  The patient was later on feeling fine, discussed with surgery.  The patient was then able to discharge to home and follow with the surgeon in about 3-5 days.  Discharged home with Synthroid 0.5 mg 1 tablet p.o. daily, Plavix 75 mg p.o. daily, folic acid 1 mg p.o. daily, Diovan 80 mg p.o. daily, Renagel 2 tablets 800 mg p.o. twice a day, Lasix 40 mg p.o.  2 tablets twice a day, lovastatin 20 mg p.o. daily, Coreg 3.125 mg p.o. twice a day, nebulizer therapy every 3 hours as needed, also Phenergan 25 mg p.o. q.8 hours for nausea and vomiting, Pepcid 20 mg p.o. daily, Vicodin 1 tablet p.o. q.6 hours p.r.n. as needed, and Levaquin 250 mg p.o. every other day for the next 5 days.  The patient also had Premarin that she was taking, advised to discontinue because of increased risk of heart disease and stroke explained to the patient.  Discharged home.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>discharge summary,</t>
+          <t xml:space="preserve">discharge summary, end-stage renal disease, lymphoma, cholecystitis, congestive heart failure, skin lymphoma, gallbladder wall, laparoscopic cholecystectomy </t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>533</v>
+        <v>505</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Discharge Summary; long; discharge summary; diagnoses + symptoms + medications</t>
+          <t>Discharge Summary; medium; discharge summary; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J15" s="2" t="n">
-        <v>3966</v>
+        <v>3911</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
@@ -1389,17 +1377,17 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0.5607529305680794</v>
+        <v>0.5958633904418396</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; procedures; imaging; past history; treatment plans; surgery</t>
+          <t>diagnoses; symptoms; medications; laboratory values; vital signs; procedures; imaging; past history; surgery</t>
         </is>
       </c>
     </row>
     <row r="16" ht="110" customHeight="1">
       <c r="A16" s="2" t="n">
-        <v>3864</v>
+        <v>3846</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
@@ -1408,35 +1396,39 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Closed Head Injury </t>
+          <t xml:space="preserve"> Fall &amp; Laceration </t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Status post a high-speed motor vehicle accident in which patient was ejected from the vehicle.</t>
+          <t xml:space="preserve"> Patient running to catch a taxi and stumbled, fell and struck his face on the sidewalk.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>CHIEF COMPLAINT:,  Status post motor vehicle accident.,HISTORY OF PRESENT ILLNESS: , The patient is a 17-year-old white male who is status post a high-speed motor vehicle accident in which he was ejected from the vehicle.  He denies loss of consciousness, although the EMT people report that he did have loss of consciousness.  The patient was stable en route.  Upon arrival, he complained of headache.,PAST MEDICAL HISTORY:,  Medical:  None.  Surgical:  None.,REVIEW OF SYSTEMS: , CARDIAC:  No history.  PULMONARY:  Some morning cough.  (Patient is a smoker.),MEDICATIONS:,  None.,ALLERGIES:,  ALLERGIC TO PENICILLIN, CAUSES SKIN RASH.,PHYSICAL EXAMINATION:,VITAL SIGNS:  Blood pressure 120/80, pulse 82, respirations 20, temperature 36.8°.,HEENT:  Contusion over right occipital area.  Tympanic membranes benign.,NECK:  Nontender.,CHEST:  Atraumatic, nontender.,LUNGS:  Clear to auscultation and percussion.,ABDOMEN:  Flat, soft, and nontender.,BACK:  Atraumatic, nontender.,PELVIS:  Stable,EXTREMITIES:  Contusion over right forearm.  No bone deformity or crepitus.,RECTAL:  Normal sphincter tone; guaiac negative.,NEUROLOGIC:  Glasgow coma scale 15.  Pupils equal, round, reactive to light.  Patient moves all 4 extremities without focal deficit.,LABORATORY DATA: , Serial hematocrits 42.4, and 40.4.  White blood count 6.3.  Ethanol:  None.  Amylase 66.  Urinalysis normal.  PT 12.6, PTT 29.  Chem-7 panel within normal limits.,X-rays of cervical spine and lumbosacral spine within normal limits.  X-rays of pelvis and chest within normal limits.,ASSESSMENT:,1.  Closed head injury.,2.  Rule out intra-abdominal injury.,PLAN:,  The patient will be admitted to the trauma surgery service for continued evaluation and treatment for closed head injury as well as possible intra-abdominal injury.</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr"/>
+          <t>CC:,  Fall and laceration.,HPI: , Mr. B is a 42-year-old man who was running to catch a taxi when he stumbled, fell and struck his face on the sidewalk.  He denies loss of consciousness but says he was dazed for a while after it happened.  He complains of pain over the chin and right forehead where he has abrasions.  He denies neck pain, back pain, extremity pain or pain in the abdomen.,PMH: , Hypertension.,MEDS:,  None.,ROS: , As above.  Otherwise negative.,PHYSICAL EXAM: , This is a gentleman in full C-spine precautions on a backboard brought by EMS.  He is in no apparent distress.  ,Vital Signs:  BP 165/95 HR 80 RR 12 Temp 98.4 SpO2 95% ,HEENT:  No palpable step offs, there is blood over the right fronto-parietal area where there is a small 1cm laceration and surrounding abrasion.  Also, 2 cm laceration over the base of the chin without communication to the oro-pharynx.  No other trauma noted.  No septal hematoma.  No other facial bony tenderness.  ,Neck:  Nontender ,Chest:  Breathing comfortably; equal breath sounds.  ,Heart:  Regular rhythm.,Abd:  Benign.,Ext:  No tenderness or deformity; pulses are equal throughout; good cap refill ,Neuro:  Awake and alert; slight slurring of speech and cognitive slowing consistent with alcohol; moves all extremities; cranial nerves normal.  ,COURSE IN THE ED:,  Patient arrived and was placed on monitors.  An IV had been placed in the field and labs were drawn.  X-rays of the C spine show no fracture and I've removed the C-collar.  The lacerations were explored and no foreign body found.  They were irrigated and closed with simple interrupted sutures.  Labs showed normal CBC, Chem-7, and U/A except there was moderate protein in the urine.  The blood alcohol returned at 0.146.  A banana bag is ordered and his care will be turned over to Dr. G for further evaluation and care.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>emergency room reports, loss of consciousness, laceration, fall, course in the ed, placed on monitors, fell and struck, abrasions,</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="n">
-        <v>232</v>
+        <v>302</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Emergency Room Reports; short; other narrative/sectioned; diagnoses + symptoms + medications</t>
+          <t>Emergency Room Reports; medium; other narrative/sectioned; lower text complexity; symptoms + laboratory values + vital signs</t>
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>3864</v>
+        <v>3846</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
@@ -1445,21 +1437,21 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>higher</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>0.6975879170423805</v>
+        <v>0.36547565374211</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; imaging; past history; treatment plans; surgery; assessment/plan</t>
+          <t>symptoms; laboratory values; vital signs; imaging</t>
         </is>
       </c>
     </row>
     <row r="17" ht="110" customHeight="1">
       <c r="A17" s="2" t="n">
-        <v>3838</v>
+        <v>3826</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
@@ -1468,22 +1460,26 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Head Injury </t>
+          <t xml:space="preserve"> Mastoiditis - Discharge Summary </t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Head injury, anxiety, and hypertensive emergency.</t>
+          <t xml:space="preserve"> Suspected mastoiditis ruled out, right acute otitis media, and severe ear pain resolving.  The patient is an 11-year-old male who was admitted from the ER after a CT scan suggested that the child had mastoiditis.  </t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>CHIEF COMPLAINT:,  Head injury.,HISTORY: , This 16-year-old female presents to Children's Hospital via paramedic ambulance with a complaint at approximately 6 p.m. while she was at band practice using her flag device.  She struck herself in the head with the flag.  There was no loss of consciousness.  She did feel dizzy.  She complained of a headache.  She was able to walk.  She continued to participate in her flag practice.  She got dizzier.  She sat down for a while and walked and during the second period of walking, she had some episodes of diplopia, felt that she might faint and was assisted to the ground and was transported via paramedic ambulance to Children's Hospital for further evaluation.,PAST MEDICAL HISTORY: , Hypertension.,ALLERGIES:,  DENIED TO ME; HOWEVER, IT IS NOTED BEFORE SEVERAL ACCORDING TO MEDITECH.,CURRENT MEDICATIONS: , Enalapril.,PAST SURGICAL HISTORY: , She had some kind of an abdominal obstruction as an infant.,SOCIAL HISTORY: , She is here with mother and father who lives at home.  There is no smoking at home.  There is second-hand smoke exposure.,FAMILY HISTORY:  ,No noted family history of infectious disease exposure.,IMMUNIZATIONS:,  She is up-to-date on her shots, otherwise negative.,REVIEW OF SYSTEMS:  ,On the 10-plus systems reviewed with the section of those noted on the template.,PHYSICAL EXAMINATION:,VITAL SIGNS:  Her temperature 100 degrees, pulse 86, respirations 20, and her initial blood pressure 166/116, and a weight of 55.8 kg.,GENERAL:  She is supine awake, alert, cooperative, and active child.,HEENT:  Head atraumatic, normocephalic.  Pupils equal, round, reactive to light.  Extraocular motions intact and conjugate.  Clear TMs, nose and oropharynx.  Moist oral mucosa without noted lesions.,NECK:  Supple, full painless nontender range motion.,CHEST:  Clear to auscultation, equal, stable to palpation.,HEART:  Regular without rubs or murmurs.,ABDOMEN:  No abdominal bruits are heard.,EXTREMITIES:  Equal femoral pulses are appreciated.  Equal radial and dorsalis pedis pulses are appreciated.  He moves all extremities without difficulty.  Nontender.  No deformity.  No swelling.,SKIN:  There was no significant bruising, lesions or rash about her abdomen.  No significant bruising, lesions or rash.,NEUROLOGIC:  Symmetric face and extremity motion.  Ambulates without difficulty.  She is awake, alert, and appropriate.,MEDICAL DECISION MAKING:,  The differential entertained includes head injury, anxiety, and hypertensive emergency.  She is evaluated in the emergency department with serial blood pressure examinations, which are noted to return to a more baseline state for her 130s/90s.  Her laboratory data shows a mildly elevated creatinine of 1.3.  Urine is within normal.  Urinalysis showing no signs of infection.  Head CT read by staff has no significant intracranial pathology.  No mass shift, bleed or fracture per Dr. X.  A 12-lead EKG reviewed preliminarily by myself noting normal sinus rhythm, normal axis rates of 90.  No significant ST-T wave changes.  No significant change from previous 09/2007 EKG.  Her headache has resolved.  She is feeling better.  I spoke with Dr. X at 0206 hours consulting Nephrology regarding this patient's presentation with the plan for home.  Follow up with her regular doctor.  Blood pressures have normalized for her.  She should return to emergency department on concern.  They are to call the family to Nephrology Clinic next week for optimization of her blood pressure control with a working diagnosis of head injury, hypertension, and syncope.</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr"/>
+          <t>DISCHARGE DIAGNOSES:  ,1.  Suspected mastoiditis ruled out.,2.  Right acute otitis media.,3.  Severe ear pain resolving.,HISTORY OF PRESENT ILLNESS: , The patient is an 11-year-old male who was admitted from the ER after a CT scan suggested that the child had mastoiditis.  The child has had very severe ear pain and blood draining from the right ear.  The child had a temperature maximum of 101.4 in the ER.  The patient was admitted and started on IV Unasyn, which he tolerated well and required Morphine and Vicodin for pain control.  In the first 12 hours after admission, the patient's pain decreased and also swelling of his cervical area decreased.  The patient was evaluated by Dr. X from the ENT while in house.  After reviewing the CT scan, it was felt that the CT scan was not consistent with mastoiditis.  The child was continued on IV fluid and narcotics for pain as well as Unasyn until the time of discharge.  At the time of discharge his pain is markedly decreased about 2/10 and swelling in the area has improved.  The patient is also able to take p.o. well.,DISCHARGE PHYSICAL EXAMINATION:,GENERAL:  The patient is alert, in no respiratory distress.,VITAL SIGNS:  His temperature is 97.6, heart rate 83, blood pressure 105/57, respiratory rate 16 on room air.,HEENT:  Right ear shows no redness.  The area behind his ear is nontender.  There is a large posterior chains node that is nontender and the swelling in this area has decreased markedly.,NECK:  Supple.,CHEST:  Clear breath sounds.,CARDIAC:  Normal S1, S2 without murmur.,ABDOMEN:  Soft.  There is no hepatosplenomegaly or tenderness.,SKIN:  Warm and well perfused.,DISCHARGE WEIGHT: , 38.7 kg.,DISCHARGE CONDITION: , Good.,DISCHARGE DIET:,  Regular as tolerated.,DISCHARGE MEDICATIONS:  ,1.  Ciprodex Otic Solution in the right ear twice daily.,2.  Augmentin 500 mg three times daily x10 days.,FOLLOW UP:  ,1.  Dr. Y in one week (ENT).,2.  The primary care physician in 2 to 3 days.,TIME SPENT: , Approximate discharge time is 28 minutes.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
       <c r="G17" s="2" t="n">
-        <v>519</v>
+        <v>318</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1492,15 +1488,15 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Emergency Room Reports; medium; other narrative/sectioned; diagnoses + symptoms + medications</t>
+          <t>Emergency Room Reports; medium; discharge summary; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J17" s="2" t="n">
-        <v>3838</v>
+        <v>3826</v>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>other narrative/sectioned</t>
+          <t>discharge summary</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1509,17 +1505,17 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>0.8070897204688909</v>
+        <v>0.631311992786294</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; imaging; past history; treatment plans; follow-up; surgery</t>
+          <t>diagnoses; symptoms; medications; vital signs; imaging; past history; follow-up</t>
         </is>
       </c>
     </row>
     <row r="18" ht="110" customHeight="1">
       <c r="A18" s="2" t="n">
-        <v>3818</v>
+        <v>3860</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
@@ -1528,39 +1524,39 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Shone complex </t>
+          <t xml:space="preserve"> Consult/ER Report - OB/GYN </t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Complete heart block with pacemaker malfunction and  a history of Shone complex.</t>
+          <t xml:space="preserve"> A female with unknown gestational age who presents to the ED after a suicide attempt.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>HISTORY AND PHYSICAL:  ,The patient is a 13-year-old, who has a history of Shone complex and has a complete heart block.  He is on the pacemaker.  He had a coarctation of the aorta and that was repaired when he was an infant.  He was followed in our Cardiology Clinic here and has been doing well.  However last night, he was sleeping, and he states he felt as if he has having a dream, and there was thunder in this dream, which woke him up.  He then felt that his defibrillator was going off and this has continued and feels like his heart rate is not normal.  Thus, his dad put him in the car and transported him here.  He has been evaluated here.  He had some scar tissue at one point when the internal pacemaker was not working properly and had to have that replaced.  It was 2 a.m. when he woke, and again, he was brought here by private vehicle.  He was well prior to going to bed.  No cough, cold, runny nose, fever.  No trauma has been noted.,PAST MEDICAL HISTORY:,  Shone complex, pacemaker dependent.,MEDICATIONS: , He is on no medications at this time.,ALLERGIES:,  He has no allergies.,IMMUNIZATIONS:,  Up to date.,SOCIAL HISTORY: , He lives with his parents.,FAMILY HISTORY: , Negative.,REVIEW OF SYSTEM: , Twelve asked, all negative, except as noted above.,PHYSICAL EXAMINATION:,GENERAL:  This is an awake, alert male, who appears to be in mild distress.,HEENT:  Pupils are equal, round, and reactive to light.  Extraocular movements are intact.  His TMs are clear.  His nares are clear.  The mucous membranes are pink and moist.  Throat is clear.,NECK:  Supple without lymphadenopathy or masses.  Trachea is midline.,LUNGS:  Clear.,HEART:  Shows bradycardia at 53.  He has good distal pulses.,ABDOMEN:  Soft, nontender.  Positive bowel sounds.  No guarding, no rebound.  No rashes are seen.,HOSPITAL COURSE:,  Initial blood pressure is 164/90.  He was moved in room 1.  He was placed on nasal cannula.  Pulse ox was 100%, which is normal.  We placed him on a monitor.  We did an EKG; it has not appear to be capturing his pacemaker at this time.  Shortly after the patient's arrival, the Medtronic technician came and worked out his pacemaker.  Medtronic representative informed me that the lead that he has in place has been recalled because it has been prone to microfractures, oversensing, and automatic defibrillation.  As noted, he was transferred to room 1, placed on a monitor, pulse ox.  An IV was placed.  A standard blood work was sent.  A chest x-ray was done showing normal heart size, lead appeared to be in placed.  There was no evidence of pulmonary edema.  His pacemaker did not appear to be capturing.  We placed him on transthoracic leads.  However, it is difficult to get good placement with these because of the area where his pacemaker was placed.  The Medtronic technician initially turned off his defibrillation mode and turned down his sensor.  However, we could not get our transthoracic pacer to capture his heart.  When the Medtronic representative turned off the pacemaker, the heart rate seemed to drop into the 40s.  The patient appeared to be in pain.  We placed it back on a rate of 60 at that time.  He has remained in sinus bradycardia, but no evidence of ectopic beats.  No widening of his QRS complex.  I spoke with Cardiology.  Cardiology service has come in, has evaluated him at bedside with me.  Again, we turned up the transthoracic pacer, but it is again not seem to be picking up, and his heart rate is still going with the Medtronic's internal pacemaker.  So with the ICU physician on call, Dr. X, he has agreed with taking this young man to the ICU.,An hour after presentation here, the ICU was ready for bed.  I accompanied the patient up to the ICU.  He remained awake and alert.  Initially, he was complaining of a lot of chest pain.  Once the defibrillator was turned off, he had no more pain.  He was transported to the Pediatrics PICU and delivered in stable condition.,LABORATORY DATA: , CBC was normal.  Chem-20 was normal as well.,IMPRESSION:  ,Complete heart block with pacemaker malfunction.,PLAN:  ,He is admitted to the ICU.,TIME SEEN: , Critical care time outside billable procedures was 45 minutes with this patient.  I should note that a 12-lead EKG was done here showing sinus bradycardia, normal intervals otherwise.</t>
+          <t>The patient states that she has abnormal menstrual periods and cannot remember the first day of her last normal menstrual period.  She states that she had spotting for three months daily until approximately two weeks ago, when she believes that she passed a fetus.  She states that upon removal of a tampon, she saw a tadpole like structure and believed it to be a fetus.  However, she states she did not know that she was pregnant at this time.  She denies any abdominal pain or vaginal bleeding.  She states that the pregnancy is unplanned; however, she would desire to continue the pregnancy.,PAST MEDICAL HISTORY:  Diabetes mellitus which resolved after weight loss associated with gastric bypass surgery.,PAST SURGICAL HISTORY:,1.  Gastric bypass.,2.  Bilateral carpal tunnel release.,3.  Laparoscopic cholecystectomy.,4.  Hernia repair after gastric bypass surgery.,5.  Thoracotomy.,6.  Knee surgery.,MEDICATIONS:,1.  Lexapro 10 mg daily.,2.  Tramadol 50 mg tablets two by mouth four times a day.,3.  Ambien 10 mg tablets one by mouth at bedtime.,ALLERGIES:  AMOXICILLIN CAUSES THROAT SWELLING.  AVELOX CAUSES IV SITE SWELLING.,SOCIAL HISTORY:  The patient denies tobacco, ethanol, or drug use.  She is currently separated from her partner who is the father of her 21-month-old daughter.  She currently lives with her parents in Greenville.  However, she was visiting the estranged boyfriend in Wilkesboro, this week.,GYN HISTORY:  The patient denies history of abnormal Pap smears or STDs.,OBSTETRICAL HISTORY:  Gravida 1 was a term spontaneous vaginal delivery, complicated only by increased blood pressures at the time of delivery.  Gravida 2 is current.,REVIEW OF SYSTEMS:  The 14-point review of systems was negative with the exception as noted in the HPI.,PHYSICAL EXAMINATION:,VITAL SIGNS:  Blood pressure 134/45, pulse 130, respirations 28.  Oxygen saturation 100%.,GENERAL:  Patient lying quietly on a stretcher.  No acute distress.,HEENT:  Normocephalic, atraumatic.  Slightly dry mucous membranes.,CARDIOVASCULAR EXAM:  Regular rate and rhythm with tachycardia.,CHEST:  Clear to auscultation bilaterally.,ABDOMEN:  Soft, nontender, nondistended with positive bowel sounds.  No rebound or guarding.,SKIN:  Normal turgor.  No jaundice.  No rashes noted.,EXTREMITIES:  No clubbing, cyanosis, or edema.,NEUROLOGIC:  Cranial nerves II through XII grossly intact.,PSYCHIATRIC:  Flat affect.  Normal verbal response.,ASSESSMENT AND PLAN:  A 34-year-old Caucasian female, gravida 2 para 1-0-0-1, at unknown gestation who presents after suicide attempt.,1.  Given the substances taken, medications are unlikely to affect the development of the fetus.  There have been no reported human anomalies associated with Ambien or tramadol use.  There is, however, a 4% risk of congenital anomalies in the general population.,2.  Recommend quantitative HCG and transvaginal ultrasound for pregnancy dating.,3.  Recommend prenatal vitamins.,4.  The patient to follow up as an outpatient for routine prenatal care.,</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="n">
-        <v>717</v>
+        <v>418</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Emergency Room Reports; long; history and physical; diagnoses + symptoms + medications</t>
+          <t>Emergency Room Reports; medium; consultation; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J18" s="2" t="n">
-        <v>3818</v>
+        <v>3860</v>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>history and physical</t>
+          <t>consultation</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1569,17 +1565,17 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>0.7195671776375112</v>
+        <v>0.8509355275022543</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; imaging; past history; treatment plans; follow-up; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="19" ht="110" customHeight="1">
       <c r="A19" s="2" t="n">
-        <v>3859</v>
+        <v>3847</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
@@ -1588,58 +1584,62 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Consult - ICU Management </t>
+          <t xml:space="preserve"> Fiberoptic Bronchoscopy with Lavage </t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Consultation for ICU management for a patient with possible portal vein and superior mesenteric vein thrombus leading to mesenteric ischemia.</t>
+          <t xml:space="preserve"> Emergent fiberoptic bronchoscopy with lavage.   Status post multiple trauma/motor vehicle accident.  Acute respiratory failure.  Acute respiratory distress/ventilator asynchrony.  Hypoxemia.  Complete atelectasis of left lung.  Clots partially obstructing the endotracheal tube and completely obstructing the entire left main stem and entire left bronchial system.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>REASON FOR CONSULTATION: , ICU management.,HISTORY OF PRESENT ILLNESS: , The patient is a 43-year-old gentleman who presented from an outside hospital with complaints of right upper quadrant pain in the abdomen, which revealed possible portal vein and superior mesenteric vein thrombus leading to mesenteric ischemia.  The patient was transferred to the ABCD Hospital where he had a weeklong course with progressive improvement in his status after aggressive care including intubation, fluid resuscitation, and watchful waiting.  The patient clinically improved; however, his white count remained elevated with the intermittent fevers prompting a CT scan.  Repeat CT scan showed a loculated area of ischemic bowel with perforation in the left upper abdomen.  The patient was taken emergently to the operating room last night by the General Surgery Service where proximal half of the jejunum was noted to be liquified with 3 perforations.  This section of small bowel was resected, and a wound VAC placed for damage control.  Plan was to return the patient to the Operating Room tomorrow for further exploration and possible re-anastomosis of the bowel.  The patient is currently intubated, sedated, and on pressors for septic shock and in the down ICU.,PAST MEDICAL HISTORY:,  Prior to coming into the hospital for this current episode, the patient had hypertension, diabetes, and GERD.,PAST SURGICAL HISTORY:,  Included a cardiac cath with no interventions taken.,HOME MEDICATIONS:,  Include Lantus insulin as well as oral hypoglycemics.,CURRENT MEDS:,  Include Levophed, Ativan, fentanyl drips, cefepime, Flagyl, fluconazole, and vancomycin.  Nexium, Synthroid, hydrocortisone, and Angiomax, which is currently on hold.,REVIEW OF SYSTEMS:,  Unable to be obtained secondary to the patient's intubated and sedated status.,ALLERGIES: , None.,FAMILY HISTORY:,  Includes diabetes on his father side of the family.  No other information is provided.,SOCIAL HISTORY:,  Includes tobacco use as well as alcohol use.,PHYSICAL EXAMINATION:,GENERAL: The patient is currently intubated and sedated on Levophed drip.,VITAL SIGNS: Temperature is 100.6, systolic is 110/60 with MAP of 80, and heart rate is 120, sinus rhythm.,NEUROLOGIC: Neurologically, he is sedated, on Ativan with fentanyl drip as well.  He does arouse with suctioning, but is unable to open his eyes to commands.,HEAD AND NECK EXAMINATION: His pupils are equal, round, reactive, and constricted.  He has no scleral icterus.  His mucous membranes are pink, but dry.  He has an EG tube, which is currently 24-cm at the lip.  He has a left-sided subclavian vein catheter, triple lumen.,NECK: His neck is without masses or lymphadenopathy or JVD.,CHEST: Chest has diminished breath sounds bilaterally.,ABDOMEN: Abdomen is soft, but distended with a wound VAC in place.  Groins demonstrate a left-sided femoral outline.,EXTREMITIES: His bilateral upper extremities are edematous as well as his bilateral lower extremities; however, his right is more than it is in the left.  His toes are cool, and pulses are not palpable.,LABORATORY EXAMINATION: , Laboratory examination reveals an ABG of 7.34, CO2 of 30, O2 of 108, base excess of -8, bicarb of 16.1, sodium of 144, potassium of 6.5, chloride of 122, CO2 18, BUN 43, creatinine 2.0, glucose 172, calcium 6.6, phosphorus 1.1, mag 1.8, albumin is 1.6, cortisone level random is 22.  After stimulation with cosyntropin, they were still 22 and then 21 at 30 and 60 minutes respectively.  LFTs are all normal.  Amylase and lipase are normal.  Triglycerides are 73, INR is 2.2, PTT is 48.3, white count 20.7, hemoglobin 9.6, and platelets of 211.  UA was done, which also shows a specific gravity of 1.047, 1+ protein, trace glucose, large amount of blood, and many bacteria.  Chest x-rays performed and show the tip of the EG tube at level of the carina with some right upper lobe congestion, but otherwise clear costophrenic angles.  Tip of the left subclavian vein catheter is appropriate, and there is no pneumothorax noted.,ASSESSMENT AND PLAN:,  This is a 43-year-old gentleman who is acutely ill, in critical condition with mesenteric ischemia secondary to visceral venous occlusion.  He is status post small bowel resection.  We plan to go back to operating room tomorrow for further debridement and possible closure.  Neurologically, the patient initially had question of encephalopathy while in the hospital secondary to slow awakening after previous intubation; however, he did clear eventually, and was able to follow commands.  I did not suspect any sort of pathologic abnormality of his neurologic status as he has further CT scan of his brain, which was normal.  Currently, we will keep him sedated and on fentanyl drip to ease pain and facilitate ventilation on the respirator.  We will form daily sedation holidays to assess his neurologic status and avoid over sedating with Ativan.,1.  Cardiovascular.  The patient currently is in septic shock requiring vasopressors maintained on MAP greater than 70.  We will continue to try to wean the vasopressin after continued volume loading, also place SvO2 catheter to assess his oxygen delivery and consumption given his state of shock.  Currently, his rhythm is of sinus tachycardia, I do not suspect AFib or any other arrhythmia at this time.  If he does not improve as expected with volume resuscitation and with resolution of his sepsis, we will obtain an echocardiogram to assess his cardiac function.  Once he is off the vasopressors, we will try low-dose beta blockade as tolerated to reduce his rate.,2.  Pulmonology.  Currently, the patient is on full vent support with a rate of 20, tidal volume of 550, pressure support of 10, PEEP of 6, and FiO2 of 60.  We will wean his FiO2 as tolerated to keep his saturation greater than 90% and wean his PEEP as tolerated to reduce preload compromise.  We will keep the head of bed elevated and start chlorhexidine as swish and swallow for VAP prevention.,3.  Gastrointestinal.  The patient has known mesenteric venous occlusion secondary to the thrombus formation at the portal vein as well as the SMV.  He is status post immediate resection of jejunum leaving a blind proximal jejunum and blind distal jejunum.  We will maintain NG tube as he has a blind stump there, and we will preclude any further administration of any meds through this NG tube.  I will keep him on GI prophylaxis as he is intubated.  We will currently hold his TPN as he is undergoing a large amount of volume changes as well as he is undergoing electrolyte changes.  He will have a long-term TPN after this acute episode.  His LFTs are all normal currently.  Once he is postop tomorrow, we will restart the Angiomax for his venous occlusion.,4.  Renal.  The patient currently is in the acute renal insufficiency with anuria and an increase in his creatinine as well as his potassium.  His critical hyperkalemia which is requiring dosing of dextrose insulin, bicarb, and calcium; we will recheck his potassium levels after this cocktail.  He currently is started to make more urine since being volume resuscitated with Hespan as well as bicarb drip.  Hopefully given his increased urine output, he will start to eliminate some potassium and will not need dialysis.  We will re-consult Nephrology at this time.,5.  Endocrine.  The patient has adrenal insufficiency based on lack of stem to cosyntropin.  We will start hydrocortisone 50 q.6h.,6.  Infectious Disease.  Currently, the patient is on broad-spectrum antibiotic prophylaxis imperially.  Given his bowel ischemia, we will continue these, and appreciate ID service's input.,7.  Hematology.  Hematologically, the patient has a hypercoagulable syndrome, also had HIT secondary to his heparin administration.  We will restart the Angiomax once he is back from the OR tomorrow.  Currently, his INR is 2.2.  Therefore, he should be covered at the moment.  Appreciate the Hematology's input in this matter.,Please note the total critical care time spent at the bedside excluding central line placement was 1 hour.</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr"/>
+          <t>PREOPERATIVE DIAGNOSES:,1.  Status post multiple trauma/motor vehicle accident.,2.  Acute respiratory failure.,3.  Acute respiratory distress/ventilator asynchrony.,4.  Hypoxemia.,5.  Complete atelectasis of left lung.,POSTOPERATIVE DIAGNOSES:,1.  Status post multiple trauma/motor vehicle accident.,2.  Acute respiratory failure.,3.  Acute respiratory distress/ventilator asynchrony.,4.  Hypoxemia.,5.  Complete atelectasis of left lung.,6.  Clots partially obstructing the endotracheal tube and completely obstructing the entire left main stem and entire left bronchial system.,PROCEDURE PERFORMED: ,Emergent fiberoptic plus bronchoscopy with lavage.,LOCATION OF PROCEDURE:  ,ICU.  Room #164.,ANESTHESIA/SEDATION:,  Propofol drip, Brevital 75 mg, morphine 5 mg, and Versed 8 mg.,HISTORY,:  The patient is a 44-year-old male who was admitted to ABCD Hospital on 09/04/03 status post MVA with multiple trauma and subsequently diagnosed with multiple spine fractures as well as bilateral pulmonary contusions, requiring ventilatory assistance.  The patient was noted with acute respiratory distress on ventilator support with both ventilator asynchrony and progressive desaturation.  Chest x-ray as noted above revealed complete atelectasis of the left lung.  The patient was subsequently sedated and received one dose of paralytic as noted above followed by emergent fiberoptic flexible bronchoscopy.,PROCEDURE DETAIL,:  A bronchoscope was inserted through the oroendotracheal tube, which was partially obstructed with blood clots.  These were lavaged with several aliquots of normal saline until cleared.  The bronchoscope required removal because the tissue/clots were obstructing the bronchoscope.  The bronchoscope was reinserted on several occasions until cleared and advanced to the main carina.  The endotracheal tube was noted to be in good position.  The bronchoscope was advanced through the distal trachea.  There was a white tissue completely obstructing the left main stem at the carina.  The bronchoscope was advanced to this region and several aliquots of normal saline lavage were instilled and suctioned.  Again this partially obstructed the bronchoscope requiring several times removing the bronchoscope to clear the lumen.  The bronchoscope subsequently was advanced into the left mainstem and subsequently left upper and lower lobes.  There was diffuse mucus impactions/tissue as well as intermittent clots.  There was no evidence of any active bleeding noted.  Bronchoscope was adjusted and the left lung lavaged until no evidence of any endobronchial obstruction is noted.  Bronchoscope was then withdrawn to the main carina and advanced into the right bronchial system.  There is no plugging or obstruction of the right bronchial system.  The bronchoscope was then withdrawn to the main carina and slowly withdrawn as the position of endotracheal tube was verified, approximately 4 cm above the main carina.  The bronchoscope was then completely withdrawn as the patient was maintained on ventilator support during and postprocedure.  Throughout the procedure, pulse oximetry was greater than 95% throughout.  There is no hemodynamic instability or variability noted during the procedure.  Postprocedure chest x-ray is pending at this time.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">emergency room reports, multiple trauma, motor vehicle accident, acute respiratory failure, acute respiratory distress, ventilator asynchrony, hypoxemia, atelectasis, bronchoscopy, lavage, fiberoptic bronchoscopy, endotracheal tube, acute respiratory, asynchrony, bronchoscope, fiberoptic, endotracheal, bronchial, ventilatory, tube, respiratory, </t>
+        </is>
+      </c>
       <c r="G19" s="2" t="n">
-        <v>1258</v>
+        <v>440</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Emergency Room Reports; long; consultation; diagnoses + symptoms + medications</t>
+          <t>Emergency Room Reports; medium; procedure/operative; middle text complexity; diagnoses + medications + vital signs</t>
         </is>
       </c>
       <c r="J19" s="2" t="n">
-        <v>3859</v>
+        <v>3847</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>consultation</t>
+          <t>procedure/operative</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>higher</t>
+          <t>middle</t>
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0.9758791704238052</v>
+        <v>0.5204012623985572</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; follow-up; surgery; assessment/plan</t>
+          <t>diagnoses; medications; vital signs; procedures; imaging</t>
         </is>
       </c>
     </row>
     <row r="20" ht="110" customHeight="1">
       <c r="A20" s="2" t="n">
-        <v>3800</v>
+        <v>3808</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
@@ -1648,62 +1648,58 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Diabetes Mellitus - SOAP Note - 2 </t>
+          <t xml:space="preserve"> Acute Cystitis &amp; Diabetes Type II </t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Patient today with ongoing issues with diabetic control.</t>
+          <t xml:space="preserve"> The patient complaining of abdominal pain, has a long-standing history of diabetes treated with Micronase daily.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>SUBJECTIVE:,  I am asked to see the patient today with ongoing issues around her diabetic control.  We have been fairly aggressively, downwardly adjusting her insulins, both the Lantus insulin, which we had been giving at night as well as her sliding scale Humalog insulin prior to meals.  Despite frequent decreases in her insulin regimen, she continues to have somewhat low blood glucoses, most notably in the morning when the glucoses have been in the 70s despite decreasing her Lantus insulin from around 84 units down to 60 units, which is a considerable change.  What I cannot explain is why her glucoses have not really climbed at all despite the decrease in insulin.  The staff reports to me that her appetite is good and that she is eating as well as ever.  I talked to Anna today.  She feels a little fatigued.  Otherwise, she is doing well.,PHYSICAL EXAMINATION:  ,Vitals as in the chart.  The patient is a pleasant and cooperative.  She is in no apparent distress.,ASSESSMENT AND PLAN: , Diabetes, still with some problematic low blood glucoses, most notably in the morning.  To address this situation, I am going to hold her Lantus insulin tonight and decrease and then change the administration time to in the morning.  She will get 55 units in the morning.  I am also decreasing once again her Humalog sliding scale insulin prior to meals.  I will review the blood glucoses again next week.,</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>endocrinology, diabetic control, insulin prior to meals, low blood glucoses, sliding scale, lantus insulin, diabetes, mellitus, lantus, glucoses,</t>
-        </is>
-      </c>
+          <t>HISTORY OF PRESENT ILLNESS: , The patient is a 45-year-old male complaining of abdominal pain.  The patient also has a long-standing history of diabetes which is treated with Micronase daily.,PAST MEDICAL HISTORY: , There is no significant past medical history noted today.,PHYSICAL EXAMINATION:,HEENT:  Patient denies ear abnormalities, nose abnormalities and throat abnormalities.,Cardio:  Patient has history of elevated cholesterol, but does not have ASHD, hypertension and PVD.,Resp:  Patient denies asthma, lung infections and lung lesions.,GI:  Patient denies colon abnormalities, gall bladder problems, liver abnormalities and peptic ulcer disease.,GU:  Patient has history of Urinary tract disorder, but does not have Bladder disorder and Kidney disorder.,Endocrine:  Patient has history of diabetes, but does not have hormonal irregularities and thyroid abnormalities.,Dermatology:  Patient denies allergic reactions, rashes and skin lesions.,MEDS:,  Micronase 2.5 mg Tab PO QAM #30.  Bactrim 400/80 Tab PO BID #30.,SOCIAL HISTORY:,  No known history of drug or alcohol abuse.  Work, diet, and exercise patterns are within normal limits.,FAMILY HISTORY:,  No significant family history.,REVIEW OF SYSTEMS:,  Non-contributory.,Vital Signs:  Height = 72 in.  Weight =184 lbs.  Upright BP = 120/80 mmHg.  Pulse = 80 bpm.  Resp =12 pm.  Patient is afebrile.,Neck:  The neck is supple.  There is no jugular venous distension.  The thyroid is nontender, or normal size and conto.,Lungs:  Lung expansion and excursions are symmetric.  The lungs are clear to auscultation and percussion.,Cardio:  There is a regular rhythm.  SI and S2 are normal.  No abnormal heart sounds are detected.  Blood pressure is equal bilaterally.,Abdomen:  Normal bowel sounds are present.  The abdomen is soft; The abdomen is nontender; without organomegaly; There is no CVA tenderness.  No hernias are noted.,Extremities:  There is no clubbing, cyanosis, or edema.,ASSESSMENT: , Diabetes type II uncontrolled.  Acute cystitis.,PLAN: , Endocrinology Consult, complete CBC.  ,RX: , Micronase 2.5 mg Tab PO QAM #30, Bactrim 400/80 Tab PO BID #30.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="n">
-        <v>237</v>
+        <v>299</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Endocrinology; short; SOAP-style; diagnoses + treatment plans + assessment/plan</t>
+          <t>Endocrinology; medium; other narrative/sectioned; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J20" s="2" t="n">
-        <v>3800</v>
+        <v>3808</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>SOAP-style</t>
+          <t>other narrative/sectioned</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>middle</t>
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>0.1243800721370604</v>
+        <v>0.5951307484220019</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; treatment plans; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; past history; treatment plans; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="21" ht="110" customHeight="1">
       <c r="A21" s="2" t="n">
-        <v>3798</v>
+        <v>3805</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
@@ -1712,26 +1708,26 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Post Hemithyroidectomy </t>
+          <t xml:space="preserve"> Completion Thyroidectomy </t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The patient with left completion hemithyroidectomy and reimplantation of the left parathyroid and left sternocleidomastoid region in the inferior 1/3rd region.  Papillary carcinoma of the follicular variant of the thyroid in the right lobe, status post right hemithyroidectomy.</t>
+          <t xml:space="preserve"> Completion thyroidectomy with limited right paratracheal node dissection.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>PREOPERATIVE DIAGNOSES: , Papillary carcinoma of the follicular variant of the thyroid in the right lobe, status post right hemithyroidectomy.,POSTOPERATIVE DIAGNOSES: , Papillary carcinoma of the follicular variant of the thyroid in the right lobe, status post right hemithyroidectomy.,PROCEDURE:  ,The patient with left completion hemithyroidectomy and reimplantation of the left parathyroid and left sternocleidomastoid region in the inferior 1/3rd region.,FINDINGS: , Normal-appearing thyroid gland with a possible lump in the inferior aspect, there was a parathyroid gland that by frozen section _________  was not thyroid, it was reimplanted to the left lower sternocleidomastoid region.,ESTIMATED BLOOD LOSS:  ,Approximately 10 mL.,FLUIDS: , Crystalloid only.,COMPLICATIONS: , None.,DRAINS: , Rubber band drain in the neck.,CONDITION:,  Stable.,PROCEDURE:  ,The patient placed supine under general anesthesia.  First, a shoulder roll was placed, 1% lidocaine and 1:100,000 epinephrine was injected into the old scar, natural skin fold, and Betadine prep.  Sterile dressing was placed.  The laryngeal monitoring was noted to be working fine.  Then, an incision was made in this area in a curvilinear fashion through the old scar, taken through the fat and the platysma level.  The strap muscles were found and there was scar tissue along the trachea and the strap muscles were elevated off of the left thyroid, the thyroid gland was then found.  Then, using bipolar cautery and a Coblation dissector, the thyroid gland inferiorly was dissected off and the parathyroid gland was left inferiorly and there was scar tissue that was released and laterally, the thyroid gland was released, then came into the Berry ligaments.  The Berry ligament was dissected off and the gland came off all the way to the superior and inferior thyroid vessels, which were crossed with the Harmonic scalpel and removed.  No bleeding was seen.  There was a small nick in the external jugular vein that was tied with a 4-0 Vicryl suture ligature.  After this was completed, on examining the specimen, there appeared to be a lobule on it and it was sent off as possibly parathyroid, therefore it was reimplanted in the left lower sternocleidomastoid region using the silk suture ligature.  After this was completed, no bleeding was seen.  The laryngeal nerve could be seen and intact and then Rubber band  drain was placed throughout the neck along the thyroid bed and 4-0 Vicryl was used to close the strap muscles in an interrupted fashion along with the platysma region and subcutaneous region and a running 5-0 nylon was used to close the skin and Mastisol and Steri-Strips were placed along the skin edges and then on awakening, both laryngeal nerves were working normally.  Procedure was then terminated at that time.</t>
+          <t>TITLE OF OPERATION:,  Completion thyroidectomy with limited right paratracheal node dissection.,INDICATION FOR SURGERY:,  A 49-year-old woman with a history of a left dominant nodule in her thyroid gland, who subsequently underwent left thyroid lobectomy and isthmusectomy, was found to have multifocal papillary thyroid carcinoma throughout her left thyroid lobe and isthmus.  Consideration given to completion thyroidectomy.  Risks, benefits, and alternatives of this procedure was discussed with the patient in great detail.  Risks included but were not limited to anesthesia, bleeding, infection, injury to nerves including vocal fold paralysis, hoarseness, low calcium, scar, cosmetic deformity, need for thyroid hormone replacement, and also need for further management.  The patient understood all of this and then wished to proceed.,PREOP DIAGNOSIS:,  Multifocal thyroid carcinoma and previous left thyroid lobectomy resection specimen.,POSTOP DIAGNOSIS: , Multifocal thyroid carcinoma and previous left thyroid lobectomy resection specimen.,PROCEDURE DETAIL:,  After identifying the patient, the patient was placed supine in the operating room table.  After establishment of general anesthesia via orotracheal intubation with a number 6 nerve integrity monitoring system endotracheal tube, the eyes were protected with Tegaderm.  Nerve integrity monitoring system endotracheal tube was confirmed to be working adequately and secured.  The previous skin incision for a thyroidectomy was then planned, then incorporated into an ellipse.  The patient was prepped and draped in a sterile fashion.  Subsequently, the ellipse around the previous incision was deformed.  The scar was then excised.  Subplatysmal flaps were raised to the thyroid notch and sternal notch respectively.  Strap muscles were isolated in the midline and dissected and mobilized from the thyroid lobe on the right side.  There was some dense fibrosis and inflammation surrounding the right thyroid lobe.  Careful dissection along the thyroid lobe allowed for identification of the superior thyroid artery and vein which were individually ligated with a Harmonic scalpel.  The right inferior and superior parathyroid glands were identified and preserved and recurrent laryngeal nerve was identified and traced superiorly, then preserved.  Of note is that there were multiple lymph nodes in the paratracheal region on the right side.  These lymph nodes were carefully dissected away from the recurrent laryngeal nerve, trachea, and the carotid artery, and sent as a separate specimen labeled right paratracheal lymph nodes.  The wound was copiously irrigated.  Valsalva maneuver was given.  Surgicel was placed in the wound bed.  Strap muscles were reapproximated in the midline with 3-0 Vicryl and incision was then closed with interrupted 3-0 Vicryl and Indermil for the skin.  The patient was extubated in the operating room table, sent to the postanesthesia care unit in good condition.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>endocrinology, thyroid, rubber band drain, berry ligaments, papillary carcinoma, follicular variant, strap muscles, thyroid gland, sternocleidomastoid, parathyroid, hemithyroidectomy,</t>
+          <t xml:space="preserve">endocrinology, multifocal thyroid carcinoma, thyroid lobectomy, thyroid, papillary, thyroid lobe, isthmus, completion thyroidectomy, thyroidectomy, paratracheal, lobectomy, </t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>434</v>
+        <v>423</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1740,15 +1736,15 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Endocrinology; medium; procedure/operative; diagnoses + procedures + surgery</t>
+          <t>Endocrinology; medium; other narrative/sectioned; middle text complexity; diagnoses + procedures + past history</t>
         </is>
       </c>
       <c r="J21" s="2" t="n">
-        <v>3798</v>
+        <v>3805</v>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>procedure/operative</t>
+          <t>other narrative/sectioned</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -1757,17 +1753,17 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>0.4576758340847611</v>
+        <v>0.4482078449053201</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; procedures; surgery</t>
+          <t>diagnoses; procedures; past history; treatment plans; surgery</t>
         </is>
       </c>
     </row>
     <row r="22" ht="110" customHeight="1">
       <c r="A22" s="2" t="n">
-        <v>3797</v>
+        <v>3811</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
@@ -1776,39 +1772,43 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Thyroid Mass Consult </t>
+          <t xml:space="preserve"> Acquired Hypothyroidism Followup </t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Thyroid mass diagnosed as papillary carcinoma.  The patient is a 16-year-old young lady with a history of thyroid mass that is now biopsy proven as papillary.  The pattern of miliary metastatic lesions in the chest is consistent with this diagnosis.</t>
+          <t xml:space="preserve"> Return visit to the endocrine clinic for acquired hypothyroidism, papillary carcinoma of the thyroid gland status post total thyroidectomy in 1992, and diabetes mellitus.</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>REASON FOR CONSULTATION: , Thyroid mass diagnosed as papillary carcinoma.,HISTORY OF PRESENT ILLNESS:  ,The patient is a 16-year-old young lady, who was referred from the Pediatric Endocrinology Department by Dr. X for evaluation and surgical recommendations regarding treatment of a mass in her thyroid, which has now been proven to be papillary carcinoma on fine needle aspiration biopsy.  The patient's parents relayed that they first noted a relatively small but noticeable mass in the middle portion of her thyroid gland about 2004.  An ultrasound examination had reportedly been done in the past and the mass is being observed.  When it began to enlarge recently, she was referred to the Pediatric Endocrinology Department and had an evaluation there.  The patient was referred for fine needle aspiration and the reports recently returned a diagnosis of papillary thyroid carcinoma.  The patient has not had any hoarseness, difficulty swallowing, or any symptoms of endocrine dysfunction.  She has no weight changes consistent with either hyper or hypothyroidism.  There is no family history of thyroid cancer in her family.  She has no notable discomfort with this lesion.  There have been no skin changes.  Historically, she does not have a history of any prior head and neck radiation or treatment of any unusual endocrinopathy.,PAST MEDICAL HISTORY:,  Essentially unremarkable.  The patient has never been hospitalized in the past for any major illnesses.  She has had no prior surgical procedures.,IMMUNIZATIONS: , Current and up to date.,ALLERGIES: , She has no known drug allergies.,CURRENT MEDICATIONS:  ,Currently taking no routine medications.  She describes her pain level currently as zero.,FAMILY HISTORY: , There is no significant family history, although the patient's father does note that his mother had a thyroid surgery at some point in life, but it was not known whether this was for cancer, but he suspects it might have been for goiter.  This was done in Tijuana.  His mom is from central portion of Mexico.  There is no family history of multiple endocrine neoplasia syndromes.,SOCIAL HISTORY:  ,The patient is a junior at Hoover High School.  She lives with her mom in Fresno.,REVIEW OF SYSTEMS: , A careful 12-system review was completely normal except for the problems related to the thyroid mass.,PHYSICAL EXAMINATION:,GENERAL:  The patient is a 55.7 kg, nondysmorphic, quiet, and perhaps slightly apprehensive young lady, who was in no acute distress.  She was alert and oriented x3 and had an appropriate affect.,HEENT:  The head and neck examination is most significant.  There is mild amount of facial acne.  The patient's head, eyes, ears, nose, and throat appeared to be grossly normal.,NECK:  There is a slightly visible midline bulge in the region of the thyroid isthmus.  A firm nodule is present there, and there is also some nodularity in the right lobe of the thyroid.  This mass is relatively hard, slightly fixed, but not tethered to surrounding tissues, skin, or muscles that I can determine.  There are some shotty adenopathy in the area.  No supraclavicular nodes were noted.,CHEST:  Excursions are symmetric with good air entry.,LUNGS:  Clear.,CARDIOVASCULAR:  Normal.  There is no tachycardia or murmur noted.,ABDOMEN:  Benign.,EXTREMITIES:  Extremities are anatomically correct with full range of motion.,GENITOURINARY:  External genitourinary exam was deferred at this time and can be performed later during anesthesia.  This is same as too for her rectal examination.,SKIN:  There is no acute rash, purpura, or petechiae.,NEUROLOGIC:  Normal and no focal deficits.  Her voice is strong and clear.  There is no evidence of dysphonia or vocal cord malfunction.,DIAGNOSTIC STUDIES: , I reviewed laboratory data from the Diagnostics Lab, which included a mild abnormality in the AST at 11, which is slightly lower than the normal range.  T4 and TSH levels were recorded as normal.  Free thyroxine was normal, and the serum pregnancy test was negative.  There was no level of thyroglobulin recorded on this.  A urinalysis and comprehensive metabolic panel was unremarkable.  A chest x-ray was obtained, which I personally reviewed.  There is a diffuse pattern of tiny nodules in both lungs typical of miliary metastatic disease that is often seen in patients with metastatic thyroid carcinoma.,IMPRESSION/PLAN: , The patient is a 16-year-old young lady with a history of thyroid mass that is now biopsy proven as papillary.  The pattern of miliary metastatic lesions in the chest is consistent with this diagnosis and is unfortunate in that it generally means a more advanced stage of disease.  I spent approximately 30 minutes with the patient and her family today discussing the surgical aspects of the treatment of this disease.  During this time, we talked about performing a total thyroidectomy to eradicate as much of the native thyroid tissue and remove the primary source of the cancer in anticipation of radioactive iodine therapy.  We talked about sentinel node dissection, and we spent significant amount of time talking about the possibility of hypoparathyroidism if all four of the parathyroid glands were damaged during this operation.  We also discussed the recurrent laryngeal and external laryngeal branches of the nerve supplying the vocal cord function and how they cane be damaged during the thyroidectomy as well.  I answered as many of the family's questions as they could mount during this stressful time with this recent information supplied to them.  I also did talk to them about the chest x-ray pattern, which was complete __________ as the film was just on the day prior to my clinic visit.  This will have some impact on the postoperative adjunctive therapy.  The radiologist commented about the risk of pulmonary fibrosis and the use of radioactive iodine in this situation, but it seems likely that is going to be necessary to attempt to treat this disease in the patient's case.  I did discuss with them the possibility of having to take large doses of calcium and vitamin D in the event of hypoparathyroidism if that does happen, and we also talked about possibly sparing parathyroid tissue and reimplanting it in a muscle belly either in the neck or forearm if that becomes a necessity.  All of the family's questions have been answered.  This is a very anxious and anxiety provoking time in the family.  I have made every effort to get the patient under schedule within the next 48 hours to have this operation done.  We are tentatively planning on proceeding this upcoming Friday afternoon with total thyroidectomy.</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr"/>
+          <t>PROBLEM LIST:,1.  Acquired hypothyroidism.,2.  Papillary carcinoma of the thyroid gland, status post total thyroidectomy in 1992.,3.  Diabetes mellitus.,4.  Insomnia with sleep apnea.,HISTORY OF PRESENT ILLNESS: , This is a return visit to the endocrine clinic for the patient with history as noted above.  She is 45 years old.  Her last visit was about 6 months ago.  Since that time, the patient states her health has remained unchanged.  Currently, primary complaint is one of fatigue that she feels throughout the day.  She states, however, she is doing well with CPAP and wakes up feeling refreshed but tends to tire out later in the day.  In terms of her thyroid issues, the patient states that she is not having signs or symptoms of thyroid excess or hypothyroidism.  She is not reporting temperature intolerance, palpitations, muscle weakness, tremors, nausea, vomiting, constipation, hyperdefecation or diarrhea.  Her weight has been stable.  She is not reporting proximal muscle weakness.,CURRENT MEDICATIONS:,1.  Levothyroxine 125 micrograms p.o. once daily.,2.  CPAP.,3.  Glucotrol.,4.  Avandamet.,5.  Synthroid.,6.  Byetta injected twice daily.,REVIEW OF SYSTEMS: , As stated in the HPI.  She is not reporting polyuria, polydipsia or polyphagia.  She is not reporting fevers, chills, sweats, visual acuity changes, nausea, vomiting, constipation or diarrhea.  She is not having any lightheadedness, weakness, chest pain, shortness of breath, difficulty breathing, orthopnea or dyspnea on exertion.,PHYSICAL EXAMINATION:,GENERAL:  She is an overweight, very pleasant woman, in no acute distress.  VITAL SIGNS:  Temperature 96.9, pulse 85, respirations not counted, blood pressure 135/65, and weight 85.7 kg.  NECK:  Reveals well healed surgical scar in the anteroinferior aspect of the neck.  There is no palpable thyroid tissue noted on this examination today.  There is no lymphadenopathy.  THORAX:  Reveals lungs that are clear, PA and lateral, without adventitious sounds.  CARDIOVASCULAR:  Demonstrated regular rate and rhythm.  S1 and S2 without murmur.  No S3, no S4 is auscultated.  EXTREMITIES:  Deep tendon reflexes 2+/4 without a delayed relaxation phase.  No fine resting tremor of the outstretched upper extremity.  SKIN, HAIR, AND NAILS:  All are unremarkable.,LABORATORY DATABASE: , Lab data on 08/29/07 showed the following:  Thyroglobulin quantitative less than 0.5 and thyroglobulin antibody less than 20, free T4 1.35, and TSH suppressed at 0.121.,ASSESSMENT AND PLAN:,This is a 45-year-old woman with history as noted above.,1.  Acquired hypothyroidism, status post total thyroidectomy for papillary carcinoma in 1992.,2.  Plan to continue following thyroglobulin levels.,3.  Plan to obtain a free T4, TSH, and thyroglobulin levels today.,4.  Have the patient call the clinic next week for followup and continued management of her hypothyroid state.,5.  Plan today is to repeat her thyroid function studies.  This case was discussed with Dr. X and the recommendation.  We are giving the patient today is for us to taper her medication to get her TSH somewhere between 0.41 or less.  Therefore, labs have been drawn.  We plan to see the patient back in approximately 6 months or sooner.  A repeat body scan will not been done, the one in 03/06 was negative.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">endocrinology, thyroid function studies, thyroid gland, diabetes mellitus, papillary carcinoma, total thyroidectomy, acquired hypothyroidism, carcinoma, thyroidectomy, thyroglobulin, hypothyroidism, </t>
+        </is>
+      </c>
       <c r="G22" s="2" t="n">
-        <v>1037</v>
+        <v>486</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Endocrinology; long; consultation; diagnoses + symptoms + medications</t>
+          <t>Endocrinology; medium; follow-up/progress; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J22" s="2" t="n">
-        <v>3797</v>
+        <v>3811</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>consultation</t>
+          <t>follow-up/progress</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -1817,17 +1817,17 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>0.8055117222723174</v>
+        <v>0.8002705139765555</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; procedures; imaging; past history; treatment plans; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; laboratory values; vital signs; past history; treatment plans; follow-up; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="23" ht="110" customHeight="1">
       <c r="A23" s="2" t="n">
-        <v>3604</v>
+        <v>3608</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
@@ -1836,39 +1836,39 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CT Abdomen &amp; Pelvis - 5 </t>
+          <t xml:space="preserve"> CT Abdomen &amp; Pelvis </t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  CT abdomen without contrast and pelvis without contrast, reconstruction.</t>
+          <t xml:space="preserve"> CT Abdomen &amp; Pelvis W&amp;WO Contrast</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>EXAM: , CT abdomen without contrast and pelvis without contrast, reconstruction.,REASON FOR EXAM: , Right lower quadrant pain, rule out appendicitis.,TECHNIQUE:  ,Noncontrast CT abdomen and pelvis.  An intravenous line could not be obtained for the use of intravenous contrast material.,FINDINGS: , The appendix is normal.  There is a moderate amount of stool throughout the colon.  There is no evidence of a small bowel obstruction or evidence of pericolonic inflammatory process.  Examination of the extreme lung bases appear clear, no pleural effusions.  The visualized portions of the liver, spleen, adrenal glands, and pancreas appear normal given the lack of contrast.  There is a small hiatal hernia.  There is no intrarenal stone or evidence of obstruction bilaterally.  There is a questionable vague region of low density in the left anterior mid pole region, this may indicate a tiny cyst, but it is not well seen given the lack of contrast.  This can be correlated with a followup ultrasound if necessary.  The gallbladder has been resected.  There is no abdominal free fluid or pathologic adenopathy.  There is abdominal atherosclerosis without evidence of an aneurysm.,Dedicated scans of the pelvis disclosed phleboliths, but no free fluid or adenopathy.  There are surgical clips present.  There is a tiny airdrop within the bladder.  If this patient has not had a recent catheterization, correlate for signs and symptoms of urinary tract infection.,IMPRESSION:,1.Normal appendix.,2.Moderate stool throughout the colon.,3.No intrarenal stones.,4.Tiny airdrop within the bladder.  If this patient has not had a recent catheterization, correlate for signs and symptoms of urinary tract infection.  The report was faxed upon dictation.</t>
+          <t>EXAM:,  CT Abdomen &amp; Pelvis W&amp;WO Contrast, ,REASON FOR EXAM: , Status post aortobiiliac graft repair. , ,TECHNIQUE: , 5 mm spiral thick spiral CT scanning was performed through the entire abdomen and pelvis utilizing intravenous dynamic bolus contrast enhancement.  No oral or rectal contrast was utilized.  Comparison is made with the prior CT abdomen and pelvis dated 10/20/05.  There has been no significant change in size of the abdominal aortic aneurysm centered roughly at the renal artery origin level which has dimensions of 3.7 cm transversely x 3.4 AP.  Just below this level is the top of the endoluminal graft repair with numerous surrounding surgical clips.  The size of the native aneurysm component at this level is stable at 5.5 cm in diameter with mural thrombus surrounding the enhancing endolumen.  There is no abnormal entrance of contrast agent into the mural thrombus to indicate an endoluminal leak.  Further distally, there is extension of the graft into both proximal common iliac arteries without evidence for endoluminal leak at this level either.  No exoluminal leakage is identified at any level.  There is no retroperitoneal hematoma present.  The findings are unchanged from the prior exam.  ,The liver, spleen, pancreas, adrenals and right kidney are unremarkable with moderate diffuse atrophy of the pancreas present.  There is advanced atrophy of the left kidney.  No hydronephrosis is present.  No acute findings are identified elsewhere in the abdomen. ,The lung bases are clear. ,Concerning the remainder of the pelvis, no acute pathology is identified.  There is prominent streak artifact from the left total hip replacement.  There is diffuse moderate sigmoid diverticulosis without evidence for diverticulitis.  The bladder grossly appears normal.  A hysterectomy has been performed.  ,IMPRESSION:,1.  No complications identified regarding endoluminal aortoiliac graft repair as described.  The findings are stable compared to the study of 10/20/04.  ,2.  Stable mild aneurysm of aortic aneurysm, centered roughly at renal artery level.  ,3.  No other acute findings noted. ,4.  Advanced left renal atrophy.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>gastroenterology, reconstruction, appendicitis, urinary tract infection, ct abdomen, abdomen, ct, pelvis, contrast, noncontrast,</t>
+          <t>gastroenterology, aortobiiliac graft repair, renal atrophy, ct abdomen &amp; pelvis, w&amp;wo contrast, aortic aneurysm, renal artery, mural thrombus, endoluminal leak, ct abdomen, ct, contrast, pelvis, abdomen,</t>
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>259</v>
+        <v>324</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Gastroenterology; short; diagnostic report; diagnoses + symptoms + procedures</t>
+          <t>Gastroenterology; medium; diagnostic report; lower text complexity; diagnoses + imaging + surgery</t>
         </is>
       </c>
       <c r="J23" s="2" t="n">
-        <v>3604</v>
+        <v>3608</v>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
@@ -1881,17 +1881,17 @@
         </is>
       </c>
       <c r="M23" s="2" t="n">
-        <v>0.3426510369702435</v>
+        <v>0.3290126239855726</v>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; procedures; imaging; follow-up; surgery</t>
+          <t>diagnoses; imaging; surgery</t>
         </is>
       </c>
     </row>
     <row r="24" ht="110" customHeight="1">
       <c r="A24" s="2" t="n">
-        <v>3472</v>
+        <v>3685</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
@@ -1900,22 +1900,26 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Rectal Bleeding - 1-year-old </t>
+          <t xml:space="preserve"> Admission History &amp; Physical - Nausea </t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Pediatric Gastroenterology - Rectal Bleeding Consult.</t>
+          <t xml:space="preserve"> Patient status post gastric bypass surgery, developed nausea and right upper quadrant pain.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS:,  This is a 1-year-old male patient who was admitted on 12/23/2007 with a history of rectal bleeding.  He was doing well until about 2 days prior to admission and when he passes hard stools, there was bright red blood in the stool.  He had one more episode that day of stool; the stool was hard with blood in it.  Then, he had one episode of rectal bleeding yesterday and again one stool today, which was soft and consistent with dark red blood in it.  No history of fever, no diarrhea, no history of easy bruising.  Excessive bleeding from minor cut.  He has been slightly fussy.,PAST MEDICAL HISTORY:  ,Nothing significant.,PREGNANCY DELIVERY AND NURSERY COURSE: , He was born full term without complications.,PAST SURGICAL HISTORY: , None.,SIGNIFICANT ILLNESS AND REVIEW OF SYSTEMS: , Negative for heart disease, lung disease, history of cancer, blood pressure problems, or bleeding problems.,DIET:,  Regular table food, 24 ounces of regular milk.  He is n.p.o. now.,TRAVEL HISTORY: , Negative.,IMMUNIZATION: , Up-to-date.,ALLERGIES: , None.,MEDICATIONS: , None, but he is on IV Zantac now.,SOCIAL HISTORY: , He lives with parents and siblings.,FAMILY HISTORY:,  Nothing significant.,LABORATORY EVALUATION: , On 12/24/2007, WBC 8.4, hemoglobin 7.6, hematocrit 23.2 and platelets 314,000.  Sodium 135, potassium 4.7, chloride 110, CO2 20, BUN 6 and creatinine 0.3.  Albumin 3.3.  AST 56 and ALT 26.  CRP less than 0.3.  Stool rate is still negative.,DIAGNOSTIC DATA: , CT scan of the abdomen was read as normal.,PHYSICAL EXAMINATION:  ,VITAL SIGNS:  Temperature 99.5 degrees Fahrenheit, pulse 142 per minute and respirations 28 per minute.  Weight 9.6 kilogram.,GENERAL:  He is alert and active child in no apparent distress.,HEENT:  Atraumatic and normocephalic.  Pupils are equal, round and reactive to light.  Extraocular movements, conjunctivae and sclerae fair.  Nasal mucosa pink and moist.  Pharynx is clear.,NECK:  Supple without thyromegaly or masses.,LUNGS:  Good air entry bilaterally.  No rales or wheezing.,ABDOMEN:  Soft and nondistended.  Bowel sounds positive.  No mass palpable.,GENITALIA:  Normal male.,RECTAL:  Deferred, but there was no perianal lesion.,MUSCULOSKELETAL:  Full range of movement.  No edema.  No cyanosis.,CNS:  Alert, active and playful.,IMPRESSION: , A 1-year-old male patient with history of rectal bleeding.  Possibilities include Meckel's diverticulum, polyp, infection and vascular malformation.,PLAN:,  To proceed with Meckel scan today.  If Meckel scan is negative, we will consider upper endoscopy and colonoscopy.  We will start colon clean out if Meckel scan is negative.  We will send his stool for C. diff toxin, culture, blood for RAST test for cow milk, soy, wheat and egg.  Monitor hemoglobin.</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr"/>
+          <t>CHIEF COMPLAINT: , Nausea.,PRESENT ILLNESS: , The patient is a 28-year-old, who is status post gastric bypass surgery nearly one year ago.  He has lost about 200 pounds and was otherwise doing well until yesterday evening around 7:00-8:00 when he developed nausea and right upper quadrant pain, which apparently wrapped around toward his right side and back.  He feels like he was on it but has not done so.  He has overall malaise and a low-grade temperature of 100.3.  He denies any prior similar or lesser symptoms.  His last normal bowel movement was yesterday.  He denies any outright chills or blood per rectum.,PAST MEDICAL HISTORY: , Significant for hypertension and morbid obesity, now resolved.,PAST SURGICAL HISTORY: , Gastric bypass surgery in December 2007.,MEDICATIONS:  ,Multivitamins and calcium.,ALLERGIES: , None known.,FAMILY HISTORY:  ,Positive for diabetes mellitus in his father, who is now deceased.,SOCIAL HISTORY: , He denies tobacco or alcohol.  He has what sounds like a data entry computer job.,REVIEW OF SYSTEMS:  ,Otherwise negative.,PHYSICAL EXAMINATION:,  His temperature is 100.3, blood pressure 129/59, respirations 16, heart rate 84.  He is drowsy, but easily arousable and appropriate with conversation.  He is oriented to person, place, and situation.  He is normocephalic, atraumatic.  His sclerae are anicteric.  His mucous membranes are somewhat tacky.  His neck is supple and symmetric.  His respirations are unlabored and clear.  He has a regular rate and rhythm.  His abdomen is soft.  He has diffuse right upper quadrant tenderness, worse focally, but no rebound or guarding.  He otherwise has no organomegaly, masses, or abdominal hernias evident.  His extremities are symmetrical with no edema.  His posterior tibial pulses are palpable and symmetric.  He is grossly nonfocal neurologically.,STUDIES:,  His white blood cell count is 8.4 with 79 segs.  His hematocrit is 41.  His electrolytes are normal.  His bilirubin is 2.8.  His AST 349, ALT 186, alk-phos 138 and lipase is normal at 239.,ASSESSMENT: , Choledocholithiasis, ? cholecystitis.,PLAN: , He will be admitted and placed on IV antibiotics.  We will get an ultrasound this morning.  He will need his gallbladder out, probably with intraoperative cholangiogram.  Hopefully, the stone will pass this way.  Due to his anatomy, an ERCP would prove quite difficult if not impossible unless laparoscopic assisted.  Dr. X will see him later this morning and discuss the plan further.  The patient understands.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gastroenterology, gastric bypass surgery, nausea, choledocholithiasis, cholecystitis, ercp, gastric bypass, bypass surgery, </t>
+        </is>
+      </c>
       <c r="G24" s="2" t="n">
-        <v>410</v>
+        <v>379</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -1924,15 +1928,15 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Gastroenterology; medium; other narrative/sectioned; diagnoses + symptoms + medications</t>
+          <t>Gastroenterology; medium; history and physical; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>3472</v>
+        <v>3685</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>other narrative/sectioned</t>
+          <t>history and physical</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -1941,17 +1945,17 @@
         </is>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0.800777727682597</v>
+        <v>0.7628494138863842</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; imaging; past history; treatment plans; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="25" ht="110" customHeight="1">
       <c r="A25" s="2" t="n">
-        <v>3525</v>
+        <v>3606</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
@@ -1960,58 +1964,62 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> GI Consultation - 3 </t>
+          <t xml:space="preserve"> CT Abdomen &amp; Pelvis - 3 </t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> GI Consultation for Chrohn's disease.</t>
+          <t xml:space="preserve"> CT of the abdomen and pelvis without contrast.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>PROBLEM:  ,Prescription evaluation for Crohn's disease., ,HISTORY: , This is a 46-year-old male who is here for a refill of Imuran.  He is taking it at a dose of 100 mg per day.  He is status post resection of the terminal ileum and has experienced intermittent obstructive symptoms for the past several years.  In fact, he had an episode three weeks ago in which he was seen at the emergency room after experiencing sudden onset of abdominal pain and vomiting. An x-ray was performed, which showed no signs of obstruction per his report.  He thinks that the inciting factor of this incident was too many grapes eaten the day before.  He has had similar symptoms suggestive of obstruction when eating oranges or other high-residue fruits in the past.  The patient's normal bowel pattern is loose stools and this is unchanged recently.  He has not had any rectal bleeding. He asks today about a rope-like vein on his anterior right arm that has been a little tender and enlarged after he was in the emergency room and they had difficulty with IV insertion.  He has not had any fever, red streaking up the arm, or enlargement of lymph nodes.  The tenderness has now completely resolved.  , ,He had a colonoscopy performed in August of 2003, by Dr. S.  An anastomotic stricture was found at the terminal ileum/cecum junction.  Dr. S recommended that if the patient experienced crampy abdominal pain or other symptoms of obstruction, that he may consider balloon dilation.  No active Crohn's disease was found during the colonoscopy.  , ,Earlier this year, he experienced a non-specific hepatitis with elevation of his liver function tests.  At that time he was taking a lot of Tylenol for migraine-type headaches.  Under Dr. S's recommendation, he stopped the Imuran for one month and reduced his dose of Tylenol.  Since that time his liver enzymes have normalized and he has restarted the Imuran with no problems.  , ,He also reports heartburn that is occurring on a slightly more frequent basis than it has in the past.  It used to occur once a week only, but has now increased in frequency to twice a week.  He takes over-the-counter H2 blockers as needed, as well as Tums.  He associates the onset of his symptoms with eating spicy Mexican food., ,PAST MEDICAL HISTORY: , Reviewed and unchanged.,ALLERGIES: , No known allergies to medications.,OPERATIONS: , Unchanged.,ILLNESSES: , Crohn's disease, vitamin B12 deficiency.,MEDICATIONS:,  Imuran, Nascobal, Vicodin p.r.n., ,REVIEW OF SYSTEMS: , Dated 08/04/04 is reviewed and noted.  Please see pertinent GI issues as discussed above.  Otherwise unremarkable., ,PHYSICAL EXAMINATION:  , GENERAL:  Pleasant male in no acute distress.  Well nourished and well developed. SKIN: indurated, cord-like superficial vein on the right anterior forearm, approx. 3 cm in length.  Non-tender to palpation. No erythema or red streaking.  No edema. LYMPH:  No epitrochlear or axillary lymph node enlargement or tenderness on the right side. , ,DATA REVIEWED: Labs from June 8th and July 19th reviewed.  Liver function tests normal with AST 14 and ALT 44.  WBCs were slightly low at 4.8.  Hemoglobin dropped slightly from 14.1 on 6/8 to 12.9 on 7/19. Hematocrit dropped slightly as well from 43.2 on 6/804 to 40.0 on 7/19/04.  These results were reviewed by Dr. S and lab results letter sent., ,IMPRESSION:  ,1. Crohn's disease, status post terminal ileum resection, on Imuran.  Intermittent symptoms of bowel obstruction.  Last episode three weeks ago.,2.  History of non-specific hepatitis while taking high doses of Tylenol.  Now resolved. ,2.  Increased frequency of reflux symptoms.,3.  Superficial thrombophlebitis, resolving. ,4.  Slightly low H&amp;H., ,PLAN:  ,1.  We discussed Dr. S's recommendation that the patient undergo balloon dilation for recurrent bowel obstruction type symptoms.  The patient emphatically states that he does not want to consider dilation at this time.  The patient is strongly encouraged to call us when he does experience any obstructive symptoms, including abdominal pain, nausea, vomiting, or change in bowel habits.  He states understanding of this. Advised to maintain low residue diet to avoid obstructions. ,2.  Continue with liver panel and ABC every month per Dr. S's instructions.,3.  Continue Imuran 100 mg per day.,4.  Continue to minimize Tylenol use.  The patient is wondering if he can take another type of medication for migraines that is not Tylenol or antiinflammatories or aspirin.  Dr. S is consulted and agrees that Imitrex is an acceptable alternative for migraine headaches since he does not have advanced liver disease. The patient will make an appointment with his primary care provider to discuss this further. ,5.  Reviewed the importance of prophylactic treatment of reflux-type symptoms.  Encouraged the patient to take over-the-counter H2 blockers on a daily basis to prevent symptoms from occurring.  The patient will try this and if he remains symptomatic, then he will call our office and a prescription for Zantac 150 mg per day will be provided.  Reviewed the potential need for upper endoscopy should his symptoms continue or become more frequent.  He does not want to undergo any type of procedure such as that at this time.,6.</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr"/>
+          <t>EXAM: , CT of the abdomen and pelvis without contrast.,HISTORY: , Lower abdominal pain.,FINDINGS:,  Limited views of the lung bases demonstrate linear density most likely representing dependent atelectasis.  There is a 1.6 cm nodular density at the left posterior sulcus.,Noncontrast technique limits evaluation of the solid abdominal organs.  Cardiomegaly and atherosclerotic calcifications are seen.,Hepatomegaly is observed.  There is calcification within the right lobe of the liver likely related to granulomatous changes.  Subtle irregularity of the liver contour is noted, suggestive of cirrhosis.  There is splenomegaly seen.  There are two low-attenuation lesions seen in the posterior aspect of the spleen, which are incompletely characterized that may represent splenic cyst.  The pancreas appears atrophic.  There is a left renal nodule seen, which measures 1.9 cm with a Hounsfield unit density of approximately 29, which is indeterminate.,There is mild bilateral perinephric stranding.  There is an 8-mm fat density lesion in the anterior inner polar region of the left kidney, compatible in appearance with angiomyolipoma.  There is a 1-cm low-attenuation lesion in the upper pole of the right kidney, likely representing a cyst, but incompletely characterized on this examination.  Bilateral ureters appear normal in caliber along their visualized course.  The bladder is partially distended with urine, but otherwise unremarkable.,Postsurgical changes of hysterectomy are noted.  There are pelvic phlebolith seen.  There is a calcified soft tissue density lesion in the right pelvis, which may represent an ovary with calcification, as it appears continuous with the right gonadal vein.,Scattered colonic diverticula are observed.  The appendix is within normal limits.  The small bowel is unremarkable.  There is an anterior abdominal wall hernia noted containing herniated mesenteric fat.  The hernia neck measures approximately 2.7 cm.  There is stranding of the fat within the hernia sac.,There are extensive degenerative changes of the right hip noted with changes suggestive of avascular necrosis.  Degenerative changes of the spine are observed.,IMPRESSION:,1.  Anterior abdominal wall hernia with mesenteric fat-containing stranding, suggestive of incarcerated fat.,2.  Nodule in the left lower lobe, recommend follow up in 3 months.,3.  Indeterminate left adrenal nodule, could be further assessed with dedicated adrenal protocol CT or MRI.,4.  Hepatomegaly with changes suggestive of cirrhosis.  There is also splenomegaly observed.,5.  Low-attenuation lesions in the spleen may represent cyst, that are incompletely characterized on this examination.,6.  Fat density lesion in the left kidney, likely represents angiomyolipoma.,7.  Fat density soft tissue lesion in the region of the right adnexa, this contains calcifications and may represent an ovary or possibly dermoid cyst.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>gastroenterology, abdominal pain, cardiomegaly, atherosclerotic calcifications, hepatomegaly, perinephric stranding, low attenuation lesions, abdominal, calcifications, lesions, abdomen,</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="n">
-        <v>833</v>
+        <v>408</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Gastroenterology; long; consultation; diagnoses + symptoms + medications</t>
+          <t>Gastroenterology; medium; diagnostic report; middle text complexity; diagnoses + symptoms + imaging</t>
         </is>
       </c>
       <c r="J25" s="2" t="n">
-        <v>3525</v>
+        <v>3606</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>consultation</t>
+          <t>diagnostic report</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>higher</t>
+          <t>middle</t>
         </is>
       </c>
       <c r="M25" s="2" t="n">
-        <v>0.9021077547339945</v>
+        <v>0.472497745716862</v>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; procedures; imaging; past history; treatment plans; follow-up; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; imaging; treatment plans; follow-up</t>
         </is>
       </c>
     </row>
     <row r="26" ht="110" customHeight="1">
       <c r="A26" s="2" t="n">
-        <v>3362</v>
+        <v>3341</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
@@ -2020,39 +2028,39 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Gen Med Consult - 23 </t>
+          <t xml:space="preserve"> Gen Med Consult - 41 </t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Patient in with mom for possible ear infection.</t>
+          <t xml:space="preserve"> Backache, stomachache, and dysuria for the last two days - Urinary dysuria, left flank pain, pharyngitis.</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>SUBJECTIVE:,  Mom brings the patient in today for possible ear infection.  He is complaining of left ear pain today.  He was treated on 04/14/2004, with amoxicillin for left otitis and Mom said he did seem to get better but just started complaining of the left ear pain today.  He has not had any fever but the congestion has continued to be very thick and purulent.  It has never really resolved.  He has a loose, productive-sounding cough but not consistently and not keeping him up at night.  No wheezing or shortness of breath.,PAST MEDICAL HISTORY:,  He has had some wheezing in the past but nothing recently.,FAMILY HISTORY: , All siblings are on antibiotics for ear infections and URIs.,OBJECTIVE:,General:  The patient is a 5-year-old male.  Alert and cooperative.  No acute distress.,Neck:  Supple without adenopathy.,HEENT:  Ear canals clear.  TMs, bilaterally, have distorted light reflexes but no erythema.  Gray in color.  Oropharynx pink and moist with a lot of postnasal discharge.  Nares are swollen and red.  Thick, purulent drainage.  Eyes are a little puffy.,Chest:  Respirations regular, nonlabored.,Lungs:  Clear to auscultation throughout.,Heart:  Regular rhythm without murmur.,Skin:  Warm, dry, pink.  Moist mucus membranes.  No rash.,ASSESSMENT:,  Ongoing purulent rhinitis.  Probable sinusitis and serous otitis.,PLAN:,  Change to Omnicef two teaspoons daily for 10 days.  Frequent saline in the nose.  Also, there was some redness around the nares with a little bit of yellow crusting.  It appeared to be the start of impetigo, so hold off on the Rhinocort for a few days and then restart.  Use a little Neosporin for now.</t>
+          <t>SUBJECTIVE:,  The patient complains of backache, stomachache, and dysuria for the last two days.  Fever just started today and cough.  She has history of kidney stones less than a year ago and had a urinary tract infection at that time.  Her back started hurting last night.,PAST MEDICAL HISTORY:,  She denies sexual activities since two years ago.  Her last menstrual period was 06/01/2004.  Her periods have been irregular.  She started menarche at 10 years of age and she is still irregular and it runs in Mom’s side of the family.  Mom and maternal aunt have had total hysterectomies.  She also is diagnosed with abnormal valve has to be on SBE prophylaxis, sees Dr. XYZ Allen.  She avoids decongestants.  She is limited on her activity secondary to her heart condition.,MEDICATION:,  Cylert.,ALLERGIES: , No known drug allergies.,OBJECTIVE:,Vital Signs:  Blood pressure is 124/72.  Temperature 99.2.  Respirations 20 unlabored.  Weight:  137 pounds.,HEENT:  Normocephalic.  Conjunctivae noninjected.  No mattering noted.  Her TMs are bilaterally clear, nonerythematous.  Throat clear, good mucous membrane moisture, but she did have erythema and edema at her posterior soft palate.,Neck:  Supple.  Increased lymphadenopathy noted in the submandibular nodes, but no axillary nodes and no hepatosplenomegaly.,Respiratory:  Clear.  No wheezes, no crackles, no tachypnea, and no retractions.,Cardiovascular:  Regular rate and rhythm.  S1 and S2 normal, no murmur.,Abdomen:  Soft.  No organomegaly.  She did have exquisite tenderness to palpation of the left upper quadrant and flank area, but the spleen was not palpable.  She has no suprapubic tenderness.,Extremities:  She has good range of motion of upper and lower extremities.  Good ambulation.,Her UA was positive for 2+ leukocyte esterase, positive nitrites, 1+ protein, 2+ ketones, 4+ blood, greater than 50 white blood cells, 10-20 rbc’s, and 1+ bacteria.  Culture and sensitivity is pending.  Her Strep test is negative.  Culture is pending.,ASSESSMENT:,1.  Urinary dysuria.,2.  Left flank pain.,3.  Pharyngitis.,PLAN:,  A 1 g of Rocephin IM was given.  Call Dr. B's office tomorrow morning incase a second IM dose is needed.  If not then she will fill a prescription for Omnicef 300 mg capsule 1 p.o. b.i.d. for 10 days total and then we will await the culture and sensitivity results to see if this is appropriate drug.  Push fluids.  Await strep culture report.  Follow up with Dr. XYZ if no better or symptoms worsen.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>general medicine, ear infection, productive-sounding cough, purulent rhinitis, serous otitis, sinusitis, wheezing, ear, amoxicillin,</t>
+          <t xml:space="preserve">general medicine, backache, stomachache, dysuria, cylert, urinary dysuria, pharyngitis, culture and sensitivity, tenderness, urinary, infection, </t>
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>253</v>
+        <v>374</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>General Medicine; short; SOAP-style; diagnoses + symptoms + past history</t>
+          <t>General Medicine; medium; SOAP-style; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J26" s="2" t="n">
-        <v>3362</v>
+        <v>3341</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -2061,21 +2069,21 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>higher</t>
         </is>
       </c>
       <c r="M26" s="2" t="n">
-        <v>0.3677299368800721</v>
+        <v>0.6918958521190262</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; past history; treatment plans; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; past history; treatment plans; follow-up; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="27" ht="110" customHeight="1">
       <c r="A27" s="2" t="n">
-        <v>3375</v>
+        <v>3319</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
@@ -2084,26 +2092,22 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Gen Med Consult - 15 </t>
+          <t xml:space="preserve"> Gen Med H&amp;P - 2 </t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Complaint of mood swings and tearfulness.</t>
+          <t xml:space="preserve"> Weakness, malaise dyspnea on exertion, 15-pound weight loss - Bilateral pneumonia, hepatitis, renal insufficiency, </t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS:,  A 50-year-old female comes to the clinic with complaint of mood swings and tearfulness.  This has been problematic over the last several months and is just worsening to the point where it is impairing her work.  Her boss asks her if she was actually on drugs in which she said no.  She stated may be she needed to be, meaning taking some medications.  The patient had been prescribed Wellbutrin in the past and responded well to it; however, at that time it was prescribed for obsessive-compulsive type disorder relating to overeating and therefore her insurance would not cover the medication.  She has not been on any other antidepressants in the past.  She is not having any suicidal ideation but is having difficulty concentrating, rapid mood swings with tearfulness, and insomnia.  She denies any hot flashes or night sweats.  She underwent TAH with BSO in December of 2003.,FAMILY HISTORY: , Benign breast lump in her mother; however, her paternal grandmother had breast cancer.  The patient denies any palpitations, urinary incontinence, hair loss, or other concerns.  She was recently treated for sinusitis.,ALLERGIES:,  She is allergic to Sulfa.,CURRENT MEDICATIONS:,  Recently finished Minocin and Duraphen II DM.,PHYSICAL EXAMINATION:,General:  A well-developed and well-nourished female, conscious, alert, oriented times three in no acute distress.  Mood is dysthymic.  Affect is tearful.,Skin:  Without rash.,Eyes:  PERRLA.  Conjunctivae are clear.,Neck:  Supple with adenopathy or thyromegaly.,Lungs:  Clear.,Heart:  Regular rate and rhythm without murmur.,ASSESSMENT:,1.  Postsurgical menopause.,2.  Mood swings.,PLAN:,  I spent about 30 minutes with the patient discussing treatment options.  I do believe that her moods would greatly benefit from hormone replacement therapy; however, she is reluctant to do this because of family history of breast cancer.  We will try starting her back on Wellbutrin XL 150 mg daily.  She may increase to 300 mg daily after three to seven days.  Samples provided initially.  If she is not obtaining adequate relief from medication alone, we will then suggest that we explore the use of hormone replacement therapy.  I also recommended increasing her exercise.  We will also obtain some screening lab work including CBC, UA, TSH, chemistry panel, and lipid profile.  Follow up here in two weeks or sooner if any other problems.  She is needing her annual breast exam as well.</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>general medicine, tearfulness, mood swings, menopause, postsurgical menopause, mood swings and tearfulness, hormone replacement therapy, breast cancer, wellbutrin,</t>
-        </is>
-      </c>
+          <t>HISTORY OF PRESENT ILLNESS: , This is a 43-year-old black man with no apparent past medical history who presented to the emergency room with the chief complaint of weakness, malaise and dyspnea on exertion for approximately one month.  The patient also reports a 15-pound weight loss.  He denies fever, chills and sweats.  He denies cough and diarrhea.  He has mild anorexia.,PAST MEDICAL HISTORY:,  Essentially unremarkable except for chest wall cysts which apparently have been biopsied by a dermatologist in the past, and he was given a benign diagnosis.  He had a recent PPD which was negative in August 1994.,MEDICATIONS: , None.,ALLERGIES: , No known drug allergies.,SOCIAL HISTORY: , He occasionally drinks and is a nonsmoker.  The patient participated in homosexual activity in Haiti during 1982 which he described as "very active." Denies intravenous drug use.  The patient is currently employed.,FAMILY HISTORY:,  Unremarkable.,PHYSICAL EXAMINATION:,GENERAL:  This is a thin, black cachectic man speaking in full sentences with oxygen.,VITAL SIGNS:  Blood pressure 96/56, heart rate 120.  No change with orthostatics.  Temperature 101.6 degrees Fahrenheit.  Respirations 30.,HEENT:  Funduscopic examination normal.  He has oral thrush.,LYMPH:  He has marked adenopathy including right bilateral epitrochlear and posterior cervical nodes.,NECK:  No goiter, no jugular venous distention.,CHEST:  Bilateral basilar crackles, and egophony at the right and left middle lung fields.,HEART:  Regular rate and rhythm, no murmur, rub or gallop.,ABDOMEN:  Soft and nontender.,GENITOURINARY:  Normal.,RECTAL:  Unremarkable.,SKIN:  The patient has multiple, subcutaneous mobile nodules on the chest wall that are nontender.  He has very pale palms., ,LABORATORY AND X-RAY DATA: , Sodium 133, potassium 5.3, BUN 29, creatinine 1.8.  Hemoglobin 14, white count 7100, platelet count 515.  Total protein 10, albumin 3.1, AST 131, ALT 31.  Urinalysis shows 1+ protein, trace blood.  Total bilirubin 2.4, direct bilirubin 0.1.  Arterial blood gases:  pH 7.46, pC02 32, p02 46 on room air.  Electrocardiogram shows normal sinus rhythm.  Chest x-ray shows bilateral alveolar and interstitial infiltrates.,IMPRESSION:,1.  Bilateral pneumonia; suspect atypical pneumonia, rule out Pneumocystis carinii pneumonia and tuberculosis.,2.  Thrush.,3.  Elevated unconjugated bilirubins.,4.  Hepatitis.,5.  Elevated globulin fraction.,6.  Renal insufficiency.,7.  Subcutaneous nodules.,8.  Risky sexual behavior in 1982 in Haiti.,PLAN:,1.  Induced sputum, rule out Pneumocystis carinii pneumonia and tuberculosis.,2.  Begin intravenous Bactrim and erythromycin.,3.  Begin prednisone.,4.  Oxygen.,5.  Nystatin swish and swallow.,6.  Dermatologic biopsy of lesions.,7.  Check HIV and RPR.,8.  Administer Pneumovax, tetanus shot and Heptavax if indicated.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="n">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -2112,34 +2116,34 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>General Medicine; medium; consultation; diagnoses + symptoms + medications</t>
+          <t>General Medicine; medium; history and physical; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J27" s="2" t="n">
-        <v>3375</v>
+        <v>3319</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>consultation</t>
+          <t>history and physical</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>higher</t>
         </is>
       </c>
       <c r="M27" s="2" t="n">
-        <v>0.5342087466185753</v>
+        <v>0.8847497745716864</v>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; past history; treatment plans; follow-up; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="28" ht="110" customHeight="1">
       <c r="A28" s="2" t="n">
-        <v>3319</v>
+        <v>3381</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
@@ -2148,22 +2152,22 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Gen Med H&amp;P - 2 </t>
+          <t xml:space="preserve"> Gen Med Consult - 13 </t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Weakness, malaise dyspnea on exertion, 15-pound weight loss - Bilateral pneumonia, hepatitis, renal insufficiency, </t>
+          <t xml:space="preserve"> Consult for hypertension and a med check.  History of osteoarthritis, osteoporosis, hypothyroidism, allergic rhinitis and kidney stones.</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS: , This is a 43-year-old black man with no apparent past medical history who presented to the emergency room with the chief complaint of weakness, malaise and dyspnea on exertion for approximately one month.  The patient also reports a 15-pound weight loss.  He denies fever, chills and sweats.  He denies cough and diarrhea.  He has mild anorexia.,PAST MEDICAL HISTORY:,  Essentially unremarkable except for chest wall cysts which apparently have been biopsied by a dermatologist in the past, and he was given a benign diagnosis.  He had a recent PPD which was negative in August 1994.,MEDICATIONS: , None.,ALLERGIES: , No known drug allergies.,SOCIAL HISTORY: , He occasionally drinks and is a nonsmoker.  The patient participated in homosexual activity in Haiti during 1982 which he described as "very active." Denies intravenous drug use.  The patient is currently employed.,FAMILY HISTORY:,  Unremarkable.,PHYSICAL EXAMINATION:,GENERAL:  This is a thin, black cachectic man speaking in full sentences with oxygen.,VITAL SIGNS:  Blood pressure 96/56, heart rate 120.  No change with orthostatics.  Temperature 101.6 degrees Fahrenheit.  Respirations 30.,HEENT:  Funduscopic examination normal.  He has oral thrush.,LYMPH:  He has marked adenopathy including right bilateral epitrochlear and posterior cervical nodes.,NECK:  No goiter, no jugular venous distention.,CHEST:  Bilateral basilar crackles, and egophony at the right and left middle lung fields.,HEART:  Regular rate and rhythm, no murmur, rub or gallop.,ABDOMEN:  Soft and nontender.,GENITOURINARY:  Normal.,RECTAL:  Unremarkable.,SKIN:  The patient has multiple, subcutaneous mobile nodules on the chest wall that are nontender.  He has very pale palms., ,LABORATORY AND X-RAY DATA: , Sodium 133, potassium 5.3, BUN 29, creatinine 1.8.  Hemoglobin 14, white count 7100, platelet count 515.  Total protein 10, albumin 3.1, AST 131, ALT 31.  Urinalysis shows 1+ protein, trace blood.  Total bilirubin 2.4, direct bilirubin 0.1.  Arterial blood gases:  pH 7.46, pC02 32, p02 46 on room air.  Electrocardiogram shows normal sinus rhythm.  Chest x-ray shows bilateral alveolar and interstitial infiltrates.,IMPRESSION:,1.  Bilateral pneumonia; suspect atypical pneumonia, rule out Pneumocystis carinii pneumonia and tuberculosis.,2.  Thrush.,3.  Elevated unconjugated bilirubins.,4.  Hepatitis.,5.  Elevated globulin fraction.,6.  Renal insufficiency.,7.  Subcutaneous nodules.,8.  Risky sexual behavior in 1982 in Haiti.,PLAN:,1.  Induced sputum, rule out Pneumocystis carinii pneumonia and tuberculosis.,2.  Begin intravenous Bactrim and erythromycin.,3.  Begin prednisone.,4.  Oxygen.,5.  Nystatin swish and swallow.,6.  Dermatologic biopsy of lesions.,7.  Check HIV and RPR.,8.  Administer Pneumovax, tetanus shot and Heptavax if indicated.</t>
+          <t>SUBJECTIVE:,  The patient is a 76-year-old white female who presents to the clinic today originally for hypertension and a med check.  She has a history of hypertension, osteoarthritis, osteoporosis, hypothyroidism, allergic rhinitis and kidney stones.  Since her last visit she has been followed by Dr. Kumar.  Those issues are stable.  She has had no fever or chills, cough, congestion, nausea, vomiting, chest pain, chest pressure.,PAST MEDICAL HISTORY:,  She has an intolerance to Prevacid.,CURRENT MEDICATIONS:,  Evista 60 daily, Levothroid 0.05 mg daily, Claritin 10 daily, Celebrex 200 daily, HCTZ 25 daily and amitriptyline p.r.n.,PAST SURGICAL HISTORY:,  Bilateral mastectomies, tonsillectomy, EGD, flex sig in 2001 and a heart cath.,FAMILY HISTORY: , Father passed away at 81; mother of multiple myeloma at 83.,SOCIAL HISTORY:,  She is married.  A 76-year-old who used to smoke a pack a day and quit in 1985.  She is retired.,REVIEW OF SYSTEMS:,  Essentially negative in HEENT, chest, cardiovascular, GI, GU, musculoskeletal, or neurologic.,OBJECTIVE:,  Temperature is 97.5 degrees.  Blood pressure is 168/70.  Pulse is 88.  Weight is 129 pounds.,GENERAL:  She is an elderly 76-year-old in no acute distress.,HEENT:  Atraumatic.  Extraocular muscles were intact.  Pupils equal, round and reactive to light and accommodation.  Tympanic membranes are clear, dry and intact.  Sinuses and throat are clear.  Neck is soft, supple.  No meningeal signs are present.  No thyromegaly is present.,CHEST:  Clear to auscultation.,CARDIOVASCULAR:  Regular rate and rhythm without murmur.,ABDOMEN:  Soft, nontender.  Bowel sounds are positive.  No organomegaly or peritoneal signs are present.,EXTREMITIES:  Moving all extremities.  Peripheral pulses are normal.  No edema is present.,NEUROLOGIC:  Alert and oriented.  Cranial nerves II-XII grossly intact.  Strength 5+/5 globally.  Reflexes 2+/IV globally.  Romberg is negative.  There is no numbness, tingling, weakness or other neurologic deficit present.,BREASTS:  Surgically absent but there are no lumps, lesions, masses, discharge or adenopathy present.,BACK:  Straight.,SKIN:  Clear.,GENITALIA:  Deferred as she has been followed by Dr. XYZ many times this year.  She does have a history of some elevated cholesterol.,ASSESSMENT:,1.  Hypertension, suboptimal control.,2.  Hypothyroidism.,3.  Arthritis.,4.  Allergic rhinitis.,5.  History of kidney stones.,6.  Osteoporosis.,PLAN:,1.  CBC, complete metabolic profile, UA for hypertension.,2.  Chest x-ray for history of breast cancer.,3.  DEXA scan, full body for osteoporosis.,4.  Flex is up to date.,5.  Pneumovax has been given in the last five years.,6.  Lipid profile for elevated cholesterol.,7.  Refill meds.,8.  Follow up every three to six months for blood pressure check or sooner p.r.n. problems.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="n">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -2172,15 +2176,15 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>General Medicine; medium; history and physical; diagnoses + symptoms + medications</t>
+          <t>General Medicine; medium; SOAP-style; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J28" s="2" t="n">
-        <v>3319</v>
+        <v>3381</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>history and physical</t>
+          <t>SOAP-style</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -2189,17 +2193,17 @@
         </is>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0.8847497745716864</v>
+        <v>0.8136271415689811</v>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; imaging; past history; treatment plans; follow-up; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="29" ht="110" customHeight="1">
       <c r="A29" s="2" t="n">
-        <v>3287</v>
+        <v>3290</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
@@ -2208,35 +2212,35 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> H&amp;P - Gen Med - 2 </t>
+          <t xml:space="preserve"> H&amp;P - Gen Med - 1  </t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> History of diabetes, osteoarthritis, atrial fibrillation, hypertension, asthma, obstructive sleep apnea on CPAP, diabetic foot ulcer, anemia, and left lower extremity cellulitis.</t>
+          <t xml:space="preserve"> An 85-year-old female with diarrhea, vomiting, and abdominal pain.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS:, The patient is a 71-year-old Caucasian female with a history of diabetes, osteoarthritis, atrial fibrillation, hypertension, asthma, obstructive sleep apnea on CPAP, diabetic foot ulcer, anemia and left lower extremity cellulitis. She was brought in by the EMS service to Erlanger emergency department with pulseless electrical activity. Her husband states that he was at home with his wife, when she presented to him complaining of fever and chills. She became acutely unresponsive. She was noted to have worsening of her breathing. She took several of her MDIs and then was placed on her CPAP. He went to notify EMS and when he returned, she was found to not be breathing. He stated that she was noted to have no breathing in excess of 10 minutes. He states that the EMS system arrived at the home and she was found not breathing. The patient was intubated at the scene and upon arrival to Erlanger Medical Center, she was found to have pupils fixed and dilated. She was seen by me in the emergency department and was on Neo-Synephrine, dopamine with a blood pressure of 97/22 with a rapid heart rate and again, in an unresponsive state.,REVIEW OF SYSTEMS:, Review of systems was not obtainable.,PAST MEDICAL HISTORY:, Diabetes, osteoarthritis, hypertension, asthma, atrial fibrillation, diabetic foot ulcer and anemia.,PAST SURGICAL HISTORY:, Noncontributory to above.,FAMILY HISTORY:, Mother with history of coronary artery disease.,SOCIAL HISTORY:, The patient is married. She uses no ethanol, no tobacco and no illicits. She has a very support family unit.,MEDICATIONS:, Augmentin; Detrol LA; lisinopril.,IMMUNIZATIONS:, Immunizations were up to date for influenza, negative for Pneumovax.,ALLERGIES:, PENICILLIN.,LABORATORY AT PRESENTATION:, White blood cell count 11, hemoglobin 10.5, hematocrit 32.2, platelets 175,000. Sodium 148, potassium 5.2, BUN 30, creatinine 2.2 and glucose 216. PT was 22.4.,RADIOLOGIC DATA:, Chest x-ray revealed a diffuse pulmonary edema.,PHYSICAL EXAMINATION:,VITAL SIGNS: Blood pressure 97/52, pulse of 79, respirations 16, O2 sat 100%.,HEENT: The patient's pupils were again, fixed and dilated and intubated on the monitor.,CHEST: Poor air movement bilateral with bilateral rales.,CARDIOVASCULAR: Regular rate and rhythm.,ABDOMEN: The abdomen was obese, nondistended and nontender.,EXTREMITIES: Left diabetic foot had oozing pus drainage from the foot.,GU: Foley catheter was in place.,IMPRESSION AND PLAN:,1. Acute cardiac arrest with pulseless electrical activity with hypotensive shock and respiratory failure: Will continue ventilator support. Will rule out pulmonary embolus, rule out myocardial infarction. Continue pressors. The patient is currently on dopamine, Neo-Synephrine and Levophed.,2. Acute respiratory distress syndrome: Will continue ventilatory support.,3. Questionable sepsis: Will obtain blood cultures, intravenous vancomycin and Rocephin given.,4. Hypotensive shock: Will continue pressors. Will check random cortisol. Hydrocortisone was added.,Further inpatient management for this patient will be provided by Dr. R. The patient's status was discussed with her daughter and her husband. The husband states that his wife has been very ill in the past with multiple admissions, but he had never seen her as severely ill as with this event. He states that she completely was not breathing at all and he is aware of the severity of her illness and the gravity of her current prognosis. Will obtain the assistance with cardiology with this admission and will continue pressors and supportive therapy. The family will make an assessment and final decision concerning her long-term management after a 24 hour period.</t>
+          <t>CHIEF COMPLAINT:, Diarrhea, vomiting, and abdominal pain.,HISTORY OF PRESENT ILLNESS:, The patient is an 85-year-old female who presents with a chief complaint as described above. The patient is a very poor historian and is extremely hard of hearing, and therefore, very little history is available. She was found by EMS sitting on the toilet having diarrhea, and apparently had also just vomited. Upon my questioning of the patient, she can confirm that she has been sick to her stomach and has vomited. She cannot tell me how many times. She is also unable to describe the vomitus. She also tells me that her belly has been hurting. I am unable to get any further history from the patient because, again, she is an extremely poor historian and very hard of hearing.,PAST MEDICAL HISTORY:, Per the ER documentation is hypertension, diverticulosis, blindness, and sciatica.,MEDICATIONS:, Lorazepam 0.5 mg, dosing interval is not noted; Tylenol PM; Klor-Con 10 mEq; Lexapro; calcium with vitamin D.,ALLERGIES:, SHE IS ALLERGIC TO PENICILLIN.,FAMILY HISTORY:, Unknown.,SOCIAL HISTORY:, Also unknown.,REVIEW OF SYSTEMS:, Unobtainable secondary to the patient's condition.,PHYSICAL EXAMINATION:,VITAL SIGNS: Pulse 80. Respiratory rate 18. Blood pressure 130/80. Temperature 97.6.,GENERAL: Elderly black female who is initially sleeping upon my evaluation, but is easily arousable.,NECK: No JVD. No thyromegaly.,EARS, NOSE, AND THROAT: Her oropharynx is dry. Her hearing is very diminished.,CARDIOVASCULAR: Regular rhythm. No lower extremity edema.,GI: Mild epigastric tenderness to palpation without guarding or rebound. Bowel sounds are normoactive.,RESPIRATORY: Clear to auscultation bilaterally with a normal effort.,SKIN: Warm, dry, no erythema.,NEUROLOGICAL: The patient attempts to answer questions when asked, but is very hard of hearing. She is seen to move all extremities spontaneously.,DIAGNOSTIC DATA:, White count 9.6, hemoglobin 15.9, hematocrit 48.2, platelet count 345, PTT 24, PT 13.3, INR 0.99, sodium 135, potassium 3.3, chloride 95, bicarb 20, BUN 54, creatinine 2.2, glucose 165, calcium 10.3, magnesium 2.5, total protein 8.2, albumin 3.8, AST 33, ALT 26, alkaline phosphatase 92. Cardiac isoenzymes negative x1. EKG shows sinus rhythm with a rate of 96 and a prolonged QT interval.,ASSESSMENT AND PLAN:,1. Pancreatitis. Will treat symptomatically with morphine and Zofran, and also IV fluids. Will keep NPO.,2. Diarrhea. Will check stool studies.,3. Volume depletion. IV fluids.,4. Hyperglycemia. It is unknown whether the patient is diabetic. I will treat her with sliding scale insulin.,5. Hypertension. If the patient takes blood pressure medications, it is not listed on the only medication listing that is available. I will prescribe clonidine as needed.,6. Renal failure. Her baseline is unknown. This is at least partly prerenal. Will replace volume with IV fluids and monitor her renal function.,7. Hypokalemia. Will replace per protocol.,8. Hypercalcemia. This is actually rather severe when adjusted for the patient's low albumin. Her true calcium level comes out to somewhere around 12. For now, I will just treat her with IV fluids and Lasix, and monitor her calcium level.,9. Protein gap. This, in combination with the calcium, may be suggestive of multiple myeloma. It is my understanding that the family is seeking hospice placement for the patient right now. I would have to discuss with the family before undertaking any workup for multiple myeloma or other malignancy.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="n">
-        <v>545</v>
+        <v>524</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>General Medicine; long; history and physical; diagnoses + symptoms + medications</t>
+          <t>General Medicine; medium; history and physical; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J29" s="2" t="n">
-        <v>3287</v>
+        <v>3290</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
@@ -2249,17 +2253,17 @@
         </is>
       </c>
       <c r="M29" s="2" t="n">
-        <v>0.8654756537421101</v>
+        <v>0.8744364292155093</v>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; past history; treatment plans; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="30" ht="110" customHeight="1">
       <c r="A30" s="2" t="n">
-        <v>3150</v>
+        <v>3186</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
@@ -2268,39 +2272,39 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Lymph Node Excisional Biopsy </t>
+          <t xml:space="preserve"> Biopsy - Cervical Lymph Node </t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Left axillary lymph node excisional biopsy.  Left axillary adenopathy.</t>
+          <t xml:space="preserve"> Excisional biopsy of right cervical lymph node.</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>PREOPERATIVE DIAGNOSIS: , Left axillary adenopathy.,POSTOPERATIVE DIAGNOSIS: , Left axillary adenopathy.,PROCEDURE: , Left axillary lymph node excisional biopsy.,ANESTHESIA:,  LMA.,INDICATIONS: , Patient is a very pleasant woman who in 2006 had breast conservation therapy with radiation only.  Note, she refused her CMF adjuvant therapy and this was for a triple-negative infiltrating ductal carcinoma of the breast.  Patient has been following with Dr. Diener and Dr. Wilmot.  I believe that genetic counseling had been recommended to her and obviously the CMF was recommended, but she declined both.  She presented to the office with left axillary adenopathy in view of the high-risk nature of her lesion.  I recommended that she have this lymph node removed.  The procedure, purpose, risk, expected benefits, potential complications, alternative forms of therapy were discussed with her and she was agreeable to surgery.,TECHNIQUE: , Patient was identified, then taken into the operating room where after induction of appropriate anesthesia, her left chest, neck, axilla, and arm were prepped with Betadine solution, draped in a sterile fashion.  An incision was made at the hairline, carried down by sharp dissection through the clavipectoral fascia.  I was able to easily palpate the lymph node and grasp it with a figure-of-eight 2-0 silk suture and by sharp dissection, was carried to hemoclip all attached structures.  The lymph node was excised in its entirety.  The wound was irrigated.  The lymph node sent to pathology.  The wound was then closed.  Hemostasis was assured and the patient was taken to recovery room in stable condition.</t>
+          <t>PREOPERATIVE DIAGNOSIS: , Cervical lymphadenopathy.,POSTOPERATIVE DIAGNOSIS:,  Cervical lymphadenopathy.,PROCEDURE: , Excisional biopsy of right cervical lymph node.,ANESTHESIA: , General endotracheal anesthesia.,SPECIMEN: , Right cervical lymph node.,EBL: , 10 cc.,COMPLICATIONS: , None.,FINDINGS:,  Enlarged level 2 lymph node was identified and removed and sent for pathologic examination.,FLUIDS: , Please see anesthesia report.,URINE OUTPUT: , None recorded during the case.,INDICATIONS FOR PROCEDURE: , This is a 43-year-old female with a several-year history of persistent cervical lymphadenopathy.  She reports that it is painful to palpation on the right and has had multiple CT scans as well as an FNA which were all nondiagnostic.  After risks and benefits of surgery were discussed with the patient, an informed consent was obtained.  She was scheduled for an excisional biopsy of the right cervical lymph node.,PROCEDURE IN DETAIL: , The patient was taken to the operating room and placed in the supine position.  She was anesthetized with general endotracheal anesthesia.  The neck was then prepped and draped in the sterile fashion.  Again, noted on palpation there was an enlarged level 2 cervical lymph node.,A 3-cm horizontal incision was made over this lymph node.  Dissection was carried down until the sternocleidomastoid muscle was identified.  The enlarged lymph node that measured approximately 2 cm in diameter was identified and was removed and sent to Pathology for touch prep evaluation.  The area was then explored for any other enlarged lymph nodes.  None were identified, and hemostasis was achieved with electrocautery.  A quarter-inch Penrose drain was placed in the wound.,The wound was then irrigated and closed with 3-0 interrupted Vicryl sutures for a deep closure followed by a running 4-0 Prolene subcuticular suture.  Mastisol and Steri-Strip were placed over the incision, and sterile bandage was applied.  The patient tolerated this procedure well and was extubated without complications and transported to the recovery room in stable condition.  She will return to the office tomorrow in followup to have the Penrose drain removed.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>hematology - oncology, axillary lymph node excisional biopsy, sharp dissection, excisional biopsy, lymph node, axillary, excisional, biopsy</t>
+          <t xml:space="preserve">hematology - oncology, lymphadenopathy, excisional biopsy, fna, mastisol, penrose drain, cervical, cervical lymph node, endotracheal anesthesia, lymph node, sternocleidomastoid, cervical lymph, lymph, anesthesia, </t>
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>249</v>
+        <v>318</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Hematology - Oncology; short; procedure/operative; diagnoses + procedures + treatment plans</t>
+          <t>Hematology - Oncology; medium; procedure/operative; middle text complexity; diagnoses + procedures + imaging</t>
         </is>
       </c>
       <c r="J30" s="2" t="n">
-        <v>3150</v>
+        <v>3186</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
@@ -2309,15 +2313,15 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>middle</t>
         </is>
       </c>
       <c r="M30" s="2" t="n">
-        <v>0.3123872858431019</v>
+        <v>0.5526375112714157</v>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; procedures; treatment plans; surgery</t>
+          <t>diagnoses; procedures; imaging; past history; follow-up; surgery</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2364,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Hematology - Oncology; medium; follow-up/progress; diagnoses + symptoms + laboratory values</t>
+          <t>Hematology - Oncology; medium; follow-up/progress; higher text complexity; diagnoses + symptoms + laboratory values</t>
         </is>
       </c>
       <c r="J31" s="2" t="n">
@@ -2387,7 +2391,7 @@
     </row>
     <row r="32" ht="110" customHeight="1">
       <c r="A32" s="2" t="n">
-        <v>3119</v>
+        <v>3159</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
@@ -2396,62 +2400,58 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Symes Amputation - Hallux </t>
+          <t xml:space="preserve"> Hematology Consult </t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Excision of mass, left second toe and distal Symes amputation, left hallux with excisional biopsy.  Mass, left second toe.  Tumor.  Left hallux bone invasion of the distal phalanx.</t>
+          <t xml:space="preserve"> Leukocytosis, acute deep venous thrombosis, right lower extremity with bilateral pulmonary embolism, on intravenous heparin complicated with acute renal failure for evaluation.</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>PREOPERATIVE DIAGNOSES:,1.  Mass, left second toe.,2.  Tumor.,3.  Left hallux bone invasion of the distal phalanx.,POSTOPERATIVE DIAGNOSES:,1.  Mass, left second toe.,2.  Tumor.,3.  Left hallux with bone invasion of the distal phalanx.,PROCEDURE PERFORMED:,1.  Excision of mass, left second toe.,2.  Distal Syme's amputation, left hallux with excisional biopsy.,HISTORY: , This 47-year-old Caucasian male presents to ABCD General Hospital with a history of tissue mass on his left foot.  The patient states that the mass has been present for approximately two weeks and has been rapidly growing in size.  The patient also has history of shave biopsy in the past.  The patient does state that he desires surgical excision at this time.,PROCEDURE IN DETAIL:,  An IV was instituted by the Department of Anesthesia in the preoperative holding area.  The patient was transported from the operating room and placed on the operating room table in the supine position with the safety belt across his lap.  Copious amount of Webril was placed around the left ankle followed by a blood pressure cuff.  After adequate sedation by the Department of Anesthesia, a total of 6 cc mixed with 1% lidocaine plain with 0.5% Marcaine plain was injected in a digital block fashion at the base of the left hallux as well as the left second toe.,The foot was then prepped and draped in the usual sterile orthopedic fashion.  The foot was elevated from the operating table and exsanguinated with an Esmarch bandage.  Care was taken with the exsanguination to perform exsanguination below the level of the digits so as not to rupture the masses.  The foot was lowered to the operating table.  The stockinet was reflected and the foot was cleansed with wet and dry sponge.  A distal Syme's incision was planned over the distal aspect of the left hallux.  The incision was performed with a #10 blade and deepened with #15 down to the level of bone.  The dorsal skin flap was removed and dissected in toto off of the distal phalanx.  There was noted to be in growth of the soft tissue mass into the dorsal cortex with erosion in the dorsal cortex and exposure of cortical bone at the distal phalanx.  The tissue was sent to Pathology where Dr. Green stated that a frozen sample would be of less use for examining for cancer.  Dr. Green did state that he felt that there was an adequate incomplete excision of the soft tissue for specimen.  At this time, a sagittal saw was then used to resect all ends of bone of the distal phalanx.  The area was inspected for any remaining suspicious tissues.  Any suspicious tissue was removed.  The area was then flushed with copious amounts of sterile saline.  The skin was then reapproximated with #4-0 nylon with a combination of simple and vertical mattress sutures.,Attention was then directed to the left second toe.  There was noted to be a dorsolateral mass over the dorsal distal aspect of the left second toe.  A linear incision was made just medial to the tissue mass.  The mass was then dissected from the overlying skin and off of the underlying capsule.  This tissue mass was hard, round, and pearly-gray in appearance.  It does not invade into any other surrounding tissues.  The area was then flushed with copious amounts of sterile saline and the skin was closed with #4-0 nylon.  Dressings consisted of Owen silk soaked in Betadine, 4x4s, Kling, Kerlix, and an Ace wrap.  The pneumatic ankle tourniquet was released and immediate hyperemic flush was noted to all five digits of the left foot.  The patient tolerated the above procedure and anesthesia well without complications.  The patient was transported to PACU with vital signs stable and vascular status intact.  The patient was given postoperative pain prescription for Vicodin and instructed to follow up with Dr. Bonnani in his office as directed.  The patient will be contacted immediately pending the results of pathology.  Cultures obtained in the case were aerobic and anaerobic gram stain, Silver stain, and a CBC.</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>hematology - oncology, distal phalanx, mass, tumor., hallux bone, phalanx, symes amputation, excisional biopsy, distal, amputation, invasion, toe, symes, incision, flushed, excision, tissue, hallux</t>
-        </is>
-      </c>
+          <t>REASON FOR CONSULTATION:,  Acute deep venous thrombosis, right lower extremity with bilateral pulmonary embolism, on intravenous heparin complicated with acute renal failure for evaluation.,HISTORY OF PRESENTING ILLNESS:  ,Briefly, this is a 36-year-old robust Caucasian gentleman with no significant past medical or surgical history, who works as a sales representative, doing a lot of traveling by plane and car and attending several sales shows, developed acute shortness of breath with an episode of syncope this weekend and was brought in by paramedics to Hospital.  A V/Q scan revealed multiple pulmonary perfusion defects consistent with high probability pulmonary embolism.  A Doppler venous study of the lower extremity also revealed nonocclusive right popliteal vein thrombosis.  A CT of the abdomen and pelvis revealed normal-appearing liver, spleen, and pancreas; however, the right kidney appeared smaller compared to left and suggesting possibility of renal infarct.  Renal function on admission was within normal range; however, serial renal function showed rapid increase in creatinine to 5 today.  He has been on intravenous heparin and hemodialysis is being planned for tomorrow.  Reviewing his history, there is no family members with hypercoagulable state or prior history of any thrombotic complication.  He denies any recent injury to his lower extremity and in fact denied any calf pain or swelling.,PAST MEDICAL AND SURGICAL HISTORY:  ,Unremarkable.,SOCIAL HISTORY: , He is married and has 1 son.  He has a brother who is healthy.  There is no history of tobacco use or alcohol use.,FAMILY HISTORY:,  No family history of hypercoagulable condition.,MEDICATIONS:  ,Advil p.r.n.,ALLERGIES: , NONE.,REVIEW OF SYSTEMS: , Essentially unremarkable except for sudden onset dyspnea on easy exertion complicated with episode of syncope.  He denied any hemoptysis.  He denied any calf swelling or pain.  Lately, he has been traveling and has been sitting behind a desk for a long period of time.,PHYSICAL EXAMINATION:,GENERAL:  He is a robust young gentleman, awake, alert, and hemodynamically stable.,HEENT:  Sclerae anicteric.  Conjunctivae normal.  Oropharynx normal.,NECK:  No adenopathy or thyromegaly.  No jugular venous distention.,HEART:  Regular.,LUNGS:  Bilateral air entry.,ABDOMEN:  Obese and benign.,EXTREMITIES:  No calf swelling or calf tenderness appreciated.,SKIN:  No petechiae or ecchymosis.,NEUROLOGIC:  Nonfocal.,LABORATORY FINDINGS:,  Blood count obtained showed a white count of 16.8, hemoglobin 14.8 g percent, hematocrit 44.6%, MCV 94, and platelet count 209,000.  Liver profile normal.  Thyroid study revealed a TSH of 1.3.  Prothrombin time/INR 1.5, partial thromboplastin time 78.6 seconds.  Renal function, BUN 44 and creatinine 5.7.  Echocardiogram revealed left ventricular hypertrophy with ejection fraction of 65%, no intramural thrombus noted.,IMPRESSION:,1.  Bilateral pulmonary embolism, most consistent with emboli from right lower extremity, on intravenous heparin, rule out hereditary hypercoagulable state.,2.  Leukocytosis, most likely leukemoid reaction secondary to acute pulmonary embolism/renal infarction, doubt presence of myeloproliferative disorder.,3.  Acute renal failure secondary to embolic right renal infarction.,4.  Obesity.,PLAN: , From hematologic standpoint, we will await hypercoagulable studies, which have all been sent on admission to see if a hereditary component is at play.  For now, we will continue intravenous heparin and subsequent oral anticoagulation with Coumadin.  In view of worsening renal function, may need temporary hemodialysis until renal function improves.  I discussed at length with the patient's wife at the bedside.</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="n">
-        <v>660</v>
+        <v>512</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Hematology - Oncology; long; procedure/operative; diagnoses + symptoms + medications</t>
+          <t>Hematology - Oncology; medium; consultation; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J32" s="2" t="n">
-        <v>3119</v>
+        <v>3159</v>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>procedure/operative</t>
+          <t>consultation</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>higher</t>
         </is>
       </c>
       <c r="M32" s="2" t="n">
-        <v>0.5547790802524797</v>
+        <v>0.845299819657349</v>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; procedures; past history; follow-up; surgery</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; imaging; past history; treatment plans; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="33" ht="110" customHeight="1">
       <c r="A33" s="2" t="n">
-        <v>2920</v>
+        <v>2964</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
@@ -2460,39 +2460,39 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CT Head - 2 </t>
+          <t xml:space="preserve"> Carotid Ultrasound </t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The patient is a 79-year-old man with adult hydrocephalus who was found to have large bilateral effusions on a CT scan.  The patient's subdural effusions are still noticeable, but they are improving.</t>
+          <t xml:space="preserve"> Bilateral carotid ultrasound.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>REASON FOR CT SCAN: , The patient is a 79-year-old man with adult hydrocephalus who was found to have large bilateral effusions on a CT scan performed on January 16, 2008.  I changed the shunt setting from 1.5 to 2.0 on February 12, 2008 and his family obtained this repeat CT scan to determine whether his subdural effusions were improving.,CT scan from 03/11/2008 demonstrates frontal horn span at the level of foramen of Munro of 2.6 cm.  The 3rd ventricular contour which is flat with a 3rd ventricular span of 10 mm.  There is a single shunt, which enters on the right occipital side and ends in the left lateral ventricle.  He has symmetric bilateral subdurals that are less than 1 cm in breadth each, which is a reduction from the report from January 16, 2008, which states that he had a subdural hygroma, maximum size 1.3 cm on the right and 1.1 cm on the left.,ASSESSMENT: , The patient's subdural effusions are still noticeable, but they are improving at the setting of 2.0.,PLAN: , I would like to see the patient with a new head CT in about three months, at which time we can decide whether 2.0 is the appropriate setting for him to remain at or whether we can consider changing the shunt setting.</t>
+          <t>EXAM:,  Bilateral carotid ultrasound.,REASON FOR EXAM: , Headache.,TECHNIQUE:  ,Color grayscale and Doppler analysis is employed.,FINDINGS:,  On the grayscale images, the right common carotid artery demonstrates patency with mild intimal thickening only.  At the level of the carotid bifurcation, there is heterogeneous hard plaque present, but without grayscale evidence of greater than 50% stenosis.  Right common carotid waveform is normal with a peak systolic velocity of 0.474 m/second and an end-diastolic velocity of 0.131 m/second.  The right ECA is patent as well with the velocity measurement 0.910 m/second.,The right internal carotid artery at the bifurcation demonstrates plaque formation, but no evidence of greater than 50% stenosis.  Proximal peak systolic velocity in the internal carotid artery is 0.463 m/second with proximal end-diastolic velocity of 0.170.  The mid internal carotid peak systolic velocity is 0.564 m/second, and mid ICA end-diastolic velocity is 0.199 m/second.  Right ICA distal PSV 0.580 m/second, right ICA distal EDV 0.204 m/second.  Vertebral flow is antegrade on the right at 0.469 m/second.,On the left, the common carotid artery demonstrates intimal thickening, but is otherwise patent.  At the level of the bifurcation, however, there is more pronounced plaque formation with approximately 50% stenosis by the grayscale analysis.  See the velocity measurements below:,Left carotid ECA measurement 0.938 m/second.  Left common carotid PSV 0.686 m/second, and left common carotid end-diastolic velocity 0.137 m/second.,Left internal carotid artery again demonstrates prominent focus of hard plaque with up to at least 50% stenosis.  This should be further assessed with CTA for more precise measurement.  The left proximal ICA/PSV 0.955 m/second, left proximal ICA/EDV 0.287 m/second.  There is spectral broadening in the proximal aspect of the carotid waveform.  The left carotid ICA mid PSV 0.895, left carotid ICA mid EDV 0.278 with also spectral broadening present.,The left distal ICA/PSV 0.561, left distal ICA/EDV 0.206, again the spectral broadening present.  Vertebral flow is antegrade at 0.468 m/second.,IMPRESSION: , The study demonstrates bilateral hard plaque at the bifurcation, left greater than right.  There is at least 50% stenosis of the left internal carotid artery at its bifurcation and a followup CTA is recommended for further assessment.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>neurology, ct scan, subdural, adult hydrocephalus, bilateral effusions, shunt setting, subdural effusions, hydrocephalus, ventricular, scan, ct,</t>
+          <t>neurology, doppler analysis, headache, edv, ica, eca, psv, distal ica/edv, hard plaque, bilateral carotid ultrasound, peak systolic velocity, internal carotid artery, plaque formation, carotid ultrasound, carotid artery, carotid, stenosis, proximal, artery, velocity</t>
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>217</v>
+        <v>348</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Neurology; short; diagnostic report; diagnoses + imaging + treatment plans</t>
+          <t>Neurology; medium; diagnostic report; middle text complexity; diagnoses + imaging + treatment plans</t>
         </is>
       </c>
       <c r="J33" s="2" t="n">
-        <v>2920</v>
+        <v>2964</v>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
@@ -2501,21 +2501,21 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>middle</t>
         </is>
       </c>
       <c r="M33" s="2" t="n">
-        <v>0.2989179440937781</v>
+        <v>0.3897655545536519</v>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; imaging; treatment plans; assessment/plan</t>
+          <t>diagnoses; imaging; treatment plans; follow-up</t>
         </is>
       </c>
     </row>
     <row r="34" ht="110" customHeight="1">
       <c r="A34" s="2" t="n">
-        <v>2868</v>
+        <v>2936</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
@@ -2524,62 +2524,62 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Headache - Office Visit </t>
+          <t xml:space="preserve"> Craniotomy - Frontotemporal - 1 </t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The patient with continued problems with her headaches. </t>
+          <t xml:space="preserve"> Acute left subdural hematoma.  Left frontal temporal craniotomy for evacuation of acute subdural hematoma.  CT imaging reveals an acute left subdural hematoma, which is hemispheric.</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>She also had EMG/nerve conduction studies since she was last seen in our office that showed severe left ulnar neuropathy, moderate right ulnar neuropathy, bilateral mild-to-moderate carpal tunnel and diabetic neuropathy.  She was referred to Dr. XYZ and will be seeing him on August 8, 2006.,She was also never referred to the endocrine clinic to deal with her poor diabetes control.  Her last hemoglobin A1c was 10.,PAST MEDICAL HISTORY:,  Diabetes, hypertension, elevated lipids, status post CVA, and diabetic retinopathy.,MEDICATIONS: , Glyburide, Avandia, metformin, lisinopril, Lipitor, aspirin, metoprolol and Zonegran.,PHYSICAL EXAMINATION:,  Blood pressure was 140/70, heart rate was 76, respiratory rate was 18, and weight was 226 pounds.  On general exam she has an area of tenderness on palpation in the left parietal region of her scalp.  Neurological exam is detailed on our H&amp;P form.  Her neurological exam is within normal limits.,IMPRESSION AND PLAN:,  For her headaches we are going to titrate Zonegran up to 200 mg q.h.s. to try to maximize the Zonegran therapy.  If this is not effective, when she comes back on August 7, 2006 we will then consider other anticonvulsants such as Neurontin or Lyrica.  We also discussed with Ms. Hawkins the possibility of nerve block injection; however, at this point she is not interested.,She will be seeing Dr. XYZ for her neuropathies.,We made an appointment in endocrine clinic today for a counseling in terms of better diabetes control and she is responsible for trying to get her referral from her primary care physician to go for this consult.</t>
+          <t>PREOPERATIVE DIAGNOSIS:,  Acute left subdural hematoma.,POSTOPERATIVE DIAGNOSIS:,  Acute left subdural hematoma.,PROCEDURE:,  Left frontal temporal craniotomy for evacuation of acute subdural hematoma.,DESCRIPTION OF PROCEDURE: , This is a 76-year-old man who has a history of acute leukemia.  He is currently in the phase of his therapy where he has developed a profound thrombocytopenia and white cell deficiency.  He presents after a fall in the hospital in which he apparently struck his head and now has a progressive neurologic deterioration consistent with an intracerebral injury.  His CT imaging reveals an acute left subdural hematoma, which is hemispheric.,The patient was brought to the operating room, placed under satisfactory general endotracheal anesthesia.  He had previously been intubated and taken to the Intensive Care Unit and now is brought for emergency craniotomy.  The images were brought up on the electronic imaging and confirmed that this was a left-sided condition.  He was fixed in a three-point headrest.  His scalp was shaved and prepared with Betadine, iodine and alcohol.  We made a small curved incision over the temporal, parietal, frontal region.  The scalp was reflected.  A single bur hole was made at the frontoparietal junction and then a 4x6cm bur hole was created.  After completing the bur hole flap, the dura was opened and a gelatinous mass of subdural was peeled away from the brain.  The brain actually looked relatively relaxed; and after removal of the hematoma, the brain sort of slowly came back up.  We investigated the subdural space forward and backward as we could and yet careful not to disrupt any venous bleeding as we close to the midline.  After we felt that we had an adequate decompression, the dura was reapproximated and we filled the subdural space with saline.  We placed a small drain in the extra dural space and then replaced the bone flap and secured this with the bone plates.  The scalp was reapproximated, and the patient was awakened and taken to the CT scanner for a postoperative scan to ensure that there was no new hemorrhage or any other intracerebral pathology that warranted treatment.  Given that this actual skin looked good with apparent removal of about 80% of the subdural we elected to take patient to the Intensive Care Unit for further management.,I was present for the entire procedure and supervised this.  I confirmed prior to closing the skin that we had correct sponge and needle counts and the only foreign body was the drain.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>neurology, nerve conduction studies, emg, zonegran therapy, ulnar neuropathy, endocrine clinic, diabetes control, neurological exam, headache, zonegran</t>
+          <t xml:space="preserve">neurology, subdural, hematoma, temporal craniotomy, craniotomy, subdural space, bur hole, subdural hematoma, </t>
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>252</v>
+        <v>404</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Neurology; short; follow-up/progress; diagnoses + medications + laboratory values</t>
+          <t>Neurology; medium; procedure/operative; lower text complexity; diagnoses + procedures + imaging</t>
         </is>
       </c>
       <c r="J34" s="2" t="n">
-        <v>2868</v>
+        <v>2936</v>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>follow-up/progress</t>
+          <t>procedure/operative</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="M34" s="2" t="n">
-        <v>0.4283701532912534</v>
+        <v>0.3485685302073941</v>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; medications; laboratory values; vital signs; past history; treatment plans; follow-up; assessment/plan</t>
+          <t>diagnoses; procedures; imaging; past history; treatment plans; surgery</t>
         </is>
       </c>
     </row>
     <row r="35" ht="110" customHeight="1">
       <c r="A35" s="2" t="n">
-        <v>2964</v>
+        <v>2756</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
@@ -2588,26 +2588,26 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Carotid Ultrasound </t>
+          <t xml:space="preserve"> Wilson's Disease - Letter </t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Bilateral carotid ultrasound.</t>
+          <t xml:space="preserve"> A pleasant gentleman with a history of Wilson's disease who has been treated with penicillamine.</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>EXAM:,  Bilateral carotid ultrasound.,REASON FOR EXAM: , Headache.,TECHNIQUE:  ,Color grayscale and Doppler analysis is employed.,FINDINGS:,  On the grayscale images, the right common carotid artery demonstrates patency with mild intimal thickening only.  At the level of the carotid bifurcation, there is heterogeneous hard plaque present, but without grayscale evidence of greater than 50% stenosis.  Right common carotid waveform is normal with a peak systolic velocity of 0.474 m/second and an end-diastolic velocity of 0.131 m/second.  The right ECA is patent as well with the velocity measurement 0.910 m/second.,The right internal carotid artery at the bifurcation demonstrates plaque formation, but no evidence of greater than 50% stenosis.  Proximal peak systolic velocity in the internal carotid artery is 0.463 m/second with proximal end-diastolic velocity of 0.170.  The mid internal carotid peak systolic velocity is 0.564 m/second, and mid ICA end-diastolic velocity is 0.199 m/second.  Right ICA distal PSV 0.580 m/second, right ICA distal EDV 0.204 m/second.  Vertebral flow is antegrade on the right at 0.469 m/second.,On the left, the common carotid artery demonstrates intimal thickening, but is otherwise patent.  At the level of the bifurcation, however, there is more pronounced plaque formation with approximately 50% stenosis by the grayscale analysis.  See the velocity measurements below:,Left carotid ECA measurement 0.938 m/second.  Left common carotid PSV 0.686 m/second, and left common carotid end-diastolic velocity 0.137 m/second.,Left internal carotid artery again demonstrates prominent focus of hard plaque with up to at least 50% stenosis.  This should be further assessed with CTA for more precise measurement.  The left proximal ICA/PSV 0.955 m/second, left proximal ICA/EDV 0.287 m/second.  There is spectral broadening in the proximal aspect of the carotid waveform.  The left carotid ICA mid PSV 0.895, left carotid ICA mid EDV 0.278 with also spectral broadening present.,The left distal ICA/PSV 0.561, left distal ICA/EDV 0.206, again the spectral broadening present.  Vertebral flow is antegrade at 0.468 m/second.,IMPRESSION: , The study demonstrates bilateral hard plaque at the bifurcation, left greater than right.  There is at least 50% stenosis of the left internal carotid artery at its bifurcation and a followup CTA is recommended for further assessment.</t>
+          <t>Doctor's Address,Dear Doctor:,This letter is an introduction to my patient, A, who you will be seeing in the near future.  He is a pleasant gentleman with a history of Wilson's disease.  It has been treated with penicillamine.  He was diagnosed with this at age 14.  He was on his way to South Carolina for a trip when he developed shortness of breath, palpitations, and chest discomfort.  He went to the closest hospital that they were near in Randolph, North Carolina and he was found to be in atrial fibrillation with rapid rate.  He was admitted there and observed.  He converted to normal sinus rhythm spontaneously and so he required no further interventions.  He was started on Lopressor, which he has tolerated well.  An echocardiogram was performed, which revealed mild-to-moderate left atrial enlargement.  Normal ejection fraction.  No other significant valvular abnormality.  He reported to physicians there that he had cirrhosis related to his Wilson's disease.  Therefore hepatologist was consulted.  There was a recommendation to avoid Coumadin secondary to his questionable significant liver disease, therefore he was placed on aspirin 325 mg once a day.,In discussion with Mr. A and review of his chart that I have available, it is unclear as to the status of his liver disease, however, he has never had a liver biopsy, so his diagnosis of cirrhosis that they were concerned about in North Carolina is in doubt.  His LFTs have remained normal and his copper level has been undetectable on his current dose of penicillamine.,I would appreciate your input into the long term management of his anticoagulation and also any recommendations you would have about rhythm control.  He is in normal sinus rhythm as of my evaluation of him on 06/12/2008.  He is tolerating his metoprolol and aspirin without any difficulty.  I guess the big question remains is what level of risk that is entailed by placing him on Coumadin therapy due to his potentially paroxysmal atrial fibrillation and evidence of left atrial enlargement that would place him in increased risk of recurrent episodes.,I appreciate your input regarding this friendly gentleman.  His current medicines include penicillamine 250 mg p.o. four times a day, metoprolol 12.5 mg twice a day, and aspirin 325 mg a day.,If you have any questions regarding his care, please feel free to call me to discuss his case.  Otherwise, I will look forward to hearing back from you regarding his evaluation.  Thank you as always for your care of our patient.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>neurology, doppler analysis, headache, edv, ica, eca, psv, distal ica/edv, hard plaque, bilateral carotid ultrasound, peak systolic velocity, internal carotid artery, plaque formation, carotid ultrasound, carotid artery, carotid, stenosis, proximal, artery, velocity</t>
+          <t>neurology, atrial enlargement, wilson's disease, penicillamine,</t>
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>348</v>
+        <v>409</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
@@ -2616,34 +2616,34 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Neurology; medium; diagnostic report; diagnoses + imaging + treatment plans</t>
+          <t>Neurology; medium; other narrative/sectioned; lower text complexity; diagnoses + medications + procedures</t>
         </is>
       </c>
       <c r="J35" s="2" t="n">
-        <v>2964</v>
+        <v>2756</v>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>diagnostic report</t>
+          <t>other narrative/sectioned</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="M35" s="2" t="n">
-        <v>0.3897655545536519</v>
+        <v>0.3789449954914337</v>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; imaging; treatment plans; follow-up</t>
+          <t>diagnoses; medications; procedures; imaging; past history; treatment plans</t>
         </is>
       </c>
     </row>
     <row r="36" ht="110" customHeight="1">
       <c r="A36" s="2" t="n">
-        <v>2796</v>
+        <v>2946</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
@@ -2652,35 +2652,35 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Neurologic Consultation - 5 </t>
+          <t xml:space="preserve"> Consult - Migraine </t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Approximately one and a half years ago, patient fell down while walking in the living room from the bedroom.  At that time, he reports both legs gave away on him and he fell.  He reported that he had some lightheadedness just before he fell and was slightly confused, but was aware of what was happening around him.</t>
+          <t xml:space="preserve"> The patient is a 36-year-old female with past medical history of migraine headaches, who was brought to the ER after she was having uncontrolled headaches.  In the ER, the patient had a CT scan done, which was reported negative, and lumbar puncture with normal pressure and the cell count, and was admitted for followup.</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS: ,The patient is a 79-year-old right-handed man who reports that approximately one and a half years ago, he fell down while walking in the living room from the bedroom.  At that time, he reports both legs gave away on him and he fell.  He reported that he had some lightheadedness just before he fell and was slightly confused, but was aware of what was happening around him.  He was able to get up shortly after falling and according to the patient and his son, subsequently returned back to normal.,He was then well until the 3rd of July 2008 when his legs again gave way on him.  This was not preceded by lightheadedness.  He was rushed to the hospital and was found to have pneumonia, and the fall was blamed on the pneumonia.  He started using a walker from that time, prior to that he was able to walk approximately two miles per day.  He again had a fall in August of 2008 after his legs gave way.  Again, there was no lightheadedness associated with this.  He was again found to have pneumonia and again was admitted to hospital after which he went to rehabilitation and was able to use his walker again after this.  He did not, however, return to the pre-July baseline.  In October of 2008, after another fall, he was found to have pneumonia again and shingles.  He is currently in a Chronic Rehabilitation Unit.  He cannot use a walker and uses a wheelchair for everything.  He states that his hands have been numb, involving all the fingers of both hands for the past three weeks.  He is also losing muscle bulk in his hands and has noticed some general weakness of his hands.  He does, however, note that strength in his hands has not been normal since July 2008, but it is clearly getting worse.  He has been aware of some fasciculations in his legs starting in August 2008, these are present both in the lower legs and the thighs.  He does not report any cramps, problems with swallowing or problems with breathing.  He reports that he has had constipation alternating with diarrhea, although there has been no loss of control of either his bowel or bladder.  He has had some problems with blood pressure drops, and does feel presyncopal when he stands.  He also reports that he has no feeling in his feet, and that his feet feel like sponges.  This has been present for about nine months.  He has also lost joint position sense in his feet for approximately nine months.,PAST MEDICAL HISTORY:,1.  Pneumonia.  He has had recurrent episodes of pneumonia, which started at approximately age 20.  These have been treated repeatedly over the years, and on average he has tended to have an episode of pneumonia once every five years, although this has been far more frequent in the past year.  He is usually treated with antibiotics and then discharged.  There is no known history of bronchiectasis, inherited lung disease or another chronic pulmonary cause for the repeated pneumonia.,2.  He has had a catheter placed for urinary retention, his urologist has told him that he thinks that this may be due to prostate enlargement.  The patient does not have any history of diabetes and does not report any other medical problems.  He has lost approximately 18 pounds in the past month.,3.  He had an appendectomy in the 1940s.,4.  He had an ankle resection in 1975.,SOCIAL HISTORY:  ,The patient stopped smoking 27 years ago, he smoked approximately two packs a day with combined cigarettes and cigars.  He has not smoked for the past 27 years.  He hardly ever uses alcohol.  He is currently retired.,FAMILY HISTORY: , There is no family history of neuropathy, pes cavus, foot deformities, or neuromuscular diseases.  His aunt has a history of type II diabetes.,CURRENT MEDICATIONS: , Fludrocortisone 0.1 mg p.o. q.d., midodrine 5 mg p.o. q.i.d., Cymbalta 30 mg p.o. per day, Prilosec 20 mg p.o. per day, Lortab 10 mg p.o. per day, Amoxil 500 mg p.o. per day, vitamin B12 1000 mcg weekly, vitamin D 1000 units per day, Metamucil p.r.n., enteric-coated aspirin once a day, Colace 200 mg p.o. q.d., Senokot three tablets p.o. p.r.n., Reglan 10 mg p.o. q.6h., Xanax 0.25 mg p.o. q.8h. p.r.n., Ambien 5 mg p.o. q.h.s. p.r.n. and Dilaudid 2 mg tablets p.o. q.3h. p.r.n., Protonix 40 mg per day, and Megace 400 mg per day.,ALLERGIES:,  He has no medication or food allergies.,REVIEW OF SYSTEMS:,  Please see the health questionnaire and clinical notes from today.,GENERAL PHYSICAL EXAMINATION:,VITAL SIGNS:  BP was 137/60, P was 89, and his weight could not be measured because he was in a wheelchair.  His pain score was 0.,APPEARANCE:  No acute distress.  He is pleasant and well-groomed.,HEENT:  Atraumatic, normocephalic.  No carotid bruits appreciated.,LUNGS:  There were few coarse crackles in both lung bases.,CARDIOVASCULAR:  Revealed a normal first and second heart sound, with no third or fourth heart sound and no murmurs.  The pulse was regular and of normal volume.,ABDOMEN:  Soft with no masses and normal bowel sounds.  There were no carotid bruits.,EXTREMITIES:  No contractures appreciated.,NEUROLOGICAL EXAM:,MSE:  His orientation, language, calculations, 100-7 tests were all normal.  There was atrophy and fasciculations in both the arms and legs.,CRANIAL NERVES:  Cranial nerve examination was normal with the exception that there was some mild atrophy of his tongue and possible fasciculations.  His palatal movement was normal and gag reflex was normal.,MOTOR:  Strength was decreased in all muscle groups as follows:  Deltoid 4/4, biceps 4+/4+, triceps 5/5, wrist extensors 4+/4+, finger extensors 4-/4-, finger flexors 4-/4-, interossei 4-/4-, hip flexors 4+/4+, hip extensors 4+/4+, knee extensors 4/4, and knee flexors 4/4.  Foot dorsiflexion, plantar flexion, eversion, toe extension and toe flexion was all 0 to 1.  There was atrophy in both hands and general atrophy of the lower limb muscles.  The feet were both cold and showed dystrophic features.  Fasciculations were present mainly in the hands.  There was evidence of dysmetria and past pointing in the left hand.,REFLEXES:  Reflexes were 0 in all sites in the arms and legs.  The jaw reflex was 2+.  Vibration was severely decreased at the elbow and wrist and was absent in the fingers.  Vibration was absent in the toes and ankle bilaterally and was severely decreased at the knee.  Joint position sense was absent in the toes and severely decreased in the fingers.  Pin perception was absent in the feet and was decreased to the upper thighs.  Pin was decreased or absent in the fingers and decreased above the elbows.  The same distribution of sensory loss was found with monofilament testing.,COORDINATION:  Coordination was barely normal in the right hand.  Rapid alternating movements were decreased in the left hand greater than the right hand.  The patient was unable to stand and therefore gait, Romberg's test and balance could not be assessed.,DIAGNOSTIC STUDIES: , Previous diagnostic studies and patient reports.  There were extensive patient reports, all of which were reviewed.  A previous x-ray study of the lateral chest performed in October 2008 showed poor inspiration with basilar atelectasis and an infiltrate.  An x-ray of the cervical, thoracic and lumbar spine showed some evidence of lumbar spinal stenosis.  A CTA of the neck with and without contrast performed in November 2008 showed minor stenosis in the left carotid, a mild hard and soft plaque in the right carotid with approximately 55% stenosis.  The posterior circulation showed a slightly dominant right vertebral artery with no stenosis.  There was no significant stenosis, but there was minor extracranial stenosis noted.  An MRI of the brain with and without contrast performed in November 2008 showed no evidence of an acute infarct, major vascular occlusion, and no abnormal enhancement with gadolinium administration.  There was also no significant sinusitis or mastoiditis.  This was an essentially normal brain MRI.  A CBC performed in January 2009 showed an elevated white cell count of 11.3, a low red cell count of 3.43, elevated MCH of 32.4 and the rest of the study was normal.  An electrolyte study performed in January 2009 showed a sodium which was low at 127, a calcium which was low at 8.3, and a low protein of 5.2 and albumin of 3.1.  The glucose was 86.  TSH performed in January 2009 was 1.57, which is within the normal range.  Vitamin B12 was greater than a 1000, which is normal and the folate was 18.2, which was normal.  A myocardial stress study performed in December 2008 showed normal myocardial perfusion with Persantine Cardiolite SPECT.  The ECG was non-diagnostic.  There was normal regional wall motion of the left ventricle.  The left ventricular ejection fraction was 68%, which is within the normal range for males.  A CT of the lumbar spine without contrast performed in December 2008 showed a broad-based disc bulge at L1-L2, L2-L3, L3-L4 and L4-L5.  At L5-S1, in addition to the broad-based disc bulge, there was also an osteophyte complex and evidence of flavum hypertrophy without canal stenosis.  There was severe bilateral neural foraminal stenosis at L5-S1 and moderate neural foraminal stenosis at L1-L4.  An echocardiogram was performed in November 2008 and showed mild left atrial enlargement, normal left ventricular systolic function, mild concentric left ventricular hypertrophy, scleral degenerative changes in the aortic and mitral apparatus, mild mitral regurgitation, mild tricuspid regurgitation and mild to moderate aortic regurgitation.,DIAGNOSTIC IMPRESSION:  ,The patient presents with a severe neuropathy with marked large fiber sensory as well as motor findings.  He is diffusely weak as well as atrophic in all muscle groups both in his upper and lower extremities, although he is disproportionately weak in his lower extremities.  His proprioceptive and vibratory loss is severe in both the distal upper and lower extremities, signifying that he either has a severe sensory neuropathy or has involvement of the dorsal root ganglia.  According to the history, which was carefully checked, the initial onset of these symptoms goes back one and a half years, although there has only been significant progression in his condition since July 2008.  As indicated below, further diagnostic studies including a detailed nerve conduction and EMG test today showed evidence of a severe sensory, motor, and axonal neuropathy and in addition there was evidence of a diffuse polyradiculopathy.  There was no involvement of the tongue on EMG.  The laboratory testing as indicated below failed to show a specific cause for the neuropathy.  We are still, however, waiting for the paraneoplastic antibodies, which were send out lab to the Mayo Clinic.  This type of very severe sensorimotor neuropathy with significant proprioceptive loss may be seen in several conditions including peripheral nerve vasculitis due to a variety of disorders such as SLE, Sjogren's, rheumatoid arthritis, and mixed connective tissue disease.  In addition, it may also be seen with certain toxins, particularly chemotherapeutic agents.  The patient did not receive any of these.  It may also be seen as part of a paraneoplastic syndrome.  Although the patient does not have any specific clinical symptoms of a cancer, it is noted that he has had an 18-pound weight loss in the past month and does have a remote history of smoking.  We have requested that he obtain a CT of his chest, abdomen and pelvis while he is in Acute Rehabilitation.  The verbal reports of these possibly did not show any evidence of a cancer.  We did also request that he obtain a gallium scan to see if there was any evidence of an unsuspected neoplasm.  The patient did undergo a nerve and muscle biopsy, this was a radial nerve and biceps muscle biopsy from the left arm.  This showed evidence of severe axonal loss.  There was no evidence of a vasculitis.  The vessels did show some mild intimal changes that would be consistent with atherosclerosis.  There were a few perivascular changes; however, there was no clear evidence of a necrotizing vasculitis even on multiple sections.  The muscle biopsy showed severe muscle fiber atrophy, with evidence of fiber grouping.  Again, there was no evidence of inflammation or vasculitis.  Evaluation so far has also shown no evidence of an amyloid neuropathy, no evidence of a monoclonal gammopathy, of sarcoidosis, and again there is no past history of a significant toxin or infective cause for the neuropathy.  Specifically, there is no history of HIV exposure.  We would await the results of the gallium scan and of the paraneoplastic antibodies to see if these are helpful in making a diagnosis.  At this point, because of the severity and the axonal nature of the neuropathy, there is no specific therapy that will reverse the course of the illness, unless we find a specific etiology that can be stopped or reversed.  I have discussed these issues at length with the patient and with his son.  We also addressed whether or not there might be a previously undiagnosed inherited neuropathy.  I think this is unlikely given the short history and the rapid progression of the disorder.,There is also no family history that we can detect a neuropathy, and the patient does not have the typical phenotype for a chronic inherited neuropathy such as Charcot-Marie-Tooth disease type 2.  However, since I have only seen the patient on one occasion and do not know what his previous examination showed two years ago, I cannot be certain that there may not have been the presence of a neuropathy preceding this.,PLAN:,1.  Nerve conduction and EMG will be performed today.  The results were indicated above.,2.  The following laboratory studies were requested including electrolytes, CBC, thyroid function tests, B12, ANA, C-reactive protein, complement, cryoglobulins, double-stranded DNA antibodies, folate level, hemoglobin A1c, immunofixation electrophoresis, P-ANCA, C-ANCA, protein electrophoresis, rheumatoid factor, paraneoplastic antibody studies requested from the Mayo Clinic, B12.  These studies showed minor changes, which included a low sodium level of 129 as previously noted, a low creatinine of 0.74, low calcium of 8.6, low total protein of 5.7.  The B12 was greater than 2000.  The immunoelectrophoresis, ANA, double-stranded DNA, ANCA, hemoglobin A1c, folate, cryoglobulins, complement, C-reactive protein were all normal or negative.  The B12 level was greater than 2000.  Liver function tests were normal.  The glucose was 90.  ESR was 10.  Hemoglobin A1c was 5.5.,3.  A left radial sensory and left biceps biopsy were requested and have been performed and interpreted as indicated above.,4.  CT of chest, abdomen and pelvis.,5.  Whole body gallium scan for evidence of an underlying neoplasm.,6.  The patient will go to the Rehabilitation Facility for Acute Rehabilitation and Training.,7.  We have not made any changes to his medication.  He does have some mild orthostatic changes; however, he is adequately controlled with midodrine at a dose of 2.5 mg three times a day as needed up to 5 mg four times a day.  Usually, he uses a lower dose of 2.5 three times a day to 5 mg three times a day.,8.  Followup will be as determined by the family.</t>
+          <t>HISTORY OF PRESENT ILLNESS: , The patient is a 36-year-old female with past medical history of migraine headaches, who was brought to the ER after she was having uncontrolled headaches.  In the ER, the patient had a CT scan done, which was reported negative, and lumbar puncture with normal pressure and the cell count, and was admitted for followup.  Neurology consult was called to evaluate the patient in view of the current symptomatology.  The headaches were refractory to the treatment.  The patient has been on Topamax and Maxalt in the past, but did not work and according to the patient she got more confused.,PAST MEDICAL HISTORY: , History of migraine.,PAST SURGICAL HISTORY:  ,Significant for partial oophorectomy, appendectomy, and abdominoplasty.,SOCIAL HISTORY:  ,No history of any smoking, alcohol, or drug abuse.  The patient is a registered nurse by profession.,MEDICATIONS: , Currently taking no medication.,ALLERGIES: , No known allergies.,FAMILY HISTORY:,  Nothing significant.,REVIEW OF SYSTEMS: , The patient was considered to ask systemic review including neurology, psychiatry, sleep, ENT, ophthalmology, pulmonary, cardiology, gastroenterology, genitourinary, hematology, rheumatology, dermatology, allergy, immunology, endocrinology, toxicology, oncology, and was found to be positive for the symptoms mentioned in the history of the presenting illness.,PHYSICAL EXAMINATION,VITAL SIGNS:  Blood pressure of 115/66, heart rate of 69, respiratory rate of 13, temperature normal, and pulse oximetry 98% on room air at the time of initial evaluation.,HEENT:  Head, normocephalic, atraumatic.  Neck supple.  Throat clear.  No discharge from the ears or nose.  No discoloration of conjunctivae and sclerae.  No bruits auscultated over temple, orbits, or the neck.,LUNGS:  Clear to auscultation.,CARDIOVASCULAR:  Normal heart sounds.,ABDOMEN:  Benign.,EXTREMITIES:  No edema, clubbing or cyanosis.,SKIN:  No rash.  No neurocutaneous disorder.,MENTAL STATUS:  The patient is awake, alert and oriented to place and person.  Speech is fluent.  No language deficits.  Mood normal.  Affect is clear.  Memory and insight is normal.  No abnormality with thought processing and thought content.  Cranial nerve examination intact II through XII.  Motor examination:  Normal bulk, tone and power.  Deep tendon reflexes symmetrical.  Downgoing toes.  No sign of any myelopathy.  Cortical sensation intact.  Peripheral sensation grossly intact.  Vibratory sense not tested.  Gait not tested.  Coordination is normal with no dysmetria.,IMPRESSION: , Intractable headaches, by description to be migraines.  Complicated migraines by clinical criteria.  Rule out sinusitis.  Rule out vasculitis including temporal and arthritis, lupus, polyarthritis, moyamoya disease, Takayasu and Kawasaki disease.,PLAN AND RECOMMENDATIONS: , The patient to be given a trial of the prednisone with a plan to taper off in 6 days, as she already had received 50 mg today.  Depakote as a part of migraine prophylaxis and Fioricet on p.r.n. basis.,The patient to get vasculitis workup, as it has not been ordered by the primary care physician initially.  The patient already had MRI of the brain and the cervical spine.  MRI of the brain reported negative and cervical spine as shown signs of disk protrusion at C5 and C6 level, which will not explain of the temporal headache.  Plan and followup discussed with the patient in detail.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="2" t="n">
-        <v>2460</v>
+        <v>490</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Neurology; long; consultation; diagnoses + symptoms + medications</t>
+          <t>Neurology; medium; consultation; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J36" s="2" t="n">
-        <v>2796</v>
+        <v>2946</v>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
@@ -2693,17 +2693,17 @@
         </is>
       </c>
       <c r="M36" s="2" t="n">
-        <v>0.9954350766456268</v>
+        <v>0.7585099188458071</v>
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; imaging; past history; treatment plans; follow-up; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; imaging; past history; treatment plans; follow-up; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="37" ht="110" customHeight="1">
       <c r="A37" s="2" t="n">
-        <v>2270</v>
+        <v>2359</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
@@ -2712,56 +2712,52 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Closed Reduction - 1 </t>
+          <t xml:space="preserve"> Ankle Sprain - H&amp;P </t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Right distal both-bone forearm fracture.  Closed reduction under conscious sedation and application of a splint was warranted.</t>
+          <t xml:space="preserve"> History and Physical for right ankle sprain</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>PREOPERATIVE DIAGNOSIS: , Right distal both-bone forearm fracture.,POSTOPERATIVE DIAGNOSIS: , Right distal both-bone forearm fracture.,INDICATIONS:,  Mr. ABC is a 10-year-old boy who suffered a fall resulting in a right distal both-bone forearm fracture.  Upon evaluation by Orthopedic Surgery team in the emergency department, it was determined that a closed reduction under conscious sedation and application of a splint was warranted.  This was discussed with the parents who expressed verbal and written consent.,PROCEDURE:,  Conscious sedation was achieved via propofol via the emergency department staff.  Afterwards, traction with re-creation of the injury pattern was utilized to achieve reduction of the patient's fracture.  This was confirmed with image intensifier.  Subsequently, the patient was placed into a splint.  The patient was aroused from conscious sedation and at this time it was noted that he had full sensation throughout radial, median, and ulnar nerve distributions and positive extensor pollicis longus, flexor pollicis longus, dorsal and palmar interossei.,DISPOSITION:  ,Post-reduction x-rays revealed good alignment in the AP x-rays.  The lateral x-rays also revealed adequate reduction.  At this time, we will allow the patient to be discharged home and have him follow up with Dr. XYZ in one week.</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">orthopedic, closed reduction, distal both bone forearm, emergency department, pollicis longus, bone forearm, forearm fracture, conscious sedation, emergency, department, pollicis, longus, splint, distal, bone, forearm, conscious, sedation, fracture, reduction, </t>
-        </is>
-      </c>
+          <t>CHIEF COMPLAINT:,  Right ankle sprain.,HISTORY OF PRESENT ILLNESS: , This is a 56-year-old female who fell on November 26, 2007 at 11:30 a.m. while at work.  She did not recall the specifics of her injury but she thinks that her right foot inverted and subsequently noticed pain in the right ankle.  She describes no other injury at this time.,PAST MEDICAL HISTORY: , Hypertension and anxiety.,PAST SURGICAL HISTORY: , None.,MEDICATIONS: , She takes Lexapro and a blood pressure pill, but does not know anything more about the names and the doses.,ALLERGIES:,  No known drug allergies.,SOCIAL HISTORY: , The patient lives here locally.  She does not report any significant alcohol or illicit drug use.  She works full time.,FAMILY HISTORY:,  Noncontributory.,REVIEW OF SYSTEMS:,Pulm:  No cough, No wheezing, No shortness of breath,CV:  No chest pain or palpitations,GI:  No abdominal pain.  No nausea, vomiting, or diarrhea.,PHYSICAL EXAM:,GENERAL APPEARANCE:  No acute distress,VITAL SIGNS:  Temperature 97.8, blood pressure 122/74, heart rate 76, respirations 24, weight 250 lbs, O2 sat 95% on R.A.,NECK:  Supple.  No lymphadenopathy.  No thyromegaly.,CHEST:  Clear to auscultation bilaterally.,HEART:  Regular rate and rhythm.  No murmurs.,ABDOMEN:  Non-distended, nontender, normal active bowel sounds.,EXTREMITIES:  No Clubbing, No Cyanosis, No edema.,MUSCULOSKELETAL:  The spine is straight and there is no significant muscle spasm or tenderness there.  Both knees appear to be non-traumatic with no deformity or significant tenderness.  The right ankle has some swelling just below the right lateral malleolus and the dorsum of the foot is tender.  There is decreased range of motion and some mild ecchymosis noted around the ankle.,DIAGNOSTIC DATA: , X-ray of the right ankle reveals no acute fracture by my observation.  Radiologic interpretation is pending., ,IMPRESSION:,  Right ankle sprain.,PLAN:,1.  Motrin 800 mg t.i.d.,2.  Tylenol 1 gm q.i.d. as needed.,3.  Walking cast is prescribed.,4.  I told the patient to call back if any problems.  The next morning she called back complaining of worsening pain and I called in some Vicodin ES 1-2 p.o. q.  8 hours p.r.n. pain #60 with no refills.</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr"/>
       <c r="G37" s="2" t="n">
-        <v>191</v>
+        <v>326</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Orthopedic; short; procedure/operative; diagnoses + procedures + imaging</t>
+          <t>Orthopedic; medium; history and physical; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J37" s="2" t="n">
-        <v>2270</v>
+        <v>2359</v>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>procedure/operative</t>
+          <t>history and physical</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>higher</t>
         </is>
       </c>
       <c r="M37" s="2" t="n">
-        <v>0.2753043282236249</v>
+        <v>0.7403629395852119</v>
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; procedures; imaging; follow-up; surgery</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; imaging; past history; treatment plans; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2800,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Orthopedic; medium; other narrative/sectioned; diagnoses + symptoms + medications</t>
+          <t>Orthopedic; medium; other narrative/sectioned; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J38" s="2" t="n">
@@ -2831,7 +2827,7 @@
     </row>
     <row r="39" ht="110" customHeight="1">
       <c r="A39" s="2" t="n">
-        <v>2078</v>
+        <v>2059</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
@@ -2840,39 +2836,39 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Physical Therapy - Low Back Pain  </t>
+          <t xml:space="preserve"> Rotator cuff syndrome - H&amp;P </t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The patient is a 26-year-old female, referred to Physical Therapy for low back pain.  The patient has a history of traumatic injury to low back.</t>
+          <t xml:space="preserve"> Shoulder pain, right shoulder diffusely - Rotator cuff syndrome, right.</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS: , The patient is a 26-year-old female, referred to Physical Therapy for low back pain.  The patient has a history of traumatic injury to low back.  The patient stated initial injury occurred eight years ago, when she fell at a ABC Store.  The patient stated she received physical therapy, one to two visits and received modality treatment only, specifically electrical stimulation and heat pack per patient recollection.  The patient stated that she has had continuous low-back pain at varying degrees for the past eight years since that fall.  The patient gave birth in August 2008 and since the childbirth, has experienced low back pain.  The patient also states that she fell four to five days ago, while mopping her floor.  The patient stated that she landed on her tailbone and symptoms have increased since that fall.  The patient stated that her initial physician examination with Dr. X was on 01/10/09, and has a followup appointment on 02/10/09.,PAST MEDICAL HISTORY: , The patient denies high blood pressure, diabetes, heart disease, lung disease, thyroid, kidney, or bladder dysfunctions.  The patient stated that she quit smoking prior to her past childbirth and is currently not pregnant.  The patient has had a C-section and also an appendectomy.  The patient was involved in a motor vehicle accident four to five years ago and at that time, the patient did not require any physical therapy nor did she report any complaints of increased back pain following that accident.,MEDICATIONS: , Patient currently states she is taking:,1.  Vicodin 500 mg two times a day.,2.  Risperdal.,3.  Zoloft.,4.  Stool softeners.,5.  Prenatal pills.,DIAGNOSTIC IMAGERY:  ,The patient states she has not had an MRI performed on her lumbar spine.  The patient also states that Dr. X took x-rays two weeks ago, and no fractures were found at that time.  Per physician note, dated 12/10/08, Dr. X dictated that the x-ray showed an anterior grade 1 spondylolisthesis of L5 over S1, and requested Physical Therapy to evaluate and treat.,SUBJECTIVE:  ,The patient states that pain is constant in nature with a baseline of 6-7/10 with pain increasing to 10/10 during the night or in cold weather.  The patient states that pain is dramatically less, when the weather is warmer.  The patient also states that pain worsens as the day progresses, in that she also hard time getting out of bed in the morning.  The patient states that she does not sleep at night well and sleeps less than one hour at a time.,Aggravating factors include, sitting for periods greater than 20 minutes or lying supine on her back.  Easing factors include side lying position in she attempts to sleep.,OBJECTIVE: , AGE:  26 years old.  HEIGHT:  5 feet 2 inches.  WEIGHT:  The patient is an obese 26-year-old female.,ACTIVE RANGE OF MOTION: , Lumbar spine, flexion, lateral flexion and rotation all within functional limits without complaints of pain or soreness while performing them during evaluation.,PALPATION:  ,The patient complained of bilateral SI joint point tenderness.  The patient also complained of left greater trochanter hip point tenderness.  The patient also complained of bilateral paraspinal tenderness on cervical spine to lumbar spine.,STRENGTH:  ,RIGHT LOWER EXTREMITY:,Knee extension 5/5, hip flexion 5/5, knee flexion 4/5, internal and external hip rotation was 4/5.  With manual muscle testing of knee flexion, hip, internal and external rotation, the patient reports an increase in right SI joint pain to 8/10.,LEFT LOWER EXTREMITY:,Hip flexion 5/5, knee extension 5/5, knee flexion 4/5, hip internal and external rotation 4/5, with slight increase in pain level with manual muscle testing and resistance.  It must be noted that PT did not apply as much resistance during manual muscle testing, secondary to the 8/10 pain elicited during the right lower extremity.,NEUROLOGICAL:  ,The patient subjectively complains of numbness with tingling in her bilateral extremities when she sits longer than 25 minutes.  However, they subside when she stands.  The patient did complain of this numbness and tingling during the evaluation and the patient was seated for a period of 20 minutes.  Upon standing, the patient stated that the numbness and tingling subsides almost immediately.  The patient stated that Dr. X told her that he believes that during her past childbirth when the epidural was being administered that there was a possibility that a sensory nerve may have been also affected during the epidural less causing the numbness and tingling in her bilateral lower extremities.  The patient does not demonstrate any sensation deficits with gentle pressure to the lumbar spine and during manual muscle testing.,GAIT:  ,The patient ambulated out of the examination room, while carrying her baby in a car seat.,ASSESSMENT:  ,The patient is a 26-year-old overweight female, referred to Physical Therapy for low back pain.  The patient presents with lower extremity weakness, which may be contributing to her lumbosacral pain, in that she has poor lumbar stabilization with dynamic ADLs, transfers, and gait activity when fatigued.  At this time, the patient may benefit from skilled physical therapy to address her decreased strength and core stability in order to improve her ADL, transfer, and mobility skills.,PROGNOSIS: , The patient's prognosis for physical therapy is good for dictated goals.,SHORT-TERM GOALS TO BE ACHIEVED IN TWO WEEKS:,1.  The patient will be able to sit for greater than 25 minutes without complaints of paraesthesia or pain in her bilateral lower extremities or bilateral SI joints.,2.  The patient will increase bilateral hip internal and external rotation to 4/5 with SI joint pain less than or equal to 5/10.,3.  The patient will report 25% improvement in her functional and ADL activities.,4.  Pain will be less than 4/10 while performing __________ while at PT session.,LONG-TERM GOALS TO BE ACCOMPLISHED IN ONE MONTH:,1.  The patient will be independent with home exercise program.,2.  Bilateral hamstring, bilateral hip internal and external rotation strength to be 4+/5 with SI joint pain less than or equal to 2/10, while performing manual muscle test.,3.  The patient will report 60% improvement or greater in functional transfers in general ADL activity.,4.  The patient will be able to sit greater than or equal to 45 minutes without complaint of lumbosacral pain.,5.  The patient will be able to sleep greater than 2 hours without pain.,TREATMENT PLAN:,1.  Therapeutic exercises to increase lower extremity strength and assist with lumbar sacral stability.</t>
+          <t>CHIEF COMPLAINT:  ,This 18 year old male presents today with shoulder pain right.  Location:  He indicates the problem location is the right shoulder diffusely.  Quality:  Quality of the pain is described by the patient as aching, throbbing and tolerable.  Patient relates pain on a scale from 0 to 10 as 5/10.  Severity:  The severity has worsened over the past 3 months.  Timing (onset/frequency):  Onset was gradual and after pitching a baseball game.  Modifying Factors:  Patient's condition is aggravated by throwing.  He participates with difficulty in basketball.  Past conservative treatments include NSAID and muscle relaxant medications.,ALLERGIES: , No known medical allergies.,MEDICATION HISTORY:,  None.,PAST MEDICAL HISTORY:  ,Childhood Illnesses: (+) strep throat (+) mumps (+) chickenpox,PAST SURGICAL HISTORY:,  No previous surgeries.,FAMILY HISTORY:,  Patient admits a family history of arthritis associated with mother.,SOCIAL HISTORY: , Patient denies smoking, alcohol abuse, illicit drug use and STDs.,REVIEW OF SYSTEMS:,Musculoskeletal: (+) joint or musculoskeletal symptoms (+) stiffness in AM.,Psychiatric: (-) psychiatric or emotional difficulties.,Eyes: (-) visual disturbance or change.,Neurological: (-) neurological symptoms or problems Endocrine: (-) endocrine-related symptoms.,Allergic / Immunologic: (-) allergic or immunologic symptoms.,Ears, Nose, Mouth, Throat: (-) symptoms involving ear, nose, mouth, or throat.,Gastrointestinal: (-) GI symptoms.,Genitourinary: (-) GU symptoms.,Constitutional Symptoms: (-) constitutional symptoms such as fever, headache, nausea, dizziness.,Cardiovascular: (-) cardiovascular problems or chest symptoms.,Respiratory: (-)breathing difficulties, respiratory symptoms.,Physical Exam:  BP Standing:  116/68 Resp:  16 HR:  68 Temp:  98.1 Height:  5 ft.  11 in.  Weight:  165 lbs.  Patient is a 18 year old male who appears pleasant, in no apparent distress, his given age, well developed, well nourished and with good attention to hygiene and body habitus.  Oriented to person, place and time.  Right shoulder shows evidence of swelling and tenderness.  Radial pulses are 2 /4, bilateral.  Brachial pulses are 2 /4, bilateral.,Appearance:  Normal.,Tenderness:  Anterior - moderate, Biceps - none, Posterior - moderate and Subacromial - moderate right.,Range of Motion:  Right shoulder ROM shows decreased flexion, decreased extension, decreased adduction, decreased abduction, decreased internal rotation, decreased external rotation.  L shoulder normal.,Strength:  External rotation - fair.  Internal rotation - poor right.,AC Joint:  Pain with ABD and cross-chest - mild right.,Rotator Cuff:  Impingement - moderate.  Painful arc - moderate right.,Instability:  None.,TEST &amp; X-RAY RESULTS:,  X-rays of the shoulder were performed.  X-ray of right shoulder reveals cuff arthropathy present.,IMPRESSION: , Rotator cuff syndrome, right.,PLAN: , Diagnosis of a rotator cuff tendinitis and shoulder impingement were discussed.  I noted that this is a very common condition resulting in significant difficulties with use of the arm.  Several treatment options and their potential benefits were described.  Nonsteroidal anti-inflammatories can be helpful but typically are slow acting.  Cortisone shots can be very effective and are quite safe.  Often more than one injection may be required.  Physical therapy can also be helpful, particularly if there is any loss of shoulder mobility or strength.  If these treatments fail to resolve symptoms, an MRI or shoulder arthrogram may be required to rule out a rotator cuff tear.  Injected shoulder joint and with Celestone Soluspan 1.0 cc .  Ordered x-rays of shoulder right.,PRESCRIPTIONS:,  Vioxx Dosage:  25 mg tablet Sig:  TID Dispense:  60 Refills:  0 Allow Generic:  Yes,PATIENT INSTRUCTIONS:,  Patient was instructed to restrict activity.  Patient was given instructions on RICE therapy.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr"/>
       <c r="G39" s="2" t="n">
-        <v>1033</v>
+        <v>526</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Orthopedic; long; SOAP-style; diagnoses + symptoms + medications</t>
+          <t>Orthopedic; medium; history and physical; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J39" s="2" t="n">
-        <v>2078</v>
+        <v>2059</v>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>SOAP-style</t>
+          <t>history and physical</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -2881,17 +2877,17 @@
         </is>
       </c>
       <c r="M39" s="2" t="n">
-        <v>0.8933724075743913</v>
+        <v>0.8419183949504058</v>
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; imaging; past history; treatment plans; follow-up; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; vital signs; imaging; past history; treatment plans; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="40" ht="110" customHeight="1">
       <c r="A40" s="2" t="n">
-        <v>1618</v>
+        <v>1571</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
@@ -2900,39 +2896,39 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Mayoview </t>
+          <t xml:space="preserve"> MRI Knee - 4 </t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Resting Myoview and adenosine Myoview SPECT</t>
+          <t xml:space="preserve"> MRI left knee without contrast.</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>PROCEDURE DONE:  ,Resting Myoview and adenosine Myoview SPECT.,INDICATIONS:,  Chest pain.,PROCEDURE:,  13.3 mCi of Tc-99m tetrofosmin was injected and resting Myoview SPECT was obtained.  Pharmacologic stress testing was done using adenosine infusion.  Patient received 38 mg of adenosine infused at 140 mcg/kg/minute over a period of four minutes.  Two minutes during adenosine infusion, 31.6 mCi of Tc-99m tetrofosmin was injected.  Resting heart rate was 90 beats per minute.  Resting blood pressure was 130/70.  Peak heart rate obtained during adenosine infusion was 102 beats per minute.  Blood pressure obtained during adenosine infusion was 112/70.  During adenosine infusion, patient experienced dizziness and shortness of breath.  No significant ST segment, T wave changes, or arrhythmias were seen.,Resting Myoview and adenosine Myoview SPECT showed uniform uptake of isotope throughout myocardium without any perfusion defect.  Gated dynamic imaging showed normal wall motion and normal systolic thickening throughout left ventricular myocardium.  Left ventricular ejection fraction obtained during adenosine Myoview SPECT was 77%.  Lung heart ratio was 0.40.  TID ratio was 0.88.,IMPRESSION:,  Normal adenosine Myoview myocardial perfusion SPECT.  Normal left ventricular regional and global function with left ventricular ejection fraction of 77%.</t>
+          <t>EXAM:,MRI OF THE LEFT KNEE WITHOUT CONTRAST,CLINICAL:,Left knee pain. Twisting injury.,FINDINGS:,The images reveal a sizable joint effusion. The joint effusion appears to be complex with mixed signal intensity material within. The patella is slightly laterally tilted towards the left. The mid portion of the patella cartilage shows some increased signal and focal injury to the patellar cartilage is suspected. Mildly increased bone signal overlying the inferolateral portion of the patella is identified. No significant degenerative changes about the patella can be seen. The quadriceps tendon as well as the infrapatellar ligament both look intact. There is some prepatellar soft tissue edema.,The bone signal shows a couple of small areas of cystic change in the proximal aspect of the tibia. NO significant areas of bone edema are appreciated.,There is soft tissue edema along the lateral aspect of the knee. There is a partial tear of the lateral collateral ligament complex. The medial collateral ligament complex looks intact. A small amount of edema is identified immediately adjacent to the medial collateral ligament complex.,The posterior cruciate ligament looks intact. The anterior cruciate ligament is thickened with significant increased signal. I suspect at least a high grade partial tear.,The posterior horn of the medial meniscus shows some myxoid degenerative changes. The posterior horn and anterior horn of the lateral meniscus likewise shows myxoid degenerative type changes. I don’t see a definite tear extending to the articular surface.,IMPRESSION:,Sizeable joint effusion which is complex and may contain blood products.,Myxoid degenerative type changes medial and lateral meniscus with no definite evidence of a tear.,Soft tissue swelling and partial tear of the lateral collateral ligament complex.,At least high grade partial tear of the anterior cruciate ligament with significant thickening and increased signal of this structure.,The posterior cruciate ligament is intact.,Injury to the patellar cartilage as above.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>radiology, myoview, gated dynamic imaging, myoview spect, resting myoview, spect, tc-99m, adenosine myoview, adenosine infusion, ejection fraction, myocardium, systolic thickening, tetrofosmin, adenosine myoview spect, adenosine,</t>
+          <t>radiology, lateral collateral ligament, medial collateral ligament, posterior cruciate ligament, anterior cruciate ligament, collateral ligament complex, myxoid degenerative, partial tear, collateral ligament, ligament complex, cruciate ligament, mri, effusion, cartilage, collateral, cruciate, knee, tear, ligament</t>
         </is>
       </c>
       <c r="G40" s="2" t="n">
-        <v>184</v>
+        <v>298</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Radiology; short; diagnostic report; diagnoses + symptoms + medications</t>
+          <t>Radiology; medium; diagnostic report; lower text complexity; diagnoses + symptoms + imaging</t>
         </is>
       </c>
       <c r="J40" s="2" t="n">
-        <v>1618</v>
+        <v>1571</v>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
@@ -2945,17 +2941,17 @@
         </is>
       </c>
       <c r="M40" s="2" t="n">
-        <v>0.3524008115419297</v>
+        <v>0.147204688908927</v>
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; vital signs; procedures; imaging</t>
+          <t>diagnoses; symptoms; imaging</t>
         </is>
       </c>
     </row>
     <row r="41" ht="110" customHeight="1">
       <c r="A41" s="2" t="n">
-        <v>1663</v>
+        <v>1516</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
@@ -2964,26 +2960,26 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CT-Guided Biopsy - Kidney </t>
+          <t xml:space="preserve"> Transesophageal Echocardiogram - 3 </t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CT-guided needle placement, CT-guided biopsy of right renal mass, and embolization of biopsy tract with gelfoam.</t>
+          <t xml:space="preserve"> Transesophageal echocardiographic examination report.   Aortic valve replacement.  Assessment of stenotic valve.  Evaluation for thrombus on the valve.</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>REASON FOR EXAM:  This 60-year-old female who was found to have a solid indeterminate mass involving the inferior pole of the right kidney was referred for percutaneous biopsy under CT guidance at the request of Dr. X.,PROCEDURE:  The procedure risks and possible complications including, but not limited to severe hemorrhage which could result in emergent surgery, were explained to the patient.  The patient understood.  All questions were answered, and informed consent was obtained.  With the patient in the prone position, noncontrasted CT localization images were obtained through the kidney.  Conscious sedation was utilized with the patient being monitored.  The patient was administered divided dose of Versed and fentanyl intravenously.,Following sterile preparation and local anesthesia to the posterior aspect of the right flank, an 18-gauge co-axial Temno-type needle was directed into the inferior pole right renal mass from the posterior oblique approach.  Two biopsy specimens were obtained and placed in 10% formalin solution.  CT documented needle placement.  Following the biopsy, there was active bleeding through the stylet, as well as a small hematoma about the inferior aspect of the right kidney posteriorly.  I placed several torpedo pledgets of Gelfoam through the co-axial sheath into the site of bleeding.  The bleeding stopped.  The co-axial sheath was then removed.  Bandage was applied.  Hemostasis was obtained.  The patient was placed in the supine position.  Postbiopsy CT images were then obtained.  The patient's hematoma appeared stable.  The patient was without complaints of pain or discomfort.  The patient was then sent to her room with plans of observing for approximately 4 hours and then to be discharged, as stable.  The patient was instructed to remain at bedrest for the remaining portions of the day at home and patient is to followup with Dr. Fieldstone for the results and follow-up care.,FINDINGS:  Initial noncontrasted CT localization images reveals the presence of an approximately 2.1 cm cortical mass involving the posterior aspect of the inferior pole of the right kidney.  Images obtained during the biopsy reveals the cutting portion of the biopsy needle to extend through the mass.  Images obtained following the biopsy reveals the development of a small hematoma posterior to the right kidney in its inferior pole adjacent to the mass.  There are small droplets of air within the hematoma.  No hydronephrosis is identified.,CONCLUSION:,1.  Percutaneous biopsy of inferior pole right renal mass under computed tomography guidance with specimen sent to laboratory in 10% formalin solution.,2.  Development of a small hematoma adjacent to the inferior pole of the right kidney with active bleeding through the biopsy needle stopped by tract embolization with Gelfoam pledgets.</t>
+          <t>REASON FOR EXAM: , Aortic valve replacement.  Assessment of stenotic valve.  Evaluation for thrombus on the valve.,PREOPERATIVE DIAGNOSIS:  ,Atrial valve replacement.,POSTOPERATIVE DIAGNOSES:,  Moderate stenosis of aortic valve replacement.  Mild mitral regurgitation.  Normal left ventricular function.,PROCEDURES IN DETAIL: , The procedure was explained to the patient with risks and benefits.  The patient agreed and signed the consent form.  The patient received a total of 3 mg of Versed and 50 mcg of fentanyl for conscious sedation and pain control.  The oropharynx anesthetized with benzocaine spray and lidocaine solution.,Esophageal intubation was done with no difficulty with the second attempt.  In a semi-Fowler position, the probe was passed to transthoracic views at about 40 to 42 cm.  Multiple pictures obtained.  Assessment of the peak velocity was done later.,The probe was pulled to the mid esophageal level.  Different pictures including short-axis views of the aortic valve was done.  Extubation done with no problems and no blood on the probe.  The patient tolerated the procedure well with no immediate postprocedure complications.,INTERPRETATION: , The left atrium was mildly dilated.  No masses or thrombi were seen.  The left atrial appendage was free of thrombus.  Pulse wave interrogation showed peak velocities of 60 cm per second.,The left ventricle was normal in size and contractility with mild LVH.  EF is normal and preserved.,The right atrium and right ventricle were both normal in size.,Mitral valve showed no vegetations or prolapse.  There was mild-to-moderate regurgitation on color flow interrogation.  Aortic valve was well-seated mechanical valve, bileaflet with acoustic shadowing beyond the valve noticed.  No perivalvular leak was noticed.  There was increased velocity across the valve with peak velocity of 3.2 m/sec with calculated aortic valve area by continuity equation at 1.2 cm2 indicative of moderate aortic valve stenosis based on criteria for native heart valves.,No AIC.,Pulmonic valve was somewhat difficult to see because of acoustic shadowing from the aortic valve.  Overall showed no abnormalities.  The tricuspid valve was structurally normal.,Interatrial septum appeared to be intact, confirmed by color flow interrogation as well as agitated saline contrast study.,The aorta and aortic arch were unremarkable.  No dissection.,IMPRESSION:,1.  Mildly dilated left atrium.,2.  Mild-to-moderate regurgitation.,3.  Well-seated mechanical aortic valve with peak velocity of 3.2 m/sec and calculated valve area of 1.2 cm2 consistent with moderate aortic stenosis.  Reevaluation in two to three years with transthoracic echocardiogram will be recommended.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>radiology, embolization, ct localization, gelfoam pledgets, ct guided needle placement, ct guided biopsy, needle placement, renal mass, ct guided, inferior pole, ct, biopsy, hematoma, kidney, mass,</t>
+          <t xml:space="preserve">radiology, aortic valve replacement, stenotic valve, thrombus, stenosis, ventricular, esophageal, peak velocity, valve replacement, aortic valve, aortic, transesophageal, valve, oropharynx, atrium, interrogation, atrial, moderate, </t>
         </is>
       </c>
       <c r="G41" s="2" t="n">
-        <v>426</v>
+        <v>384</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
@@ -2992,15 +2988,15 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Radiology; medium; diagnostic report; symptoms + laboratory values + procedures</t>
+          <t>Radiology; medium; procedure/operative; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J41" s="2" t="n">
-        <v>1663</v>
+        <v>1516</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>diagnostic report</t>
+          <t>procedure/operative</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
@@ -3009,17 +3005,17 @@
         </is>
       </c>
       <c r="M41" s="2" t="n">
-        <v>0.3975428313796213</v>
+        <v>0.5675157799819658</v>
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>symptoms; laboratory values; procedures; imaging; follow-up; surgery</t>
+          <t>diagnoses; symptoms; medications; vital signs; procedures; imaging; treatment plans</t>
         </is>
       </c>
     </row>
     <row r="42" ht="110" customHeight="1">
       <c r="A42" s="2" t="n">
-        <v>1639</v>
+        <v>1663</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
@@ -3028,39 +3024,39 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Fetal Anatomical Survey </t>
+          <t xml:space="preserve"> CT-Guided Biopsy - Kidney </t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The patient is a 39-year-old gravida 3, para 2, who is now at 20 weeks and 2 days gestation.  This pregnancy is a twin gestation.  The patient presents for her fetal anatomical survey.  </t>
+          <t xml:space="preserve"> CT-guided needle placement, CT-guided biopsy of right renal mass, and embolization of biopsy tract with gelfoam.</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>PAST MEDICAL HISTORY:  ,The patient denies any significant past medical history.,PAST SURGICAL HISTORY: , The patient denies any significant surgical history.,MEDICATIONS: , The patient takes no medications.,ALLERGIES: , No known drug allergies.,SOCIAL HISTORY: , She denies use of cigarettes, alcohol or drugs.,FAMILY HISTORY: , No family history of birth defects, mental retardation or any psychiatric history.,DETAILS: , I performed a transabdominal ultrasound today using a 4 MHz transducer.  There is a twin gestation in the vertex transverse lie with an anterior placenta and a normal amount of amniotic fluid surrounding both of the twins.  The fetal biometry of twin A is as follows.  The biparietal diameter is 4.9 cm consistent with 20 weeks and 5 days, head circumference 17.6 cm consistent with 20 weeks and 1 day, the abdominal circumference is 15.0 cm consistent with 20 weeks and 2 days, and femur length is 3.1 cm consistent with 19 weeks and 5 days, and the humeral length is 3.0 cm consistent with 20 weeks and 0 day.  The average gestational age by ultrasound is 20 weeks and 1 day and the estimated fetal weight is 353 g.  The following structures are seen as normal on the fetal anatomical survey, the shape of the fetal head, the choroid plexuses, the cerebellum, nuchal fold thickness, the fetal spine and fetal face, the four-chamber view of the fetal heart, the outflow tracts of the fetal heart, the stomach, the kidneys, and cord insertion site, the bladder, the extremities, the genitalia, the cord, which appeared to have three vessels and the placenta.,Limited in views of baby A with a nasolabial region.,The following is the fetal biometry for twin B. The biparietal diameter is 4.7 cm consistent with 20 weeks and 2 days, head circumference 17.5 cm consistent with 20 weeks and 0 day, the abdominal circumference is 15.5 cm consistent with 20 weeks and 5 days, the femur length is 3.3 cm consistent with 20 weeks and 3 days, and the humeral length is 3.1 cm consistent with 20 weeks and 2 days, the average gestational age by ultrasound is 22 weeks and 2 days, and the estimated fetal weight is 384 g.  The following structures were seen as normal on the fetal anatomical survey.  The shape of the fetal head, the choroid plexuses, the cerebellum, nuchal fold thickness, the fetal spine and fetal face, the four-chamber view of the fetal heart, the outflow tracts of the fetal heart, the stomach, the kidneys, and cord insertion site, the bladder, the extremities, the genitalia, the cord, which appeared to have three vessels, and the placenta.  Limited on today's ultrasound the views of nasolabial region.,In summary, this is a twin gestation, which may well be monochorionic at 20 weeks and 1 day.  There is like gender and a single placenta.  One cannot determine with certainty whether or not this is a monochorionic or dichorionic gestation from the ultrasound today.,I sat with the patient and her husband and discussed alternative findings and the complications.  We focused our discussion today on the association of twin pregnancy with preterm delivery.  We discussed the fact that the average single intrauterine pregnancy delivers at 40 weeks' gestation while the average twin delivery occurs at 35 weeks' gestation.  We discussed the fact that 15% of twins deliver prior to 32 weeks' gestation.  These are the twins which we have the most concern regarding the long-term prospects of prematurity.  We discussed several etiologies of preterm delivery including preterm labor, incompetent cervix, premature rupture of the fetal membranes as well as early delivery from preeclampsia and growth restriction.  We discussed the use of serial transvaginal ultrasound to assess for early cervical change and the use of serial transabdominal ultrasound to assess for normal interval growth.  We discussed the need for frequent office visits to screen for preeclampsia.  We also discussed treatment options such as cervical cerclage, bedrest, tocolytic medications, and antenatal steroids.  I would recommend that the patient return in two weeks for further cervical assessment and assessment of fetal growth and well-being.,In closing, I do want to thank you very much for involving me in the care of your delightful patient.  I did review all of the above findings and recommendations with the patient today at the time of her visit.  Please do not hesitate to contact me if I could be of any further help to you.,Total visit time 40 minutes.</t>
+          <t>REASON FOR EXAM:  This 60-year-old female who was found to have a solid indeterminate mass involving the inferior pole of the right kidney was referred for percutaneous biopsy under CT guidance at the request of Dr. X.,PROCEDURE:  The procedure risks and possible complications including, but not limited to severe hemorrhage which could result in emergent surgery, were explained to the patient.  The patient understood.  All questions were answered, and informed consent was obtained.  With the patient in the prone position, noncontrasted CT localization images were obtained through the kidney.  Conscious sedation was utilized with the patient being monitored.  The patient was administered divided dose of Versed and fentanyl intravenously.,Following sterile preparation and local anesthesia to the posterior aspect of the right flank, an 18-gauge co-axial Temno-type needle was directed into the inferior pole right renal mass from the posterior oblique approach.  Two biopsy specimens were obtained and placed in 10% formalin solution.  CT documented needle placement.  Following the biopsy, there was active bleeding through the stylet, as well as a small hematoma about the inferior aspect of the right kidney posteriorly.  I placed several torpedo pledgets of Gelfoam through the co-axial sheath into the site of bleeding.  The bleeding stopped.  The co-axial sheath was then removed.  Bandage was applied.  Hemostasis was obtained.  The patient was placed in the supine position.  Postbiopsy CT images were then obtained.  The patient's hematoma appeared stable.  The patient was without complaints of pain or discomfort.  The patient was then sent to her room with plans of observing for approximately 4 hours and then to be discharged, as stable.  The patient was instructed to remain at bedrest for the remaining portions of the day at home and patient is to followup with Dr. Fieldstone for the results and follow-up care.,FINDINGS:  Initial noncontrasted CT localization images reveals the presence of an approximately 2.1 cm cortical mass involving the posterior aspect of the inferior pole of the right kidney.  Images obtained during the biopsy reveals the cutting portion of the biopsy needle to extend through the mass.  Images obtained following the biopsy reveals the development of a small hematoma posterior to the right kidney in its inferior pole adjacent to the mass.  There are small droplets of air within the hematoma.  No hydronephrosis is identified.,CONCLUSION:,1.  Percutaneous biopsy of inferior pole right renal mass under computed tomography guidance with specimen sent to laboratory in 10% formalin solution.,2.  Development of a small hematoma adjacent to the inferior pole of the right kidney with active bleeding through the biopsy needle stopped by tract embolization with Gelfoam pledgets.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>radiology, vaginal delivery, transducer, transabdominal ultrasound, placenta, amniotic fluid, fetal anatomical survey, preterm delivery, twin gestation, gestation, infant, fetal, anatomical, delivery, ultrasound,</t>
+          <t>radiology, embolization, ct localization, gelfoam pledgets, ct guided needle placement, ct guided biopsy, needle placement, renal mass, ct guided, inferior pole, ct, biopsy, hematoma, kidney, mass,</t>
         </is>
       </c>
       <c r="G42" s="2" t="n">
-        <v>729</v>
+        <v>426</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Radiology; long; diagnostic report; diagnoses + medications + allergies</t>
+          <t>Radiology; medium; diagnostic report; middle text complexity; symptoms + laboratory values + procedures</t>
         </is>
       </c>
       <c r="J42" s="2" t="n">
-        <v>1639</v>
+        <v>1663</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -3069,21 +3065,21 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>higher</t>
+          <t>middle</t>
         </is>
       </c>
       <c r="M42" s="2" t="n">
-        <v>0.738334084761046</v>
+        <v>0.3975428313796213</v>
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; medications; allergies; imaging; past history; treatment plans; follow-up; surgery</t>
+          <t>symptoms; laboratory values; procedures; imaging; follow-up; surgery</t>
         </is>
       </c>
     </row>
     <row r="43" ht="110" customHeight="1">
       <c r="A43" s="2" t="n">
-        <v>1307</v>
+        <v>1394</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
@@ -3092,43 +3088,43 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> SOAP - Temporal Mass </t>
+          <t xml:space="preserve"> Fundoplication &amp; Gastrostomy Followup </t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> MRI demonstrated right contrast-enhancing temporal mass.</t>
+          <t xml:space="preserve"> Followup of laparoscopic fundoplication and gastrostomy.  Laparoscopic fundoplication and gastrostomy was done because of the need for enteral feeding access.</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>SUBJECTIVE: , The patient is a 55-year-old African-American male that was last seen in clinic on 07/29/2008 with diagnosis of new onset seizures and an MRI scan, which demonstrated right contrast-enhancing temporal mass.  Given the characteristics of this mass and his new onset seizures, it is significantly concerning for a high-grade glioma.  ,OBJECTIVE: , The patient is alert and oriented times three, GCS of 15.  Cranial nerves II to XII are grossly intact.  Motor exam demonstrates 5/5 strength in all four extremities.  Sensation is intact to light touch, pain, temperature, and proprioception.  Cerebellar exam is intact.  Gait is normal and tandem on heels and toes.  Speech is appropriate.  Judgment is intact.  Pupils are equal and reactive to light.,ASSESSMENT AND PLAN: , The patient is a 55-year-old African-American male with a new diagnosis of rim-enhancing right temporal mass.  Given the characteristics of the MRI scan, it is highly likely that he demonstrates high-grade glioma and concerning for glioblastoma multiforme.  We have discussed in length the possible benefits of biopsy, surgical resection, medical management, as well as chemotherapy, radiation treatments, and doing nothing.  Given the high probability that the mass represents a high-grade glioma, the patient, after weighing the risks and the benefits of surgery, has agreed to undergo a surgical biopsy and resection of the mass as well as concomitant chemotherapy and radiation as the diagnosis demonstrates a high-grade glioma.  The patient has signed consent for his right temporal craniotomy for biopsy and likely resection of right temporal brain tumor.  He agrees that he will be n.p.o. after mid night on Wednesday night.  He is sent for preoperative assessment with the Anesthesiology tomorrow morning.  He has undergone vocational rehab assessment.</t>
+          <t>REASON FOR VISIT: , Followup of laparoscopic fundoplication and gastrostomy.,HISTORY OF PRESENT ILLNESS: , The patient is a delightful baby girl, who is now nearly 8 months of age and had a tracheostomy for subglottic stenosis.  Laparoscopic fundoplication and gastrostomy was done because of the need for enteral feeding access and to protect her airway at a time when it is either going to heal enough to improve and allow decannulation or eventually prove that she will need laryngotracheoplasty.  Dr. X is following The patient for this and currently plans are to perform a repeat endoscopic exam every couple of months to assist the status of her airway caliber.,The patient had a laparoscopic fundoplication and gastrostomy on 10/05/2007.  She has done well since that time.  She has had some episodes of retching intermittently and these seemed to be unpredictable.  She also had some diarrhea and poor feeding tolerance about a week ago but that has also resolved.  The patient currently takes about 1 ounce to 1.5 ounce of her feedings by mouth and the rest is given by G-tube.  She seems otherwise happy and is not having an excessive amount of stools.  Her parents have not noted any significant problems with the gastrostomy site.,The patient's exam today is excellent.  Her belly is soft and nontender.  All of her laparoscopic trocar sites are healing with a normal amount of induration, but there is no evidence of hernia or infection.  We removed The patient's gastrostomy button today and showed her parents how to reinsert one without difficulty.  The site of the gastrostomy is excellent.  There is not even a hint of granulation tissue or erythema, and I am very happy with the overall appearance.,IMPRESSION: , The patient is doing exceptionally well status post laparoscope fundoplication and gastrostomy.  Hopefully, the exquisite control of acid reflux by fundoplication will help her airway heal, and if she does well, allow decannulation in the future.  If she does require laryngotracheoplasty, the protection from acid reflux will be important to healing of that procedure as well.,PLAN:  ,The patient will follow up as needed for problems related to gastrostomy.  We will see her when she comes in the hospital for endoscopic exams and possibly laryngotracheoplasty in the future.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>soap / chart / progress notes, new onset seizures, temporal mass, cerebellar exam, glioma, temporal, massNOTE</t>
+          <t xml:space="preserve">soap / chart / progress notes, decannulation, enteral feeding, feeding access, laparoscopic fundoplication, gastrostomy, airway, laryngotracheoplasty, laparoscopic, fundoplication, </t>
         </is>
       </c>
       <c r="G43" s="2" t="n">
-        <v>279</v>
+        <v>370</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>SOAP / Chart / Progress Notes; short; SOAP-style; diagnoses + symptoms + procedures</t>
+          <t>SOAP / Chart / Progress Notes; medium; follow-up/progress; lower text complexity; diagnoses + procedures + past history</t>
         </is>
       </c>
       <c r="J43" s="2" t="n">
-        <v>1307</v>
+        <v>1394</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>SOAP-style</t>
+          <t>follow-up/progress</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -3137,17 +3133,17 @@
         </is>
       </c>
       <c r="M43" s="2" t="n">
-        <v>0.3710550045085662</v>
+        <v>0.345299819657349</v>
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; procedures; imaging; treatment plans; surgery; assessment/plan</t>
+          <t>diagnoses; procedures; past history; treatment plans; follow-up; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="44" ht="110" customHeight="1">
       <c r="A44" s="2" t="n">
-        <v>1396</v>
+        <v>1384</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
@@ -3156,26 +3152,26 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Gen Med Progress Note - 11 </t>
+          <t xml:space="preserve"> Gen Med Progress Note - 7 </t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 5-month recheck on type II diabetes mellitus, as well as hypertension.</t>
+          <t xml:space="preserve"> Patient with a three-day history of emesis and a four-day history of diarrhea</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>SUBJECTIVE:,  The patient is a 66-year-old female who presents to the clinic today for a five-month recheck on her type II diabetes mellitus, as well as hypertension.  While here she had a couple of other issues as well.  She stated that she has been having some right shoulder pain.  She denies any injury but certain range of motion does cause it to hurt.  No weakness, numbness or tingling.  As far as her diabetes she states that she only checks her blood sugars in the morning and those have all been ranging less than 100.  She has not been checking any two hours after meals.  Her blood pressures when she does check them have been running normal as well but she does not have any record of these present with her.  No other issues or concerns.  Upon review of her chart it did show that she had a benign breast biopsy done back on 06/11/04 and was told to have a repeat mammogram in six months but she has never had that done so she is needing to have this done as well.,ALLERGIES: , None.,MEDICATIONS:,  She is on Hyzaar 50/12.5 one-half p.o. daily, coated aspirin daily, lovastatin 40 mg one-half tab p.o. daily, multivitamin daily, metformin 500 mg one tab p.o. b.i.d.; however, she has been skipping her second dose during the day.,SOCIAL HISTORY:,  She is a nonsmoker.,REVIEW OF SYSTEMS:,  As noted above.,OBJECTIVE:,Vital Signs:  Temperature:  98.2.  Pulse:  64.  Respirations:  16.  Blood pressure:  110/56.  Weight:  169.,General:  Alert and oriented x 3.  No acute distress noted.,Neck:  No lymphadenopathy, thyromegaly, JVD or bruits.,Lungs:  Clear to auscultation.,Heart:  Regular rate and rhythm without murmur or gallops present.,Breasts:  Exam performed with a female nurse present.  The breasts do have some scars present underneath them bilaterally from prior breast reduction surgery.  There is no axillary adenopathy or tenderness.  Breasts appear to be symmetric.  There was no nipple discharge or retraction.  No breast tissue retraction noted in either the sitting or the supine position.  Upon palpation there were no palpable lumps or bumps and no palpable discharge.,Musculoskeletal:  She did have full range of motion of her shoulders.  She did have tenderness upon palpation over the right bicipital tendon.  There is no swelling, crepitus or discoloration noted.,MEDICAL DECISION MAKING:  Most recent hemoglobin A1c was 5.6% back in October 2004.  Most recent lipid checks were obtained back in July 2004.  We have not had this checked since that time.,ASSESSMENT:,1.  Type II diabetes mellitus.,2.  Hypertension.,3.  Right shoulder pain.,4.  Hyperlipidemia.,PLAN:,1.  She is going to go to lab to obtain a hemoglobin A1c, BMP, lipids, CPK, liver enzymes and quantitative microalbumin.,2.  We are going to set her up for a diagnostic bilateral mammogram due to a history of abnormal mammogram in the past which subsequently showed a benign breast cyst.,3.  I told her for her shoulder to take ibuprofen 600 mg three times daily with her meals for a minimum of the next one week.,4.  She is going to follow up in the clinic in three months for a complete comprehensive examination.  If any questions, concerns or problems arise between now and then she should let us know.</t>
+          <t>SUBJECTIVE:,  The patient is a 7-year-old male who comes in today with a three-day history of emesis and a four-day history of diarrhea.  Apparently, his brother had similar symptoms.  They had eaten some chicken and then ate some more of it the next day, and I could not quite understand what the problem was because there is a little bit of language barrier, although dad was trying very hard to explain to me what had happened.  But any way, after he and his brother got done eating with chicken, they both felt bad and have continued to feel bad.  The patient has had diarrhea five to six times a day for the last four days and then he had emesis pretty frequently three days ago and then has just had a couple of it each day in the last two days.  He has not had any emesis today.  He has urinated this morning.  His parents are both concerned because he had a fever of 103 last night.  Also, he ate half of a hamburger yesterday and he tried drinking some milk and that is when he had an emesis.  He has been drinking Pedialyte, Gatorade, white grape juice, and 7Up, otherwise he has not been eating anything.,MEDICATIONS:  ,None.,ALLERGIES:  ,He has no known drug allergies.,REVIEW OF SYSTEMS:,  Negative as far as sore throat, earache, or cough.,PHYSICAL EXAMINATION:,General:  He is awake and alert, no acute distress.,Vital Signs:  Blood pressure:  106/75.  Temperature:  99.  Pulse:  112.  Weight is 54 pounds.,HEENT:  His TMs are normal bilaterally.  Posterior pharynx is unremarkable.,Neck:  Without adenopathy or thyromegaly.,Lungs:  Clear to auscultation.,Heart:  Regular rate and rhythm without murmur.,Abdomen:  Benign.,Skin:  Turgor is intact.  His capillary refill is less than 3 seconds.,LABORATORY: , White blood cell count is 5.3 with 69 segs, 15 lymphs, and 13 monos.  His platelet count on his CBC is 215.,ASSESSMENT:,  Viral gastroenteritis.,PLAN:,  The parents did point out to me a rash that he had on his buttock.  There were some small almost pinpoint erythematous patches of papules that have a scab on them.  I did not see any evidence of petechiae.  Therefore, I just reassured them that this is a viral gastroenteritis.  I recommended that they stop giving him juice and just go with the Gatorade and water.  He is to stay away from milk products until his diarrhea and stomach upset have calmed down.  We talked about BRAT diet and slowly advancing his diet as he tolerates.  They have used some Kaopectate, which did not really help with the diarrhea.  Otherwise follow up as needed.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve">soap / chart / progress notes, diarrhea, emesis, history of, gastroenteritis, viral, brat diet, progress note, </t>
         </is>
       </c>
       <c r="G44" s="2" t="n">
-        <v>514</v>
+        <v>419</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -3184,34 +3180,34 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>SOAP / Chart / Progress Notes; medium; SOAP-style; diagnoses + symptoms + medications</t>
+          <t>SOAP / Chart / Progress Notes; medium; follow-up/progress; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J44" s="2" t="n">
-        <v>1396</v>
+        <v>1384</v>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>SOAP-style</t>
+          <t>follow-up/progress</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>higher</t>
+          <t>middle</t>
         </is>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0.7346145175834085</v>
+        <v>0.6001465284039675</v>
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; past history; treatment plans; follow-up; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; past history; treatment plans; follow-up; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="45" ht="110" customHeight="1">
       <c r="A45" s="2" t="n">
-        <v>1392</v>
+        <v>1396</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
@@ -3220,39 +3216,39 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Foot Pain - SOAP </t>
+          <t xml:space="preserve"> Gen Med Progress Note - 11 </t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Patient having foot pain.</t>
+          <t xml:space="preserve"> 5-month recheck on type II diabetes mellitus, as well as hypertension.</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>SUBJECTIVE:,  This 32-year-old female comes in again still having not got a primary care physician.  She said she was at Dr. XYZ office today for her appointment, and they cancelled her appointment because she has not gotten her Project Access insurance into affect.  She says that Project Access is trying to find her a doctor.  She is not currently on Project Access, and so she is here to get something for the pain in her foot.  I did notice that she went in to see Dr. XYZ for a primary care physician on 05/14/2004.  She said she does not have a primary care physician.  She was in here just last week and saw Dr. XYZ for back pain and was put on pain medicines and muscle relaxers.  She has been in here multiple times for different kinds of pain.  This pain she is having is in her foot.  She had surgery on it, and she has plates and screws.  She said she was suppose to see Dr. XYZ about getting some of the hardware out of it.  The appointment was cancelled, and that is why she came here.  It started hurting a lot yesterday, but she had this previous appointment with Dr. XYZ so she thought she would take care of it there, but they would not see her.  She did not injure her foot in any way recently.  It is chronically painful.  Every time she does very much exercise it hurts more.  We have x-rayed it in the past.  She has some hardware there.  It does not appear to be grossly abnormal or causing any loosening or problems on x-ray.,PHYSICAL EXAM: , Examination of her foot shows some well-healed surgical scars.  On the top of her foot she has two, and then on the lateral aspect below her ankle she has a long scar.  They are all old, and the surgery was done over a year ago.  She is walking with a very slight limp.  There is no redness.  No heat.  No swelling of the foot or the ankle.  It is mildly tender around the medial side of the foot just inferior to the medial malleolus.  It is not warm or red.,ASSESSMENT:,  Foot pain.,PLAN:,  She has been in here before.  She seems very pleasant.  Thought maybe she certainly might be having some significant pain, so I gave her some Lortab 7.5 to take with a refill.  After she left, I got to thinking about it and looked into her record.  She has been in here multiple times for pain medicine.  She has a primary care physician, and now she is telling us she does not have a primary care physician even though she had seen Dr. XYZ not too long ago.  We called Dr. XYZ office.  Dr. XYZ nurse said that the patient did not have an appointment today.  She has an appointment on June 15, 2004, for a postop check.  They did not tell her they would not see her today because of insurance, so the patient was lying to me.  We will keep that in mind the next time she returns, because she will likely be back.  She did say that Project Access will be approving her insurance next week, so she will be able to see Dr. XYZ soon.</t>
+          <t>SUBJECTIVE:,  The patient is a 66-year-old female who presents to the clinic today for a five-month recheck on her type II diabetes mellitus, as well as hypertension.  While here she had a couple of other issues as well.  She stated that she has been having some right shoulder pain.  She denies any injury but certain range of motion does cause it to hurt.  No weakness, numbness or tingling.  As far as her diabetes she states that she only checks her blood sugars in the morning and those have all been ranging less than 100.  She has not been checking any two hours after meals.  Her blood pressures when she does check them have been running normal as well but she does not have any record of these present with her.  No other issues or concerns.  Upon review of her chart it did show that she had a benign breast biopsy done back on 06/11/04 and was told to have a repeat mammogram in six months but she has never had that done so she is needing to have this done as well.,ALLERGIES: , None.,MEDICATIONS:,  She is on Hyzaar 50/12.5 one-half p.o. daily, coated aspirin daily, lovastatin 40 mg one-half tab p.o. daily, multivitamin daily, metformin 500 mg one tab p.o. b.i.d.; however, she has been skipping her second dose during the day.,SOCIAL HISTORY:,  She is a nonsmoker.,REVIEW OF SYSTEMS:,  As noted above.,OBJECTIVE:,Vital Signs:  Temperature:  98.2.  Pulse:  64.  Respirations:  16.  Blood pressure:  110/56.  Weight:  169.,General:  Alert and oriented x 3.  No acute distress noted.,Neck:  No lymphadenopathy, thyromegaly, JVD or bruits.,Lungs:  Clear to auscultation.,Heart:  Regular rate and rhythm without murmur or gallops present.,Breasts:  Exam performed with a female nurse present.  The breasts do have some scars present underneath them bilaterally from prior breast reduction surgery.  There is no axillary adenopathy or tenderness.  Breasts appear to be symmetric.  There was no nipple discharge or retraction.  No breast tissue retraction noted in either the sitting or the supine position.  Upon palpation there were no palpable lumps or bumps and no palpable discharge.,Musculoskeletal:  She did have full range of motion of her shoulders.  She did have tenderness upon palpation over the right bicipital tendon.  There is no swelling, crepitus or discoloration noted.,MEDICAL DECISION MAKING:  Most recent hemoglobin A1c was 5.6% back in October 2004.  Most recent lipid checks were obtained back in July 2004.  We have not had this checked since that time.,ASSESSMENT:,1.  Type II diabetes mellitus.,2.  Hypertension.,3.  Right shoulder pain.,4.  Hyperlipidemia.,PLAN:,1.  She is going to go to lab to obtain a hemoglobin A1c, BMP, lipids, CPK, liver enzymes and quantitative microalbumin.,2.  We are going to set her up for a diagnostic bilateral mammogram due to a history of abnormal mammogram in the past which subsequently showed a benign breast cyst.,3.  I told her for her shoulder to take ibuprofen 600 mg three times daily with her meals for a minimum of the next one week.,4.  She is going to follow up in the clinic in three months for a complete comprehensive examination.  If any questions, concerns or problems arise between now and then she should let us know.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>soap / chart / progress notes, soap, foot pain, primary care physician, project access, insurance, foot, project, access, care, appointment</t>
+          <t> </t>
         </is>
       </c>
       <c r="G45" s="2" t="n">
-        <v>543</v>
+        <v>514</v>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>SOAP / Chart / Progress Notes; long; SOAP-style; diagnoses + symptoms + medications</t>
+          <t>SOAP / Chart / Progress Notes; medium; SOAP-style; higher text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J45" s="2" t="n">
-        <v>1392</v>
+        <v>1396</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
@@ -3261,21 +3257,21 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>higher</t>
         </is>
       </c>
       <c r="M45" s="2" t="n">
-        <v>0.3392132551848512</v>
+        <v>0.7346145175834085</v>
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; imaging; treatment plans; follow-up; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; vital signs; procedures; past history; treatment plans; follow-up; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="46" ht="110" customHeight="1">
       <c r="A46" s="2" t="n">
-        <v>783</v>
+        <v>343</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
@@ -3284,39 +3280,39 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Foreign Body Removal - Thigh </t>
+          <t xml:space="preserve"> Shockwave Lithotripsy </t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Removal of foreign body of right thigh.  Foreign body of the right thigh, sewing needle.</t>
+          <t xml:space="preserve"> Right shockwave lithotripsy, cystoscopy, and stent removal x2.</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>PREPROCEDURE DIAGNOSIS:,  Foreign body of the right thigh.,POSTOPERATIVE DIAGNOSIS: , Foreign body of the right thigh, sewing needle.,PROCEDURE:  ,Removal of foreign body of right thigh.,HISTORY:  ,This is a 71-year-old lady who has been referred because there is a mass in the right thigh.  The patient comes with an ultrasound and apparently was diagnosed with a blood clot.  On physical examination, blood pressure was 152/76 and temperature was 95.0.  The patient is 5 feet 1 inch and weighs 170.  On examination of her right thigh, there is a transverse area of ecchymosis in the upper third of the thigh.  There is a palpation of a very sharp object just under the skin.  The patient desires for this to be removed.,DESCRIPTION OF PROCEDURE: , After obtaining informed consent in our office, the area was prepped and draped in usual fashion.  Xylocaine 1% was infiltrated in the end of the object that was the sharpest and a small incision was made there and then I pushed the foreign body through partially and then grabbed it with a hemostat and took it out and it was a 1-1/2-inch sewing needle.,Compression was applied for a few minutes and then a Band-Aid was applied.,The patient was given a tetanus toxoid 0.5 cc IM shot injection and then she was dismissed with instructions of return if inflammatory signs develop.</t>
+          <t>PREOPERATIVE DIAGNOSIS:,  Right renal stone.,POSTOPERATIVE DIAGNOSIS:  ,Right renal stone.,PROCEDURE: , Right shockwave lithotripsy, cystoscopy, and stent removal x2.,ANESTHESIA: , LMA.,ESTIMATED BLOOD LOSS:,  Minimal.  The patient was given antibiotics preoperatively.,HISTORY: , This is a 47-year-old male who presented with right renal stone and right UPJ stone.  The right UPJ stone was removed using ureteroscopy and laser lithotripsy and the stone in the kidney.  The plan was for shockwave lithotripsy.  The patient had duplicated system on the right side.  Risk of anesthesia, bleeding, infection, pain, MI, DVT, PE was discussed.  Options such as watchful waiting, passing the stone on its own, and shockwave lithotripsy were discussed.  The patient wanted to proceed with the shockwave to break the stone into small pieces as possible to allow the stones to pass easily.  Consent was obtained.,DETAILS OF THE OPERATION:  ,The patient was brought to the OR.  Anesthesia was applied.  The patient was placed in the supine position.  Using Dornier lithotriptor total of 2500 shocks were applied.  Energy levels were slowly started at O2 increased up to 7; gradually the stone seem to have broken into smaller pieces as the number of shocks went up.  The shocks were started at 60 per minute and slowly increased up to 90 per minute.  The patient's heart rate and blood pressure were stable throughout the entire procedure.,After the end of the shockwave lithotripsy the patient was placed in dorsal lithotomy position.  The patient was prepped and draped in usual sterile fashion and cystoscopy was done.  Using graspers, the stent was grasped x2 and pulled out, both stents were removed.  The patient tolerated the procedure well.  The patient was brought to recovery in stable condition.  The plan was for the patient to follow up with us and plan for KUB in about two to three months.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>surgery, removal of foreign body, sewing needle, foreign body</t>
+          <t>surgery, renal stone, stent removal, upj stone, shockwave lithotripsy, cystoscopy, stent, renal, shocks, upj, shockwave, lithotripsy, stone</t>
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>222</v>
+        <v>296</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Surgery; short; procedure/operative; diagnoses + vital signs + procedures</t>
+          <t>Surgery; medium; procedure/operative; lower text complexity; diagnoses + symptoms + procedures</t>
         </is>
       </c>
       <c r="J46" s="2" t="n">
-        <v>783</v>
+        <v>343</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
@@ -3329,17 +3325,17 @@
         </is>
       </c>
       <c r="M46" s="2" t="n">
-        <v>0.3787759242560866</v>
+        <v>0.3752254283137962</v>
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; vital signs; procedures; imaging; follow-up; surgery</t>
+          <t>diagnoses; symptoms; procedures; treatment plans; follow-up; surgery</t>
         </is>
       </c>
     </row>
     <row r="47" ht="110" customHeight="1">
       <c r="A47" s="2" t="n">
-        <v>422</v>
+        <v>1190</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
@@ -3348,26 +3344,26 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Plantar Fasciotomy </t>
+          <t xml:space="preserve"> AV Fistula - 4 </t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Plantar fascitis, left foot.  Partial plantar fasciotomy.</t>
+          <t xml:space="preserve"> Creation of autologous right brachiobasilic arteriovenous fistula - first stage.</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>PREOPERATIVE DIAGNOSIS:,  Plantar fascitis, left foot.,POSTOPERATIVE DIAGNOSIS: , Plantar fascitis, left foot.,PROCEDURE PERFORMED: , Partial plantar fasciotomy, left foot.,ANESTHESIA:,  10 cc of 0.5% Marcaine plain with TIVA.,HISTORY:  ,This 35-year-old Caucasian female presents to ABCD General Hospital with above chief complaint.  The patient states she has extreme pain with plantar fascitis in her left foot and has attempted conservative treatment including orthotics without long-term relief of symptoms and desires surgical treatment.  The patient has been NPO since mid night.  Consent is signed and in the chart.  No known drug allergies.,Details Of Procedure:  An IV was instituted by the Department of Anesthesia in the preoperative holding area.  The patient was transported to the operating room and placed on the operating table in supine position with a safety belt across the stomach.  Copious amounts of Webril were placed on the left ankle followed by blood pressure cuff.  After adequate sedation by the Department of Anesthesia, a total of 10 cc of 0.5% Marcaine plain was injected into the surgical site both medially and laterally across the plantar fascia.  The foot was then prepped and draped in the usual sterile orthopedic fashion.  An Esmarch bandage was applied for exsanguination and the pneumatic ankle tourniquet was inflated to 250 mmHg.  The foot was then reflected on the operating, stockinet reflected, and the foot cleansed with a wet and dry sponge.  Attention was then directed to the plantar medial aspect of the left heel.  An approximately 0.75 cm incision was then created in the plantar fat pad over the area of maximal tenderness.,The incision was then deepened with a combination of sharp and blunt dissection until the plantar fascia was palpated.  A #15 blade was then used to transect the medial and central bands of the plantar fascia.  Care was taken to preserve the lateral fibroids.  The foot was dorsiflexed against resistance as the fibers were released and there was noted to be increased laxity after release of the fibers on the plantar aspect of the foot indicating that plantar fascia has in fact been transacted.  The air was then flushed with copious amounts of sterile saline.  The skin incision was then closed with #3-0 nylon in simple interrupted fashion.  Dressings consisted of #0-1 silk, 4 x 4s, Kling, Kerlix, and Coban.  The pneumatic ankle tourniquet was released and immediate hyperemic flush was noted throughout all digits of the left foot.  The patient tolerated the above procedure and anesthesia well without complications.  The patient was transported to the PACU with vital signs stable and vascular status intact to the left foot.  Intraoperatively, an additional 80 cc of 1% lidocaine was injected for additional anesthesia in the case.  The patient is to be nonweightbearing on the left lower extremity with crutches.  The patient is given postoperative pain prescriptions for Vicodin ES, one q3-4h. p.o. p.r.n. for pain as well as Celebrex 200 mg one p.o. b.i.d.  The patient is to follow-up with Dr. X as directed.</t>
+          <t>PREOPERATIVE DIAGNOSES,1.  End-stage renal disease.,2.  Left subclavian vein occlusion.,3.  Status post chronic tracheostomy.,4.  Status post coronary artery bypass grafting.,5.  Right subclavian vein stenosis.,POSTOPERATIVE DIAGNOSES,1.  End-stage renal disease.,2.  Left subclavian vein occlusion.,3.  Status post chronic tracheostomy.,4.  Status post coronary artery bypass grafting.,5.  Right subclavian vein stenosis.,OPERATIVE PROCEDURE,Creation of autologous right brachiobasilic arteriovenous fistula - first stage.,INDICATIONS FOR THE PROCEDURE,This patient has a known left subclavian vein occlusion.  The right subclavian vein has an estimated 50% stenosis.  The patient has a catheter traversed in the right innominate vein.  The right basilic vein was judged to be suitable for usage on vein mapping.,OPERATIVE FINDINGS,The basilic vein was of an adequate size, but somewhat sclerotic.  A first stage autologous right brachiobasilic arteriovenous fistula was created.  A grade 2 was felt at completion.,OPERATIVE PROCEDURE IN DETAIL,After informed consent was obtained, the patient was taken to the operating room.  The patient was placed in the supine position.  The patient received regional nerve block.  The patient also received intravenous sedation.  The right arm was prepped and draped in the usual sterile fashion.  We used ultrasound to locate the basilic vein at the cubital fossa.,A small transverse incision was made slightly above the basilic vein.  The basilic vein was identified and immobilized.  The basilic vein was of a good size, but somewhat sclerotic.  The underlying fascia was incised and the brachial artery was identified and immobilized.  The brachial artery was normal.  We then divided the basilic vein distally.  The distal end was ligated using silk suture.  The brachial artery was clamped proximally and distally.  A small longitudinal arteriotomy was made in the brachial artery.  We did not give heparin.  The end of the basilic vein was then sewn end-to-side to the brachial artery using a running 7-0 Prolene suture.  ,Just prior to completion of the anastomosis, it was flushed and anastomosis was completed.  Flow was then established.  A grade 2 was felt in the outflow basilic fistula.  Hemostasis was secured.  The wound was then closed in layers using interrupted PDS sutures for the fascia and a running 4-0 Monocryl subcuticular suture for the skin.  A sterile dry dressing was applied.,The patient tolerated the procedure well.  There were no operative complications.  The sponge, instrument, and needle counts were correct at the end of the case.  I was present and participated in all aspects of the procedure.  The patient was transferred to the recovery room in satisfactory condition.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>surgery, foot, plantar fasciotomy, plantar fascitis, plantar fascia, plantar, fasciotomy, ankle, medially, fascitis, fascia</t>
+          <t xml:space="preserve">surgery, end-stage renal disease, left subclavian vein occlusion, arteriovenous fistula, artery bypass grafting, autologous, basilic vein, brachial artery, brachiobasilic, clamped, fistula, sclerotic, subclavian vein, subclavian vein stenosis, tracheostomy, brachiobasilic arteriovenous fistula, subclavian vein occlusion, vein occlusion, subclavian, basilic, artery, </t>
         </is>
       </c>
       <c r="G47" s="2" t="n">
-        <v>489</v>
+        <v>398</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
@@ -3376,34 +3372,34 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>Surgery; medium; procedure/operative; diagnoses + symptoms + medications</t>
+          <t>Surgery; medium; other narrative/sectioned; lower text complexity; diagnoses + procedures + imaging</t>
         </is>
       </c>
       <c r="J47" s="2" t="n">
-        <v>422</v>
+        <v>1190</v>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>procedure/operative</t>
+          <t>other narrative/sectioned</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>middle</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0.5703899909828674</v>
+        <v>0.3529643823264202</v>
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; procedures; treatment plans; follow-up; surgery</t>
+          <t>diagnoses; procedures; imaging; surgery</t>
         </is>
       </c>
     </row>
     <row r="48" ht="110" customHeight="1">
       <c r="A48" s="2" t="n">
-        <v>768</v>
+        <v>422</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
@@ -3412,39 +3408,39 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Gangrene Surgery </t>
+          <t xml:space="preserve"> Plantar Fasciotomy </t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Gangrene osteomyelitis, right second toe.  The patient is a 58-year-old female with poorly controlled diabetes with severe lower extremity lymphedema.  The patient has history of previous right foot infection requiring first ray resection.</t>
+          <t xml:space="preserve"> Plantar fascitis, left foot.  Partial plantar fasciotomy.</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>PREOPERATIVE DIAGNOSIS: , Gangrene osteomyelitis, right second toe.,POSTOPERATIVE DIAGNOSIS: , Gangrene osteomyelitis, right second toe.,OPERATIVE REPORT:  ,The patient is a 58-year-old female with poorly controlled diabetes with severe lower extremity lymphedema.  The patient has history of previous right foot infection requiring first ray resection.  The patient has ulcerations of right second toe dorsally at the proximal interphalangeal joint, which has failed to respond to conservative treatment.  The patient now has exposed bone and osteomyelitis in the second toe.  The patient has been on IV antibiotics as an outpatient and has failed to respond to these and presents today for surgical intervention.,After an IV was started by the Department of Anesthesia, the patient was taken back to the operating room and placed on the operative table in the supine position.  A restraint belt was placed around the patient's waist using copious amounts of Webril and an ankle pneumatic tourniquet was placed around the patient's right ankle and the patient was made comfortable by the Department of Anesthesia.  After adequate amounts of sedation had been given to the patient, we administered a block of 10 cc of 0.5% Marcaine plain in proximal digital block around the second digit.  The foot and ankle were then prepped in the normal sterile orthopedic manner.  The foot was elevated and an Esmarch bandage applied to exsanguinate the foot.  The tourniquet was then inflated to 250 mmHg and the foot was brought back onto the table.  Using Band-Aid scissors, the stockinet was cut and reflected and using a wet and dry sponge, the foot was wiped, cleaned, and the second toe identified.,Using a skin scrape, a racket type incision was planned around the second toe to allow also remodelling of previous operative site.  Using a fresh #10 blade, skin incision was made circumferentially in the racket-shaped manner around the second digit.  Then, using a fresh #15 blade, the incision was deepened and was taken down to the level of the second metatarsophalangeal joint.  Care was taken to identify bleeders and cautery was used as necessary for hemostasis.  After cleaning up all the soft tissue attachments, the second digit was disarticulated down to the level of the metatarsophalangeal joint.  The head of the second metatarsal was inspected and was noted to have good glistening white cartilage with no areas of erosion evident by visual examination.  Attention was then directed to closure of the wound.  All remaining tissue was noted to be healthy and granular in appearance with no necrotic tissue evident.  Areas of subcutaneous tissue were then removed through a sharp dissection in order to allow better approximation of the skin edges.  Due to long-standing lower extremity lymphedema and postoperative changes on previous surgery, I thought that we were unable to close the incision in entirety.  Therefore, after copious amounts of irrigation using sterile saline, it was determined to use modified dental rolls using #4-0 gauze to remove tension from the skin.  Deep vertical mattress sutures were used in order to reapproximate more closely, the skin edges and bring the plantar flap of skin up to the dorsal skin.  This was obtained using #2-0 nylon suture.  Following this, the remaining exposed tissue from the wound was covered using moist to dry saline soaked 4 x 4 gauze.  The wound was then dressed using 4 x 4 gauze fluffed with abdominal pads, then using Kling and Kerlix and an ACE bandage to provide compression.  The tourniquet was deflated at 42 minutes' time and hemostasis was noted to be achieved.  The ACE bandage was extended up to just below the knee and no bleeding striking to the bandages was appreciated.  The patient tolerated the procedure well and was escorted to the Postanesthesia Care Unit with vital signs stable and vascular status intact, as was evidenced by capillary bleeding, which was present during the procedure.  Sedation was given postoperative introductions, which include to remain nonweightbearing to her right foot.  The patient was instructed to keep the foot elevated and to apply ice behind her knee as necessary, no more than 20 minutes each hour.  The patient was instructed to continue her regular medications.  The patient was to continue IV antibiotic course and was given prescription for Vicoprofen to be taken q.4h. p.r.n. for moderate to severe pain #30.  The patient will followup with Podiatry on Monday morning at 8:30 in the Podiatry Clinic for dressing change and evaluation of her foot at that time.,The patient was instructed as to signs and symptoms of infection, was instructed to return to the Emergency Department immediately if these should present.  The second digit was sent to Pathology for gross and micro.</t>
+          <t>PREOPERATIVE DIAGNOSIS:,  Plantar fascitis, left foot.,POSTOPERATIVE DIAGNOSIS: , Plantar fascitis, left foot.,PROCEDURE PERFORMED: , Partial plantar fasciotomy, left foot.,ANESTHESIA:,  10 cc of 0.5% Marcaine plain with TIVA.,HISTORY:  ,This 35-year-old Caucasian female presents to ABCD General Hospital with above chief complaint.  The patient states she has extreme pain with plantar fascitis in her left foot and has attempted conservative treatment including orthotics without long-term relief of symptoms and desires surgical treatment.  The patient has been NPO since mid night.  Consent is signed and in the chart.  No known drug allergies.,Details Of Procedure:  An IV was instituted by the Department of Anesthesia in the preoperative holding area.  The patient was transported to the operating room and placed on the operating table in supine position with a safety belt across the stomach.  Copious amounts of Webril were placed on the left ankle followed by blood pressure cuff.  After adequate sedation by the Department of Anesthesia, a total of 10 cc of 0.5% Marcaine plain was injected into the surgical site both medially and laterally across the plantar fascia.  The foot was then prepped and draped in the usual sterile orthopedic fashion.  An Esmarch bandage was applied for exsanguination and the pneumatic ankle tourniquet was inflated to 250 mmHg.  The foot was then reflected on the operating, stockinet reflected, and the foot cleansed with a wet and dry sponge.  Attention was then directed to the plantar medial aspect of the left heel.  An approximately 0.75 cm incision was then created in the plantar fat pad over the area of maximal tenderness.,The incision was then deepened with a combination of sharp and blunt dissection until the plantar fascia was palpated.  A #15 blade was then used to transect the medial and central bands of the plantar fascia.  Care was taken to preserve the lateral fibroids.  The foot was dorsiflexed against resistance as the fibers were released and there was noted to be increased laxity after release of the fibers on the plantar aspect of the foot indicating that plantar fascia has in fact been transacted.  The air was then flushed with copious amounts of sterile saline.  The skin incision was then closed with #3-0 nylon in simple interrupted fashion.  Dressings consisted of #0-1 silk, 4 x 4s, Kling, Kerlix, and Coban.  The pneumatic ankle tourniquet was released and immediate hyperemic flush was noted throughout all digits of the left foot.  The patient tolerated the above procedure and anesthesia well without complications.  The patient was transported to the PACU with vital signs stable and vascular status intact to the left foot.  Intraoperatively, an additional 80 cc of 1% lidocaine was injected for additional anesthesia in the case.  The patient is to be nonweightbearing on the left lower extremity with crutches.  The patient is given postoperative pain prescriptions for Vicodin ES, one q3-4h. p.o. p.r.n. for pain as well as Celebrex 200 mg one p.o. b.i.d.  The patient is to follow-up with Dr. X as directed.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>surgery, dorsally, toe, ulcerations, foot infection, ray resection, metatarsophalangeal joint, ace bandage, gangrene osteomyelitis, foot, infection, gangrene, digital,</t>
+          <t>surgery, foot, plantar fasciotomy, plantar fascitis, plantar fascia, plantar, fasciotomy, ankle, medially, fascitis, fascia</t>
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>767</v>
+        <v>489</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Surgery; long; procedure/operative; diagnoses + symptoms + medications</t>
+          <t>Surgery; medium; procedure/operative; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J48" s="2" t="n">
-        <v>768</v>
+        <v>422</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
@@ -3457,17 +3453,17 @@
         </is>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0.6022317403065824</v>
+        <v>0.5703899909828674</v>
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; procedures; past history; treatment plans; follow-up; surgery</t>
+          <t>diagnoses; symptoms; medications; allergies; procedures; treatment plans; follow-up; surgery</t>
         </is>
       </c>
     </row>
     <row r="49" ht="110" customHeight="1">
       <c r="A49" s="2" t="n">
-        <v>113</v>
+        <v>85</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
@@ -3476,43 +3472,43 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Hydrocelectomy. </t>
+          <t xml:space="preserve"> Neurogenic Bladder - Consult </t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Left hydrocelectomy.   This is a 67-year-old male with pain, left scrotum.  He has had an elevated PSA and also has erectile dysfunction.  He comes in now for a left hydrocelectomy.  Physical exam confirmed obvious hydrocele, left scrotum.</t>
+          <t xml:space="preserve"> Neurogenic bladder, in a patient catheterizing himself 3 times a day, changing his catheter 3 times a week</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>PREOPERATIVE DIAGNOSIS: , Left hydrocele.,OPERATION: , Left hydrocelectomy.,POSTOPERATIVE DIAGNOSIS: , Left hydrocele.,ANESTHESIA: , General,INDICATIONS AND STUDIES: , This is a 67-year-old male with pain, left scrotum.  He has had an elevated PSA and also has erectile dysfunction.  He comes in now for a left hydrocelectomy.  Physical exam confirmed obvious hydrocele, left scrotum, approximately 8 cm.  Laboratory data included a hematocrit of 43.5, hemoglobin of 15.0, and white count 4700.  Creatinine 1.3, sodium 141, and potassium 4.0.  Calcium 8.6.  Chest x-ray was unremarkable.  EKG was normal.,PROCEDURE: , The patient was satisfactorily given general anesthesia, prepped and draped in supine position, and left scrotal incision was made, carried down to the tunica vaginalis forming the hydrocele.  This was dissected free from the scrotal wall back to the base of the testicle and then excised back to the spermatic cord.  In the fashion, the hydrocele was excised and fluid drained.,Cord was infiltrated with 5 mL of 0.25% Marcaine.  The edges of the tunica vaginalis adjacent to the spermatic cord were oversewn with interrupted 3-0 Vicryl sutures for hemostasis.  The left testicle was replaced into the left scrotal compartment and affixed to the overlying Dartos fascia with a 3-0 Vicryl suture through the edge of the tunica vaginalis and the overlying Dartos fascia.,The left scrotal incision was closed, first closing the Dartos fascia with interrupted 3-0 Vicryl sutures.  Skin was closed with an interrupted running 4-0 chromic suture.  A sterile dressing was applied.  The patient was sent to the recovery room in good condition, upon awakening from general anesthesia.  Plan is to discharge the patient and see him back in the office in a week or 2 in followup.  Further plans will depend upon how he does.</t>
+          <t>HISTORY OF PRESENT ILLNESS: , The patient presents today as a consultation from Dr. ABC's office regarding the above.  He has history of neurogenic bladder, and on intermittent self-catheterization 3 times a day.  However, June 24, 2008, he was seen in the ER, and with fever, weakness, possible urosepsis.  He had a blood culture, which was positive for Staphylococcus epidermidis, as well as urine culture noted for same bacteria.  He was treated on IV antibiotics, Dr. XYZ also saw the patient.  Discharged home.  Not taking any antibiotics.  Today in the office, the patient denies any dysuria, gross hematuria, fever, chills.  He is catheterizing 3 times a day, changing his catheter weekly.  Does have history of renal transplant, which has been followed by Dr. X and is on chronic steroids.  Renal ultrasound, June 23, 2008, was noted for mild hydronephrosis of renal transplant with fluid in the pericapsular space.  Creatinine, July 7, 2008 was 2.0, BUN 36, and patient tells me this is being followed by Dr. X.  No interval complaints today, no issues with catheterization or any gross hematuria.,IMPRESSION:  ,1.  Neurogenic bladder, in a patient catheterizing himself 3 times a day, changing his catheter 3 times a week, we again reviewed the technique of catheterization, and he has no issues with this.,2.  Recurrent urinary tract infection, in a patient who has been hospitalized twice within the last few months, he is on steroids for renal transplant, which has most likely been overall reducing his immune system.  He is asymptomatic today.  No complaints today.,PLAN:,  Following a detailed discussion with the patient, we elected to proceed with intermittent self-catheterization, changing catheter weekly, and technique has been discussed as above.  Based on the recent culture, we will place him on Keflex nighttime prophylaxis, for the next three months or so.  He will call if any concerns.  Follow up as previously scheduled in September for re-assessment.  All questions answered.  The patient is seen and evaluated by myself.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>urology, hydrocele, erectile dysfunction, spermatic cord, tunica vaginalis, vicryl sutures, dartos fascia, hydrocelectomy, psa, testicle, scrotum, scrotal,</t>
+          <t>urology, neurogenic bladder, catheterizing, catheter, urinary tract infection, self-catheterization, intermittent self catheterization, renal transplant, catheterization,</t>
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>283</v>
+        <v>323</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Urology; short; procedure/operative; diagnoses + symptoms + laboratory values</t>
+          <t>Urology; medium; consultation; middle text complexity; diagnoses + symptoms + laboratory values</t>
         </is>
       </c>
       <c r="J49" s="2" t="n">
-        <v>113</v>
+        <v>85</v>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>procedure/operative</t>
+          <t>consultation</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
@@ -3521,17 +3517,17 @@
         </is>
       </c>
       <c r="M49" s="2" t="n">
-        <v>0.5389990982867449</v>
+        <v>0.4687218214607755</v>
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; laboratory values; procedures; imaging; treatment plans; follow-up; surgery</t>
+          <t>diagnoses; symptoms; laboratory values; procedures; imaging; past history; treatment plans; follow-up; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="50" ht="110" customHeight="1">
       <c r="A50" s="2" t="n">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
@@ -3540,26 +3536,26 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Erectile Dysfunction - Followup </t>
+          <t xml:space="preserve"> Flank Pain - Consult - 1 </t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Some improvement of erectile dysfunction, on low dose of Cialis, with no side effects.  </t>
+          <t xml:space="preserve"> Left flank pain, ureteral stone.</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>HISTORY OF PRESENT ILLNESS: , The patient presents today for followup, history of erectile dysfunction, last visit started on Cialis 10 mg.  He indicates that he has noticed some mild improvement of his symptoms, with no side effect.  On this dose, he is having firm erection, able to penetrate, lasting for about 10 or so minutes.  No chest pain, no nitroglycerin usage, no fever, no chills.  No dysuria, gross hematuria, fever, chills.  Daytime frequency every three hours, nocturia times 0, good stream.  He does have a history of elevated PSA and biopsy June of this year was noted for high grade PIN, mid left biopsy, with two specimens being too small to evaluate.  PSA 11.6.  Dr. X's notes are reviewed.,IMPRESSION:  ,1.  Some improvement of erectile dysfunction, on low dose of Cialis, with no side effects.  The patient has multiple risk factors, but denies using any nitroglycerin or any cardiac issues at this time.  We reviewed options of increasing the medication, versus trying other medications, options of penile prosthesis, Caverject injection use as well as working pump is reviewed.,2.  Elevated PSA in a patient with a recent biopsy showing high-grade PIN, as well as two specimens not being large enough to evaluate.  The patient tells me he has met with his primary care physician and after discussion, he is in consideration of repeating a prostate ultrasound and biopsy.  However, he would like to meet with Dr. X to discuss these prior to biopsy.,PLAN: , Following detailed discussion, the patient wishes to proceed with Cialis 20 mg, samples are provided as well as Levitra 10 mg, may increase this to 20 mg and understand administration of each and contraindication as well as potential side effects are reviewed.  The patient not to use them at the same time.  Will call if any other concern.  In the meantime, he is scheduled to meet with Dr. X, with a prior PSA in consideration of a possible repeating prostate ultrasound and biopsy.  He declined scheduling this at this time.  All questions answered.</t>
+          <t>REASON FOR CONSULTATION: , Left flank pain, ureteral stone.,BRIEF HISTORY: , The patient is a 76-year-old female who was referred to us from Dr. X for left flank pain.  The patient was found to have a left ureteral stone measuring about 1.3 cm in size per the patient's history.  The patient has had pain in the abdomen and across the back for the last four to five days.  The patient has some nausea and vomiting.  The patient wants something done for the stone.  The patient denies any hematuria, dysuria, burning or pain.  The patient denies any fevers.,PAST MEDICAL HISTORY: , Negative.,PAST SURGICAL HISTORY:  ,Years ago she had surgery that she does not recall.,MEDICATIONS: , None.,ALLERGIES: , None.,REVIEW OF SYSTEMS: , Denies any seizure disorder, chest pain, denies any shortness of breath, denies any dysuria, burning or pain, denies any nausea or vomiting at this time.  The patient does have a history of nausea and vomiting, but is doing better.,PHYSICAL EXAMINATION:,VITAL SIGNS:  The patient is afebrile.  Vitals are stable.,HEART:  Regular rate and rhythm.,ABDOMEN:  Soft, left-sided flank pain and left lower abdominal pain.,The rest of the exam is benign.,LABORATORY DATA: , White count of 7.8, hemoglobin 13.8, and platelets 234,000.  The patient's creatinine is 0.92.,ASSESSMENT:,1.  Left flank pain.,2.  Left ureteral stone.,3.  Nausea and vomiting.,PLAN: , Plan for laser lithotripsy tomorrow.  Options such as watchful waiting, laser lithotripsy, and shockwave lithotripsy were discussed.  The patient has a pretty enlarged stone.  Failure of the procedure if the stone is significantly impacted into the ureteral wall was discussed.  The patient understood that the success of the surgery may be or may not be 100%, that she may require shockwave lithotripsy if we are unable to get the entire stone out in one sitting.  The patient understood all the risk, benefits of the procedure and wanted to proceed.  Need for stent was also discussed with the patient.  The patient will be scheduled for surgery tomorrow.  Plan for continuation of the antibiotics, obtain urinalysis and culture, and plan for KUB to evaluate for the exact location of the stone prior to surgery tomorrow.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>urology, improvement of erectile dysfunction, erectile dysfunction, erectile, dysfunction, cialis, psa, biopsy,</t>
+          <t xml:space="preserve">urology, flank pain, ureteral stone, shockwave lithotripsy, shockwave, nausea, vomiting, lithotripsy, ureteral, stone, </t>
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -3568,15 +3564,15 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Urology; medium; follow-up/progress; diagnoses + symptoms + medications</t>
+          <t>Urology; medium; consultation; middle text complexity; diagnoses + symptoms + medications</t>
         </is>
       </c>
       <c r="J50" s="2" t="n">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>follow-up/progress</t>
+          <t>consultation</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
@@ -3585,17 +3581,17 @@
         </is>
       </c>
       <c r="M50" s="2" t="n">
-        <v>0.3959084761045987</v>
+        <v>0.5969341749323716</v>
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; procedures; imaging; past history; treatment plans; follow-up; assessment/plan</t>
+          <t>diagnoses; symptoms; medications; allergies; laboratory values; procedures; past history; treatment plans; surgery; assessment/plan</t>
         </is>
       </c>
     </row>
     <row r="51" ht="110" customHeight="1">
       <c r="A51" s="2" t="n">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
@@ -3604,52 +3600,56 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Elevated PSA - H&amp;P </t>
+          <t xml:space="preserve"> I&amp;D - Penoscrotal Abscess </t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Abnormal serum PSA of 16 ng/ml, dribbling urine, inability to empty bladder, nocturia, urinary hesitancy and slow urine stream.</t>
+          <t xml:space="preserve"> Incision and drainage of the penoscrotal abscess, packing, penile biopsy, cystoscopy, and urethral dilation.</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>CHIEF COMPLAINT:, This 61-year-old male presents today with recent finding of abnormal serum PSA of 16 ng/ml. Associated signs and symptoms: Associated signs and symptoms include dribbling urine, inability to empty bladder, nocturia, urinary hesitancy and urine stream is slow.  Timing (onset/frequency): Onset was 6 months ago. Patient denies fever and chills and denies flank pain.,ALLERGIES: ,Patient admits allergies to adhesive tape resulting in severe rash. Patient denies an allergy to anesthesia.,MEDICATION HISTORY:, Patient is not currently taking any medications.,PAST MEDICAL HISTORY:, Childhood Illnesses: (+) asthma, Cardiovascular Hx: (-) angina, Renal / Urinary Hx: (-) kidney problems.,PAST SURGICAL HISTORY:, Patient admits past surgical history of appendectomy in 1992.,SOCIAL HISTORY:, Patient admits alcohol use, Drinking is described as heavy, Patient denies illegal drug use, Patient denies STD history, Patient denies tobacco use.,FAMILY HISTORY:, Patient admits a family history of gout attacks associated with father.,REVIEW OF SYSTEMS:, Unremarkable with exception of chief complaint.,PHYSICAL EXAM: ,BP Sitting: 120/80 Resp: 20 HR: 72 Temp: 98.6,The patient is a pleasant, 61-year-old male in no apparent distress who looks his given age, is well-developed and nourished with good attention to hygiene and body habitus.,Neck: Neck is normal and symmetrical, without swelling or tenderness. Thyroid is smooth and symmetric with no enlargement, tenderness or masses noted.,Respiratory: Respirations are even without use of accessory muscles and no intercostal retractions noted. Breathing is not labored, diaphragmatic, or abdominal. Lungs clear to auscultation with no rales, rhonchi, wheezes, or rubs noted.,Cardiovascular: Normal S1 and S2 without murmurs, gallop, rubs or clicks.  Peripheral pulses full to palpation, no varicosities, extremities warm with no edema or tenderness.,Gastrointestinal: Abdominal organs, bladder, kidney: No abnormalities, without masses, tenderness, or rigidity. Hernia: absent; no inguinal, femoral, or ventral hernias noted. Liver and/or Spleen: no abnormalities, tenderness, or masses noted. Stool specimen not indicated.,Genitourinary: Anus and perineum: no abnormalities. No fissures, edema, dimples, or tenderness noted.,Scrotum: no abnormalities. No lesions, rash, or sebaceous cyst noted.,Epididymides: no abnormalities, masses, or spermatocele, without enlargement, induration, or tenderness.,Testes: symmetrical; no abnormalities, tenderness, hydrocele, or masses noted.,Urethral Meatus: no abnormalities; no hypospadias, lesions, polyps, or discharge noted.,Penis: no abnormalities; circumcised; no phimosis, Peyronie's, condylomata, or lumps noted.,Prostate: size 60 gr, RT&gt;LT and firm.,Seminal Vesicles: no abnormalities; symmetrical; no tenderness, induration, or nodules noted.,Sphincter tone: no abnormalities; good tone; without hemorrhoids or masses.,Skin/Extremities: Skin is warm and dry with normal turgor and there is no icterus. No skin rash, subcutaneous nodules, lesions or ulcers observed.,Neurological/Psychiatric: Oriented to person, place and time. Mood and affect normal, appropriate to situation, without depression, anxiety, or agitation.,TEST RESULTS:, No tests to report at this time.,IMPRESSION: ,Elevated prostate specific antigen (PSA).,PLAN:, Cystoscopy in the office.,DIAGNOSTIC &amp; LAB ORDERS:, Ordered serum creatinine. Urinalysis and C &amp; S ordered using clean-catch specimen. Ordered free prostate specific antigen (PSA). Ordered ultrasound of prostate.,I have discussed the findings of this follow-up evaluation with the patient. The discussion included a complete verbal explanation of any changes in the examination results, diagnosis and current treatment plan. Discussed the possibility of a TURP surgical procedure; risks, complications, benefits, and alternative measures discussed. There are no activity restrictions . Instructed Ben to avoid caffeinated or alcoholic beverages and excessively spiced foods. Questions answered. If any questions should arise after returning home I have encouraged the patient to feel free to call the office at 327-8850.,PRESCRIPTIONS: , Proscar Dosage: 5 mg tablet Sig: once daily Dispense: 30 Refills: 0 Allow Generic: No,PATIENT INSTRUCTIONS:,  Patient completed benign prostatic hypertrophy questionnaire.</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr"/>
+          <t>PREOPERATIVE DIAGNOSIS: , Penoscrotal abscess.,POSTOPERATIVE DIAGNOSIS:,  Penoscrotal abscess.,OPERATION: , Incision and drainage of the penoscrotal abscess, packing, penile biopsy, cystoscopy, and urethral dilation.,BRIEF HISTORY: , The patient is a 75-year-old male presented with penoscrotal abscess.  Options such as watchful waiting, drainage, and antibiotics were discussed.  Risks of anesthesia, bleeding, infection, pain, MI, DVT, PE, completely the infection turning into necrotizing fascitis, Fournier's gangrene were discussed.  The patient already had significant phimotic changes and disfigurement of the penis.  For further debridement the patient was told that his penis is not going to be viable, he may need a total or partial penectomy now or in the future.  Risks of decreased penile sensation, pain, Foley, other unexpected issues were discussed.  The patient understood all the complications and wanted to proceed with the procedure.,DETAIL OF THE OPERATION:  ,The patient was brought to the OR.  The patient was placed in dorsal lithotomy position.  The patient was prepped and draped in the usual fashion.  Pictures were taken prior to starting the procedure for documentation.  The patient had an open sore on the right side of the penis measuring about 1 cm in size with pouring pus out using blunt dissection.  The penile area was opened up distally to allow the pus to come out.  The dissection around the proximal scrotum was done to make sure there are no other pus pockets.  The corporal body was intact, but the distal part of the corpora was completely eroded and had a fungating mass, which was biopsied and sent for permanent pathology analysis.,Urethra was identified at the distal tip, which was dilated and using 23-French cystoscope cystoscopy was done, which showed some urethral narrowing in the distal part of the urethra.  The rest of the bladder appeared normal.  The prostatic urethra was slightly enlarged.  There are no stones or tumors inside the bladder.  There were moderate trabeculations inside the bladder.  Otherwise, the bladder and the urethra appeared normal.  There was a significantly fungating mass involving the distal part of the urethra almost possibility to have including the fungating wart or fungating squamous cell carcinoma.  Again biopsies were sent for pathology analysis.  Prior to urine irrigation anaerobic aerobic cultures were sent, irrigation with over 2 L of fluid was performed.  After irrigation, packing was done with Kerlix.  The patient was brought to recovery in a stable condition.  Please note that 18-French Foley was kept in place.  Electrocautery was used at the end of the procedure to obtain hemostasis as much as possible, but there was fungating mass with slight bleeding packing was done and tight scrotal Kling was applied.  The patient was brought to Recovery in a stable condition after applying 0.5% Marcaine about 20 mL were injected around for local anesthesia.</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">urology, i&amp;d, penoscrotal, penile biopsy, cystoscopy, urethral dilation, incision and drainage, fungating mass, penoscrotal abscess, abscess, urethral, </t>
+        </is>
+      </c>
       <c r="G51" s="2" t="n">
-        <v>574</v>
+        <v>453</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Urology; long; history and physical; diagnoses + symptoms + medications</t>
+          <t>Urology; medium; procedure/operative; lower text complexity; diagnoses + symptoms + procedures</t>
         </is>
       </c>
       <c r="J51" s="2" t="n">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>history and physical</t>
+          <t>procedure/operative</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>higher</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="M51" s="2" t="n">
-        <v>0.8476104598737602</v>
+        <v>0.3762962128043282</v>
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>diagnoses; symptoms; medications; allergies; vital signs; procedures; imaging; past history; treatment plans; follow-up; surgery; assessment/plan</t>
+          <t>diagnoses; symptoms; procedures; surgery</t>
         </is>
       </c>
     </row>

</xml_diff>